<commit_message>
docs(sim-548): pause the joint fit by owner decision — the fit runs on the final model; the resume order (the pool-window test first) stamped in the plan, the changelog, the backlog and the guide
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -164,21 +164,20 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -567,23 +566,23 @@
   <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11.28515625" customWidth="1" style="18" min="1" max="1"/>
-    <col width="17" bestFit="1" customWidth="1" style="18" min="2" max="2"/>
-    <col width="26.140625" customWidth="1" style="18" min="3" max="3"/>
-    <col width="71.42578125" customWidth="1" style="18" min="4" max="4"/>
-    <col width="70.85546875" customWidth="1" style="18" min="5" max="5"/>
-    <col width="71.42578125" customWidth="1" style="18" min="6" max="6"/>
+    <col width="11.28515625" customWidth="1" style="17" min="1" max="1"/>
+    <col width="17" bestFit="1" customWidth="1" style="17" min="2" max="2"/>
+    <col width="26.140625" customWidth="1" style="17" min="3" max="3"/>
+    <col width="71.42578125" customWidth="1" style="17" min="4" max="4"/>
+    <col width="70.85546875" customWidth="1" style="17" min="5" max="5"/>
+    <col width="71.42578125" customWidth="1" style="17" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20.25" customHeight="1" s="18">
-      <c r="A1" s="15" t="inlineStr">
+    <row r="1" ht="20.25" customHeight="1" s="17">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>MLB Baseball Simulation Platform — Open Ticket Backlog</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>NEXT FREE TICKET ID: SIM-550</t>
         </is>
@@ -605,7 +604,7 @@
           <t>Title</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -621,7 +620,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="405" customHeight="1" s="18">
+    <row r="5" ht="405" customHeight="1" s="17">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>P1</t>
@@ -649,11 +648,11 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>STATUS 2026-09-15 (06:30 UTC): PLAN v2 IN EXECUTION (owner: 'implement your plan'). Built: the skill table, the calibration layer (scripts/sim548_calibrate_markets.py), the offline joint fit for the pitch draws (scripts/sim548_offline_fit.py), the designed-experiment runner (scripts/sim548_design.py); 11 unit tests. First calibration read on held-out 2024 games: the strikeout map (b 0.15) brings the market LEVEL with the line; batter props pass. The offline fit (78 settings) and the pool-totals lane on today's production are running. The Docker VM is now 16 CPU / 19.5 GiB. STATUS 2026-09-15: the 1,000-game baseline of production READ (scripts/sim548_baseline_1000_skill.txt; CHANGES.md 2026-09-15). Worst market: strikeouts (+0.022 Brier behind the line) - but the sim's discrimination now equals the line's (AUC 0.55 vs 0.54); the gap is a 9.5-point low bias and a 3x over-spread = calibration-layer work. The moneyline's gap (+0.011) is a stale win-probability curve in /data/calibration.json that maps raw 0.545-0.618 to 0.500 (owner decision: retire it now or refit on raw probabilities). The run level is real: totals over-predicted by 4.6-5.3 points; the batter excess sits in the weak third of hitters (the batter weight too flat). STATUS 2026-09-14 (evening): the split FLIPPED ON in production by owner decision (16 / 16 / 8; no 2025 hold-out); the 1,000-game accuracy baseline of the flipped production RUNNING (games 251-1000 of 2024 in three chunks, scripts/sim548_baseline_1000.sh; the first 250 = scripts/sim548_accuracy_split.json), done ~04:40 UTC 2026-09-15; the per-market skill table (scripts/sim548_market_skill.py) reads it. STATUS 2026-09-14 (later): plan v2 DRAFTED for the owner's review - docs/audit/2026-09-14-sim548-joint-fit-plan.md (one model; a composite objective over every market; an offline joint fit of every draw's weights; a ~20-arm designed experiment on the full simulator; the 2025 hold-out; a per-market calibration layer; no per-market weight sets). Eight owner decisions listed in its section 9. STATUS 2026-09-14: Part A4 RAN - the pitch / pitch-result split (16 / 16 / 8) as a paired accuracy arm over production with the fatigue weight at 0.5: starter strikeouts -0.0155 Brier [-0.0258, -0.0050] (the gap to the closing line halved; AUC 0.51 -&gt; 0.55, the line 0.58; a 6.5-point LOW bias), the moneyline -0.0050 (AUC 0.49 -&gt; 0.58), batter props flat; one guard worse beyond its range (the first-five total +0.0113, whose baseline row is the outlier of four reports). NEXT: Part C, the 2025 hold-out (a production baseline + a split arm on 250 games of 2025; ~6.5 h); the split flips if the strikeout sign holds and no guard worsens on both seasons. The owner asked whether a one-weight-at-a-time ladder can miss interactions between weights (it can: one concentration budget, both actors on the same outcome, the chain from the pitch draw to the result draw); the answer proposes a return pass, a 3x3 grid on the pitcher / batter pair, and an offline joint fit on real held-out pitches before the full-game confirmations - to be written into the plan on the owner's word. Follow docs/audit/2026-09-14-sim548-accuracy-fit-plan.md. Per weight: (1) the 35-minute probe screen (does it move a market probability at all, and the new discrimination read); (2) a ladder of values, each a 2.5-hour paired arm of scripts/clv_backtest.py on the fixed 250-game 2024 list against the production baseline, read with scripts/sim518_pair_accuracy.py and the new per-market skill table; (3) the choice: the best strikeout-market improvement, the smallest power among ties, every other market not worse; (4) the 2025 hold-out; (5) the flip. First cycle: SIM_PITCH_PITCHER_POWER over 1/2/4/8/16 plus the built pitch/pitch-result split at 16/16/8; if the pitcher score carries no strikeout information at any power, add a results similarity (the pitcher's own strikeout and walk rates against the row pitcher's) as one more draw weight and ladder that. Second cycle: the batter powers on the hit markets. About two days of compute per cycle on the current 6-CPU Docker VM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="94.5" customHeight="1" s="18">
+          <t>STATUS 2026-09-16 (04:42 UTC): PAUSED by owner decision - the fit runs once the model is in its final state; the owner works on other tickets first. The four-factor design on the full simulator stopped at run 3 of 21 (runs 1-2 kept in scripts/sim548_design_20260915/); the offline fit v2 READ (per pitch flat wins, between pitchers sharp wins, per start flat within noise - the design decides); everything committed (5f6a0ef). The resume order is in docs/audit/2026-09-14-sim548-joint-fit-plan.md s11: the pool-window test first (does a ten-season pool cure the sharp draw's starvation; do old rows predict worse at equal similarity; the recency decay is an unfitted weight), then the design on the chosen pool, then the 2025 hold-out, the flip, the calibration layer. Any change to the pool, the bundle, the profiles or the draw code before the resume invalidates the two finished runs (expected). STATUS 2026-09-15 (06:30 UTC): PLAN v2 IN EXECUTION (owner: 'implement your plan'). Built: the skill table, the calibration layer (scripts/sim548_calibrate_markets.py), the offline joint fit for the pitch draws (scripts/sim548_offline_fit.py), the designed-experiment runner (scripts/sim548_design.py); 11 unit tests. First calibration read on held-out 2024 games: the strikeout map (b 0.15) brings the market LEVEL with the line; batter props pass. The offline fit (78 settings) and the pool-totals lane on today's production are running. The Docker VM is now 16 CPU / 19.5 GiB. STATUS 2026-09-15: the 1,000-game baseline of production READ (scripts/sim548_baseline_1000_skill.txt; CHANGES.md 2026-09-15). Worst market: strikeouts (+0.022 Brier behind the line) - but the sim's discrimination now equals the line's (AUC 0.55 vs 0.54); the gap is a 9.5-point low bias and a 3x over-spread = calibration-layer work. The moneyline's gap (+0.011) is a stale win-probability curve in /data/calibration.json that maps raw 0.545-0.618 to 0.500 (owner decision: retire it now or refit on raw probabilities). The run level is real: totals over-predicted by 4.6-5.3 points; the batter excess sits in the weak third of hitters (the batter weight too flat). STATUS 2026-09-14 (evening): the split FLIPPED ON in production by owner decision (16 / 16 / 8; no 2025 hold-out); the 1,000-game accuracy baseline of the flipped production RUNNING (games 251-1000 of 2024 in three chunks, scripts/sim548_baseline_1000.sh; the first 250 = scripts/sim548_accuracy_split.json), done ~04:40 UTC 2026-09-15; the per-market skill table (scripts/sim548_market_skill.py) reads it. STATUS 2026-09-14 (later): plan v2 DRAFTED for the owner's review - docs/audit/2026-09-14-sim548-joint-fit-plan.md (one model; a composite objective over every market; an offline joint fit of every draw's weights; a ~20-arm designed experiment on the full simulator; the 2025 hold-out; a per-market calibration layer; no per-market weight sets). Eight owner decisions listed in its section 9. STATUS 2026-09-14: Part A4 RAN - the pitch / pitch-result split (16 / 16 / 8) as a paired accuracy arm over production with the fatigue weight at 0.5: starter strikeouts -0.0155 Brier [-0.0258, -0.0050] (the gap to the closing line halved; AUC 0.51 -&gt; 0.55, the line 0.58; a 6.5-point LOW bias), the moneyline -0.0050 (AUC 0.49 -&gt; 0.58), batter props flat; one guard worse beyond its range (the first-five total +0.0113, whose baseline row is the outlier of four reports). NEXT: Part C, the 2025 hold-out (a production baseline + a split arm on 250 games of 2025; ~6.5 h); the split flips if the strikeout sign holds and no guard worsens on both seasons. The owner asked whether a one-weight-at-a-time ladder can miss interactions between weights (it can: one concentration budget, both actors on the same outcome, the chain from the pitch draw to the result draw); the answer proposes a return pass, a 3x3 grid on the pitcher / batter pair, and an offline joint fit on real held-out pitches before the full-game confirmations - to be written into the plan on the owner's word. Follow docs/audit/2026-09-14-sim548-accuracy-fit-plan.md. Per weight: (1) the 35-minute probe screen (does it move a market probability at all, and the new discrimination read); (2) a ladder of values, each a 2.5-hour paired arm of scripts/clv_backtest.py on the fixed 250-game 2024 list against the production baseline, read with scripts/sim518_pair_accuracy.py and the new per-market skill table; (3) the choice: the best strikeout-market improvement, the smallest power among ties, every other market not worse; (4) the 2025 hold-out; (5) the flip. First cycle: SIM_PITCH_PITCHER_POWER over 1/2/4/8/16 plus the built pitch/pitch-result split at 16/16/8; if the pitcher score carries no strikeout information at any power, add a results similarity (the pitcher's own strikeout and walk rates against the row pitcher's) as one more draw weight and ladder that. Second cycle: the batter powers on the hit markets. About two days of compute per cycle on the current 6-CPU Docker VM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="94.5" customHeight="1" s="17">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>P1</t>
@@ -685,7 +684,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="81" customHeight="1" s="18">
+    <row r="7" ht="81" customHeight="1" s="17">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>P2</t>
@@ -717,7 +716,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="81" customHeight="1" s="18">
+    <row r="8" ht="81" customHeight="1" s="17">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>x</t>
@@ -749,7 +748,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="94.5" customHeight="1" s="18">
+    <row r="9" ht="94.5" customHeight="1" s="17">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>P2</t>
@@ -781,7 +780,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="229.5" customHeight="1" s="18">
+    <row r="10" ht="229.5" customHeight="1" s="17">
       <c r="A10" s="6" t="inlineStr">
         <is>
           <t>P2</t>
@@ -813,7 +812,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="94.5" customHeight="1" s="18">
+    <row r="11" ht="121.5" customHeight="1" s="17">
       <c r="A11" s="6" t="inlineStr">
         <is>
           <t>P2</t>
@@ -821,164 +820,164 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
+          <t>SIM-549</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Fix the first-five run line in the accuracy comparison: two separate bets, not two sides of one</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>The book lists the first-five run line as two separate bets: 'the home team leads by two or more after five innings' (home -1.5) and 'the away team leads by two or more after five' (away -1.5). Both can lose (a tie or a one-run lead), so both are plus money, and the loader stores them faithfully (game 744796: home -1.5 at +350, away -1.5 at +150). The accuracy comparison (scripts/clv_backtest.py, the segment-market scorer added 2026-09-12) treats the two prices as the two sides of ONE bet and removes the book's margin as if they had to add to one. That inflates the market's probability of 'home covers -1.5' (from about 0.21 to 0.36 on that pair), so the closing line reads as badly calibrated (its mean probability 14 points above the outcome rate) and the simulator reads as beating it by 0.032 of Brier on 250 games of 2024 — an artefact. Every read that uses this market's line (the skill table, the composite objective, the hypothetical return) is wrong for it. The full-game run line is a real two-way pair (home +1.5 / away -1.5) and is scored correctly. Found 2026-09-14 by the overround check in the skill-table read (the two implied probabilities add to 0.76; a two-way pair adds to about 1.05); the owner identified the cause. Until it is fixed the f5_runline row is excluded from every accuracy read.</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>(1) The accuracy comparison scores the first-five run line as TWO records per game — home -1.5 and away -1.5 — each with its own simulator probability from the per-iteration first-five linescore (the lead of two or more), its own outcome from the official inning grid, and its own market probability from its single price with the book's margin removed by the margin of the same game's two-way first-five markets (never by pairing it with the other team's price). (2) A unit test on a real payload holds this: two records, both priced from their own line, a tie graded as a loss for both. (3) The skill table's overround check accepts the market again (or treats one-sided markets by their own rule) and the f5_runline row re-enters the reads. (4) The 2024 baseline's f5_runline rows are re-scored from the stored reports' prices without re-running the simulator. (5) CHANGES.md records the fix.</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>In scripts/clv_backtest.py's segment scorer, give the run-line kind a one-sided branch: when the stored home and away spreads have the same sign, the market is two separate bets. Price each from its own American odds; take the margin from the same game's f5 total and f5 moneyline pairs (the mean overround, about 1.05) and divide the implied probability by it. Emit two AccuracyRecords (side = home / away, line = -1.5). The simulator's probability for each side comes from simulation/game_market_distributions.py's run-line rule applied per side. Add the overround assertion as a per-market log line in the backtest so a future market with the same shape is caught at load, not at read time. Re-score the existing 2024 reports with a small script that rewrites the f5_runline records from the stored prices (no simulation needed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="94.5" customHeight="1" s="17">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
           <t>SIM-451</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Re-check that every play-selection group has enough data</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>The simulator picks each pitch by first grouping similar past pitches into small buckets (based on things like the count and which bases have runners), then drawing an outcome from the most similar bucket. This check re-measures how many real pitches fall into each of the roughly 2,880 buckets, to make sure none is so small that its draw becomes unreliable. It needs to be re-run because the number of buckets is about to double once the new pitch-realism factors go live.</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>The bucket-size check has been re-run on the current data, and the platform has a documented minimum acceptable bucket size based on the results.</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>Re-run the existing bucket-coverage measurement script once the pitch-realism-factor rebuild finishes, and use its results to set the minimum bucket size.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="81" customHeight="1" s="18">
-      <c r="A12" s="6" t="inlineStr">
+    <row r="13" ht="81" customHeight="1" s="17">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>SIM-519</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Build the live, schedule-driven game day view</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>The public-facing screen that lists all of today's games should pull its list directly from Major League Baseball's own public schedule and mark each game as upcoming, in progress, or finished. Right now it pulls its game list only from the platform's own database, which can miss games or show stale information. This is a multi-part project; each part can be finished and checked off on its own.</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>The day view lists every game the league's real schedule shows for that day, with the correct status, sourced live from the league rather than only from the platform's own stored data.</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Build a connection to the league's public schedule feed, use it to drive the list of games shown, and keep layering the platform's simulations, projections, and odds on top of that live list.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="135" customHeight="1" s="18">
-      <c r="A13" s="6" t="inlineStr">
+    <row r="14" ht="135" customHeight="1" s="17">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>SIM-546</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Show the twelve segment and team markets in the API and on the game page</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>The odds tables now hold every game market the book posts, and the backtest prices and grades all of them. But the betting API's edge endpoint and the game page still show only the three full-game markets: the moneyline, the run line and the total. The cause is the simulation cache. It stores each game's score arrays, not its runs by inning. The twelve segment markets settle on the first inning, the first five innings, one team's runs, or which team scored first. Those need the per-inning runs of every simulated game. The pricing code already exists (simulation/game_market_distributions.py); only the cache and the API surface are missing.</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>The simulation cache carries each simulated game's runs by inning. The edge endpoint returns an edge report for every one of the fifteen game markets when odds are supplied or found. The game page's betting card shows them. The existing three markets are unchanged.</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>Extend the cached simulation result with the per-inning run grids (the same light form the backtest workers carry). Build the edge reports for the twelve markets from simulation/game_market_distributions.py: a two-way market through the existing report builder; a three-way market with the three-way de-vig. Add the markets to the edge endpoint's market list and the betting card. Keep the frontend data-driven.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="121.5" customHeight="1" s="18">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="15" ht="67.5" customHeight="1" s="17">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>SIM-549</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Fix the first-five run line in the accuracy comparison: two separate bets, not two sides of one</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>The book lists the first-five run line as two separate bets: 'the home team leads by two or more after five innings' (home -1.5) and 'the away team leads by two or more after five' (away -1.5). Both can lose (a tie or a one-run lead), so both are plus money, and the loader stores them faithfully (game 744796: home -1.5 at +350, away -1.5 at +150). The accuracy comparison (scripts/clv_backtest.py, the segment-market scorer added 2026-09-12) treats the two prices as the two sides of ONE bet and removes the book's margin as if they had to add to one. That inflates the market's probability of 'home covers -1.5' (from about 0.21 to 0.36 on that pair), so the closing line reads as badly calibrated (its mean probability 14 points above the outcome rate) and the simulator reads as beating it by 0.032 of Brier on 250 games of 2024 — an artefact. Every read that uses this market's line (the skill table, the composite objective, the hypothetical return) is wrong for it. The full-game run line is a real two-way pair (home +1.5 / away -1.5) and is scored correctly. Found 2026-09-14 by the overround check in the skill-table read (the two implied probabilities add to 0.76; a two-way pair adds to about 1.05); the owner identified the cause. Until it is fixed the f5_runline row is excluded from every accuracy read.</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>(1) The accuracy comparison scores the first-five run line as TWO records per game — home -1.5 and away -1.5 — each with its own simulator probability from the per-iteration first-five linescore (the lead of two or more), its own outcome from the official inning grid, and its own market probability from its single price with the book's margin removed by the margin of the same game's two-way first-five markets (never by pairing it with the other team's price). (2) A unit test on a real payload holds this: two records, both priced from their own line, a tie graded as a loss for both. (3) The skill table's overround check accepts the market again (or treats one-sided markets by their own rule) and the f5_runline row re-enters the reads. (4) The 2024 baseline's f5_runline rows are re-scored from the stored reports' prices without re-running the simulator. (5) CHANGES.md records the fix.</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>In scripts/clv_backtest.py's segment scorer, give the run-line kind a one-sided branch: when the stored home and away spreads have the same sign, the market is two separate bets. Price each from its own American odds; take the margin from the same game's f5 total and f5 moneyline pairs (the mean overround, about 1.05) and divide the implied probability by it. Emit two AccuracyRecords (side = home / away, line = -1.5). The simulator's probability for each side comes from simulation/game_market_distributions.py's run-line rule applied per side. Add the overround assertion as a per-market log line in the backtest so a future market with the same shape is caught at load, not at read time. Re-score the existing 2024 reports with a small script that rewrites the f5_runline records from the stored prices (no simulation needed).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="67.5" customHeight="1" s="18">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>SIM-526</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Turn on the catcher pitch-receiving factor</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="67.5" customHeight="1" s="17">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>SIM-526</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Turn on the catcher pitch-receiving factor</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="67.5" customHeight="1" s="18">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
           <t>SIM-524</t>
@@ -1005,7 +1004,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="67.5" customHeight="1" s="18">
+    <row r="17" ht="67.5" customHeight="1" s="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1037,7 +1036,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="54" customHeight="1" s="18">
+    <row r="18" ht="54" customHeight="1" s="17">
       <c r="A18" s="7" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1069,7 +1068,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="54" customHeight="1" s="18">
+    <row r="19" ht="54" customHeight="1" s="17">
       <c r="A19" s="7" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1101,7 +1100,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="40.5" customHeight="1" s="18">
+    <row r="20" ht="40.5" customHeight="1" s="17">
       <c r="A20" s="7" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1133,7 +1132,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="67.5" customHeight="1" s="18">
+    <row r="21" ht="67.5" customHeight="1" s="17">
       <c r="A21" s="7" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1165,7 +1164,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="67.5" customHeight="1" s="18">
+    <row r="22" ht="67.5" customHeight="1" s="17">
       <c r="A22" s="7" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1197,7 +1196,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="67.5" customHeight="1" s="18">
+    <row r="23" ht="67.5" customHeight="1" s="17">
       <c r="A23" s="7" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1229,7 +1228,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="67.5" customHeight="1" s="18">
+    <row r="24" ht="67.5" customHeight="1" s="17">
       <c r="A24" s="7" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1261,7 +1260,7 @@
         </is>
       </c>
     </row>
-    <row r="25" s="18">
+    <row r="25" ht="121.5" customHeight="1" s="17">
       <c r="A25" s="7" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1293,10 +1292,10 @@
         </is>
       </c>
     </row>
-    <row r="26" s="18">
-      <c r="D26" s="16" t="n"/>
-    </row>
-    <row r="27" s="18">
+    <row r="26">
+      <c r="D26" s="13" t="n"/>
+    </row>
+    <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>Priority key:</t>
@@ -1312,7 +1311,7 @@
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D27" s="17" t="inlineStr">
+      <c r="D27" s="14" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>

</xml_diff>

<commit_message>
docs(sim-558): close the ticket — the lane on the fixed code (the SIM-559 lane of 2026-10-07) moved no band, the row deleted, the leftovers resolved by SIM-559 or re-homed on SIM-519
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="18" min="1" max="1"/>
@@ -782,35 +782,35 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="243" customHeight="1" s="18">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
+    <row r="10" ht="94.5" customHeight="1" s="18">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SIM-558</t>
+          <t>SIM-443d</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Give every game its real starting pitcher on both sides, and refuse a game with a starter missing</t>
+          <t>Restrict what the SQL query tool can read</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>The simulator found each side's starting pitcher in the lineup table, by the pitcher position code. That table holds one row for each player, with the LAST position he played. Three kinds of game break it. (1) A two-way starter, who pitches and bats as the designated hitter, is coded DH, so his side has no pitcher: 80 team-games of 2017-2026, all one player. (2) A position player who finished a lopsided game on the mound is coded as a pitcher and is picked ahead of the real starter: 308 team-games. (3) An announced starter who was scratched before his first pitch: 9 team-games. Together 392 of the 22,742 Final games (1.7%), and 192 of the 9,457 games of the 2023-2026 pool window. With the home starter missing the game was refused with a 'not found' error (41 games). With the away starter missing (39 games) the game ran: the loop swaps the pitcher at each half inning and, with no away pitcher to swap in, left the home pitcher on the mound against his own team. Game 823372 (2026-06-10), one of the 45 games of the balanced certifying set, is one of the 39: home-team pitchers threw about 40% of the plate appearances to their own batters, the home starter's box line held both teams' outs, and the real away starter had no line and no prop. In the other 317 team-games the simulator ran a position player, or a scratched pitcher, as the starter. Found 2026-10-04 during the design of the pitcher-outs credit (SIM-557). Count, cause and measurement: CHANGES.md, 2026-10-05.</t>
+          <t>The platform includes a tool that lets a user run their own read-only database queries from the website. It only blocks queries that would change data, but does not restrict which parts of the database can be read, so a user could query internal system tables that list other database accounts and their passwords.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>On every Final game of 2017-2026 each side's starter equals the starter the official box score names: scripts/sim558_starter_census.py reads 0 missing and 0 different (before the fix: 80 missing, 317 wrong). The resolver and the game driver both refuse a game with a starter missing on one side, before the first pitch, with a message that names the side. Unit tests pin the three cases, the refusal on both paths, and that each half inning opens with the fielding side's pitcher. The unit lane is green. The code is reviewed, committed and running in the app. The next 45 x 130 acceptance lane runs on the fixed code; the paired read of game 823372 (390 game-sims an arm) predicts that no band changes its verdict: every band total moves by 0.11% or less.</t>
+          <t>The SQL query tool only allows reading from the platform's approved data tables, and requests to read internal system tables are blocked.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>BUILT AND MEASURED 2026-10-05; COMMITTED AND MERGED INTO MASTER 2026-10-06, the app restarted on it. Open: the next 45 x 130 acceptance lane, held by the owner until another fix is in. simulation/lineup_resolver.py: fetch_box_starters reads raw.game_player_stats.p_started; the box's starter replaces the lineup's sequence-1 pitcher row (a recorded pitching change still wins); the starter's throwing hand is fetched when the lineup does not list him; build_game_state refuses a missing pitcher on either side. simulation/sim_loop.py: simulate_game refuses a game that names one side's starter and not the other's (a game with neither id is the fixed matchup of the no-database tests and still plays). tests/unit/test_sim558_starter_resolution.py, 22 tests. The count is scripts/sim558_starter_census.py; the paired read is scripts/sim558_game_probe.py. No data run and no migration. NOT in this ticket: (a) the lineup loader should store each player's STARTING position (allPositions[0] in the box feed), then re-load the lineups; the same last-position coding leaves 26% of team-games with a fielding position missing from the defense map; (b) a game with no box yet (the live slate, SIM-519) needs the schedule's probable pitcher for a two-way starter; (c) scripts/sim523_game_set.py finds starters by the same position code.</t>
+          <t>Add a list of allowed tables to the query tool's safety check, and reject any query that reaches outside that list.</t>
         </is>
       </c>
     </row>
@@ -822,31 +822,31 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SIM-443d</t>
+          <t>SIM-443e</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Restrict what the SQL query tool can read</t>
+          <t>Turn on the read-only database connection for the SQL tool</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>The platform includes a tool that lets a user run their own read-only database queries from the website. It only blocks queries that would change data, but does not restrict which parts of the database can be read, so a user could query internal system tables that list other database accounts and their passwords.</t>
+          <t>The SQL query tool was built to use a separate, limited-permission database connection for safety, but the setting that turns that connection on is currently switched off, so the tool quietly falls back to the full administrator database connection instead.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>The SQL query tool only allows reading from the platform's approved data tables, and requests to read internal system tables are blocked.</t>
+          <t>The SQL query tool is confirmed to be using the limited, read-only database connection rather than the administrator connection.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Add a list of allowed tables to the query tool's safety check, and reject any query that reaches outside that list.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="94.5" customHeight="1" s="18">
+          <t>Turn on and set the read-only connection's configuration value, then confirm the tool uses it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="81" customHeight="1" s="18">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>P3</t>
@@ -854,31 +854,31 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>SIM-443e</t>
+          <t>SIM-443a</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Turn on the read-only database connection for the SQL tool</t>
+          <t>Stop exposing database ports to the network</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>The SQL query tool was built to use a separate, limited-permission database connection for safety, but the setting that turns that connection on is currently switched off, so the tool quietly falls back to the full administrator database connection instead.</t>
+          <t>The main database, the cache, and the application are all currently reachable from any computer on the network, not just the local machine, because their network connections are open to every network instead of limited to the local computer.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>The SQL query tool is confirmed to be using the limited, read-only database connection rather than the administrator connection.</t>
+          <t>The database, cache, and application ports are reachable only from the local machine, and the application still works normally.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Turn on and set the read-only connection's configuration value, then confirm the tool uses it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="81" customHeight="1" s="18">
+          <t>Change each service's network setting in the deployment configuration to bind only to the local machine's own address.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="135" customHeight="1" s="18">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>P3</t>
@@ -886,31 +886,31 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>SIM-443a</t>
+          <t>SIM-443b</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Stop exposing database ports to the network</t>
+          <t>Remove the default database password and admin access</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>The main database, the cache, and the application are all currently reachable from any computer on the network, not just the local machine, because their network connections are open to every network instead of limited to the local computer.</t>
+          <t>The database's password is stored in plain, readable text in a file that is checked into the project's shared code, and the account using it has full administrator-level access rather than only the access it actually needs.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>The database, cache, and application ports are reachable only from the local machine, and the application still works normally.</t>
+          <t>The database password is no longer stored in the shared project files, and the application uses an account with only the specific permissions it needs.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Change each service's network setting in the deployment configuration to bind only to the local machine's own address.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="135" customHeight="1" s="18">
+          <t>Move the password into a secrets manager or environment variable outside the shared code, and create a limited-permission database account for the application.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="67.5" customHeight="1" s="18">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>P3</t>
@@ -918,27 +918,27 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>SIM-443b</t>
+          <t>SIM-443c</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Remove the default database password and admin access</t>
+          <t>Require login on the API</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>The database's password is stored in plain, readable text in a file that is checked into the project's shared code, and the account using it has full administrator-level access rather than only the access it actually needs.</t>
+          <t>The programming interface (API) that the website and other tools use to pull data from the platform currently lets any request through with no login check whenever a certain setting is left unset, which is the default. This means anyone who can reach the server can pull the full pitch-by-pitch dataset with no credentials.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>The database password is no longer stored in the shared project files, and the application uses an account with only the specific permissions it needs.</t>
+          <t>Every route that provides data or triggers work requires a valid login by default, with no setting that silently disables that requirement.</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Move the password into a secrets manager or environment variable outside the shared code, and create a limited-permission database account for the application.</t>
+          <t>Fix the login check so it fails closed (requires login) unless deliberately configured otherwise, and re-test that all data routes are covered.</t>
         </is>
       </c>
     </row>
@@ -950,27 +950,27 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>SIM-443c</t>
+          <t>SIM-443f</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Require login on the API</t>
+          <t>Secure the shared cache (Redis)</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>The programming interface (API) that the website and other tools use to pull data from the platform currently lets any request through with no login check whenever a certain setting is left unset, which is the default. This means anyone who can reach the server can pull the full pitch-by-pitch dataset with no credentials.</t>
+          <t>The platform's shared, fast temporary-storage system (called Redis) is reachable from other computers on the local network with no password, and it stores cached data in a format that can run arbitrary code if it is tampered with. Together, this means someone who can reach the cache could plant tampered data that later runs on the server.</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Every route that provides data or triggers work requires a valid login by default, with no setting that silently disables that requirement.</t>
+          <t>The shared cache requires a password to connect, and it is no longer reachable from the network without one.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Fix the login check so it fails closed (requires login) unless deliberately configured otherwise, and re-test that all data routes are covered.</t>
+          <t>Set a password on the cache and restrict its network access the same way as the other services; consider switching away from a data format that can execute code.</t>
         </is>
       </c>
     </row>
@@ -982,31 +982,31 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>SIM-443f</t>
+          <t>SIM-525</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Secure the shared cache (Redis)</t>
+          <t>Set up scheduled backups</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>The platform's shared, fast temporary-storage system (called Redis) is reachable from other computers on the local network with no password, and it stores cached data in a format that can run arbitrary code if it is tampered with. Together, this means someone who can reach the cache could plant tampered data that later runs on the server.</t>
+          <t>None of the platform's three data stores (the main statistics database, the game-simulation database, and the bundle of pre-computed data the simulator reads at startup) currently have any automatic backup. If any were lost or corrupted, rebuilding them from scratch would take roughly 12 hours of reprocessing.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>The shared cache requires a password to connect, and it is no longer reachable from the network without one.</t>
+          <t>All three data stores back up automatically on a schedule, and a real restore from that backup has been tested successfully at least once.</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Set a password on the cache and restrict its network access the same way as the other services; consider switching away from a data format that can execute code.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="67.5" customHeight="1" s="18">
+          <t>Set up a scheduled backup job for each data store and verify a real restore works before considering this finished.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1" s="18">
       <c r="A17" s="7" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1014,27 +1014,27 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>SIM-525</t>
+          <t>SIM-493</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Set up scheduled backups</t>
+          <t>Break up the oversized simulation-loop file, and run the project-wide code-hygiene refactor</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>None of the platform's three data stores (the main statistics database, the game-simulation database, and the bundle of pre-computed data the simulator reads at startup) currently have any automatic backup. If any were lost or corrupted, rebuilding them from scratch would take roughly 12 hours of reprocessing.</t>
+          <t>The single code file that runs the pitch-by-pitch game simulation has grown very large (3,258 lines) as features were added, which makes it hard to review and maintain safely. The team deliberately postponed this cleanup until the pitch-speed and pitch-realism work settled. On 2026-09-16 the owner widened the ticket to a generalized refactor of the project. Three habits have accumulated. (1) Scripts are named after the ticket that created them, not after what they do: 26 of the 43 scripts carry a SIM-number prefix, and every model change since the fatigue weight is graded with a general tool called sim518_pair_accuracy.py (the paired accuracy comparison), so a reader cannot tell a general tool from a one-off probe. (2) Run outputs sit next to code: scripts/ holds 140 ticket-prefixed files, 114 of them results (JSON, logs, text), 40 of those committed. (3) Five source files are over 2,500 lines each: the profile computor (7,732), the accuracy comparison (3,488), the simulation loop (3,258), the full-pool sampler (3,139) and the artifact builder (2,889). Smaller items: about 2,300 SIM-number tags in code comments across 220 tickets (one tag, SIM-421, has two meanings); the 'does this column exist' probe is written about 20 times across the engines, the calibrator and the league writer; the 45 SIM_* environment flags have no single registry of their defaults and owners.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>All three data stores back up automatically on a schedule, and a real restore from that backup has been tested successfully at least once.</t>
+          <t>The simulator behaves the same before and after, confirmed by the unit and regression lanes and one 45 x 130 acceptance lane on the balanced game set. Every script is named for what it does (the paired accuracy comparison first); the shell wrappers, the plans, the technical docs and CHANGES.md point at the new names. Run outputs live outside scripts/ in a results folder that git ignores; the committed ones are moved to docs/audit/ or deleted. The five files over 2,500 lines are split by responsibility. A ticket tag in a code comment says what the work was, not only its number, or is dropped where the git history already records it. One shared column-probe helper; one registry of the SIM_* flags with each flag's default and owner ticket. Ruff, mypy and CI green.</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Set up a scheduled backup job for each data store and verify a real restore works before considering this finished.</t>
+          <t>Do it in slices, one commit each, every slice behaviour-neutral. (1) Rename the paired accuracy tool to pair_accuracy.py and the other general tools by purpose; move the one-off probes under scripts/probes/. (2) Move the run outputs out of scripts/ and add the ignore rule. (3) Split sim_loop.py by responsibility (the pitch draw, the fielding stage, the runner draws, the manager decisions, the box credit), then the other four large files. (4) The shared helpers: the column probe, the flag registry. (5) The comment tags. Timing: the joint fit (SIM-548) is paused until the model is final; run slice 3 before that fit resumes or after it finishes, never while an arm is running.</t>
         </is>
       </c>
     </row>
@@ -1046,31 +1046,31 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>SIM-493</t>
+          <t>SIM-547</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Break up the oversized simulation-loop file, and run the project-wide code-hygiene refactor</t>
+          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>The single code file that runs the pitch-by-pitch game simulation has grown very large (3,258 lines) as features were added, which makes it hard to review and maintain safely. The team deliberately postponed this cleanup until the pitch-speed and pitch-realism work settled. On 2026-09-16 the owner widened the ticket to a generalized refactor of the project. Three habits have accumulated. (1) Scripts are named after the ticket that created them, not after what they do: 26 of the 43 scripts carry a SIM-number prefix, and every model change since the fatigue weight is graded with a general tool called sim518_pair_accuracy.py (the paired accuracy comparison), so a reader cannot tell a general tool from a one-off probe. (2) Run outputs sit next to code: scripts/ holds 140 ticket-prefixed files, 114 of them results (JSON, logs, text), 40 of those committed. (3) Five source files are over 2,500 lines each: the profile computor (7,732), the accuracy comparison (3,488), the simulation loop (3,258), the full-pool sampler (3,139) and the artifact builder (2,889). Smaller items: about 2,300 SIM-number tags in code comments across 220 tickets (one tag, SIM-421, has two meanings); the 'does this column exist' probe is written about 20 times across the engines, the calibrator and the league writer; the 45 SIM_* environment flags have no single registry of their defaults and owners.</t>
+          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>The simulator behaves the same before and after, confirmed by the unit and regression lanes and one 45 x 130 acceptance lane on the balanced game set. Every script is named for what it does (the paired accuracy comparison first); the shell wrappers, the plans, the technical docs and CHANGES.md point at the new names. Run outputs live outside scripts/ in a results folder that git ignores; the committed ones are moved to docs/audit/ or deleted. The five files over 2,500 lines are split by responsibility. A ticket tag in a code comment says what the work was, not only its number, or is dropped where the git history already records it. One shared column-probe helper; one registry of the SIM_* flags with each flag's default and owner ticket. Ruff, mypy and CI green.</t>
+          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Do it in slices, one commit each, every slice behaviour-neutral. (1) Rename the paired accuracy tool to pair_accuracy.py and the other general tools by purpose; move the one-off probes under scripts/probes/. (2) Move the run outputs out of scripts/ and add the ignore rule. (3) Split sim_loop.py by responsibility (the pitch draw, the fielding stage, the runner draws, the manager decisions, the box credit), then the other four large files. (4) The shared helpers: the column probe, the flag registry. (5) The comment tags. Timing: the joint fit (SIM-548) is paused until the model is final; run slice 3 before that fit resumes or after it finishes, never while an arm is running.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="54" customHeight="1" s="18">
+          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/sim427_manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40.5" customHeight="1" s="18">
       <c r="A19" s="7" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1078,31 +1078,31 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>SIM-547</t>
+          <t>SIM-526</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
+          <t>Turn on the catcher pitch-receiving factor</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
+          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
+          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/sim427_manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="40.5" customHeight="1" s="18">
+          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="229.5" customHeight="1" s="18">
       <c r="A20" s="7" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1110,98 +1110,67 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>SIM-526</t>
+          <t>SIM-556</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Turn on the catcher pitch-receiving factor</t>
+          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
+          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/steal_weight_volume_probe.py with its records (uncommitted, in the worktree pensive-taussig-ec2f7e). Filed P3 by the owner on 2026-10-01.</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
+          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="229.5" customHeight="1" s="18">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>SIM-556</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/steal_weight_volume_probe.py with its records (uncommitted, in the worktree pensive-taussig-ec2f7e). Filed P3 by the owner on 2026-10-01.</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
           <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="300" customHeight="1" s="18">
-      <c r="A22" s="15" t="n"/>
-      <c r="B22" s="15" t="n"/>
-      <c r="C22" s="15" t="n"/>
-      <c r="D22" s="16" t="n"/>
-      <c r="E22" s="15" t="n"/>
-      <c r="F22" s="15" t="n"/>
-    </row>
-    <row r="23" ht="67.5" customHeight="1" s="18">
-      <c r="A23" s="8" t="inlineStr">
+    <row r="21" ht="300" customHeight="1" s="18">
+      <c r="A21" s="15" t="n"/>
+      <c r="B21" s="15" t="n"/>
+      <c r="C21" s="15" t="n"/>
+      <c r="D21" s="16" t="n"/>
+      <c r="E21" s="15" t="n"/>
+      <c r="F21" s="15" t="n"/>
+    </row>
+    <row r="22" ht="67.5" customHeight="1" s="18">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
+      <c r="C22" s="10" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="D22" s="13" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F23" s="12" t="n"/>
-    </row>
+      <c r="F22" s="12" t="n"/>
+    </row>
+    <row r="23" ht="67.5" customHeight="1" s="18"/>
     <row r="24" ht="67.5" customHeight="1" s="18"/>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
docs(sim-546): close the ticket; the backlog row is deleted
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="18" min="1" max="1"/>
@@ -694,59 +694,59 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>SIM-546</t>
+          <t>SIM-524</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Show the twelve segment and team markets in the API and on the game page, and store each live game's closing prices</t>
+          <t>Fix the database lock that blocks nightly data rebuilds</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>The odds tables now hold every game market the book posts, and the backtest prices and grades all of them. But the betting API's edge endpoint and the game page still show only the three full-game markets: the moneyline, the run line and the total. The cause is the simulation cache. It stores each game's score arrays, not its runs by inning. The twelve segment markets settle on the first inning, the first five innings, one team's runs, or which team scored first. Those need the per-inning runs of every simulated game. The pricing code already exists (simulation/game_market_distributions.py); only the cache and the API surface are missing. A second defect, found 2026-09-30 (SIM-555): a live game never gets closing prices. The step that marks a game's closing line (mark_closing_lines and mark_closing_prop_lines in pipeline/live/live_ingestion_pipeline.py, SIM-133 / SIM-340) has no caller in production. It also promotes ONE row per game (LIMIT 1) across every market and every book, which was already wrong for more than one market and is wrong for every game since each book has its own row. So the live edge, line-movement and CLV pages see only current prices, and a game's closing rows exist only after the historical loader backfills them.</t>
+          <t>The main statistics database cannot be safely rewritten while the live application is running, because a background worker system quietly keeps a lock on the database file. The only current way to run a data rebuild is to shut down the whole live application first, which slows down every data-refresh task and adds operational risk.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>The simulation cache carries each simulated game's runs by inning. The edge endpoint returns an edge report for every one of the fifteen game markets when odds are supplied or found. The game page's betting card shows them. The existing three markets are unchanged. Every live game's last price before first pitch is stored as its closing row for every market and every book (and for every player prop and book), by a step that runs in production when the game starts, or by a nightly backfill; a unit test pins one closing row per (market, book).</t>
+          <t>A data rebuild can run successfully while the live application keeps serving requests, with no manual shutdown step required.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Extend the cached simulation result with the per-inning run grids (the same light form the backtest workers carry). Build the edge reports for the twelve markets from simulation/game_market_distributions.py: a two-way market through the existing report builder; a three-way market with the three-way de-vig. Add the markets to the edge endpoint's market list and the betting card. Keep the frontend data-driven. For the closing prices: rewrite the marker to promote the last pre-pitch current row per (market type, book), and per (player, prop market, book) for props, through the load guard's closing-stamp rule; call it from the live cycle when a game turns from Preview to Live. A nightly run of the historical loader's closing pass over the previous day's games is the fallback; it writes the same rows (the odds hash keeps them single).</t>
+          <t>Change how the background worker system starts up so it no longer holds a lock on the database file that blocks rebuild scripts from writing to it.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="81" customHeight="1" s="18">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>SIM-524</t>
+          <t>SIM-443d</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Fix the database lock that blocks nightly data rebuilds</t>
+          <t>Restrict what the SQL query tool can read</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>The main statistics database cannot be safely rewritten while the live application is running, because a background worker system quietly keeps a lock on the database file. The only current way to run a data rebuild is to shut down the whole live application first, which slows down every data-refresh task and adds operational risk.</t>
+          <t>The platform includes a tool that lets a user run their own read-only database queries from the website. It only blocks queries that would change data, but does not restrict which parts of the database can be read, so a user could query internal system tables that list other database accounts and their passwords.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>A data rebuild can run successfully while the live application keeps serving requests, with no manual shutdown step required.</t>
+          <t>The SQL query tool only allows reading from the platform's approved data tables, and requests to read internal system tables are blocked.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Change how the background worker system starts up so it no longer holds a lock on the database file that blocks rebuild scripts from writing to it.</t>
+          <t>Add a list of allowed tables to the query tool's safety check, and reject any query that reaches outside that list.</t>
         </is>
       </c>
     </row>
@@ -758,27 +758,27 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>SIM-443d</t>
+          <t>SIM-443e</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Restrict what the SQL query tool can read</t>
+          <t>Turn on the read-only database connection for the SQL tool</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>The platform includes a tool that lets a user run their own read-only database queries from the website. It only blocks queries that would change data, but does not restrict which parts of the database can be read, so a user could query internal system tables that list other database accounts and their passwords.</t>
+          <t>The SQL query tool was built to use a separate, limited-permission database connection for safety, but the setting that turns that connection on is currently switched off, so the tool quietly falls back to the full administrator database connection instead.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>The SQL query tool only allows reading from the platform's approved data tables, and requests to read internal system tables are blocked.</t>
+          <t>The SQL query tool is confirmed to be using the limited, read-only database connection rather than the administrator connection.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Add a list of allowed tables to the query tool's safety check, and reject any query that reaches outside that list.</t>
+          <t>Turn on and set the read-only connection's configuration value, then confirm the tool uses it.</t>
         </is>
       </c>
     </row>
@@ -790,27 +790,27 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SIM-443e</t>
+          <t>SIM-443a</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Turn on the read-only database connection for the SQL tool</t>
+          <t>Stop exposing database ports to the network</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>The SQL query tool was built to use a separate, limited-permission database connection for safety, but the setting that turns that connection on is currently switched off, so the tool quietly falls back to the full administrator database connection instead.</t>
+          <t>The main database, the cache, and the application are all currently reachable from any computer on the network, not just the local machine, because their network connections are open to every network instead of limited to the local computer.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>The SQL query tool is confirmed to be using the limited, read-only database connection rather than the administrator connection.</t>
+          <t>The database, cache, and application ports are reachable only from the local machine, and the application still works normally.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Turn on and set the read-only connection's configuration value, then confirm the tool uses it.</t>
+          <t>Change each service's network setting in the deployment configuration to bind only to the local machine's own address.</t>
         </is>
       </c>
     </row>
@@ -822,27 +822,27 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SIM-443a</t>
+          <t>SIM-443b</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Stop exposing database ports to the network</t>
+          <t>Remove the default database password and admin access</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>The main database, the cache, and the application are all currently reachable from any computer on the network, not just the local machine, because their network connections are open to every network instead of limited to the local computer.</t>
+          <t>The database's password is stored in plain, readable text in a file that is checked into the project's shared code, and the account using it has full administrator-level access rather than only the access it actually needs.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>The database, cache, and application ports are reachable only from the local machine, and the application still works normally.</t>
+          <t>The database password is no longer stored in the shared project files, and the application uses an account with only the specific permissions it needs.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Change each service's network setting in the deployment configuration to bind only to the local machine's own address.</t>
+          <t>Move the password into a secrets manager or environment variable outside the shared code, and create a limited-permission database account for the application.</t>
         </is>
       </c>
     </row>
@@ -854,27 +854,27 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>SIM-443b</t>
+          <t>SIM-443c</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Remove the default database password and admin access</t>
+          <t>Require login on the API</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>The database's password is stored in plain, readable text in a file that is checked into the project's shared code, and the account using it has full administrator-level access rather than only the access it actually needs.</t>
+          <t>The programming interface (API) that the website and other tools use to pull data from the platform currently lets any request through with no login check whenever a certain setting is left unset, which is the default. This means anyone who can reach the server can pull the full pitch-by-pitch dataset with no credentials.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>The database password is no longer stored in the shared project files, and the application uses an account with only the specific permissions it needs.</t>
+          <t>Every route that provides data or triggers work requires a valid login by default, with no setting that silently disables that requirement.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Move the password into a secrets manager or environment variable outside the shared code, and create a limited-permission database account for the application.</t>
+          <t>Fix the login check so it fails closed (requires login) unless deliberately configured otherwise, and re-test that all data routes are covered.</t>
         </is>
       </c>
     </row>
@@ -886,27 +886,27 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>SIM-443c</t>
+          <t>SIM-443f</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Require login on the API</t>
+          <t>Secure the shared cache (Redis)</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>The programming interface (API) that the website and other tools use to pull data from the platform currently lets any request through with no login check whenever a certain setting is left unset, which is the default. This means anyone who can reach the server can pull the full pitch-by-pitch dataset with no credentials.</t>
+          <t>The platform's shared, fast temporary-storage system (called Redis) is reachable from other computers on the local network with no password, and it stores cached data in a format that can run arbitrary code if it is tampered with. Together, this means someone who can reach the cache could plant tampered data that later runs on the server.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Every route that provides data or triggers work requires a valid login by default, with no setting that silently disables that requirement.</t>
+          <t>The shared cache requires a password to connect, and it is no longer reachable from the network without one.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Fix the login check so it fails closed (requires login) unless deliberately configured otherwise, and re-test that all data routes are covered.</t>
+          <t>Set a password on the cache and restrict its network access the same way as the other services; consider switching away from a data format that can execute code.</t>
         </is>
       </c>
     </row>
@@ -918,27 +918,27 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>SIM-443f</t>
+          <t>SIM-525</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Secure the shared cache (Redis)</t>
+          <t>Set up scheduled backups</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>The platform's shared, fast temporary-storage system (called Redis) is reachable from other computers on the local network with no password, and it stores cached data in a format that can run arbitrary code if it is tampered with. Together, this means someone who can reach the cache could plant tampered data that later runs on the server.</t>
+          <t>None of the platform's three data stores (the main statistics database, the game-simulation database, and the bundle of pre-computed data the simulator reads at startup) currently have any automatic backup. If any were lost or corrupted, rebuilding them from scratch would take roughly 12 hours of reprocessing.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>The shared cache requires a password to connect, and it is no longer reachable from the network without one.</t>
+          <t>All three data stores back up automatically on a schedule, and a real restore from that backup has been tested successfully at least once.</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Set a password on the cache and restrict its network access the same way as the other services; consider switching away from a data format that can execute code.</t>
+          <t>Set up a scheduled backup job for each data store and verify a real restore works before considering this finished.</t>
         </is>
       </c>
     </row>
@@ -950,27 +950,27 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>SIM-525</t>
+          <t>SIM-493</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Set up scheduled backups</t>
+          <t>Break up the oversized simulation-loop file, and run the project-wide code-hygiene refactor</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>None of the platform's three data stores (the main statistics database, the game-simulation database, and the bundle of pre-computed data the simulator reads at startup) currently have any automatic backup. If any were lost or corrupted, rebuilding them from scratch would take roughly 12 hours of reprocessing.</t>
+          <t>The single code file that runs the pitch-by-pitch game simulation has grown very large (3,258 lines) as features were added, which makes it hard to review and maintain safely. The team deliberately postponed this cleanup until the pitch-speed and pitch-realism work settled. On 2026-09-16 the owner widened the ticket to a generalized refactor of the project. Three habits have accumulated. (1) Scripts are named after the ticket that created them, not after what they do: 26 of the 43 scripts carry a SIM-number prefix, and every model change since the fatigue weight is graded with a general tool called sim518_pair_accuracy.py (the paired accuracy comparison), so a reader cannot tell a general tool from a one-off probe. (2) Run outputs sit next to code: scripts/ holds 140 ticket-prefixed files, 114 of them results (JSON, logs, text), 40 of those committed. (3) Five source files are over 2,500 lines each: the profile computor (7,732), the accuracy comparison (3,488), the simulation loop (3,258), the full-pool sampler (3,139) and the artifact builder (2,889). Smaller items: about 2,300 SIM-number tags in code comments across 220 tickets (one tag, SIM-421, has two meanings); the 'does this column exist' probe is written about 20 times across the engines, the calibrator and the league writer; the 45 SIM_* environment flags have no single registry of their defaults and owners.</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>All three data stores back up automatically on a schedule, and a real restore from that backup has been tested successfully at least once.</t>
+          <t>The simulator behaves the same before and after, confirmed by the unit and regression lanes and one 45 x 130 acceptance lane on the balanced game set. Every script is named for what it does (the paired accuracy comparison first); the shell wrappers, the plans, the technical docs and CHANGES.md point at the new names. Run outputs live outside scripts/ in a results folder that git ignores; the committed ones are moved to docs/audit/ or deleted. The five files over 2,500 lines are split by responsibility. A ticket tag in a code comment says what the work was, not only its number, or is dropped where the git history already records it. One shared column-probe helper; one registry of the SIM_* flags with each flag's default and owner ticket. Ruff, mypy and CI green.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Set up a scheduled backup job for each data store and verify a real restore works before considering this finished.</t>
+          <t>Do it in slices, one commit each, every slice behaviour-neutral. (1) Rename the paired accuracy tool to pair_accuracy.py and the other general tools by purpose; move the one-off probes under scripts/probes/. (2) Move the run outputs out of scripts/ and add the ignore rule. (3) Split sim_loop.py by responsibility (the pitch draw, the fielding stage, the runner draws, the manager decisions, the box credit), then the other four large files. (4) The shared helpers: the column probe, the flag registry. (5) The comment tags. Timing: the joint fit (SIM-548) is paused until the model is final; run slice 3 before that fit resumes or after it finishes, never while an arm is running.</t>
         </is>
       </c>
     </row>
@@ -982,27 +982,27 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>SIM-493</t>
+          <t>SIM-547</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Break up the oversized simulation-loop file, and run the project-wide code-hygiene refactor</t>
+          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>The single code file that runs the pitch-by-pitch game simulation has grown very large (3,258 lines) as features were added, which makes it hard to review and maintain safely. The team deliberately postponed this cleanup until the pitch-speed and pitch-realism work settled. On 2026-09-16 the owner widened the ticket to a generalized refactor of the project. Three habits have accumulated. (1) Scripts are named after the ticket that created them, not after what they do: 26 of the 43 scripts carry a SIM-number prefix, and every model change since the fatigue weight is graded with a general tool called sim518_pair_accuracy.py (the paired accuracy comparison), so a reader cannot tell a general tool from a one-off probe. (2) Run outputs sit next to code: scripts/ holds 140 ticket-prefixed files, 114 of them results (JSON, logs, text), 40 of those committed. (3) Five source files are over 2,500 lines each: the profile computor (7,732), the accuracy comparison (3,488), the simulation loop (3,258), the full-pool sampler (3,139) and the artifact builder (2,889). Smaller items: about 2,300 SIM-number tags in code comments across 220 tickets (one tag, SIM-421, has two meanings); the 'does this column exist' probe is written about 20 times across the engines, the calibrator and the league writer; the 45 SIM_* environment flags have no single registry of their defaults and owners.</t>
+          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>The simulator behaves the same before and after, confirmed by the unit and regression lanes and one 45 x 130 acceptance lane on the balanced game set. Every script is named for what it does (the paired accuracy comparison first); the shell wrappers, the plans, the technical docs and CHANGES.md point at the new names. Run outputs live outside scripts/ in a results folder that git ignores; the committed ones are moved to docs/audit/ or deleted. The five files over 2,500 lines are split by responsibility. A ticket tag in a code comment says what the work was, not only its number, or is dropped where the git history already records it. One shared column-probe helper; one registry of the SIM_* flags with each flag's default and owner ticket. Ruff, mypy and CI green.</t>
+          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Do it in slices, one commit each, every slice behaviour-neutral. (1) Rename the paired accuracy tool to pair_accuracy.py and the other general tools by purpose; move the one-off probes under scripts/probes/. (2) Move the run outputs out of scripts/ and add the ignore rule. (3) Split sim_loop.py by responsibility (the pitch draw, the fielding stage, the runner draws, the manager decisions, the box credit), then the other four large files. (4) The shared helpers: the column probe, the flag registry. (5) The comment tags. Timing: the joint fit (SIM-548) is paused until the model is final; run slice 3 before that fit resumes or after it finishes, never while an arm is running.</t>
+          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/sim427_manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
         </is>
       </c>
     </row>
@@ -1014,27 +1014,27 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>SIM-547</t>
+          <t>SIM-526</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
+          <t>Turn on the catcher pitch-receiving factor</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
+          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
+          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/sim427_manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
+          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
         </is>
       </c>
     </row>
@@ -1046,98 +1046,67 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>SIM-526</t>
+          <t>SIM-556</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Turn on the catcher pitch-receiving factor</t>
+          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
+          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/steal_weight_volume_probe.py with its records (uncommitted, in the worktree pensive-taussig-ec2f7e). Filed P3 by the owner on 2026-10-01.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
+          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
+          <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="229.5" customHeight="1" s="18">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>SIM-556</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/steal_weight_volume_probe.py with its records (uncommitted, in the worktree pensive-taussig-ec2f7e). Filed P3 by the owner on 2026-10-01.</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
-        </is>
-      </c>
+      <c r="A19" s="15" t="n"/>
+      <c r="B19" s="15" t="n"/>
+      <c r="C19" s="15" t="n"/>
+      <c r="D19" s="16" t="n"/>
+      <c r="E19" s="15" t="n"/>
+      <c r="F19" s="15" t="n"/>
     </row>
     <row r="20" ht="300" customHeight="1" s="18">
-      <c r="A20" s="15" t="n"/>
-      <c r="B20" s="15" t="n"/>
-      <c r="C20" s="15" t="n"/>
-      <c r="D20" s="16" t="n"/>
-      <c r="E20" s="15" t="n"/>
-      <c r="F20" s="15" t="n"/>
-    </row>
-    <row r="21" ht="67.5" customHeight="1" s="18">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="D20" s="13" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F21" s="12" t="n"/>
-    </row>
+      <c r="F20" s="12" t="n"/>
+    </row>
+    <row r="21" ht="67.5" customHeight="1" s="18"/>
     <row r="22" s="18"/>
     <row r="23" ht="67.5" customHeight="1" s="18"/>
     <row r="24" ht="67.5" customHeight="1" s="18"/>

</xml_diff>

<commit_message>
fix(sim-kwargs): read the park factors into memory and close the DuckDB file (SIM-524)
The app held one read-only handle on /data/baseball_sim.duckdb for its whole
life: the park-factor connection in the uvicorn server process. A DuckDB
writer needs the file free of every other process, so every rebuild needed
the app stopped. The prime now reads the run factors into a dict and closes
the file; a lookup re-reads them when the file's mtime changes (at most once
a minute) and keeps the old snapshot while a rebuild holds the lock.

The nightly profile + bundle rebuild job is turned on (08:00 UTC). The
remaining gaps (data reaches users at the next restart; a boot during a
rebuild) are filed as SIM-563.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -585,7 +585,7 @@
     <row r="2" s="18">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>NEXT FREE TICKET ID: SIM-563</t>
+          <t>NEXT FREE TICKET ID: SIM-564</t>
         </is>
       </c>
     </row>
@@ -695,27 +695,27 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>SIM-524</t>
+          <t>SIM-563</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Fix the database lock that blocks nightly data rebuilds</t>
+          <t>Get the nightly rebuild to the running app safely, without a manual restart</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>The main statistics database cannot be safely rewritten while the live application is running, because a background worker system quietly keeps a lock on the database file. The only current way to run a data rebuild is to shut down the whole live application first, which slows down every data-refresh task and adds operational risk.</t>
+          <t>Since the database-lock fix (SIM-524, 2026-10-10) the nightly rebuild runs while the app serves. Three gaps remain. (1) The app loads the player profiles and the simulation data bundle once, at start-up, so a rebuild reaches users only when someone restarts the app; only the park factors refresh on their own. (2) If the app starts, or reloads after a code edit, while a rebuild is writing, the start-up cannot read the database and some similarity engines fail to load. (3) A simulation worker that restarts during a rebuild silently runs without the intentional-walk rates, and could read a half-written data bundle.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>A data rebuild can run successfully while the live application keeps serving requests, with no manual shutdown step required.</t>
+          <t>After the 08:00 UTC rebuild finishes, the app serves the new data the same morning with no person involved, and no start-up, reload or worker restart during a rebuild runs on missing or half-written data.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Change how the background worker system starts up so it no longer holds a lock on the database file that blocks rebuild scripts from writing to it.</t>
+          <t>Have the nightly job signal the app when it finishes (for example a marker file the app watches, or a scheduler job that restarts the app after the rebuild). Make the boot-time engine builds wait and retry while a writer holds the lock. Have the parent process load the intentional-walk rates once and hand them to the workers, and write the bundle to a new folder that is swapped in only when complete.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(bundle): prune the folders of builds that died before publishing; record SIM-563
The live run's two segfaulted attempts left their staged folders, and pruning
counted them as kept versions. publish_bundle_version now writes .published;
prune deletes an unpublished folder older than the current version and keeps a
newer one (a build in progress). CHANGES.md records the run; the backlog row
is deleted.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="18" min="1" max="1"/>
@@ -688,34 +688,34 @@
       </c>
     </row>
     <row r="7" ht="81" customHeight="1" s="18">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>SIM-563</t>
+          <t>SIM-443d</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Get the nightly rebuild to the running app safely, without a manual restart</t>
+          <t>Restrict what the SQL query tool can read</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Since the database-lock fix (SIM-524, 2026-10-10) the nightly rebuild runs while the app serves. Three gaps remain. (1) The app loads the player profiles and the simulation data bundle once, at start-up, so a rebuild reaches users only when someone restarts the app; only the park factors refresh on their own. (2) If the app starts, or reloads after a code edit, while a rebuild is writing, the start-up cannot read the database and some similarity engines fail to load. (3) A simulation worker that restarts during a rebuild silently runs without the intentional-walk rates, and could read a half-written data bundle.</t>
+          <t>The platform includes a tool that lets a user run their own read-only database queries from the website. It only blocks queries that would change data, but does not restrict which parts of the database can be read, so a user could query internal system tables that list other database accounts and their passwords.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>After the 08:00 UTC rebuild finishes, the app serves the new data the same morning with no person involved, and no start-up, reload or worker restart during a rebuild runs on missing or half-written data.</t>
+          <t>The SQL query tool only allows reading from the platform's approved data tables, and requests to read internal system tables are blocked.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Have the nightly job signal the app when it finishes (for example a marker file the app watches, or a scheduler job that restarts the app after the rebuild). Make the boot-time engine builds wait and retry while a writer holds the lock. Have the parent process load the intentional-walk rates once and hand them to the workers, and write the bundle to a new folder that is swapped in only when complete.</t>
+          <t>Add a list of allowed tables to the query tool's safety check, and reject any query that reaches outside that list.</t>
         </is>
       </c>
     </row>
@@ -727,27 +727,27 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>SIM-443d</t>
+          <t>SIM-443e</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Restrict what the SQL query tool can read</t>
+          <t>Turn on the read-only database connection for the SQL tool</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>The platform includes a tool that lets a user run their own read-only database queries from the website. It only blocks queries that would change data, but does not restrict which parts of the database can be read, so a user could query internal system tables that list other database accounts and their passwords.</t>
+          <t>The SQL query tool was built to use a separate, limited-permission database connection for safety, but the setting that turns that connection on is currently switched off, so the tool quietly falls back to the full administrator database connection instead.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>The SQL query tool only allows reading from the platform's approved data tables, and requests to read internal system tables are blocked.</t>
+          <t>The SQL query tool is confirmed to be using the limited, read-only database connection rather than the administrator connection.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Add a list of allowed tables to the query tool's safety check, and reject any query that reaches outside that list.</t>
+          <t>Turn on and set the read-only connection's configuration value, then confirm the tool uses it.</t>
         </is>
       </c>
     </row>
@@ -759,27 +759,27 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>SIM-443e</t>
+          <t>SIM-443a</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Turn on the read-only database connection for the SQL tool</t>
+          <t>Stop exposing database ports to the network</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>The SQL query tool was built to use a separate, limited-permission database connection for safety, but the setting that turns that connection on is currently switched off, so the tool quietly falls back to the full administrator database connection instead.</t>
+          <t>The main database, the cache, and the application are all currently reachable from any computer on the network, not just the local machine, because their network connections are open to every network instead of limited to the local computer.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>The SQL query tool is confirmed to be using the limited, read-only database connection rather than the administrator connection.</t>
+          <t>The database, cache, and application ports are reachable only from the local machine, and the application still works normally.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Turn on and set the read-only connection's configuration value, then confirm the tool uses it.</t>
+          <t>Change each service's network setting in the deployment configuration to bind only to the local machine's own address.</t>
         </is>
       </c>
     </row>
@@ -791,27 +791,27 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SIM-443a</t>
+          <t>SIM-443b</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Stop exposing database ports to the network</t>
+          <t>Remove the default database password and admin access</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>The main database, the cache, and the application are all currently reachable from any computer on the network, not just the local machine, because their network connections are open to every network instead of limited to the local computer.</t>
+          <t>The database's password is stored in plain, readable text in a file that is checked into the project's shared code, and the account using it has full administrator-level access rather than only the access it actually needs.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>The database, cache, and application ports are reachable only from the local machine, and the application still works normally.</t>
+          <t>The database password is no longer stored in the shared project files, and the application uses an account with only the specific permissions it needs.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Change each service's network setting in the deployment configuration to bind only to the local machine's own address.</t>
+          <t>Move the password into a secrets manager or environment variable outside the shared code, and create a limited-permission database account for the application.</t>
         </is>
       </c>
     </row>
@@ -823,27 +823,27 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SIM-443b</t>
+          <t>SIM-443c</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Remove the default database password and admin access</t>
+          <t>Require login on the API</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>The database's password is stored in plain, readable text in a file that is checked into the project's shared code, and the account using it has full administrator-level access rather than only the access it actually needs.</t>
+          <t>The programming interface (API) that the website and other tools use to pull data from the platform currently lets any request through with no login check whenever a certain setting is left unset, which is the default. This means anyone who can reach the server can pull the full pitch-by-pitch dataset with no credentials.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>The database password is no longer stored in the shared project files, and the application uses an account with only the specific permissions it needs.</t>
+          <t>Every route that provides data or triggers work requires a valid login by default, with no setting that silently disables that requirement.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Move the password into a secrets manager or environment variable outside the shared code, and create a limited-permission database account for the application.</t>
+          <t>Fix the login check so it fails closed (requires login) unless deliberately configured otherwise, and re-test that all data routes are covered.</t>
         </is>
       </c>
     </row>
@@ -855,27 +855,27 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>SIM-443c</t>
+          <t>SIM-443f</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Require login on the API</t>
+          <t>Secure the shared cache (Redis)</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>The programming interface (API) that the website and other tools use to pull data from the platform currently lets any request through with no login check whenever a certain setting is left unset, which is the default. This means anyone who can reach the server can pull the full pitch-by-pitch dataset with no credentials.</t>
+          <t>The platform's shared, fast temporary-storage system (called Redis) is reachable from other computers on the local network with no password, and it stores cached data in a format that can run arbitrary code if it is tampered with. Together, this means someone who can reach the cache could plant tampered data that later runs on the server.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Every route that provides data or triggers work requires a valid login by default, with no setting that silently disables that requirement.</t>
+          <t>The shared cache requires a password to connect, and it is no longer reachable from the network without one.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Fix the login check so it fails closed (requires login) unless deliberately configured otherwise, and re-test that all data routes are covered.</t>
+          <t>Set a password on the cache and restrict its network access the same way as the other services; consider switching away from a data format that can execute code.</t>
         </is>
       </c>
     </row>
@@ -887,27 +887,27 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>SIM-443f</t>
+          <t>SIM-525</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Secure the shared cache (Redis)</t>
+          <t>Set up scheduled backups</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>The platform's shared, fast temporary-storage system (called Redis) is reachable from other computers on the local network with no password, and it stores cached data in a format that can run arbitrary code if it is tampered with. Together, this means someone who can reach the cache could plant tampered data that later runs on the server.</t>
+          <t>None of the platform's three data stores (the main statistics database, the game-simulation database, and the bundle of pre-computed data the simulator reads at startup) currently have any automatic backup. If any were lost or corrupted, rebuilding them from scratch would take roughly 12 hours of reprocessing.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>The shared cache requires a password to connect, and it is no longer reachable from the network without one.</t>
+          <t>All three data stores back up automatically on a schedule, and a real restore from that backup has been tested successfully at least once.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Set a password on the cache and restrict its network access the same way as the other services; consider switching away from a data format that can execute code.</t>
+          <t>Set up a scheduled backup job for each data store and verify a real restore works before considering this finished.</t>
         </is>
       </c>
     </row>
@@ -919,27 +919,27 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>SIM-525</t>
+          <t>SIM-493</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Set up scheduled backups</t>
+          <t>Break up the oversized simulation-loop file, and run the project-wide code-hygiene refactor</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>None of the platform's three data stores (the main statistics database, the game-simulation database, and the bundle of pre-computed data the simulator reads at startup) currently have any automatic backup. If any were lost or corrupted, rebuilding them from scratch would take roughly 12 hours of reprocessing.</t>
+          <t>The single code file that runs the pitch-by-pitch game simulation has grown very large (3,258 lines) as features were added, which makes it hard to review and maintain safely. The team deliberately postponed this cleanup until the pitch-speed and pitch-realism work settled. On 2026-09-16 the owner widened the ticket to a generalized refactor of the project. Three habits have accumulated. (1) Scripts are named after the ticket that created them, not after what they do: 26 of the 43 scripts carry a SIM-number prefix, and every model change since the fatigue weight is graded with a general tool called sim518_pair_accuracy.py (the paired accuracy comparison), so a reader cannot tell a general tool from a one-off probe. (2) Run outputs sit next to code: scripts/ holds 140 ticket-prefixed files, 114 of them results (JSON, logs, text), 40 of those committed. (3) Five source files are over 2,500 lines each: the profile computor (7,732), the accuracy comparison (3,488), the simulation loop (3,258), the full-pool sampler (3,139) and the artifact builder (2,889). Smaller items: about 2,300 SIM-number tags in code comments across 220 tickets (one tag, SIM-421, has two meanings); the 'does this column exist' probe is written about 20 times across the engines, the calibrator and the league writer; the 45 SIM_* environment flags have no single registry of their defaults and owners.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>All three data stores back up automatically on a schedule, and a real restore from that backup has been tested successfully at least once.</t>
+          <t>The simulator behaves the same before and after, confirmed by the unit and regression lanes and one 45 x 130 acceptance lane on the balanced game set. Every script is named for what it does (the paired accuracy comparison first); the shell wrappers, the plans, the technical docs and CHANGES.md point at the new names. Run outputs live outside scripts/ in a results folder that git ignores; the committed ones are moved to docs/audit/ or deleted. The five files over 2,500 lines are split by responsibility. A ticket tag in a code comment says what the work was, not only its number, or is dropped where the git history already records it. One shared column-probe helper; one registry of the SIM_* flags with each flag's default and owner ticket. Ruff, mypy and CI green.</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Set up a scheduled backup job for each data store and verify a real restore works before considering this finished.</t>
+          <t>Do it in slices, one commit each, every slice behaviour-neutral. (1) Rename the paired accuracy tool to pair_accuracy.py and the other general tools by purpose; move the one-off probes under scripts/probes/. (2) Move the run outputs out of scripts/ and add the ignore rule. (3) Split sim_loop.py by responsibility (the pitch draw, the fielding stage, the runner draws, the manager decisions, the box credit), then the other four large files. (4) The shared helpers: the column probe, the flag registry. (5) The comment tags. Timing: the joint fit (SIM-548) is paused until the model is final; run slice 3 before that fit resumes or after it finishes, never while an arm is running.</t>
         </is>
       </c>
     </row>
@@ -951,27 +951,27 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>SIM-493</t>
+          <t>SIM-547</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Break up the oversized simulation-loop file, and run the project-wide code-hygiene refactor</t>
+          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>The single code file that runs the pitch-by-pitch game simulation has grown very large (3,258 lines) as features were added, which makes it hard to review and maintain safely. The team deliberately postponed this cleanup until the pitch-speed and pitch-realism work settled. On 2026-09-16 the owner widened the ticket to a generalized refactor of the project. Three habits have accumulated. (1) Scripts are named after the ticket that created them, not after what they do: 26 of the 43 scripts carry a SIM-number prefix, and every model change since the fatigue weight is graded with a general tool called sim518_pair_accuracy.py (the paired accuracy comparison), so a reader cannot tell a general tool from a one-off probe. (2) Run outputs sit next to code: scripts/ holds 140 ticket-prefixed files, 114 of them results (JSON, logs, text), 40 of those committed. (3) Five source files are over 2,500 lines each: the profile computor (7,732), the accuracy comparison (3,488), the simulation loop (3,258), the full-pool sampler (3,139) and the artifact builder (2,889). Smaller items: about 2,300 SIM-number tags in code comments across 220 tickets (one tag, SIM-421, has two meanings); the 'does this column exist' probe is written about 20 times across the engines, the calibrator and the league writer; the 45 SIM_* environment flags have no single registry of their defaults and owners.</t>
+          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>The simulator behaves the same before and after, confirmed by the unit and regression lanes and one 45 x 130 acceptance lane on the balanced game set. Every script is named for what it does (the paired accuracy comparison first); the shell wrappers, the plans, the technical docs and CHANGES.md point at the new names. Run outputs live outside scripts/ in a results folder that git ignores; the committed ones are moved to docs/audit/ or deleted. The five files over 2,500 lines are split by responsibility. A ticket tag in a code comment says what the work was, not only its number, or is dropped where the git history already records it. One shared column-probe helper; one registry of the SIM_* flags with each flag's default and owner ticket. Ruff, mypy and CI green.</t>
+          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Do it in slices, one commit each, every slice behaviour-neutral. (1) Rename the paired accuracy tool to pair_accuracy.py and the other general tools by purpose; move the one-off probes under scripts/probes/. (2) Move the run outputs out of scripts/ and add the ignore rule. (3) Split sim_loop.py by responsibility (the pitch draw, the fielding stage, the runner draws, the manager decisions, the box credit), then the other four large files. (4) The shared helpers: the column probe, the flag registry. (5) The comment tags. Timing: the joint fit (SIM-548) is paused until the model is final; run slice 3 before that fit resumes or after it finishes, never while an arm is running.</t>
+          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/sim427_manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
         </is>
       </c>
     </row>
@@ -983,27 +983,27 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>SIM-547</t>
+          <t>SIM-526</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
+          <t>Turn on the catcher pitch-receiving factor</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
+          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
+          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/sim427_manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
+          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
         </is>
       </c>
     </row>
@@ -1015,98 +1015,67 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>SIM-526</t>
+          <t>SIM-556</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Turn on the catcher pitch-receiving factor</t>
+          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
+          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/steal_weight_volume_probe.py with its records (uncommitted, in the worktree pensive-taussig-ec2f7e). Filed P3 by the owner on 2026-10-01.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
+          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
+          <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="40.5" customHeight="1" s="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>SIM-556</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/steal_weight_volume_probe.py with its records (uncommitted, in the worktree pensive-taussig-ec2f7e). Filed P3 by the owner on 2026-10-01.</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
-        </is>
-      </c>
+      <c r="A18" s="15" t="n"/>
+      <c r="B18" s="15" t="n"/>
+      <c r="C18" s="15" t="n"/>
+      <c r="D18" s="16" t="n"/>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="15" t="n"/>
     </row>
     <row r="19" ht="229.5" customHeight="1" s="18">
-      <c r="A19" s="15" t="n"/>
-      <c r="B19" s="15" t="n"/>
-      <c r="C19" s="15" t="n"/>
-      <c r="D19" s="16" t="n"/>
-      <c r="E19" s="15" t="n"/>
-      <c r="F19" s="15" t="n"/>
-    </row>
-    <row r="20" ht="300" customHeight="1" s="18">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="D19" s="13" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F20" s="12" t="n"/>
-    </row>
+      <c r="F19" s="12" t="n"/>
+    </row>
+    <row r="20" ht="300" customHeight="1" s="18"/>
     <row r="21" ht="67.5" customHeight="1" s="18"/>
     <row r="22" s="18"/>
     <row r="23" ht="67.5" customHeight="1" s="18"/>

</xml_diff>

<commit_message>
docs: the live game-day view passes its live check and closes (SIM-519)
The started-game lineup fixes were deployed and checked on a game in
progress (849820): the lineup written from the feed, a what-if from the
latest play and a run of 100 all finished. The backlog row is deleted.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="18" min="1" max="1"/>
@@ -655,36 +655,34 @@
       </c>
     </row>
     <row r="6" ht="230.1" customHeight="1" s="18">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>SIM-519</t>
+          <t>SIM-443d</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Build the live, schedule-driven game day view</t>
+          <t>Restrict what the SQL query tool can read</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>The public-facing screen that lists all of today's games should pull its list directly from Major League Baseball's own public schedule and mark each game as upcoming, in progress, or finished. Right now it pulls its game list only from the platform's own database, which can miss games or show stale information. This is a multi-part project; each part can be finished and checked off on its own.</t>
+          <t>The platform includes a tool that lets a user run their own read-only database queries from the website. It only blocks queries that would change data, but does not restrict which parts of the database can be read, so a user could query internal system tables that list other database accounts and their passwords.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>The day view lists every game the league's real schedule shows for that day, with the correct status, sourced live from the league rather than only from the platform's own stored data.</t>
+          <t>The SQL query tool only allows reading from the platform's approved data tables, and requests to read internal system tables are blocked.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>STATUS 2026-10-09: BUILT, MERGED (e3aae8e) and DEPLOYED: all eight parts plus the owner's Daily Diamond design; migration 0029 applied; the live service and the scheduler run. Open only for the game-day live check: (1) a live card against Gameday; (2) a posted lineup, then POST /simulate; (3) the game page on a live game (SIM-562, deployed 2026-10-09 and checked on final games only): the real linescore, box score and plays refresh every 15 s, and a what-if from the latest play runs both 100-game runs. Record: CHANGES.md 2026-10-09.
-Build a connection to the league's public schedule feed, use it to drive the list of games shown, and keep layering the platform's simulations, projections, and odds on top of that live list.
-GAME-DAY CHECK 2026-10-12 (849812, live): the live card, the game page and the what-if panel's state PASS; two steps FAIL. (a) The lineup writer writes only a game still in Preview, so a game the live service first sees in progress (the laptop slept through the pregame window) never gets lineup rows. Fix: let the writer also write a live game that has no rows. (b) 'Simulate 100 from here' then answers 503, because the what-if resolves the venue and hands from raw.game_lineups. Fix: fall back to the start state's own lineups. Re-run the check on a live game. The /live 500 found the same day is fixed (906ced9). BOTH FIXES BUILT 2026-10-13: (a) the live service writes a started game's starting lineup from its feed when none is stored (on_live); (b) the what-if builds its base state from the feed's starting lineup when the table is empty. Full unit suite green. Open only for one more live check, with the laptop awake from before first pitch.</t>
+          <t>Add a list of allowed tables to the query tool's safety check, and reject any query that reaches outside that list.</t>
         </is>
       </c>
     </row>
@@ -696,27 +694,27 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>SIM-443d</t>
+          <t>SIM-443e</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Restrict what the SQL query tool can read</t>
+          <t>Turn on the read-only database connection for the SQL tool</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>The platform includes a tool that lets a user run their own read-only database queries from the website. It only blocks queries that would change data, but does not restrict which parts of the database can be read, so a user could query internal system tables that list other database accounts and their passwords.</t>
+          <t>The SQL query tool was built to use a separate, limited-permission database connection for safety, but the setting that turns that connection on is currently switched off, so the tool quietly falls back to the full administrator database connection instead.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>The SQL query tool only allows reading from the platform's approved data tables, and requests to read internal system tables are blocked.</t>
+          <t>The SQL query tool is confirmed to be using the limited, read-only database connection rather than the administrator connection.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Add a list of allowed tables to the query tool's safety check, and reject any query that reaches outside that list.</t>
+          <t>Turn on and set the read-only connection's configuration value, then confirm the tool uses it.</t>
         </is>
       </c>
     </row>
@@ -728,27 +726,27 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>SIM-443e</t>
+          <t>SIM-443a</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Turn on the read-only database connection for the SQL tool</t>
+          <t>Stop exposing database ports to the network</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>The SQL query tool was built to use a separate, limited-permission database connection for safety, but the setting that turns that connection on is currently switched off, so the tool quietly falls back to the full administrator database connection instead.</t>
+          <t>The main database, the cache, and the application are all currently reachable from any computer on the network, not just the local machine, because their network connections are open to every network instead of limited to the local computer.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>The SQL query tool is confirmed to be using the limited, read-only database connection rather than the administrator connection.</t>
+          <t>The database, cache, and application ports are reachable only from the local machine, and the application still works normally.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Turn on and set the read-only connection's configuration value, then confirm the tool uses it.</t>
+          <t>Change each service's network setting in the deployment configuration to bind only to the local machine's own address.</t>
         </is>
       </c>
     </row>
@@ -760,27 +758,27 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>SIM-443a</t>
+          <t>SIM-443b</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Stop exposing database ports to the network</t>
+          <t>Remove the default database password and admin access</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>The main database, the cache, and the application are all currently reachable from any computer on the network, not just the local machine, because their network connections are open to every network instead of limited to the local computer.</t>
+          <t>The database's password is stored in plain, readable text in a file that is checked into the project's shared code, and the account using it has full administrator-level access rather than only the access it actually needs.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>The database, cache, and application ports are reachable only from the local machine, and the application still works normally.</t>
+          <t>The database password is no longer stored in the shared project files, and the application uses an account with only the specific permissions it needs.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Change each service's network setting in the deployment configuration to bind only to the local machine's own address.</t>
+          <t>Move the password into a secrets manager or environment variable outside the shared code, and create a limited-permission database account for the application.</t>
         </is>
       </c>
     </row>
@@ -792,27 +790,27 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SIM-443b</t>
+          <t>SIM-443c</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Remove the default database password and admin access</t>
+          <t>Require login on the API</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>The database's password is stored in plain, readable text in a file that is checked into the project's shared code, and the account using it has full administrator-level access rather than only the access it actually needs.</t>
+          <t>The programming interface (API) that the website and other tools use to pull data from the platform currently lets any request through with no login check whenever a certain setting is left unset, which is the default. This means anyone who can reach the server can pull the full pitch-by-pitch dataset with no credentials.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>The database password is no longer stored in the shared project files, and the application uses an account with only the specific permissions it needs.</t>
+          <t>Every route that provides data or triggers work requires a valid login by default, with no setting that silently disables that requirement.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Move the password into a secrets manager or environment variable outside the shared code, and create a limited-permission database account for the application.</t>
+          <t>Fix the login check so it fails closed (requires login) unless deliberately configured otherwise, and re-test that all data routes are covered.</t>
         </is>
       </c>
     </row>
@@ -824,27 +822,27 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SIM-443c</t>
+          <t>SIM-443f</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Require login on the API</t>
+          <t>Secure the shared cache (Redis)</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>The programming interface (API) that the website and other tools use to pull data from the platform currently lets any request through with no login check whenever a certain setting is left unset, which is the default. This means anyone who can reach the server can pull the full pitch-by-pitch dataset with no credentials.</t>
+          <t>The platform's shared, fast temporary-storage system (called Redis) is reachable from other computers on the local network with no password, and it stores cached data in a format that can run arbitrary code if it is tampered with. Together, this means someone who can reach the cache could plant tampered data that later runs on the server.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Every route that provides data or triggers work requires a valid login by default, with no setting that silently disables that requirement.</t>
+          <t>The shared cache requires a password to connect, and it is no longer reachable from the network without one.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Fix the login check so it fails closed (requires login) unless deliberately configured otherwise, and re-test that all data routes are covered.</t>
+          <t>Set a password on the cache and restrict its network access the same way as the other services; consider switching away from a data format that can execute code.</t>
         </is>
       </c>
     </row>
@@ -856,27 +854,27 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>SIM-443f</t>
+          <t>SIM-525</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Secure the shared cache (Redis)</t>
+          <t>Set up scheduled backups</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>The platform's shared, fast temporary-storage system (called Redis) is reachable from other computers on the local network with no password, and it stores cached data in a format that can run arbitrary code if it is tampered with. Together, this means someone who can reach the cache could plant tampered data that later runs on the server.</t>
+          <t>None of the platform's three data stores (the main statistics database, the game-simulation database, and the bundle of pre-computed data the simulator reads at startup) currently have any automatic backup. If any were lost or corrupted, rebuilding them from scratch would take roughly 12 hours of reprocessing.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>The shared cache requires a password to connect, and it is no longer reachable from the network without one.</t>
+          <t>All three data stores back up automatically on a schedule, and a real restore from that backup has been tested successfully at least once.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Set a password on the cache and restrict its network access the same way as the other services; consider switching away from a data format that can execute code.</t>
+          <t>Set up a scheduled backup job for each data store and verify a real restore works before considering this finished.</t>
         </is>
       </c>
     </row>
@@ -888,27 +886,27 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>SIM-525</t>
+          <t>SIM-493</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Set up scheduled backups</t>
+          <t>Break up the oversized simulation-loop file, and run the project-wide code-hygiene refactor</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>None of the platform's three data stores (the main statistics database, the game-simulation database, and the bundle of pre-computed data the simulator reads at startup) currently have any automatic backup. If any were lost or corrupted, rebuilding them from scratch would take roughly 12 hours of reprocessing.</t>
+          <t>The single code file that runs the pitch-by-pitch game simulation has grown very large (3,258 lines) as features were added, which makes it hard to review and maintain safely. The team deliberately postponed this cleanup until the pitch-speed and pitch-realism work settled. On 2026-09-16 the owner widened the ticket to a generalized refactor of the project. Three habits have accumulated. (1) Scripts are named after the ticket that created them, not after what they do: 26 of the 43 scripts carry a SIM-number prefix, and every model change since the fatigue weight is graded with a general tool called sim518_pair_accuracy.py (the paired accuracy comparison), so a reader cannot tell a general tool from a one-off probe. (2) Run outputs sit next to code: scripts/ holds 140 ticket-prefixed files, 114 of them results (JSON, logs, text), 40 of those committed. (3) Five source files are over 2,500 lines each: the profile computor (7,732), the accuracy comparison (3,488), the simulation loop (3,258), the full-pool sampler (3,139) and the artifact builder (2,889). Smaller items: about 2,300 SIM-number tags in code comments across 220 tickets (one tag, SIM-421, has two meanings); the 'does this column exist' probe is written about 20 times across the engines, the calibrator and the league writer; the 45 SIM_* environment flags have no single registry of their defaults and owners.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>All three data stores back up automatically on a schedule, and a real restore from that backup has been tested successfully at least once.</t>
+          <t>The simulator behaves the same before and after, confirmed by the unit and regression lanes and one 45 x 130 acceptance lane on the balanced game set. Every script is named for what it does (the paired accuracy comparison first); the shell wrappers, the plans, the technical docs and CHANGES.md point at the new names. Run outputs live outside scripts/ in a results folder that git ignores; the committed ones are moved to docs/audit/ or deleted. The five files over 2,500 lines are split by responsibility. A ticket tag in a code comment says what the work was, not only its number, or is dropped where the git history already records it. One shared column-probe helper; one registry of the SIM_* flags with each flag's default and owner ticket. Ruff, mypy and CI green.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Set up a scheduled backup job for each data store and verify a real restore works before considering this finished.</t>
+          <t>Do it in slices, one commit each, every slice behaviour-neutral. (1) Rename the paired accuracy tool to pair_accuracy.py and the other general tools by purpose; move the one-off probes under scripts/probes/. (2) Move the run outputs out of scripts/ and add the ignore rule. (3) Split sim_loop.py by responsibility (the pitch draw, the fielding stage, the runner draws, the manager decisions, the box credit), then the other four large files. (4) The shared helpers: the column probe, the flag registry. (5) The comment tags. Timing: the joint fit (SIM-548) is paused until the model is final; run slice 3 before that fit resumes or after it finishes, never while an arm is running.</t>
         </is>
       </c>
     </row>
@@ -920,27 +918,27 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>SIM-493</t>
+          <t>SIM-547</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Break up the oversized simulation-loop file, and run the project-wide code-hygiene refactor</t>
+          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>The single code file that runs the pitch-by-pitch game simulation has grown very large (3,258 lines) as features were added, which makes it hard to review and maintain safely. The team deliberately postponed this cleanup until the pitch-speed and pitch-realism work settled. On 2026-09-16 the owner widened the ticket to a generalized refactor of the project. Three habits have accumulated. (1) Scripts are named after the ticket that created them, not after what they do: 26 of the 43 scripts carry a SIM-number prefix, and every model change since the fatigue weight is graded with a general tool called sim518_pair_accuracy.py (the paired accuracy comparison), so a reader cannot tell a general tool from a one-off probe. (2) Run outputs sit next to code: scripts/ holds 140 ticket-prefixed files, 114 of them results (JSON, logs, text), 40 of those committed. (3) Five source files are over 2,500 lines each: the profile computor (7,732), the accuracy comparison (3,488), the simulation loop (3,258), the full-pool sampler (3,139) and the artifact builder (2,889). Smaller items: about 2,300 SIM-number tags in code comments across 220 tickets (one tag, SIM-421, has two meanings); the 'does this column exist' probe is written about 20 times across the engines, the calibrator and the league writer; the 45 SIM_* environment flags have no single registry of their defaults and owners.</t>
+          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>The simulator behaves the same before and after, confirmed by the unit and regression lanes and one 45 x 130 acceptance lane on the balanced game set. Every script is named for what it does (the paired accuracy comparison first); the shell wrappers, the plans, the technical docs and CHANGES.md point at the new names. Run outputs live outside scripts/ in a results folder that git ignores; the committed ones are moved to docs/audit/ or deleted. The five files over 2,500 lines are split by responsibility. A ticket tag in a code comment says what the work was, not only its number, or is dropped where the git history already records it. One shared column-probe helper; one registry of the SIM_* flags with each flag's default and owner ticket. Ruff, mypy and CI green.</t>
+          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Do it in slices, one commit each, every slice behaviour-neutral. (1) Rename the paired accuracy tool to pair_accuracy.py and the other general tools by purpose; move the one-off probes under scripts/probes/. (2) Move the run outputs out of scripts/ and add the ignore rule. (3) Split sim_loop.py by responsibility (the pitch draw, the fielding stage, the runner draws, the manager decisions, the box credit), then the other four large files. (4) The shared helpers: the column probe, the flag registry. (5) The comment tags. Timing: the joint fit (SIM-548) is paused until the model is final; run slice 3 before that fit resumes or after it finishes, never while an arm is running.</t>
+          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/sim427_manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
         </is>
       </c>
     </row>
@@ -952,27 +950,27 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>SIM-547</t>
+          <t>SIM-526</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
+          <t>Turn on the catcher pitch-receiving factor</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
+          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
+          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/sim427_manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
+          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
         </is>
       </c>
     </row>
@@ -984,98 +982,67 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>SIM-526</t>
+          <t>SIM-556</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Turn on the catcher pitch-receiving factor</t>
+          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
+          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/steal_weight_volume_probe.py with its records (uncommitted, in the worktree pensive-taussig-ec2f7e). Filed P3 by the owner on 2026-10-01.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
+          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
+          <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="54" customHeight="1" s="18">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>SIM-556</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/steal_weight_volume_probe.py with its records (uncommitted, in the worktree pensive-taussig-ec2f7e). Filed P3 by the owner on 2026-10-01.</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
-        </is>
-      </c>
+      <c r="A17" s="15" t="n"/>
+      <c r="B17" s="15" t="n"/>
+      <c r="C17" s="15" t="n"/>
+      <c r="D17" s="16" t="n"/>
+      <c r="E17" s="15" t="n"/>
+      <c r="F17" s="15" t="n"/>
     </row>
     <row r="18" ht="40.5" customHeight="1" s="18">
-      <c r="A18" s="15" t="n"/>
-      <c r="B18" s="15" t="n"/>
-      <c r="C18" s="15" t="n"/>
-      <c r="D18" s="16" t="n"/>
-      <c r="E18" s="15" t="n"/>
-      <c r="F18" s="15" t="n"/>
-    </row>
-    <row r="19" ht="229.5" customHeight="1" s="18">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D19" s="13" t="inlineStr">
+      <c r="D18" s="13" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F19" s="12" t="n"/>
-    </row>
+      <c r="F18" s="12" t="n"/>
+    </row>
+    <row r="19" ht="229.5" customHeight="1" s="18"/>
     <row r="20" ht="300" customHeight="1" s="18"/>
     <row r="21" ht="67.5" customHeight="1" s="18"/>
     <row r="22" s="18"/>

</xml_diff>

<commit_message>
Record the security hardening cluster (SIM-443a-f): CHANGES, CLAUDE.md, the audit doc, the backlog
- CHANGES.md: one BUILT entry (Why, What per ticket, Tests, Rollout, Not done).
- CLAUDE.md: the 2b bullet, the jobs-container caveat in 2a, the repo map
  (db/roles, pipeline/db_dsn.py, simulation/cache_codec.py, scripts/gen_secrets.py),
  make db-roles / make gen-secrets, and the stale "the sim cache holds score
  arrays" phrase.
- docs/audit/2026-10-13-sim443-security-hardening.md: the design by track, the
  privilege inventory and the live cutover run book (owner's procedure).
- BACKLOG.xlsx: the six SIM-443 rows deleted; SIM-564/565/566 filed P3; next
  free ID SIM-567.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="18" min="1" max="1"/>
@@ -585,7 +585,7 @@
     <row r="2" s="18">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>NEXT FREE TICKET ID: SIM-564</t>
+          <t>NEXT FREE TICKET ID: SIM-567</t>
         </is>
       </c>
     </row>
@@ -662,27 +662,27 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>SIM-443d</t>
+          <t>SIM-525</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Restrict what the SQL query tool can read</t>
+          <t>Set up scheduled backups</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>The platform includes a tool that lets a user run their own read-only database queries from the website. It only blocks queries that would change data, but does not restrict which parts of the database can be read, so a user could query internal system tables that list other database accounts and their passwords.</t>
+          <t>None of the platform's three data stores (the main statistics database, the game-simulation database, and the bundle of pre-computed data the simulator reads at startup) currently have any automatic backup. If any were lost or corrupted, rebuilding them from scratch would take roughly 12 hours of reprocessing.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>The SQL query tool only allows reading from the platform's approved data tables, and requests to read internal system tables are blocked.</t>
+          <t>All three data stores back up automatically on a schedule, and a real restore from that backup has been tested successfully at least once.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Add a list of allowed tables to the query tool's safety check, and reject any query that reaches outside that list.</t>
+          <t>Set up a scheduled backup job for each data store and verify a real restore works before considering this finished.</t>
         </is>
       </c>
     </row>
@@ -694,27 +694,27 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>SIM-443e</t>
+          <t>SIM-493</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Turn on the read-only database connection for the SQL tool</t>
+          <t>Break up the oversized simulation-loop file, and run the project-wide code-hygiene refactor</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>The SQL query tool was built to use a separate, limited-permission database connection for safety, but the setting that turns that connection on is currently switched off, so the tool quietly falls back to the full administrator database connection instead.</t>
+          <t>The single code file that runs the pitch-by-pitch game simulation has grown very large (3,258 lines) as features were added, which makes it hard to review and maintain safely. The team deliberately postponed this cleanup until the pitch-speed and pitch-realism work settled. On 2026-09-16 the owner widened the ticket to a generalized refactor of the project. Three habits have accumulated. (1) Scripts are named after the ticket that created them, not after what they do: 26 of the 43 scripts carry a SIM-number prefix, and every model change since the fatigue weight is graded with a general tool called sim518_pair_accuracy.py (the paired accuracy comparison), so a reader cannot tell a general tool from a one-off probe. (2) Run outputs sit next to code: scripts/ holds 140 ticket-prefixed files, 114 of them results (JSON, logs, text), 40 of those committed. (3) Five source files are over 2,500 lines each: the profile computor (7,732), the accuracy comparison (3,488), the simulation loop (3,258), the full-pool sampler (3,139) and the artifact builder (2,889). Smaller items: about 2,300 SIM-number tags in code comments across 220 tickets (one tag, SIM-421, has two meanings); the 'does this column exist' probe is written about 20 times across the engines, the calibrator and the league writer; the 45 SIM_* environment flags have no single registry of their defaults and owners.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>The SQL query tool is confirmed to be using the limited, read-only database connection rather than the administrator connection.</t>
+          <t>The simulator behaves the same before and after, confirmed by the unit and regression lanes and one 45 x 130 acceptance lane on the balanced game set. Every script is named for what it does (the paired accuracy comparison first); the shell wrappers, the plans, the technical docs and CHANGES.md point at the new names. Run outputs live outside scripts/ in a results folder that git ignores; the committed ones are moved to docs/audit/ or deleted. The five files over 2,500 lines are split by responsibility. A ticket tag in a code comment says what the work was, not only its number, or is dropped where the git history already records it. One shared column-probe helper; one registry of the SIM_* flags with each flag's default and owner ticket. Ruff, mypy and CI green.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Turn on and set the read-only connection's configuration value, then confirm the tool uses it.</t>
+          <t>Do it in slices, one commit each, every slice behaviour-neutral. (1) Rename the paired accuracy tool to pair_accuracy.py and the other general tools by purpose; move the one-off probes under scripts/probes/. (2) Move the run outputs out of scripts/ and add the ignore rule. (3) Split sim_loop.py by responsibility (the pitch draw, the fielding stage, the runner draws, the manager decisions, the box credit), then the other four large files. (4) The shared helpers: the column probe, the flag registry. (5) The comment tags. Timing: the joint fit (SIM-548) is paused until the model is final; run slice 3 before that fit resumes or after it finishes, never while an arm is running.</t>
         </is>
       </c>
     </row>
@@ -726,27 +726,27 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>SIM-443a</t>
+          <t>SIM-547</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Stop exposing database ports to the network</t>
+          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>The main database, the cache, and the application are all currently reachable from any computer on the network, not just the local machine, because their network connections are open to every network instead of limited to the local computer.</t>
+          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>The database, cache, and application ports are reachable only from the local machine, and the application still works normally.</t>
+          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Change each service's network setting in the deployment configuration to bind only to the local machine's own address.</t>
+          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/sim427_manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
         </is>
       </c>
     </row>
@@ -758,27 +758,27 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>SIM-443b</t>
+          <t>SIM-526</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Remove the default database password and admin access</t>
+          <t>Turn on the catcher pitch-receiving factor</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>The database's password is stored in plain, readable text in a file that is checked into the project's shared code, and the account using it has full administrator-level access rather than only the access it actually needs.</t>
+          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>The database password is no longer stored in the shared project files, and the application uses an account with only the specific permissions it needs.</t>
+          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Move the password into a secrets manager or environment variable outside the shared code, and create a limited-permission database account for the application.</t>
+          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
         </is>
       </c>
     </row>
@@ -790,31 +790,31 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SIM-443c</t>
+          <t>SIM-556</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Require login on the API</t>
+          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>The programming interface (API) that the website and other tools use to pull data from the platform currently lets any request through with no login check whenever a certain setting is left unset, which is the default. This means anyone who can reach the server can pull the full pitch-by-pitch dataset with no credentials.</t>
+          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/steal_weight_volume_probe.py with its records (uncommitted, in the worktree pensive-taussig-ec2f7e). Filed P3 by the owner on 2026-10-01.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Every route that provides data or triggers work requires a valid login by default, with no setting that silently disables that requirement.</t>
+          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Fix the login check so it fails closed (requires login) unless deliberately configured otherwise, and re-test that all data routes are covered.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="81" customHeight="1" s="18">
+          <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="94.5" customHeight="1" s="18">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>P3</t>
@@ -822,31 +822,31 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SIM-443f</t>
+          <t>SIM-564</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Secure the shared cache (Redis)</t>
+          <t>Rate limiter keyed on an unverified header</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>The platform's shared, fast temporary-storage system (called Redis) is reachable from other computers on the local network with no password, and it stores cached data in a format that can run arbitrary code if it is tampered with. Together, this means someone who can reach the cache could plant tampered data that later runs on the server.</t>
+          <t>The API can limit how many requests each caller makes per minute. It tells callers apart by the X-API-Key header, but it reads that header before any check that the key is real. A caller can send a new made-up key on every request and never reach the limit, or send someone else's key and use up that person's allowance. The limiter is off by default (RATE_LIMIT_PER_MINUTE unset), so this matters only once it is turned on.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>The shared cache requires a password to connect, and it is no longer reachable from the network without one.</t>
+          <t>The rate limiter counts a request against a key only when that key is one of the configured API keys; every other request counts against the caller's address. A unit test sends many requests with random keys and gets a 429 at the limit, and a request with a real key is counted under that key.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Set a password on the cache and restrict its network access the same way as the other services; consider switching away from a data format that can execute code.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="135" customHeight="1" s="18">
+          <t>In api/auth.py RateLimitMiddleware, choose the bucket with the same key check the login uses (_presented_api_key + _key_matches against the configured keys); a key that does not match falls back to the client address. Never use the raw header text as the bucket name. Add the test to tests/unit next to the existing rate-limit tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="94.5" customHeight="1" s="18">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>P3</t>
@@ -854,31 +854,31 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>SIM-525</t>
+          <t>SIM-565</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Set up scheduled backups</t>
+          <t>Load the engine bundle with allow_pickle=False</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>None of the platform's three data stores (the main statistics database, the game-simulation database, and the bundle of pre-computed data the simulator reads at startup) currently have any automatic backup. If any were lost or corrupted, rebuilding them from scratch would take roughly 12 hours of reprocessing.</t>
+          <t>The simulator loads its prepared data files (the engine bundle) with numpy's allow_pickle=True setting, in pipeline/batch/engine_artifacts.py. That setting lets a data file carry a pickle, and loading a pickle can run code. Only our own nightly build writes the bundle, so the risk is small, but a tampered file in the data folder would run code in every simulator worker. The JSON cache work (SIM-443f) removed pickle from the Redis cache; this is the remaining pickle load on the hot path.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>All three data stores back up automatically on a schedule, and a real restore from that backup has been tested successfully at least once.</t>
+          <t>Every np.load of the bundle uses allow_pickle=False. The live bundle loads and the simulator runs a ten-game smoke with the same results as before. A unit test fails if any np.load in the loader passes allow_pickle=True.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Set up a scheduled backup job for each data store and verify a real restore works before considering this finished.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="67.5" customHeight="1" s="18">
+          <t>First list which arrays in the live bundle are object arrays (np.load each .npz with allow_pickle=False and note which fail). Rewrite those arrays in the builder as plain types (fixed-width strings, integer codes plus a JSON side file), rebuild the bundle, then switch the five np.load calls to allow_pickle=False and add the source-scan test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="94.5" customHeight="1" s="18">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>P3</t>
@@ -886,162 +886,69 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>SIM-493</t>
+          <t>SIM-566</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Break up the oversized simulation-loop file, and run the project-wide code-hygiene refactor</t>
+          <t>Move the fixed-query read routes onto the read-only pool</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>The single code file that runs the pitch-by-pitch game simulation has grown very large (3,258 lines) as features were added, which makes it hard to review and maintain safely. The team deliberately postponed this cleanup until the pitch-speed and pitch-realism work settled. On 2026-09-16 the owner widened the ticket to a generalized refactor of the project. Three habits have accumulated. (1) Scripts are named after the ticket that created them, not after what they do: 26 of the 43 scripts carry a SIM-number prefix, and every model change since the fatigue weight is graded with a general tool called sim518_pair_accuracy.py (the paired accuracy comparison), so a reader cannot tell a general tool from a one-off probe. (2) Run outputs sit next to code: scripts/ holds 140 ticket-prefixed files, 114 of them results (JSON, logs, text), 40 of those committed. (3) Five source files are over 2,500 lines each: the profile computor (7,732), the accuracy comparison (3,488), the simulation loop (3,258), the full-pool sampler (3,139) and the artifact builder (2,889). Smaller items: about 2,300 SIM-number tags in code comments across 220 tickets (one tag, SIM-421, has two meanings); the 'does this column exist' probe is written about 20 times across the engines, the calibrator and the league writer; the 45 SIM_* environment flags have no single registry of their defaults and owners.</t>
+          <t>The SQL console now runs on a database login that can only read the raw tables (SIM-443e). Other read-only routes still use the main login, which can also write: the schema browser (/api/schema), the analytics pages (/api/analytics/*) and the player pages (/api/players/*). Their queries are fixed in code, not typed by a user, so the risk is low, but a defect in one of them runs with write access it never needs.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>The simulator behaves the same before and after, confirmed by the unit and regression lanes and one 45 x 130 acceptance lane on the balanced game set. Every script is named for what it does (the paired accuracy comparison first); the shell wrappers, the plans, the technical docs and CHANGES.md point at the new names. Run outputs live outside scripts/ in a results folder that git ignores; the committed ones are moved to docs/audit/ or deleted. The five files over 2,500 lines are split by responsibility. A ticket tag in a code comment says what the work was, not only its number, or is dropped where the git history already records it. One shared column-probe helper; one registry of the SIM_* flags with each flag's default and owner ticket. Ruff, mypy and CI green.</t>
+          <t>/api/schema, /api/analytics/* and /api/players/* read through the read-only pool, and each answers 503 when that pool is missing. Every query they run reads only raw tables (or a route that needs sim.* is listed and kept on the main pool with the reason). The unit tests for those routes pass with a fake read-only pool.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Do it in slices, one commit each, every slice behaviour-neutral. (1) Rename the paired accuracy tool to pair_accuracy.py and the other general tools by purpose; move the one-off probes under scripts/probes/. (2) Move the run outputs out of scripts/ and add the ignore rule. (3) Split sim_loop.py by responsibility (the pitch draw, the fielding stage, the runner draws, the manager decisions, the box credit), then the other four large files. (4) The shared helpers: the column probe, the flag registry. (5) The comment tags. Timing: the joint fit (SIM-548) is paused until the model is final; run slice 3 before that fit resumes or after it finishes, never while an arm is running.</t>
+          <t>Move sql_runner._ro_pool(request) into api/routes/_common.py as a shared helper and switch these routes to it. Check each query for a non-raw table first; the read-only role has no access to sim.* by design. Update docs/technical/api.md.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="67.5" customHeight="1" s="18">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>SIM-547</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/sim427_manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
-        </is>
-      </c>
+      <c r="A14" s="15" t="n"/>
+      <c r="B14" s="15" t="n"/>
+      <c r="C14" s="15" t="n"/>
+      <c r="D14" s="16" t="n"/>
+      <c r="E14" s="15" t="n"/>
+      <c r="F14" s="15" t="n"/>
     </row>
     <row r="15" ht="67.5" customHeight="1" s="18">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>SIM-526</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Turn on the catcher pitch-receiving factor</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="54" customHeight="1" s="18">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>SIM-556</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/steal_weight_volume_probe.py with its records (uncommitted, in the worktree pensive-taussig-ec2f7e). Filed P3 by the owner on 2026-10-01.</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="54" customHeight="1" s="18">
-      <c r="A17" s="15" t="n"/>
-      <c r="B17" s="15" t="n"/>
-      <c r="C17" s="15" t="n"/>
-      <c r="D17" s="16" t="n"/>
-      <c r="E17" s="15" t="n"/>
-      <c r="F17" s="15" t="n"/>
-    </row>
-    <row r="18" ht="40.5" customHeight="1" s="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E18" s="11" t="inlineStr">
+      <c r="E15" s="11" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F18" s="12" t="n"/>
-    </row>
+      <c r="F15" s="12" t="n"/>
+    </row>
+    <row r="16" ht="54" customHeight="1" s="18"/>
+    <row r="17" ht="54" customHeight="1" s="18"/>
+    <row r="18" ht="40.5" customHeight="1" s="18"/>
     <row r="19" ht="229.5" customHeight="1" s="18"/>
     <row r="20" ht="300" customHeight="1" s="18"/>
     <row r="21" ht="67.5" customHeight="1" s="18"/>

</xml_diff>

<commit_message>
Record the scheduled backups and the restore drill; close SIM-525
The record (CHANGES.md 2026-10-15) and the design with both run books
(docs/audit/2026-10-14-sim525-backups-plan.md): the deploy at 04:56 UTC, the
first sets (Postgres 2.7 GiB in 267 s, DuckDB 3.6 GiB in 201 s, the bundle
561 MiB in 46 s), the negative checks, and the drill (PASS in 450 s: pg_restore
349 s, all 36 tables inside their count brackets, both copies verified).
WORKFLOW.md gets the backups-and-restore section, deploy/README.md and the
technical reference their entries, CLAUDE.md its bullets and commands. The
CLAUDE.md inserts moved the two paragraph-11 lines the acceptance tests cite,
so the citations now read 866 and 869. BACKLOG.xlsx: the SIM-525 row is
deleted; SIM-567 (pin ODDS_PROVIDER=mock in the test lane) and SIM-568 (an
off-machine copy of the sets) are filed; the next free ID is SIM-569.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="18" min="1" max="1"/>
@@ -585,7 +585,7 @@
     <row r="2" s="18">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>NEXT FREE TICKET ID: SIM-567</t>
+          <t>NEXT FREE TICKET ID: SIM-569</t>
         </is>
       </c>
     </row>
@@ -662,27 +662,27 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>SIM-525</t>
+          <t>SIM-493</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Set up scheduled backups</t>
+          <t>Break up the oversized simulation-loop file, and run the project-wide code-hygiene refactor</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>None of the platform's three data stores (the main statistics database, the game-simulation database, and the bundle of pre-computed data the simulator reads at startup) currently have any automatic backup. If any were lost or corrupted, rebuilding them from scratch would take roughly 12 hours of reprocessing.</t>
+          <t>The single code file that runs the pitch-by-pitch game simulation has grown very large (3,258 lines) as features were added, which makes it hard to review and maintain safely. The team deliberately postponed this cleanup until the pitch-speed and pitch-realism work settled. On 2026-09-16 the owner widened the ticket to a generalized refactor of the project. Three habits have accumulated. (1) Scripts are named after the ticket that created them, not after what they do: 26 of the 43 scripts carry a SIM-number prefix, and every model change since the fatigue weight is graded with a general tool called sim518_pair_accuracy.py (the paired accuracy comparison), so a reader cannot tell a general tool from a one-off probe. (2) Run outputs sit next to code: scripts/ holds 140 ticket-prefixed files, 114 of them results (JSON, logs, text), 40 of those committed. (3) Five source files are over 2,500 lines each: the profile computor (7,732), the accuracy comparison (3,488), the simulation loop (3,258), the full-pool sampler (3,139) and the artifact builder (2,889). Smaller items: about 2,300 SIM-number tags in code comments across 220 tickets (one tag, SIM-421, has two meanings); the 'does this column exist' probe is written about 20 times across the engines, the calibrator and the league writer; the 45 SIM_* environment flags have no single registry of their defaults and owners.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>All three data stores back up automatically on a schedule, and a real restore from that backup has been tested successfully at least once.</t>
+          <t>The simulator behaves the same before and after, confirmed by the unit and regression lanes and one 45 x 130 acceptance lane on the balanced game set. Every script is named for what it does (the paired accuracy comparison first); the shell wrappers, the plans, the technical docs and CHANGES.md point at the new names. Run outputs live outside scripts/ in a results folder that git ignores; the committed ones are moved to docs/audit/ or deleted. The five files over 2,500 lines are split by responsibility. A ticket tag in a code comment says what the work was, not only its number, or is dropped where the git history already records it. One shared column-probe helper; one registry of the SIM_* flags with each flag's default and owner ticket. Ruff, mypy and CI green.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Set up a scheduled backup job for each data store and verify a real restore works before considering this finished.</t>
+          <t>Do it in slices, one commit each, every slice behaviour-neutral. (1) Rename the paired accuracy tool to pair_accuracy.py and the other general tools by purpose; move the one-off probes under scripts/probes/. (2) Move the run outputs out of scripts/ and add the ignore rule. (3) Split sim_loop.py by responsibility (the pitch draw, the fielding stage, the runner draws, the manager decisions, the box credit), then the other four large files. (4) The shared helpers: the column probe, the flag registry. (5) The comment tags. Timing: the joint fit (SIM-548) is paused until the model is final; run slice 3 before that fit resumes or after it finishes, never while an arm is running.</t>
         </is>
       </c>
     </row>
@@ -694,27 +694,27 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>SIM-493</t>
+          <t>SIM-547</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Break up the oversized simulation-loop file, and run the project-wide code-hygiene refactor</t>
+          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>The single code file that runs the pitch-by-pitch game simulation has grown very large (3,258 lines) as features were added, which makes it hard to review and maintain safely. The team deliberately postponed this cleanup until the pitch-speed and pitch-realism work settled. On 2026-09-16 the owner widened the ticket to a generalized refactor of the project. Three habits have accumulated. (1) Scripts are named after the ticket that created them, not after what they do: 26 of the 43 scripts carry a SIM-number prefix, and every model change since the fatigue weight is graded with a general tool called sim518_pair_accuracy.py (the paired accuracy comparison), so a reader cannot tell a general tool from a one-off probe. (2) Run outputs sit next to code: scripts/ holds 140 ticket-prefixed files, 114 of them results (JSON, logs, text), 40 of those committed. (3) Five source files are over 2,500 lines each: the profile computor (7,732), the accuracy comparison (3,488), the simulation loop (3,258), the full-pool sampler (3,139) and the artifact builder (2,889). Smaller items: about 2,300 SIM-number tags in code comments across 220 tickets (one tag, SIM-421, has two meanings); the 'does this column exist' probe is written about 20 times across the engines, the calibrator and the league writer; the 45 SIM_* environment flags have no single registry of their defaults and owners.</t>
+          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>The simulator behaves the same before and after, confirmed by the unit and regression lanes and one 45 x 130 acceptance lane on the balanced game set. Every script is named for what it does (the paired accuracy comparison first); the shell wrappers, the plans, the technical docs and CHANGES.md point at the new names. Run outputs live outside scripts/ in a results folder that git ignores; the committed ones are moved to docs/audit/ or deleted. The five files over 2,500 lines are split by responsibility. A ticket tag in a code comment says what the work was, not only its number, or is dropped where the git history already records it. One shared column-probe helper; one registry of the SIM_* flags with each flag's default and owner ticket. Ruff, mypy and CI green.</t>
+          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Do it in slices, one commit each, every slice behaviour-neutral. (1) Rename the paired accuracy tool to pair_accuracy.py and the other general tools by purpose; move the one-off probes under scripts/probes/. (2) Move the run outputs out of scripts/ and add the ignore rule. (3) Split sim_loop.py by responsibility (the pitch draw, the fielding stage, the runner draws, the manager decisions, the box credit), then the other four large files. (4) The shared helpers: the column probe, the flag registry. (5) The comment tags. Timing: the joint fit (SIM-548) is paused until the model is final; run slice 3 before that fit resumes or after it finishes, never while an arm is running.</t>
+          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/sim427_manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
         </is>
       </c>
     </row>
@@ -726,27 +726,27 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>SIM-547</t>
+          <t>SIM-526</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
+          <t>Turn on the catcher pitch-receiving factor</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
+          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
+          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/sim427_manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
+          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
         </is>
       </c>
     </row>
@@ -758,27 +758,27 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>SIM-526</t>
+          <t>SIM-556</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Turn on the catcher pitch-receiving factor</t>
+          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
+          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/steal_weight_volume_probe.py with its records (uncommitted, in the worktree pensive-taussig-ec2f7e). Filed P3 by the owner on 2026-10-01.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
+          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
+          <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
         </is>
       </c>
     </row>
@@ -790,27 +790,27 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SIM-556</t>
+          <t>SIM-564</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
+          <t>Rate limiter keyed on an unverified header</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/steal_weight_volume_probe.py with its records (uncommitted, in the worktree pensive-taussig-ec2f7e). Filed P3 by the owner on 2026-10-01.</t>
+          <t>The API can limit how many requests each caller makes per minute. It tells callers apart by the X-API-Key header, but it reads that header before any check that the key is real. A caller can send a new made-up key on every request and never reach the limit, or send someone else's key and use up that person's allowance. The limiter is off by default (RATE_LIMIT_PER_MINUTE unset), so this matters only once it is turned on.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
+          <t>The rate limiter counts a request against a key only when that key is one of the configured API keys; every other request counts against the caller's address. A unit test sends many requests with random keys and gets a 429 at the limit, and a request with a real key is counted under that key.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
+          <t>In api/auth.py RateLimitMiddleware, choose the bucket with the same key check the login uses (_presented_api_key + _key_matches against the configured keys); a key that does not match falls back to the client address. Never use the raw header text as the bucket name. Add the test to tests/unit next to the existing rate-limit tests.</t>
         </is>
       </c>
     </row>
@@ -822,27 +822,27 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SIM-564</t>
+          <t>SIM-565</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Rate limiter keyed on an unverified header</t>
+          <t>Load the engine bundle with allow_pickle=False</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>The API can limit how many requests each caller makes per minute. It tells callers apart by the X-API-Key header, but it reads that header before any check that the key is real. A caller can send a new made-up key on every request and never reach the limit, or send someone else's key and use up that person's allowance. The limiter is off by default (RATE_LIMIT_PER_MINUTE unset), so this matters only once it is turned on.</t>
+          <t>The simulator loads its prepared data files (the engine bundle) with numpy's allow_pickle=True setting, in pipeline/batch/engine_artifacts.py. That setting lets a data file carry a pickle, and loading a pickle can run code. Only our own nightly build writes the bundle, so the risk is small, but a tampered file in the data folder would run code in every simulator worker. The JSON cache work (SIM-443f) removed pickle from the Redis cache; this is the remaining pickle load on the hot path.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>The rate limiter counts a request against a key only when that key is one of the configured API keys; every other request counts against the caller's address. A unit test sends many requests with random keys and gets a 429 at the limit, and a request with a real key is counted under that key.</t>
+          <t>Every np.load of the bundle uses allow_pickle=False. The live bundle loads and the simulator runs a ten-game smoke with the same results as before. A unit test fails if any np.load in the loader passes allow_pickle=True.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>In api/auth.py RateLimitMiddleware, choose the bucket with the same key check the login uses (_presented_api_key + _key_matches against the configured keys); a key that does not match falls back to the client address. Never use the raw header text as the bucket name. Add the test to tests/unit next to the existing rate-limit tests.</t>
+          <t>First list which arrays in the live bundle are object arrays (np.load each .npz with allow_pickle=False and note which fail). Rewrite those arrays in the builder as plain types (fixed-width strings, integer codes plus a JSON side file), rebuild the bundle, then switch the five np.load calls to allow_pickle=False and add the source-scan test.</t>
         </is>
       </c>
     </row>
@@ -854,27 +854,27 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>SIM-565</t>
+          <t>SIM-566</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Load the engine bundle with allow_pickle=False</t>
+          <t>Move the fixed-query read routes onto the read-only pool</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>The simulator loads its prepared data files (the engine bundle) with numpy's allow_pickle=True setting, in pipeline/batch/engine_artifacts.py. That setting lets a data file carry a pickle, and loading a pickle can run code. Only our own nightly build writes the bundle, so the risk is small, but a tampered file in the data folder would run code in every simulator worker. The JSON cache work (SIM-443f) removed pickle from the Redis cache; this is the remaining pickle load on the hot path.</t>
+          <t>The SQL console now runs on a database login that can only read the raw tables (SIM-443e). Other read-only routes still use the main login, which can also write: the schema browser (/api/schema), the analytics pages (/api/analytics/*) and the player pages (/api/players/*). Their queries are fixed in code, not typed by a user, so the risk is low, but a defect in one of them runs with write access it never needs.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Every np.load of the bundle uses allow_pickle=False. The live bundle loads and the simulator runs a ten-game smoke with the same results as before. A unit test fails if any np.load in the loader passes allow_pickle=True.</t>
+          <t>/api/schema, /api/analytics/* and /api/players/* read through the read-only pool, and each answers 503 when that pool is missing. Every query they run reads only raw tables (or a route that needs sim.* is listed and kept on the main pool with the reason). The unit tests for those routes pass with a fake read-only pool.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>First list which arrays in the live bundle are object arrays (np.load each .npz with allow_pickle=False and note which fail). Rewrite those arrays in the builder as plain types (fixed-width strings, integer codes plus a JSON side file), rebuild the bundle, then switch the five np.load calls to allow_pickle=False and add the source-scan test.</t>
+          <t>Move sql_runner._ro_pool(request) into api/routes/_common.py as a shared helper and switch these routes to it. Check each query for a non-raw table first; the read-only role has no access to sim.* by design. Update docs/technical/api.md.</t>
         </is>
       </c>
     </row>
@@ -886,67 +886,98 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>SIM-566</t>
+          <t>SIM-567</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Move the fixed-query read routes onto the read-only pool</t>
+          <t>Pin the test lane's odds provider to the mock</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>The SQL console now runs on a database login that can only read the raw tables (SIM-443e). Other read-only routes still use the main login, which can also write: the schema browser (/api/schema), the analytics pages (/api/analytics/*) and the player pages (/api/players/*). Their queries are fixed in code, not typed by a user, so the risk is low, but a defect in one of them runs with write access it never needs.</t>
+          <t>The unit-test lane runs inside the app container, which reads the live .env. ODDS_PROVIDER=bettingpros leaks into the tests, so twelve tests in three files (the live pipeline's prop-odds tests and the odds-vocabulary tests) call the real BettingPros provider when they build the pipeline and fail with HTTP 404. They pass with ODDS_PROVIDER=mock. CI never sees this, because CI has no .env. Found while building the scheduled backups (SIM-525) on 2026-10-15.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>/api/schema, /api/analytics/* and /api/players/* read through the read-only pool, and each answers 503 when that pool is missing. Every query they run reads only raw tables (or a route that needs sim.* is listed and kept on the main pool with the reason). The unit tests for those routes pass with a fake read-only pool.</t>
+          <t>make test-unit on the serving stack passes those three files with no environment override, and no unit test reaches the vendor.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Move sql_runner._ro_pool(request) into api/routes/_common.py as a shared helper and switch these routes to it. Check each query for a non-raw table first; the read-only role has no access to sim.* by design. Update docs/technical/api.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="67.5" customHeight="1" s="18">
-      <c r="A14" s="15" t="n"/>
-      <c r="B14" s="15" t="n"/>
-      <c r="C14" s="15" t="n"/>
-      <c r="D14" s="16" t="n"/>
-      <c r="E14" s="15" t="n"/>
-      <c r="F14" s="15" t="n"/>
+          <t>Pin ODDS_PROVIDER=mock in tests/conftest.py, the way it already pins SIM_MANAGER and AUTH_DISABLED. Also note the whole-repo mount the SIM-525 build used for the lane (-v "$(pwd -W):/app"), so the container tests read the checkout's tests/ and compose file instead of the image's stale copies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="94.5" customHeight="1" s="18">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>SIM-568</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Keep an off-machine copy of the backup sets</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>The scheduled backups (SIM-525) write the Postgres dump, the DuckDB file and the engine bundle every night to a folder on C:, the laptop's only disk (C:/Users/grego/Documents/baseball_backups, about 7 GB a night, three sets kept). They protect against a Docker disk-image loss, docker compose down -v, a bad migration or rebuild and accidental deletion. They do not protect against the disk dying or the laptop being lost.</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>The newest complete set of each store also exists on another disk or machine (an external drive, a NAS or a cloud bucket), copied automatically after the 10:00 UTC run, and one restore from that copy has been tested.</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Add a third scheduled step after the two backup jobs that syncs BACKUP_DIR to the second location (robocopy or rclone to an external drive, a OneDrive folder, or an S3-compatible bucket). Keep the per-store manifests as they are, so scripts/backup_drill.py can drill from the copy with --backup-dir.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="67.5" customHeight="1" s="18">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="15" t="n"/>
+      <c r="B15" s="15" t="n"/>
+      <c r="C15" s="15" t="n"/>
+      <c r="D15" s="16" t="n"/>
+      <c r="E15" s="15" t="n"/>
+      <c r="F15" s="15" t="n"/>
+    </row>
+    <row r="16" ht="54" customHeight="1" s="18">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F15" s="12" t="n"/>
-    </row>
-    <row r="16" ht="54" customHeight="1" s="18"/>
+      <c r="F16" s="12" t="n"/>
+    </row>
     <row r="17" ht="54" customHeight="1" s="18"/>
     <row r="18" ht="40.5" customHeight="1" s="18"/>
     <row r="19" ht="229.5" customHeight="1" s="18"/>

</xml_diff>

<commit_message>
Close the rate limiter's bucket ticket in the backlog; next free ID SIM-570 (SIM-564, SIM-569)
SIM-564 closed 2026-10-17 (CHANGES.md is its record), so its row goes.
SIM-569 was used in CHANGES.md and the commits and closed the same day,
so it never had a row; the subtitle's next free ID moves past it.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>NEXT FREE TICKET ID: SIM-569</t>
+          <t>NEXT FREE TICKET ID: SIM-570</t>
         </is>
       </c>
     </row>
@@ -783,27 +783,27 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SIM-564</t>
+          <t>SIM-565</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Rate limiter keyed on an unverified header</t>
+          <t>Load the engine bundle with allow_pickle=False</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>The API can limit how many requests each caller makes per minute. It tells callers apart by the X-API-Key header, but it reads that header before any check that the key is real. A caller can send a new made-up key on every request and never reach the limit, or send someone else's key and use up that person's allowance. The limiter is off by default (RATE_LIMIT_PER_MINUTE unset), so this matters only once it is turned on.</t>
+          <t>The simulator loads its prepared data files (the engine bundle) with numpy's allow_pickle=True setting, in pipeline/batch/engine_artifacts.py. That setting lets a data file carry a pickle, and loading a pickle can run code. Only our own nightly build writes the bundle, so the risk is small, but a tampered file in the data folder would run code in every simulator worker. The JSON cache work (SIM-443f) removed pickle from the Redis cache; this is the remaining pickle load on the hot path.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>The rate limiter counts a request against a key only when that key is one of the configured API keys; every other request counts against the caller's address. A unit test sends many requests with random keys and gets a 429 at the limit, and a request with a real key is counted under that key.</t>
+          <t>Every np.load of the bundle uses allow_pickle=False. The live bundle loads and the simulator runs a ten-game smoke with the same results as before. A unit test fails if any np.load in the loader passes allow_pickle=True.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>In api/auth.py RateLimitMiddleware, choose the bucket with the same key check the login uses (_presented_api_key + _key_matches against the configured keys); a key that does not match falls back to the client address. Never use the raw header text as the bucket name. Add the test to tests/unit next to the existing rate-limit tests.</t>
+          <t>First list which arrays in the live bundle are object arrays (np.load each .npz with allow_pickle=False and note which fail). Rewrite those arrays in the builder as plain types (fixed-width strings, integer codes plus a JSON side file), rebuild the bundle, then switch the five np.load calls to allow_pickle=False and add the source-scan test.</t>
         </is>
       </c>
     </row>
@@ -815,27 +815,27 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SIM-565</t>
+          <t>SIM-566</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Load the engine bundle with allow_pickle=False</t>
+          <t>Move the fixed-query read routes onto the read-only pool</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>The simulator loads its prepared data files (the engine bundle) with numpy's allow_pickle=True setting, in pipeline/batch/engine_artifacts.py. That setting lets a data file carry a pickle, and loading a pickle can run code. Only our own nightly build writes the bundle, so the risk is small, but a tampered file in the data folder would run code in every simulator worker. The JSON cache work (SIM-443f) removed pickle from the Redis cache; this is the remaining pickle load on the hot path.</t>
+          <t>The SQL console now runs on a database login that can only read the raw tables (SIM-443e). Other read-only routes still use the main login, which can also write: the schema browser (/api/schema), the analytics pages (/api/analytics/*) and the player pages (/api/players/*). Their queries are fixed in code, not typed by a user, so the risk is low, but a defect in one of them runs with write access it never needs.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Every np.load of the bundle uses allow_pickle=False. The live bundle loads and the simulator runs a ten-game smoke with the same results as before. A unit test fails if any np.load in the loader passes allow_pickle=True.</t>
+          <t>/api/schema, /api/analytics/* and /api/players/* read through the read-only pool, and each answers 503 when that pool is missing. Every query they run reads only raw tables (or a route that needs sim.* is listed and kept on the main pool with the reason). The unit tests for those routes pass with a fake read-only pool.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>First list which arrays in the live bundle are object arrays (np.load each .npz with allow_pickle=False and note which fail). Rewrite those arrays in the builder as plain types (fixed-width strings, integer codes plus a JSON side file), rebuild the bundle, then switch the five np.load calls to allow_pickle=False and add the source-scan test.</t>
+          <t>Move sql_runner._ro_pool(request) into api/routes/_common.py as a shared helper and switch these routes to it. Check each query for a non-raw table first; the read-only role has no access to sim.* by design. Update docs/technical/api.md.</t>
         </is>
       </c>
     </row>
@@ -847,90 +847,58 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>SIM-566</t>
+          <t>SIM-567</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Move the fixed-query read routes onto the read-only pool</t>
+          <t>Pin the test lane's odds provider to the mock</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>The SQL console now runs on a database login that can only read the raw tables (SIM-443e). Other read-only routes still use the main login, which can also write: the schema browser (/api/schema), the analytics pages (/api/analytics/*) and the player pages (/api/players/*). Their queries are fixed in code, not typed by a user, so the risk is low, but a defect in one of them runs with write access it never needs.</t>
+          <t>The unit-test lane runs inside the app container, which reads the live .env. ODDS_PROVIDER=bettingpros leaks into the tests, so twelve tests in three files (the live pipeline's prop-odds tests and the odds-vocabulary tests) call the real BettingPros provider when they build the pipeline and fail with HTTP 404. They pass with ODDS_PROVIDER=mock. CI never sees this, because CI has no .env. Found while building the scheduled backups (SIM-525) on 2026-10-15.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>/api/schema, /api/analytics/* and /api/players/* read through the read-only pool, and each answers 503 when that pool is missing. Every query they run reads only raw tables (or a route that needs sim.* is listed and kept on the main pool with the reason). The unit tests for those routes pass with a fake read-only pool.</t>
+          <t>make test-unit on the serving stack passes those three files with no environment override, and no unit test reaches the vendor.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Move sql_runner._ro_pool(request) into api/routes/_common.py as a shared helper and switch these routes to it. Check each query for a non-raw table first; the read-only role has no access to sim.* by design. Update docs/technical/api.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="94.5" customHeight="1" s="15">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>SIM-567</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Pin the test lane's odds provider to the mock</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>The unit-test lane runs inside the app container, which reads the live .env. ODDS_PROVIDER=bettingpros leaks into the tests, so twelve tests in three files (the live pipeline's prop-odds tests and the odds-vocabulary tests) call the real BettingPros provider when they build the pipeline and fail with HTTP 404. They pass with ODDS_PROVIDER=mock. CI never sees this, because CI has no .env. Found while building the scheduled backups (SIM-525) on 2026-10-15.</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>make test-unit on the serving stack passes those three files with no environment override, and no unit test reaches the vendor.</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
           <t>Pin ODDS_PROVIDER=mock in tests/conftest.py, the way it already pins SIM_MANAGER and AUTH_DISABLED. Also note the whole-repo mount the SIM-525 build used for the lane (-v "$(pwd -W):/app"), so the container tests read the checkout's tests/ and compose file instead of the image's stale copies.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="94.5" customHeight="1" s="15"/>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+    <row r="13" ht="94.5" customHeight="1" s="15"/>
+    <row r="14" ht="94.5" customHeight="1" s="15">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F15" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
     </row>
     <row r="16" ht="54" customHeight="1" s="15"/>
   </sheetData>

</xml_diff>

<commit_message>
Record the SIM-569 deploy and file the stale nginx upstream after an app recreate (SIM-570)
The app service recreated with TRUSTED_PROXY_HOSTS=nginx and read nginx's
address inside the container. Port 80 then answered 502 until nginx
restarted: nginx resolves the app's name once, at its own start, and the
recreated container had a new address. The durable fix is SIM-570 (P3);
the next free ID is SIM-571.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>NEXT FREE TICKET ID: SIM-570</t>
+          <t>NEXT FREE TICKET ID: SIM-571</t>
         </is>
       </c>
     </row>
@@ -871,34 +871,66 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="94.5" customHeight="1" s="15"/>
-    <row r="14" ht="94.5" customHeight="1" s="15">
-      <c r="A14" s="7" t="inlineStr">
+    <row r="13" ht="94.5" customHeight="1" s="15">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>SIM-570</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>nginx keeps a stale app address after the app container is recreated</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>nginx resolves the app service's name once, when nginx starts, because its upstream block has no resolver directive. A `docker compose up -d app` recreates the app container, which then gets a new address on the compose network, and nginx keeps sending traffic to the old one. Every route on port 80 answers 502 while the app itself is healthy on its own port. Found on the SIM-569 deploy (2026-10-17): the app moved from 172.19.0.8 to 172.19.0.10 and the LAN entry was down until `docker compose restart nginx`. An in-place restart (`docker compose restart app`, the nightly self-restart of SIM-563) keeps the address and does not trigger it.</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>After `docker compose up -d app` recreates the app container, `curl http://localhost/health` through nginx answers 200 within 30 seconds with no nginx restart, and the WebSocket route still proxies. deploy/README.md says what nginx does on an address change.</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>In deploy/nginx/nginx.conf add `resolver 127.0.0.11 valid=10s ipv6=off;` (Docker's embedded DNS) and proxy to a variable (`set $app http://app:8000; proxy_pass $app;`) in each location, so nginx re-resolves the name on the TTL. A variable in proxy_pass bypasses the upstream block and its `keepalive 32`: measure the latency before and after, or keep the upstream block and add `resolve` to its server line if the nginx image's version supports it. A cheaper alternative: a Makefile target that recreates app and restarts nginx together.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="94.5" customHeight="1" s="15"/>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F14" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
     </row>
     <row r="16" ht="54" customHeight="1" s="15"/>
   </sheetData>

</xml_diff>

<commit_message>
Let nginx follow the app's address after a recreate (SIM-570)
nginx looked the app's name up once, at its own start, so a recreated app
container with a new address got 502 on every route until nginx
restarted. The upstream block now carries zone, a resolver on Docker's
embedded DNS (valid=10s, ipv6 off) and resolve on the server line
(open-source nginx 1.27.3+; the image runs 1.27.5); every location keeps
proxy_pass to the group, so its keep-alive stays. The config is baked
into the nginx image: built and recreated. Proven on the stack with a
holder container that took the freed address: the app moved .10 -> .11
and the route through nginx answered 200 the second the app was healthy,
nginx untouched. Five guard tests; the README says what nginx does on an
address change; the backlog row is deleted.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -871,66 +871,34 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="94.5" customHeight="1" s="15">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>SIM-570</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>nginx keeps a stale app address after the app container is recreated</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>nginx resolves the app service's name once, when nginx starts, because its upstream block has no resolver directive. A `docker compose up -d app` recreates the app container, which then gets a new address on the compose network, and nginx keeps sending traffic to the old one. Every route on port 80 answers 502 while the app itself is healthy on its own port. Found on the SIM-569 deploy (2026-10-17): the app moved from 172.19.0.8 to 172.19.0.10 and the LAN entry was down until `docker compose restart nginx`. An in-place restart (`docker compose restart app`, the nightly self-restart of SIM-563) keeps the address and does not trigger it.</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>After `docker compose up -d app` recreates the app container, `curl http://localhost/health` through nginx answers 200 within 30 seconds with no nginx restart, and the WebSocket route still proxies. deploy/README.md says what nginx does on an address change.</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>In deploy/nginx/nginx.conf add `resolver 127.0.0.11 valid=10s ipv6=off;` (Docker's embedded DNS) and proxy to a variable (`set $app http://app:8000; proxy_pass $app;`) in each location, so nginx re-resolves the name on the TTL. A variable in proxy_pass bypasses the upstream block and its `keepalive 32`: measure the latency before and after, or keep the upstream block and add `resolve` to its server line if the nginx image's version supports it. A cheaper alternative: a Makefile target that recreates app and restarts nginx together.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="94.5" customHeight="1" s="15"/>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+    <row r="13" ht="94.5" customHeight="1" s="15"/>
+    <row r="14" ht="94.5" customHeight="1" s="15">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F15" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
     </row>
     <row r="16" ht="54" customHeight="1" s="15"/>
   </sheetData>

</xml_diff>

<commit_message>
Delete the closed SIM-565 row from the backlog
Excel released the workbook; the changelog's held note is closed. The next free ID stays SIM-571.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -582,7 +582,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -783,27 +782,27 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SIM-565</t>
+          <t>SIM-566</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Load the engine bundle with allow_pickle=False</t>
+          <t>Move the fixed-query read routes onto the read-only pool</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>The simulator loads its prepared data files (the engine bundle) with numpy's allow_pickle=True setting, in pipeline/batch/engine_artifacts.py. That setting lets a data file carry a pickle, and loading a pickle can run code. Only our own nightly build writes the bundle, so the risk is small, but a tampered file in the data folder would run code in every simulator worker. The JSON cache work (SIM-443f) removed pickle from the Redis cache; this is the remaining pickle load on the hot path.</t>
+          <t>The SQL console now runs on a database login that can only read the raw tables (SIM-443e). Other read-only routes still use the main login, which can also write: the schema browser (/api/schema), the analytics pages (/api/analytics/*) and the player pages (/api/players/*). Their queries are fixed in code, not typed by a user, so the risk is low, but a defect in one of them runs with write access it never needs.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Every np.load of the bundle uses allow_pickle=False. The live bundle loads and the simulator runs a ten-game smoke with the same results as before. A unit test fails if any np.load in the loader passes allow_pickle=True.</t>
+          <t>/api/schema, /api/analytics/* and /api/players/* read through the read-only pool, and each answers 503 when that pool is missing. Every query they run reads only raw tables (or a route that needs sim.* is listed and kept on the main pool with the reason). The unit tests for those routes pass with a fake read-only pool.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>First list which arrays in the live bundle are object arrays (np.load each .npz with allow_pickle=False and note which fail). Rewrite those arrays in the builder as plain types (fixed-width strings, integer codes plus a JSON side file), rebuild the bundle, then switch the five np.load calls to allow_pickle=False and add the source-scan test.</t>
+          <t>Move sql_runner._ro_pool(request) into api/routes/_common.py as a shared helper and switch these routes to it. Check each query for a non-raw table first; the read-only role has no access to sim.* by design. Update docs/technical/api.md.</t>
         </is>
       </c>
     </row>
@@ -815,92 +814,62 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SIM-566</t>
+          <t>SIM-567</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Move the fixed-query read routes onto the read-only pool</t>
+          <t>Pin the test lane's odds provider to the mock</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>The SQL console now runs on a database login that can only read the raw tables (SIM-443e). Other read-only routes still use the main login, which can also write: the schema browser (/api/schema), the analytics pages (/api/analytics/*) and the player pages (/api/players/*). Their queries are fixed in code, not typed by a user, so the risk is low, but a defect in one of them runs with write access it never needs.</t>
+          <t>The unit-test lane runs inside the app container, which reads the live .env. ODDS_PROVIDER=bettingpros leaks into the tests, so twelve tests in three files (the live pipeline's prop-odds tests and the odds-vocabulary tests) call the real BettingPros provider when they build the pipeline and fail with HTTP 404. They pass with ODDS_PROVIDER=mock. CI never sees this, because CI has no .env. Found while building the scheduled backups (SIM-525) on 2026-10-15.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>/api/schema, /api/analytics/* and /api/players/* read through the read-only pool, and each answers 503 when that pool is missing. Every query they run reads only raw tables (or a route that needs sim.* is listed and kept on the main pool with the reason). The unit tests for those routes pass with a fake read-only pool.</t>
+          <t>make test-unit on the serving stack passes those three files with no environment override, and no unit test reaches the vendor.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Move sql_runner._ro_pool(request) into api/routes/_common.py as a shared helper and switch these routes to it. Check each query for a non-raw table first; the read-only role has no access to sim.* by design. Update docs/technical/api.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="94.5" customHeight="1" s="15">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>SIM-567</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Pin the test lane's odds provider to the mock</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>The unit-test lane runs inside the app container, which reads the live .env. ODDS_PROVIDER=bettingpros leaks into the tests, so twelve tests in three files (the live pipeline's prop-odds tests and the odds-vocabulary tests) call the real BettingPros provider when they build the pipeline and fail with HTTP 404. They pass with ODDS_PROVIDER=mock. CI never sees this, because CI has no .env. Found while building the scheduled backups (SIM-525) on 2026-10-15.</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>make test-unit on the serving stack passes those three files with no environment override, and no unit test reaches the vendor.</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
           <t>Pin ODDS_PROVIDER=mock in tests/conftest.py, the way it already pins SIM_MANAGER and AUTH_DISABLED. Also note the whole-repo mount the SIM-525 build used for the lane (-v "$(pwd -W):/app"), so the container tests read the checkout's tests/ and compose file instead of the image's stale copies.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="94.5" customHeight="1" s="15"/>
-    <row r="14" ht="94.5" customHeight="1" s="15">
-      <c r="A14" s="7" t="inlineStr">
+    <row r="12" ht="94.5" customHeight="1" s="15"/>
+    <row r="13" ht="94.5" customHeight="1" s="15">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F14" s="11" t="n"/>
-    </row>
-    <row r="16" ht="54" customHeight="1" s="15"/>
+      <c r="F13" s="11" t="n"/>
+    </row>
+    <row r="14" s="15"/>
+    <row r="15" ht="54" customHeight="1" s="15"/>
+    <row r="16" s="15"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>

<commit_message>
Record the SIM-566 close: the changelog, the API reference, the backlog row and SIM-571
- CHANGES.md: the entry for the Data Lab read routes on the read-only pool,
  with the gates, the reviews and the deploy note.
- docs/technical/api.md: _get_ro_pool and the constant in _common.py; the
  console, players, schema, analytics and data-freshness rows read the
  read-only pool; the public.similarity reason.
- CLAUDE.md and the security-hardening audit doc: SIM-566 CLOSED 2026-10-18.
- BACKLOG.xlsx: the SIM-566 row deleted; SIM-571 filed (the analytics swing,
  whiff and called-strike filters match Statcast codes, but raw.pitches holds
  the MLB Stats API's display text, so the rates read 0 on live data); the
  next free ID is SIM-572.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>NEXT FREE TICKET ID: SIM-571</t>
+          <t>NEXT FREE TICKET ID: SIM-572</t>
         </is>
       </c>
     </row>
@@ -782,27 +782,27 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SIM-566</t>
+          <t>SIM-567</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Move the fixed-query read routes onto the read-only pool</t>
+          <t>Pin the test lane's odds provider to the mock</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>The SQL console now runs on a database login that can only read the raw tables (SIM-443e). Other read-only routes still use the main login, which can also write: the schema browser (/api/schema), the analytics pages (/api/analytics/*) and the player pages (/api/players/*). Their queries are fixed in code, not typed by a user, so the risk is low, but a defect in one of them runs with write access it never needs.</t>
+          <t>The unit-test lane runs inside the app container, which reads the live .env. ODDS_PROVIDER=bettingpros leaks into the tests, so twelve tests in three files (the live pipeline's prop-odds tests and the odds-vocabulary tests) call the real BettingPros provider when they build the pipeline and fail with HTTP 404. They pass with ODDS_PROVIDER=mock. CI never sees this, because CI has no .env. Found while building the scheduled backups (SIM-525) on 2026-10-15.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>/api/schema, /api/analytics/* and /api/players/* read through the read-only pool, and each answers 503 when that pool is missing. Every query they run reads only raw tables (or a route that needs sim.* is listed and kept on the main pool with the reason). The unit tests for those routes pass with a fake read-only pool.</t>
+          <t>make test-unit on the serving stack passes those three files with no environment override, and no unit test reaches the vendor.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Move sql_runner._ro_pool(request) into api/routes/_common.py as a shared helper and switch these routes to it. Check each query for a non-raw table first; the read-only role has no access to sim.* by design. Update docs/technical/api.md.</t>
+          <t>Pin ODDS_PROVIDER=mock in tests/conftest.py, the way it already pins SIM_MANAGER and AUTH_DISABLED. Also note the whole-repo mount the SIM-525 build used for the lane (-v "$(pwd -W):/app"), so the container tests read the checkout's tests/ and compose file instead of the image's stale copies.</t>
         </is>
       </c>
     </row>
@@ -814,27 +814,27 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SIM-567</t>
+          <t>SIM-571</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Pin the test lane's odds provider to the mock</t>
+          <t>Match the analytics swing, whiff and called-strike filters to the pitch descriptions the loader stores</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>The unit-test lane runs inside the app container, which reads the live .env. ODDS_PROVIDER=bettingpros leaks into the tests, so twelve tests in three files (the live pipeline's prop-odds tests and the odds-vocabulary tests) call the real BettingPros provider when they build the pipeline and fail with HTTP 404. They pass with ODDS_PROVIDER=mock. CI never sees this, because CI has no .env. Found while building the scheduled backups (SIM-525) on 2026-10-15.</t>
+          <t>The Data Lab analytics routes (/api/analytics/count-state, /zone and the two leaderboards) compute swing, whiff, CSW and called-strike rates from the text in raw.pitches.description. Their filters look for Statcast's snake_case codes ('swinging_strike', 'called_strike', 'foul', 'hit_into_play', 'foul_tip', 'missed_bunt', 'foul_bunt'). The table holds the MLB Stats API's display text in every season ('Swinging Strike', 'Swinging Strike (Blocked)', 'Called Strike', 'Foul', 'Foul Tip', 'In play, out(s)', 'In play, no out', 'In play, run(s)', 'Missed Bunt', 'Foul Bunt'). On live data the swing rate reads 0, the whiff rate reads null and the called-strike and CSW rates read 0 for every pitcher and zone. The frontend's dashboard cards and leaderboards show those numbers. Found on 2026-10-18 by the SIM-566 review, which ran the routes on the live database; the simulator does not read these filters.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>make test-unit on the serving stack passes those three files with no environment override, and no unit test reaches the vendor.</t>
+          <t>The swing, whiff, CSW and called-strike rates on /api/analytics/count-state, /zone, /leaderboard/pitchers and /leaderboard/batters read plausible league values on live data (a swing rate near 47%, a whiff rate near 25%, a CSW rate near 28%). The filter vocabulary is one list, documented next to the queries, and a unit test checks every value in it against the distinct descriptions the loader stores (a fixture of the real values). The Data Lab dashboard cards show the rates.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Pin ODDS_PROVIDER=mock in tests/conftest.py, the way it already pins SIM_MANAGER and AUTH_DISABLED. Also note the whole-repo mount the SIM-525 build used for the lane (-v "$(pwd -W):/app"), so the container tests read the checkout's tests/ and compose file instead of the image's stale copies.</t>
+          <t>Replace the snake_case patterns in api/routes/analytics.py (_SWING, _WHIFF, the CSW and called-strike FILTER clauses) with the display-text values the table holds, in one frozen vocabulary; or, if the loader can also store the feed's code (pipeline/etl, the play event's details.code or call code), add that column and filter on it. Read the distinct descriptions per season first (SELECT season, description, count(*) FROM raw.pitches GROUP BY 1, 2); the ten values above cover 2017-2026. Add the vocabulary test. Check the frontend's number formatting on the restored rates.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record the SIM-567 close: the changelog and the backlog row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -582,6 +582,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -782,91 +783,60 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SIM-567</t>
+          <t>SIM-571</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Pin the test lane's odds provider to the mock</t>
+          <t>Match the analytics swing, whiff and called-strike filters to the pitch descriptions the loader stores</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>The unit-test lane runs inside the app container, which reads the live .env. ODDS_PROVIDER=bettingpros leaks into the tests, so twelve tests in three files (the live pipeline's prop-odds tests and the odds-vocabulary tests) call the real BettingPros provider when they build the pipeline and fail with HTTP 404. They pass with ODDS_PROVIDER=mock. CI never sees this, because CI has no .env. Found while building the scheduled backups (SIM-525) on 2026-10-15.</t>
+          <t>The Data Lab analytics routes (/api/analytics/count-state, /zone and the two leaderboards) compute swing, whiff, CSW and called-strike rates from the text in raw.pitches.description. Their filters look for Statcast's snake_case codes ('swinging_strike', 'called_strike', 'foul', 'hit_into_play', 'foul_tip', 'missed_bunt', 'foul_bunt'). The table holds the MLB Stats API's display text in every season ('Swinging Strike', 'Swinging Strike (Blocked)', 'Called Strike', 'Foul', 'Foul Tip', 'In play, out(s)', 'In play, no out', 'In play, run(s)', 'Missed Bunt', 'Foul Bunt'). On live data the swing rate reads 0, the whiff rate reads null and the called-strike and CSW rates read 0 for every pitcher and zone. The frontend's dashboard cards and leaderboards show those numbers. Found on 2026-10-18 by the SIM-566 review, which ran the routes on the live database; the simulator does not read these filters.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>make test-unit on the serving stack passes those three files with no environment override, and no unit test reaches the vendor.</t>
+          <t>The swing, whiff, CSW and called-strike rates on /api/analytics/count-state, /zone, /leaderboard/pitchers and /leaderboard/batters read plausible league values on live data (a swing rate near 47%, a whiff rate near 25%, a CSW rate near 28%). The filter vocabulary is one list, documented next to the queries, and a unit test checks every value in it against the distinct descriptions the loader stores (a fixture of the real values). The Data Lab dashboard cards show the rates.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Pin ODDS_PROVIDER=mock in tests/conftest.py, the way it already pins SIM_MANAGER and AUTH_DISABLED. Also note the whole-repo mount the SIM-525 build used for the lane (-v "$(pwd -W):/app"), so the container tests read the checkout's tests/ and compose file instead of the image's stale copies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="94.5" customHeight="1" s="15">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>SIM-571</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Match the analytics swing, whiff and called-strike filters to the pitch descriptions the loader stores</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>The Data Lab analytics routes (/api/analytics/count-state, /zone and the two leaderboards) compute swing, whiff, CSW and called-strike rates from the text in raw.pitches.description. Their filters look for Statcast's snake_case codes ('swinging_strike', 'called_strike', 'foul', 'hit_into_play', 'foul_tip', 'missed_bunt', 'foul_bunt'). The table holds the MLB Stats API's display text in every season ('Swinging Strike', 'Swinging Strike (Blocked)', 'Called Strike', 'Foul', 'Foul Tip', 'In play, out(s)', 'In play, no out', 'In play, run(s)', 'Missed Bunt', 'Foul Bunt'). On live data the swing rate reads 0, the whiff rate reads null and the called-strike and CSW rates read 0 for every pitcher and zone. The frontend's dashboard cards and leaderboards show those numbers. Found on 2026-10-18 by the SIM-566 review, which ran the routes on the live database; the simulator does not read these filters.</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>The swing, whiff, CSW and called-strike rates on /api/analytics/count-state, /zone, /leaderboard/pitchers and /leaderboard/batters read plausible league values on live data (a swing rate near 47%, a whiff rate near 25%, a CSW rate near 28%). The filter vocabulary is one list, documented next to the queries, and a unit test checks every value in it against the distinct descriptions the loader stores (a fixture of the real values). The Data Lab dashboard cards show the rates.</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
           <t>Replace the snake_case patterns in api/routes/analytics.py (_SWING, _WHIFF, the CSW and called-strike FILTER clauses) with the display-text values the table holds, in one frozen vocabulary; or, if the loader can also store the feed's code (pipeline/etl, the play event's details.code or call code), add that column and filter on it. Read the distinct descriptions per season first (SELECT season, description, count(*) FROM raw.pitches GROUP BY 1, 2); the ten values above cover 2017-2026. Add the vocabulary test. Check the frontend's number formatting on the restored rates.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="94.5" customHeight="1" s="15"/>
-    <row r="13" ht="94.5" customHeight="1" s="15">
-      <c r="A13" s="7" t="inlineStr">
+    <row r="11" ht="94.5" customHeight="1" s="15"/>
+    <row r="12" ht="94.5" customHeight="1" s="15">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F13" s="11" t="n"/>
-    </row>
+      <c r="F12" s="11" t="n"/>
+    </row>
+    <row r="13" ht="94.5" customHeight="1" s="15"/>
     <row r="14" s="15"/>
     <row r="15" ht="54" customHeight="1" s="15"/>
     <row r="16" s="15"/>

</xml_diff>

<commit_message>
Record the SIM-571 close: the changelog, the project guide and the backlog row
The changelog records the Data Lab vocabulary fix (SIM-571).
The entry holds the build, the gates, the reviews and the fixes.
The project guide closes the follow-up on its security line, in place.
The guide gains no line, so lines 911 and 914 keep their numbers.
The ticket's row leaves BACKLOG.xlsx. The next free ID stays SIM-572.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -575,15 +575,15 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" s="15">
       <c r="A2" s="14" t="inlineStr">
         <is>
           <t>NEXT FREE TICKET ID: SIM-572</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4">
+    <row r="3" s="15"/>
+    <row r="4" s="15">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Priority</t>
@@ -775,69 +775,38 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="94.5" customHeight="1" s="15">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>SIM-571</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Match the analytics swing, whiff and called-strike filters to the pitch descriptions the loader stores</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>The Data Lab analytics routes (/api/analytics/count-state, /zone and the two leaderboards) compute swing, whiff, CSW and called-strike rates from the text in raw.pitches.description. Their filters look for Statcast's snake_case codes ('swinging_strike', 'called_strike', 'foul', 'hit_into_play', 'foul_tip', 'missed_bunt', 'foul_bunt'). The table holds the MLB Stats API's display text in every season ('Swinging Strike', 'Swinging Strike (Blocked)', 'Called Strike', 'Foul', 'Foul Tip', 'In play, out(s)', 'In play, no out', 'In play, run(s)', 'Missed Bunt', 'Foul Bunt'). On live data the swing rate reads 0, the whiff rate reads null and the called-strike and CSW rates read 0 for every pitcher and zone. The frontend's dashboard cards and leaderboards show those numbers. Found on 2026-10-18 by the SIM-566 review, which ran the routes on the live database; the simulator does not read these filters.</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>The swing, whiff, CSW and called-strike rates on /api/analytics/count-state, /zone, /leaderboard/pitchers and /leaderboard/batters read plausible league values on live data (a swing rate near 47%, a whiff rate near 25%, a CSW rate near 28%). The filter vocabulary is one list, documented next to the queries, and a unit test checks every value in it against the distinct descriptions the loader stores (a fixture of the real values). The Data Lab dashboard cards show the rates.</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>Replace the snake_case patterns in api/routes/analytics.py (_SWING, _WHIFF, the CSW and called-strike FILTER clauses) with the display-text values the table holds, in one frozen vocabulary; or, if the loader can also store the feed's code (pipeline/etl, the play event's details.code or call code), add that column and filter on it. Read the distinct descriptions per season first (SELECT season, description, count(*) FROM raw.pitches GROUP BY 1, 2); the ten values above cover 2017-2026. Add the vocabulary test. Check the frontend's number formatting on the restored rates.</t>
-        </is>
-      </c>
+    <row r="10" ht="94.5" customHeight="1" s="15"/>
+    <row r="11" ht="94.5" customHeight="1" s="15">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Priority key:</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>P0 — immediate</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>P1 — next up</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>P2 — planned</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>P3 — later</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="n"/>
     </row>
-    <row r="11" ht="94.5" customHeight="1" s="15"/>
-    <row r="12" ht="94.5" customHeight="1" s="15">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>Priority key:</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>P0 — immediate</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>P1 — next up</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>P2 — planned</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="inlineStr">
-        <is>
-          <t>P3 — later</t>
-        </is>
-      </c>
-      <c r="F12" s="11" t="n"/>
-    </row>
-    <row r="13" ht="94.5" customHeight="1" s="15"/>
-    <row r="14" s="15"/>
+    <row r="12" ht="94.5" customHeight="1" s="15"/>
+    <row r="13" s="15"/>
+    <row r="14" ht="54" customHeight="1" s="15"/>
     <row r="15" ht="54" customHeight="1" s="15"/>
     <row r="16" s="15"/>
   </sheetData>

</xml_diff>

<commit_message>
Let the Data Lab read the regular season alone by default (SIM-572)
A season of raw.pitches holds the regular season and the postseason. The
Data Lab routes bounded each read with the season alone, so the
leaderboards mixed the two. In 2025 the postseason holds 47 games and
14,085 of the 723,055 clean pitches; the batter board showed Ohtani with
63 home runs against his 55 in the regular season.

The seven routes that take season now take game_type. 'R', the default,
keeps the pitches of regular-season games through a semi-join on
raw.games. 'all' adds no filter and reads as before. The coverage routes
(kpis, by-season) take no game type. The summary page gains a "Games"
choice. The new test file holds 43 tests; the SIM-571 tests carry the
default argument and a raw.games table. The ticket is filed in
BACKLOG.xlsx; the next free ID is SIM-573.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -578,7 +578,7 @@
     <row r="2" s="15">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>NEXT FREE TICKET ID: SIM-572</t>
+          <t>NEXT FREE TICKET ID: SIM-573</t>
         </is>
       </c>
     </row>
@@ -775,36 +775,67 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="94.5" customHeight="1" s="15"/>
-    <row r="11" ht="94.5" customHeight="1" s="15">
-      <c r="A11" s="7" t="inlineStr">
+    <row r="10" ht="150" customHeight="1" s="15">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>SIM-572</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Let the Data Lab read the regular season alone (the game-type filter)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>The Data Lab's analytics routes bound each read with the season alone. A season of raw.pitches holds the regular season and the postseason, so the leaderboards and the league rates mix the two. In 2025 the postseason holds 47 games and 14,085 of the 723,055 clean pitches. The batter board shows Shohei Ohtani with 63 home runs; his regular season ended at 55. raw.games marks the type of each game: 'R' is the regular season, and 'F', 'D', 'L' and 'W' are the four postseason rounds. The review of the Data Lab vocabulary fix (SIM-571) found the defect on 2026-10-19. The simulator does not read these routes.</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>The seven Data Lab routes that read the pitches of a season take a game_type parameter. 'R', the default, reads the regular season alone. 'all' reads every game of the season, as the routes did before. The 2025 batter board reads Ohtani at 55 home runs by default and at 63 with 'all'. The two coverage routes (kpis, by-season) keep reading every game. The routes stay on the read-only pool and read raw tables only. The summary page carries a choice between the regular season and every game. docs/technical/api.md and CHANGES.md describe the parameter. The owner decides whether the default stays the regular season.</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>In api/routes/analytics.py, add one filter to each of the seven routes: game_pk IN (SELECT g.game_pk FROM raw.games g WHERE g.game_type = $n), with the type as a query argument. The filter keeps a pitch when its game has the type. A plain join would clash on the season column, which both tables hold. 'all' adds no filter, so it reads exactly as before. Tests: the captured SQL carries the filter, DuckDB runs it over a postseason row, and a guard holds the parameter on every route. STATUS 2026-10-19: built and pushed on branch claude/interesting-newton-3ca06d, not merged. The owner decides the default and the merge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="94.5" customHeight="1" s="15"/>
+    <row r="12" ht="94.5" customHeight="1" s="15">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F11" s="11" t="n"/>
-    </row>
-    <row r="12" ht="94.5" customHeight="1" s="15"/>
+      <c r="F12" s="11" t="n"/>
+    </row>
     <row r="13" s="15"/>
     <row r="14" ht="54" customHeight="1" s="15"/>
     <row r="15" ht="54" customHeight="1" s="15"/>

</xml_diff>

<commit_message>
Bring the frontend's API snapshot and its generated types back in step with the API (SIM-573)
frontend/openapi.json had not been exported since 2026-10-09. Five
tickets changed the contract since then (the live slate, the game-page
what-if, the security hardening and the Data Lab game-type filter).
The old copy also came from the host, whose Pydantic 2.10 drops
"additionalProperties": true, so 17 free-form objects were typed as
Record<string, never>.

The export ran in the app image; npm run gen:api regenerated the types;
the frontend's type-check and lint pass with no code change. Two checks
keep the copy in step: a unit test compares it with app.openapi() (it
ignores only "additionalProperties": true, whose presence depends on
the Pydantic version), and the CI frontend job regenerates the types
and fails on any difference. The ticket is filed; the next free ID is
SIM-574.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -578,7 +578,7 @@
     <row r="2" s="15">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>NEXT FREE TICKET ID: SIM-573</t>
+          <t>NEXT FREE TICKET ID: SIM-574</t>
         </is>
       </c>
     </row>
@@ -807,36 +807,67 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="94.5" customHeight="1" s="15"/>
-    <row r="12" ht="94.5" customHeight="1" s="15">
-      <c r="A12" s="7" t="inlineStr">
+    <row r="11" ht="120" customHeight="1" s="15">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>SIM-573</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Bring the frontend's API snapshot and its generated types back in step with the API</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>frontend/openapi.json is a copy of the API's contract (its OpenAPI schema). openapi-typescript turns it into frontend/src/api/schema.d.ts, the frontend's typed API client. scripts/export_openapi.py writes the copy; nothing checks that anyone runs it. The last export was the live slate's (SIM-519, 2026-10-09). On 2026-10-19 a fresh export differed from the copy by about 1,600 added and 150 removed lines: several tickets changed the contract without an export. So the generated types no longer describe the API that the frontend calls.</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>frontend/openapi.json equals a fresh export of the app, and schema.d.ts equals a fresh generation from it. The frontend's type-check and lint pass. CHANGES.md lists the contract changes the export carries, grouped by ticket. A unit test fails when the copy differs from the app's schema, and its message names the command that fixes it.</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Run scripts/export_openapi.py in the app container, then npm run gen:api in frontend/. Fix any type error that the new types expose. Add tests/unit/test_sim573_openapi_snapshot.py: it compares app.openapi() with the copy and fails with the export command. STATUS 2026-10-19: built on branch claude/interesting-newton-3ca06d, stacked on the Data Lab game-type filter (SIM-572), so the copy matches the API that the merge lands. Not merged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="94.5" customHeight="1" s="15"/>
+    <row r="13" ht="94.5" customHeight="1" s="15">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F12" s="11" t="n"/>
-    </row>
-    <row r="13" s="15"/>
+      <c r="F13" s="11" t="n"/>
+    </row>
     <row r="14" ht="54" customHeight="1" s="15"/>
     <row r="15" ht="54" customHeight="1" s="15"/>
     <row r="16" s="15"/>

</xml_diff>

<commit_message>
Record the SIM-572 and SIM-573 close: the deploy, the live check, the backlog rows and the guide
Both tickets are merged (e06ad90, b43919e) and deployed. The app reloaded
on analytics.py at 18:03 UTC; nginx was rebuilt at 18:55 UTC and serves
the summary page's "Games" choice. The live API reads Ohtani at 55 home
runs by default and 63 with game_type=all. The two closed rows leave
BACKLOG.xlsx; the next free ID stays SIM-574. CLAUDE.md gains the SIM-572
follow-up note and, in section 15, the rule that an API contract change
ships a fresh snapshot.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -775,99 +775,37 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="150" customHeight="1" s="15">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>SIM-572</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Let the Data Lab read the regular season alone (the game-type filter)</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>The Data Lab's analytics routes bound each read with the season alone. A season of raw.pitches holds the regular season and the postseason, so the leaderboards and the league rates mix the two. In 2025 the postseason holds 47 games and 14,085 of the 723,055 clean pitches. The batter board shows Shohei Ohtani with 63 home runs; his regular season ended at 55. raw.games marks the type of each game: 'R' is the regular season, and 'F', 'D', 'L' and 'W' are the four postseason rounds. The review of the Data Lab vocabulary fix (SIM-571) found the defect on 2026-10-19. The simulator does not read these routes.</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>The seven Data Lab routes that read the pitches of a season take a game_type parameter. 'R', the default, reads the regular season alone. 'all' reads every game of the season, as the routes did before. The 2025 batter board reads Ohtani at 55 home runs by default and at 63 with 'all'. The two coverage routes (kpis, by-season) keep reading every game. The routes stay on the read-only pool and read raw tables only. The summary page carries a choice between the regular season and every game. docs/technical/api.md and CHANGES.md describe the parameter. The owner decides whether the default stays the regular season.</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>In api/routes/analytics.py, add one filter to each of the seven routes: game_pk IN (SELECT g.game_pk FROM raw.games g WHERE g.game_type = $n), with the type as a query argument. The filter keeps a pitch when its game has the type. A plain join would clash on the season column, which both tables hold. 'all' adds no filter, so it reads exactly as before. Tests: the captured SQL carries the filter, DuckDB runs it over a postseason row, and a guard holds the parameter on every route. STATUS 2026-10-19: built and pushed on branch claude/interesting-newton-3ca06d, not merged. The owner decides the default and the merge.</t>
-        </is>
-      </c>
+    <row r="10" ht="94.5" customHeight="1" s="15"/>
+    <row r="11" ht="94.5" customHeight="1" s="15">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Priority key:</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>P0 — immediate</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>P1 — next up</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>P2 — planned</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>P3 — later</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="n"/>
     </row>
-    <row r="11" ht="120" customHeight="1" s="15">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>SIM-573</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Bring the frontend's API snapshot and its generated types back in step with the API</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>frontend/openapi.json is a copy of the API's contract (its OpenAPI schema). openapi-typescript turns it into frontend/src/api/schema.d.ts, the frontend's typed API client. scripts/export_openapi.py writes the copy; nothing checks that anyone runs it. The last export was the live slate's (SIM-519, 2026-10-09). On 2026-10-19 a fresh export differed from the copy by about 1,600 added and 150 removed lines: several tickets changed the contract without an export. So the generated types no longer describe the API that the frontend calls.</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>frontend/openapi.json equals a fresh export of the app, and schema.d.ts equals a fresh generation from it. The frontend's type-check and lint pass. CHANGES.md lists the contract changes the export carries, grouped by ticket. A unit test fails when the copy differs from the app's schema, and its message names the command that fixes it.</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>Run scripts/export_openapi.py in the app container, then npm run gen:api in frontend/. Fix any type error that the new types expose. Add tests/unit/test_sim573_openapi_snapshot.py: it compares app.openapi() with the copy and fails with the export command. STATUS 2026-10-19: built on branch claude/interesting-newton-3ca06d, stacked on the Data Lab game-type filter (SIM-572), so the copy matches the API that the merge lands. Not merged.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="94.5" customHeight="1" s="15"/>
-    <row r="13" ht="94.5" customHeight="1" s="15">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Priority key:</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>P0 — immediate</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>P1 — next up</t>
-        </is>
-      </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>P2 — planned</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <t>P3 — later</t>
-        </is>
-      </c>
-      <c r="F13" s="11" t="n"/>
-    </row>
+    <row r="12" s="15"/>
+    <row r="13" s="15"/>
     <row r="14" ht="54" customHeight="1" s="15"/>
     <row r="15" ht="54" customHeight="1" s="15"/>
     <row r="16" s="15"/>

</xml_diff>

<commit_message>
Record the groundwork in CHANGES.md; file SIM-574; sessions list bugs instead of editing the workbook (SIM-493)
The CHANGES.md entry records Phase A: what each slice built, the error-path
changes on purpose, the gates (the full unit lane 6,545 passed, the
regression lane 33 passed, ruff, mypy, and all three fingerprint modes
identical to fe81d79), the script moves, and the 01:30 UTC incident where the
live app hot-reloaded the branch's code and hung on a full /dev/shm until a
forced recreate on master.

SIM-574 (P3) asks whether each SIM_* flag's code default should equal its
production value; 24 differ. Next free ID SIM-575. The plan's rule 2 changes:
an area session lists each bug in its CHANGES.md entry, and the integration
pass files them, because five branches cannot merge one binary workbook. Rule
11 forbids edits in the main checkout.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -578,7 +578,7 @@
     <row r="2" s="15">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>NEXT FREE TICKET ID: SIM-574</t>
+          <t>NEXT FREE TICKET ID: SIM-575</t>
         </is>
       </c>
     </row>
@@ -775,36 +775,67 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="94.5" customHeight="1" s="15"/>
-    <row r="11" ht="94.5" customHeight="1" s="15">
-      <c r="A11" s="7" t="inlineStr">
+    <row r="10" ht="81" customHeight="1" s="15">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>SIM-574</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Make each SIM_* flag's code default equal its production value, or record why it differs</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>The simulator reads its switches and weights from SIM_* environment flags. Each flag has a default in the code (the value an unset flag reads) and a production value set in the app service of docker-compose.yml. They differ for 24 of the flags compose sets (measured 2026-10-20): for example the pitch-draw cell index is off in code and on in production, and the fence stage, the fielding class filter and the manager draw are the same. So a script, a probe or a test that forgets one flag runs a different simulator from production, silently. The registry of the flags (simulation/flags.py, the code clean-up SIM-493) now lists every default in one table, which makes the gap visible but does not close it.</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>For every registered flag the code default equals the compose value, or the registry row says in one line why it differs (for example: the unit lane's byte-identical state). The unit lane's own pins in tests/conftest.py still hold its state. The fingerprint (scripts/behaviour_fingerprint.py) of production is unchanged, because compose already sets the production values.</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Owner decision first: should an unset flag mean production or off? If production: change each default in simulation/flags.py to the compose value, keep tests/conftest.py's pins for the unit lane, and add a registry test that the defaults equal compose. If off: add the reason column to the registry and a test that compose sets every flag whose default differs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="94.5" customHeight="1" s="15"/>
+    <row r="12" s="15">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F11" s="11" t="n"/>
-    </row>
-    <row r="12" s="15"/>
+      <c r="F12" s="11" t="n"/>
+    </row>
     <row r="13" s="15"/>
     <row r="14" ht="54" customHeight="1" s="15"/>
     <row r="15" ht="54" customHeight="1" s="15"/>

</xml_diff>

<commit_message>
File the clean-up's bugs, follow the moved builder version, and correct stale prose (SIM-493, Phase C)
- BACKLOG.xlsx: the 49 defects the five area sessions and the integration pass found are
  SIM-575 to SIM-623 (ten P2, the rest P3); the SIM-493 row goes with the clean-up's close;
  the next free ID is SIM-624.
- The steal-pool rebuild's tests patch POOL_BUILDER_VERSION on pipeline.batch.profiles.pool_meta,
  the module whose global both builders read.
- Docstrings and the technical docs name the new homes: the accuracy comparison's library
  code in scripts/accuracy/, recency_weight and the pool builder in pipeline/batch/profiles/,
  and the park-factor sentinel in the API's kwargs resolver; the middleware no longer names
  the deleted park-factor flag.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -172,6 +172,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -557,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -578,7 +581,7 @@
     <row r="2" s="15">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>NEXT FREE TICKET ID: SIM-575</t>
+          <t>NEXT FREE TICKET ID: SIM-624</t>
         </is>
       </c>
     </row>
@@ -647,199 +650,1730 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="230.1" customHeight="1" s="15">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
+    <row r="6" ht="141" customHeight="1" s="15">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>SIM-493</t>
+          <t>SIM-575</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Break up the oversized simulation-loop file, and run the project-wide code-hygiene refactor</t>
+          <t>Read each manager's profile in the API's runs, so the steal draw's manager weight is not flat</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>The single code file that runs the pitch-by-pitch game simulation has grown very large (3,258 lines) as features were added, which makes it hard to review and maintain safely. The team deliberately postponed this cleanup until the pitch-speed and pitch-realism work settled. On 2026-09-16 the owner widened the ticket to a generalized refactor of the project. Three habits have accumulated. (1) Scripts are named after the ticket that created them, not after what they do: 26 of the 43 scripts carry a SIM-number prefix, and every model change since the fatigue weight is graded with a general tool called sim518_pair_accuracy.py (the paired accuracy comparison), so a reader cannot tell a general tool from a one-off probe. (2) Run outputs sit next to code: scripts/ holds 140 ticket-prefixed files, 114 of them results (JSON, logs, text), 40 of those committed. (3) Five source files are over 2,500 lines each: the profile computor (7,732), the accuracy comparison (3,488), the simulation loop (3,258), the full-pool sampler (3,139) and the artifact builder (2,889). Smaller items: about 2,300 SIM-number tags in code comments across 220 tickets (one tag, SIM-421, has two meanings); the 'does this column exist' probe is written about 20 times across the engines, the calibrator and the league writer; the 45 SIM_* environment flags have no single registry of their defaults and owners.</t>
+          <t>The steal draw weighs each row by the batting manager's measured steal rate over the league mean. The API's runs (/simulate, the projections and the what-if) never read the manager profiles. build_sim_kwargs passes con=_get_sim_duckdb(request), and nothing sets app.state.sim_duckdb since the replay store moved to app.state.replay_duckdb. So resolve_manager_profiles_onto_state(state, None) returns at once, the kwargs carry manager_profiles == {0: {}, 1: {}}, and the manager weight reads 1.0 for every team. scripts/sim_stats.py and the accuracy comparison do read the profiles, so the lanes and the users run different simulators. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>The simulator behaves the same before and after, confirmed by the unit and regression lanes and one 45 x 130 acceptance lane on the balanced game set. Every script is named for what it does (the paired accuracy comparison first); the shell wrappers, the plans, the technical docs and CHANGES.md point at the new names. Run outputs live outside scripts/ in a results folder that git ignores; the committed ones are moved to docs/audit/ or deleted. The five files over 2,500 lines are split by responsibility. A ticket tag in a code comment says what the work was, not only its number, or is dropped where the git history already records it. One shared column-probe helper; one registry of the SIM_* flags with each flag's default and owner ticket. Ruff, mypy and CI green.</t>
+          <t>An API run's kwargs carry each side's manager profile and the season's manager league means. A unit test builds the API's kwargs with no DuckDB connection on app.state and finds both.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Do it in slices, one commit each, every slice behaviour-neutral. (1) Rename the paired accuracy tool to pair_accuracy.py and the other general tools by purpose; move the one-off probes under scripts/probes/. (2) Move the run outputs out of scripts/ and add the ignore rule. (3) Split sim_loop.py by responsibility (the pitch draw, the fielding stage, the runner draws, the manager decisions, the box credit), then the other four large files. (4) The shared helpers: the column probe, the flag registry. (5) The comment tags. Timing: the joint fit (SIM-548) is paused until the model is final; run slice 3 before that fit resumes or after it finishes, never while an arm is running.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="81" customHeight="1" s="15">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>Read the profiles through open_sim_duckdb(), as the park-factor snapshot does, or load them into the boot snapshot and read them from there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="114" customHeight="1" s="15">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>SIM-576</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Write the catcher engine's feature names in the catcher's league-average row</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>The profile computor writes the catcher row of derived.league_averages with the keys framing_runs, blocking_runs and cs_rate. The catcher engine reads its eleven feature names with pj.get(f, 0.0) or 0.0, and only cs_rate matches. So the shrinkage pulls ten features toward 0.0: a constructed 300-pitch catcher reads pop time 1.95 -&gt; 1.857 s and arm strength 81 -&gt; 77.1 mph. The error reaches the catcher and catcher_throwing score matrices, which weight the steal and pickoff draws. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>The catcher's league row carries every engine feature. A missing key reads as NaN, as the steal engines do. The nightly matrices are rebuilt.</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>In pipeline/batch/profiles (the catcher league row), write the engine's eleven feature keys. In similarity/engines/catcher_similarity.py _load_league_averages, read a missing key as NaN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="127.5" customHeight="1" s="15">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>SIM-577</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Write all thirteen features in the extra-base runner's league-average row</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>The baserunner row of derived.league_averages holds extra_base_attempt_rate, extra_base_success_rate, sb_success_rate, sprint_speed and the Savant rate. The engine reads thirteen features, so the four per-situation attempt rates, stop_rate and the four per-situation success rates shrink toward 0.0. The matrix build loads the thin profiles, so the effect is large there: a 5-chance runner's first-to-third attempt rate reads 0.35 -&gt; 0.088. The error reaches the runner_adv matrix, which weights the advancement draws. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>The runner's league row carries every engine feature, and a missing key reads as NaN. The nightly matrices are rebuilt.</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Write the engine's thirteen feature keys in the computor's baserunner league row; read a missing key as NaN in similarity/engines/baserunner_similarity.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="114" customHeight="1" s="15">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>SIM-578</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Load a database NULL as NaN, not 0.0, in the baserunner, catcher, batter and manager engines</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>The _v helpers of four engines read v or 0.0. A runner with no Savant row gets sprint speed 0 ft/s (still 20 ft/s after a 5-chance shrink, many deviations below the league's 27), so his speed score is about 0 against every measured runner. A runner who never tried reads 0% success; a NULL arm strength reads 0 mph; a manager-season with no bullpen-availability rows reads available_reliever_usage_rate near 0. The two steal engines already load NaN (the running-game work, SIM-531). Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Each of the four engines loads NULL as NaN, and its kernel or shrink handles a NaN feature. The nightly matrices are rebuilt.</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Map None to NaN in each _v helper and add the features to each engine's NaN set, as the steal engines do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="114" customHeight="1" s="15">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>SIM-579</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Select the pitcher's zone-take rate before the chase rate, so the two stay in feature order</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>In similarity/engines/pitcher_similarity.py _load_profiles, the SELECT returns chase_rate, zone_take_rate and the unpack names them zone_take_rate, chase_rate. So command_vec holds them in the opposite order to COMMAND_FEATURES and the league-average vector, and the shrinkage pulls each pitcher's chase rate toward the league's zone-take rate (weight 1 - alpha, at most 2.4% at 200 pitches). The kernel itself ignores the order. The error reaches the pitcher similarity matrix. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>The SELECT order matches COMMAND_FEATURES, and a unit test pins it. The nightly matrices are rebuilt.</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Select zone_take_rate before chase_rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="114" customHeight="1" s="15">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>SIM-580</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Make the pitcher arsenal fit reproducible: order the pitch rows before the mixture fit</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>The pitch-vector query in _compute_pitcher_profiles (pipeline/batch/profiles/pitcher.py) has no ORDER BY. DuckDB's parallel Postgres scan returns the rows in a different order on every read, and the seeded mixture fit (random_state=42) depends on the row order. So every profile rebuild gives a different arsenal for nearly every pitcher (a different number of components for about one pitcher in five), and with it a different pitcher similarity matrix. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Two profile builds of the same code from the same data write the same arsenals, by content.</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Add ORDER BY game_pk, at_bat_number, pitch_number to the query. It changes every arsenal once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="87" customHeight="1" s="15">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>SIM-581</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Name only real tests in the nightly acceptance lane's required roster</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>The REQUIRED roster of .github/workflows/acceptance-nightly.yml lists test_full_pool_out_advancement_runs_sim450, test_full_pool_steal_decision_runs_sim450 and test_reach_on_error_band_sim450. No test of those names exists, and the roster step fails when a required name did not run. So the nightly lane reds on every run, whatever the bands read. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>The roster names only real tests, and one nightly run passes its roster step.</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Delete the three names, or name the tests that took their place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="114" customHeight="1" s="15">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>SIM-582</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Add last_seen_at to the two odds archive tables, so the retirement copy fits again</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Migration 0029 added last_seen_at to raw.game_odds and raw.prop_odds and not to their archives (raw.game_odds_archive, raw.prop_odds_archive, migration 0028). The retirement script copies rows with INSERT ... SELECT *, which needs the same columns in the same order, so the next retirement fails. The integration test test_schema_migrations.py::test_sim555_stamp_indexes_and_archives reds on master fe81d79 and on the clean-up branch for this reason. Found by the code clean-up (SIM-493, the integration pass, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Both archives carry last_seen_at in the live table's position, the integration test passes, and a retirement run copies a row.</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>A new Alembic migration adds last_seen_at to both archives (nullable, so the copied rows keep their value), placed after book_line_at to match the live tables; check the column order with the test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="73.5" customHeight="1" s="15">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>SIM-583</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Keep the calibrated win probability strictly between 0 and 1</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>build_validation_report fits the reliability curve with min_bin_count=1, so a bin of two games can map 0.75 to 1.0. Example: the curve [[0,0],[0.45,0.44],[0.55,0.56],[0.73,1.0],[1,1]] and home_win_pct 0.75 at n = 100 give home 1.0, away 0.0 and an interval of zero width. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>No calibrated probability is 0.0 or 1.0, and a unit test feeds the curve above.</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Fit the curve with a min_bin_count near 30, or clamp the mapped probability to [eps, 1 - eps].</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="127.5" customHeight="1" s="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>SIM-584</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Stamp the accuracy report with the bundle the run read, not the live link</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>scripts/accuracy/selection.py bundle_provenance reads the manifest times under BASEBALL_PLAY_POOL_DIR/engine_artifacts (the live link). The factory reads BASEBALL_ENGINE_ARTIFACT_DIR when it is set (simulation/production_factory.py). Seen on 2026-10-20: two runs on the same pinned bundle, before and after the nightly rebuild, carry different manifest_mtimes and identical records, so pair_accuracy.py refuses to pair them; two runs on different pinned bundles on one day would pair. The weight fit (SIM-548) pairs these reports. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>The stamp names the bundle the run read, and a test pins the pinned-directory case.</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Read the pinned directory first, as the factory does.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="81" customHeight="1" s="15">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
           <t>SIM-547</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/probes/manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="81" customHeight="1" s="15">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
+    <row r="17" ht="81" customHeight="1" s="15">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>SIM-526</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Turn on the catcher pitch-receiving factor</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="81" customHeight="1" s="15">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
+    <row r="18" ht="81" customHeight="1" s="15">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>SIM-556</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/probes/steal_weight_volume_probe.py with its records (docs/audit/records/steal_weight_volume_probe_2025.* and _2026.*; the arrays in results/steal_weight_volume/). Filed P3 by the owner on 2026-10-01.</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/probes/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="81" customHeight="1" s="15">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
+    <row r="19" ht="81" customHeight="1" s="15">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>SIM-574</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Make each SIM_* flag's code default equal its production value, or record why it differs</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>The simulator reads its switches and weights from SIM_* environment flags. Each flag has a default in the code (the value an unset flag reads) and a production value set in the app service of docker-compose.yml. They differ for 24 of the flags compose sets (measured 2026-10-20): for example the pitch-draw cell index is off in code and on in production, and the fence stage, the fielding class filter and the manager draw are the same. So a script, a probe or a test that forgets one flag runs a different simulator from production, silently. The registry of the flags (simulation/flags.py, the code clean-up SIM-493) now lists every default in one table, which makes the gap visible but does not close it.</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>For every registered flag the code default equals the compose value, or the registry row says in one line why it differs (for example: the unit lane's byte-identical state). The unit lane's own pins in tests/conftest.py still hold its state. The fingerprint (scripts/behaviour_fingerprint.py) of production is unchanged, because compose already sets the production values.</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>Owner decision first: should an unset flag mean production or off? If production: change each default in simulation/flags.py to the compose value, keep tests/conftest.py's pins for the unit lane, and add a registry test that the defaults equal compose. If off: add the reason column to the registry and a test that compose sets every flag whose default differs.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="94.5" customHeight="1" s="15"/>
-    <row r="12" s="15">
-      <c r="A12" s="7" t="inlineStr">
+    <row r="20" ht="87" customHeight="1" s="15">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>SIM-585</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Refuse CORS_ORIGINS=* while the API sends credentials</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>api/main.py sets allow_credentials=True for every origin list, and resolve_cors_origins (api/auth.py) returns ['*'] when an operator sets CORS_ORIGINS=*. Starlette then echoes the caller's Origin on a request with a cookie, so any site can read the API with the user's login. Production sets neither variable today, so the defect is latent. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>CORS_ORIGINS=* either fails the boot or turns credentials off, and a unit test pins it.</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Refuse '*' in resolve_cors_origins while credentials are on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="60" customHeight="1" s="15">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>SIM-586</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Ask the schedule only for game types raw.games accepts</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>GAME_TYPES (pipeline/live/ingestion/constants.py) is R F D L W C P; the CHECK on raw.games allows R P S A D F L W. A game of type C on the slate fails its upsert. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>The live pipeline's game types and the table's CHECK agree, and a unit test compares them.</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Drop C from GAME_TYPES, or widen the CHECK with a migration if type C games should load.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="87" customHeight="1" s="15">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>SIM-587</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Decide which calibration values the draws use, and make the code follow</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>similarity/calibration/pitcher.py fits sigma_command and eb_n_prior_pitcher, and no code reads either, so the pitcher engine keeps RBF_SIGMA_COMMAND 1.0453 and EB_N_PRIOR 5. More broadly, the nightly actor matrices apply no calibration report (build_actor_sim_matrices): make calibrate changes only the API's engines. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>The owner decides which values the draws use, and the code and the docs follow.</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Read both fields in apply_calibration and apply /data/calibration.json in the matrix build; or document the module defaults as the draws' values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="46.5" customHeight="1" s="15">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>SIM-588</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Compute the z of the requested level in GameSimSummary.from_results</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>GameSimSummary.from_results(confidence_level=0.85) computes the 95% z and labels the intervals 0.85. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Each level gets its own z, and a unit test checks 0.85.</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Use NormalDist().inv_cdf((1 + level) / 2), or raise on a level outside the table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="73.5" customHeight="1" s="15">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>SIM-589</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Treat both samples as samples in the replay chi-squared test</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>The two-sample path of replay_chi_squared.chi_squared_gof treats the reference sample as exact. Two independent samples of 1,000 Poisson(4.4) totals were rejected 52.5% of the time at alpha 0.05 over 400 trials. replay_and_test uses it. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Two samples from one distribution are rejected near alpha.</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Use scipy.stats.chi2_contingency on the pooled 2 x k table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="60" customHeight="1" s="15">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>SIM-590</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Compare the historical replay against the right side's score</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>replay_historical_games always compares the simulated HOME score. A HistoricalGame row does not say which side its runs belong to, so an away team's runs meet the simulated home runs. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>A HistoricalGame row names its side, and the replay compares like with like.</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Add a side field to HistoricalGame.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="73.5" customHeight="1" s="15">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>SIM-591</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Charge the losing pitcher with the go-ahead run, as MLB does</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>pitcher_decisions charges the pitcher on the mound at the decisive play. In a tie, A walks a batter, B relieves him and allows a double that scores the runner, and the lead holds: MLB charges A; the simulator charges B. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>The decision follows the runner's responsible pitcher, and a unit test plays the example.</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Carry each runner's responsible pitcher on the bases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="73.5" customHeight="1" s="15">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>SIM-592</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Put the batter on first after a forced reach with no batter id</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>_force_on_reach with no batter id leaves first base's runner on first after pushing him to second (b.first = state.batter_id if ... else b.first), so the base check raises; _resolve_walk assigns b.first = state.batter_id for the same case. Reachable only with a sampler and no lineup. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>The forced reach and the walk give the same bases.</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Use the walk's assignment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="73.5" customHeight="1" s="15">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>SIM-593</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Void the plate appearance after a third out on the bases in the single pre-pitch steal draw</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>With SIM_STEAL_PITCH_CLASS=0 (not production), a pickoff or a caught stealing that makes the third out before the pitch's result still ends the plate appearance, so the pitcher gets a batter faced and the batter an at-bat. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>The single draw voids the plate appearance as the running game on the pitch does.</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Apply the no-pitch void of the class-aware draw.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="60" customHeight="1" s="15">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>SIM-594</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Let the batter run on a called third strike that gets away</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Rule 5.05(a)(2) lets the batter run on any uncaught third strike. _dropped_third_strike reads swinging strikes only. Two such rows exist in 2023-2026, both in 2026. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>A called third strike that gets away can be a dropped-third-strike reach.</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Let _dropped_third_strike read a called third strike too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="46.5" customHeight="1" s="15">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>SIM-595</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Fix the article in the what-if's ineligible-player message</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>whatif.apply_changes' message for an ineligible pinch hitter reads 'is not an bench hitter'. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Each label reads with its own article.</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Put the article inside each label.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="60" customHeight="1" s="15">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>SIM-596</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Decide what the what-if does when the designated hitter takes the field</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>A designated hitter moved to the field leaves the fielder he replaced in the batting order with no position. The rule that ends the designated hitter is not modelled in simulation/whatif.py. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>The owner decides whether the what-if models the rule, and the code follows.</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Model the rule: the pitcher bats in the replaced fielder's slot, or refuse the change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="87" customHeight="1" s="15">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>SIM-597</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Write the pitching-change pool's role file in a fixed row order</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>roles.parquet (build_pitching_change_pool, pipeline/batch/artifacts/manager_pool.py) is written from a GROUP BY with no ORDER BY, so two builds of the same code from the same data write its rows in a different order. No reader uses the order, but the fingerprint's bundle mode reads a difference on every build. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Two builds give the same file, by content.</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Add ORDER BY pitcher_id, season. It changes no game.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="60" customHeight="1" s="15">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>SIM-598</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Read the runners under the names the live service sends</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>frontend/src/hooks/useGameSocket.ts reads runner_on_first / _second / _third; the live service sends on_1b / on_2b / on_3b. The hook's on_1b to on_3b are always undefined. No page reads them today. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>A game_state_update with runners fills the hook's on_1b to on_3b.</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Read gs.on_1b, gs.on_2b and gs.on_3b in mapWsState.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="73.5" customHeight="1" s="15">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>SIM-599</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Describe the slate card's odds field as it is</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>The route description (api/routes/games_slate.py) and the model (api/routes/games_models.py) call the field 'reserved for the Phase-6 odds-provider integration (SIM-405)'. The field is always None: the card's lines come from /api/betting/games/{pk}/card-odds. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Both texts say that, with a fresh API snapshot (CLAUDE.md section 15).</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Rewrite both texts; run scripts/export_openapi.py in the image and npm run gen:api.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="46.5" customHeight="1" s="15">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>SIM-600</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Name the current state in the API's version and health strings</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>api/main.py carries the app version 0.1.0-phase7, "phase": "6" on /health and "6 - Frontend Build (in progress)" on /. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>The strings name the current state, or go.</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Drop the phase keys and set the version from one constant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="87" customHeight="1" s="15">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>SIM-601</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Make the Playwright smoke tests pass while the live app runs</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>frontend/e2e/smoke.spec.ts (three specs) fail on the owner's host: a request the test does not mock goes through the preview server's proxy to localhost:8000, the live app answers 401 and the page shows the login. With API_TARGET=http://127.0.0.1:9 all 21 tests pass; CI has no backend, so CI passes. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>The e2e suite passes with the live app running.</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Set API_TARGET to a closed port in playwright.config.ts's webServer.env, or end each spec with a catch-all **/api/** route that answers 404.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="73.5" customHeight="1" s="15">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>SIM-602</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Make two API tests check what their names say</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>tests/unit/test_api_betting.py test_clv_snapshot_returns_only_series_with_clv makes a GET and asserts nothing. tests/unit/test_api_games_plays.py test_simulate_ok_without_duckdb_then_plays_404 never requests /plays. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Each test asserts what its name says.</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Add the assertions (the CLV series' filter; /plays answers 503 with no replay store), then rename the second test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="100.5" customHeight="1" s="15">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>SIM-603</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Return the fielder's infield sub-scores in the same order from query_pair as from query</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>For an infielder, similarity/engines/fielder_similarity.py query_pair returns the specialty score in tertiary_score and the error score in quaternary_score; query returns them the other way round, as the Similarity Explorer's labels expect. Two shortstops with different error rates and equal specialty values: query gives 0.0710 / 1.0000, query_pair 1.0000 / 0.0710. The composite and the matrices are right. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>query and query_pair agree on every sub-score, and a unit test compares them.</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Map the infield tuple in SimilarityResult order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="100.5" customHeight="1" s="15">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>SIM-604</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Apply the per-hand 30-PA platoon rule in the batter engine's pair score</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>similarity/engines/batter_similarity.py _score_pair disagrees with score_all on a thin platoon split. A query with 30+ PA against either hand turns the platoon weights on for any vs_hand (10 PA vs L and 200 vs R with vs_hand='L': 0.8642 against 0.8900), and a candidate under 30 PA never gets the neutral 0.5. It serves query_pair (the Explorer's pair view and the diagnostics); the matrix is unaffected. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>_score_pair and score_all agree, and a unit test compares them.</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Use score_all's per-hand rule in _score_pair.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="73.5" customHeight="1" s="15">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>SIM-605</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Keep one pitcher engine's calibration from rewriting every pitcher engine</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>PitcherSimilarityEngine.apply_calibration sets the module global ARSENAL_SCALE, and a report with no gamma resets it to 4.10. The API builds two instances. Latent: no production path calls it today. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Each instance carries its own scale.</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>Pass the instance's scale into the three readers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="60" customHeight="1" s="15">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>SIM-606</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Pick the small-mixture-component merge target in standardized units</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>enforce_min_cluster_size runs before the standardization in the arsenal build, so spin rate (hundreds of rpm) decides the merge over velocity and movement. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>The merge measures the gap in standardized units.</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>Measure the gap over the mixture's feature_stds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="73.5" customHeight="1" s="15">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>SIM-607</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Read the line-movement direction book by book</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>betting/line_movement.py _net_direction pools every book, so the first and last quotes can come from two books: (t1, bp:1, -110/-110) and (t2, bp:2, -130/+110) give direction 'toward' and a CLV, though neither book moved. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>The direction is each book's own, then aggregated.</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>Compute the direction per book, then aggregate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="73.5" customHeight="1" s="15">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>SIM-608</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Store a price that returns to an earlier value</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>The odds writer dedups on a hash with no time (ON CONFLICT (game_pk, source, odds_hash)), so -110 at t0, -120 at t1, -110 at t2 closes the series at -120. Read from the code, not checked against stored data. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>A return to an earlier price is stored, and the series closes on the last price.</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>Dedup only against the latest row of the same game, source, book, market and line type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="46.5" customHeight="1" s="15">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>SIM-609</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Raise on a wrong market or side in the line-movement series</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>line_movement_from_quotes swallows _side_columns' ValueError, so a wrong market or side gives a silent empty series. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>A wrong market or side raises.</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>Call _side_columns once before the loop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="154.5" customHeight="1" s="15">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>SIM-610</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Similarity and betting: seven small defects</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>(1) SituationSimilarityEngine.query_batch([]) raises instead of returning []. (2) The engines' and the calibrator's __main__ blocks read a DuckDB path that does not exist (../../db/schemas/baseball_simulator.duckdb); the pitcher engine's block builds and prints nothing. (3) CalibrationReport.summary() prints no row for the batter's physical weights. (4) The Similarity Explorer's batter panel (api/routes/similarity_explorer.py) shows the four-way weights 0.40/0.35/0.15/0.10. (5) A log line in batted_ball_similarity.py says 'until SIM-051 ships'. (6) tests/regression/conftest.py scales the situation fixture's index twice. (7) No writer sets is_sharp_book, so sharp_consensus is always None. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Each of the seven is fixed or retired.</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>One edit each; retire sharp_consensus if no book will be marked sharp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="127.5" customHeight="1" s="15">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>SIM-611</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Owner decisions: four similarity design points</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Not defects, design points for the owner. (1) The catcher's shrinkage prior is 15 called pitches, so alpha is at least 0.95 for every kept catcher (framing stabilizes near 1,500). (2) stop_rate is exactly one minus the overall attempt rate, so that rate counts twice in the runner's aggression distance. (3) The batter's xba / xslg and the manager's hit-and-run and double-switch rates read 0.0 for everyone and still hold their share of the kernel weight. (4) CLAUDE.md section 1 calls CLV 'the gold-standard metric'; the owner ruled on 2026-09-28 that the model is not judged by it. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>The owner rules on each point, and the code or CLAUDE.md follows.</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>Raise the catcher prior; drop stop_rate; drop the all-zero features; rewrite CLAUDE.md section 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="60" customHeight="1" s="15">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>SIM-612</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Read the pitch rebuild's before-smoke from results/</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>scripts/pitch_pool_rebuild/export.py _smoke_games opens scripts/sim553_smoke_before.json; the groundwork moved run outputs to results/sim553/. The function always prints its placeholder. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>It reads the results/ path.</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>Change the one path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="87" customHeight="1" s="15">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>SIM-613</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Print n/a in the hypothetical-return table when no bet qualifies</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>scripts/accuracy/hypothetical_return.py _fmt_row formats the means and the range with :.4f and no guard for None. With no qualifying bet the table raises TypeError, and run() prints it before it writes the report and before the zero-games check, so the run ends in a traceback with no report and no exit code 5. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>The table prints n/a, as the accuracy table does.</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>Use the _fmt_or_na guard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="73.5" customHeight="1" s="15">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>SIM-614</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Retry a sweep attempt that crashes before its first game</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>scripts/resumable_sweep.py applies its zero-progress stop (gained == 0) after a crash too, so a segfault before the first game of an attempt ends the sweep (exit 1) instead of retrying. Found by reading the code; not exercised. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>A crashed attempt with no gain retries up to --max-attempts.</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>Apply the stop only to an attempt that exited cleanly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="73.5" customHeight="1" s="15">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>SIM-615</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Retire the odds-hash backfill probe</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>scripts/probes/backfill_odds_hash.py _dedup_rows orders by received_at, a column raw.game_odds does not have, so its DELETE fails; its ODDS_COLUMNS leaves out draw_ml. Both are dormant: the unique index and the NOT NULL hash of migration 0012 ended the probe's job. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>The probe is retired.</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Delete the probe and its test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="87" customHeight="1" s="15">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>SIM-616</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Decide the minimum-sample read's two known limits</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>scripts/accuracy/confidence.py: the 0.02 floor assumes a coin-flip market, so its power is weaker than stated for a market far from 0.5 (a home-run prop); and a small sample whose observed spread is exactly zero reads as fully resolved. An adversarial review of the minimum-sample work (SIM-539) found both. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>The owner decides whether to fix or accept them.</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>A per-market 4p(1-p) correction and an upper bound on the spread.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="181.5" customHeight="1" s="15">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>SIM-617</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Correct the runtime texts that state something false</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Left unedited by the clean-up's rule. (1) The park-guard messages name the deleted SIM_PARK_FACTOR: scripts/validate_props.py, scripts/accuracy_comparison.py, tests/acceptance/conftest.py and the --help of scripts/sim_stats.py. (2) The two pool rebuilds' exit-3 texts and the steal rebuild's lock message blame the app's worker server for the DuckDB lock (the app holds no handle since SIM-524), and two steal-rebuild texts say to merge code that is merged. (3) scripts/running_game_replay.py --help says a steal can land on any pitch in production. (4) Three texts point at a module docstring section that moved in the split. (5) scripts/measure_filter_cells.py writes into docs/audit/. (6) scripts/resumable_sweep.py --help cites a deleted record. (7) The rationale strings in tests/acceptance/bands.py cite BACKLOG.md, which is gone. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Each text says what is true.</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>One edit per text; list the runtime-string changes in CHANGES.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="60" customHeight="1" s="15">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>SIM-618</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Keep one copy of the prop ground-truth readers</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>scripts/validate_props.py and scripts/accuracy/grading.py each define _fetch_official_boxscore and _fetch_pa_events. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>One reader, imported by both.</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>Move it to simulation/prop_validation.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="73.5" customHeight="1" s="15">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>SIM-619</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Run the batch-runner stress test in a CI job</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>tests/integration/test_batch_runner_stress.py carries only the slow marker. The CI slow lane runs tests/unit -m slow; the weekly integration lane and make test-integration select -m integration; the e2e job runs one file. No job runs it. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>One lane runs it.</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>Mark it integration, or add its path to the slow lane.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="87" customHeight="1" s="15">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>SIM-620</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>Delete the regression gate's dead constants and its golden-file texts</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>tests/regression/regression_config.py: only SYMMETRY_TOLERANCE has a reader; eight constants have none (the conftest hard-codes the seed 2026). The assert message in test_engine_regression.py and the regression marker text in pyproject.toml name golden files the gate does not have. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>The dead constants go, and the texts say what the gate checks.</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>Delete them and edit the two texts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="73.5" customHeight="1" s="15">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>SIM-621</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Bench the per-pitch call the loop makes</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>tests/performance/bench_simulation.py times PitcherSimilarityEngine.query() as the per-pitch cost; the loop reads the dense pitcher matrix. bench_api_simulate.py says an authoritative gate runs on target hardware with the DB-backed factory; no job does. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>The benches time what the loop runs, and the SLA text names the job that gates it.</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>Bench the matrix read; correct the SLA text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="60" customHeight="1" s="15">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>SIM-622</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Use the pinned park factor in the sim-kwargs tests</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>tests/unit/test_sim_kwargs.py uses 0.8723846078 for venue 680 in six places; the pinned 2024 table in the same file holds 0.8725842237. The tests pass (the literal is only an input). Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>One value.</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>Read it from the table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="73.5" customHeight="1" s="15">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>SIM-623</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Replace the inning-grid test's pinned scores with an outcome check</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>tests/unit/test_inning_grid.py pins the exact scores and pitch counts of ten seeds (OUTCOMES_AT_80E3F46). That works like the golden snapshots the owner ruled out on 2026-09-10: any intended change to the draw fails it. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>The test checks a property of the grid (its sum equals the final score, the halves match the outs), not ten remembered numbers.</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>Rewrite the assertions as invariants and delete the pinned table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B60" s="8" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C60" s="9" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="D60" s="12" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="E60" s="10" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F12" s="11" t="n"/>
-    </row>
-    <row r="13" s="15"/>
-    <row r="14" ht="54" customHeight="1" s="15"/>
-    <row r="15" ht="54" customHeight="1" s="15"/>
-    <row r="16" s="15"/>
+      <c r="F60" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>

<commit_message>
File the documentation rebuild's defects as SIM-625 to SIM-634 (SIM-624)
Each defect the audit found was checked in the code again, then filed as a
P3 row of BACKLOG.xlsx: the opening-line capture, the workflow triggers, the
mock odds routes, the sweep's database address, the extra pitch past the
inning limit, the Postgres schema file, the data nobody reads, the backup
path name and the env templates, the test targets, and a bundle of small
fixes. SIM-620's row keeps only what is left. The next free ID is SIM-635.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -560,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -581,7 +581,7 @@
     <row r="2" s="15">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>NEXT FREE TICKET ID: SIM-625</t>
+          <t>NEXT FREE TICKET ID: SIM-635</t>
         </is>
       </c>
     </row>
@@ -2236,17 +2236,17 @@
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>tests/regression/regression_config.py: only SYMMETRY_TOLERANCE has a reader; eight constants have none (the conftest hard-codes the seed 2026). The assert message in test_engine_regression.py and the regression marker text in pyproject.toml name golden files the gate does not have. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>tests/regression/regression_config.py: only SYMMETRY_TOLERANCE has a reader; eight constants have none (the conftest hard-codes the seed 2026), and one constant's docstring still speaks of golden files. The assert message at test_engine_regression.py:322 names golden files the gate does not have. The pyproject.toml marker text, the ci.yml header and make help were corrected by the documentation rebuild (SIM-624, 2026-10-21). Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>The dead constants go, and the texts say what the gate checks.</t>
+          <t>The dead constants go, and the assert message says what the gate checks.</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>Delete them and edit the two texts.</t>
+          <t>Delete the dead constants and edit the assert message.</t>
         </is>
       </c>
     </row>
@@ -2346,33 +2346,354 @@
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="7" t="inlineStr">
+    <row r="59" ht="132" customHeight="1" s="15">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>SIM-625</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Capture the opening lines every day</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>No scheduled job captures the opening lines. Nothing calls schedule_opening_line_job (pipeline/etl/opening_line_job.py), and the nightly closing-lines job (scripts/nightly_closing_lines.sh, 10:30 UTC) passes --line-types closing only. The venue backfill (schedule_venue_backfill_job) has no caller either. BettingPros serves the opener after the fact, so scripts/load_historical_odds.py (its default line types are opening and closing) recovers the missing rows: nothing is lost for good. The line-movement page reads the opening-to-closing series. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Each night's odds run stores the opening rows of the games it loads, and the venue backfill either runs on a schedule or is retired.</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>Pass --line-types opening closing in scripts/nightly_closing_lines.sh. Then retire opening_line_job.py, or give it a scheduler entry; decide the venue backfill the same way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="90" customHeight="1" s="15">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>SIM-626</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Point the GitHub workflows at master</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>docker-release.yml and frontend-release.yml run on a push to main (and on a published release), and the pull_request trigger of ci.yml lists main. The default branch is master, so a push never runs the two release workflows, and a pull request into master gets no pull-request run of CI (the push run still happens). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>A push to master runs both release workflows (or the owner retires them), and a pull request into master runs CI.</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>Replace main with master in the three triggers, and in the trigger comment at the head of ci.yml.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="90" customHeight="1" s="15">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>SIM-627</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>Retire the two odds routes that serve mock lines</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>GET /api/odds/{game_pk} and GET /api/odds/today/all (pipeline/live/ingestion/odds_routes.py, mounted by api/main.py) always return MockOddsAPI lines, whatever ODDS_PROVIDER says. The rows carry is_mock: true, and no frontend code calls the routes. A client that ignores the flag reads fake prices as real ones. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>The routes are gone (or serve the stored book rows), and the API snapshot is regenerated.</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>Delete both routes, then run scripts/export_openapi.py in the app image and npm run gen:api (CLAUDE.md section 15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="90" customHeight="1" s="15">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>SIM-628</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Let the resumable sweep read the database address</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>The child process of scripts/resumable_sweep.py reads BASEBALL_DB_DSN from .env with env["BASEBALL_DB_DSN"]. Since the security hardening (SIM-443b), .env carries no such key: .env.example has it commented out, and the live .env has none. So a sweep stops with KeyError before its first game. This is separate from the retry after a crash (SIM-614). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>A sweep starts on the current .env.</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>Read BASEBALL_DB_DSN from the process environment first (pipeline.db_dsn.require_dsn); read .env only when the key is set there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="104" customHeight="1" s="15">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>SIM-629</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>End a tied game at the inning limit without an extra pitch</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>simulate_game (simulation/sim_loop.py) checks state.inning &gt; max_innings only after a pitch that does not roll the half, and _game_over_after_half knows nothing of the limit. So a game tied after the API's 12 innings (max_innings 12 in simulation/sim_kwargs.py) starts the 13th, places the extra-innings runner on second and throws one pitch before it stops. That pitch can score a run or credit a box line. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>A game tied at the limit ends when the last allowed half completes, and a unit test pins it.</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>Check the limit in the roll branch, right after _game_over_after_half.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="104" customHeight="1" s="15">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>SIM-630</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>Bring the Postgres schema file up to the migrations</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>db/schemas/01_postgres_schema.sql lags the Alembic migrations. It has no raw.savant_pitch_tracking (0020), no raw.game_bullpen (0025), none of the 0029 columns (raw.game_lineups.published_at, last_seen_at on the odds tables, the run-job columns) and none of the 0030 columns of sim.sim_runs (start_at_bat and the rest). At least eight unit tests read the file to check a schema fact. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>The file matches the schema that alembic upgrade head builds, and a test holds the two equal; or the file is retired and the tests read the migrations.</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>Regenerate the file from a migrated database (pg_dump --schema-only), or retire it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="118" customHeight="1" s="15">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>SIM-631</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>Delete or wire up the data nobody reads</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Built and never read: sim.stolen_base_pool (the profile computor builds it every night), the composite catcher actor matrix (built and concentration-checked; the draws read catcher_throwing), the sim.live_games view and raw.savant_first_base_receiving. Declared and never written: derived.outfield_play_detail, derived.infield_play_detail and derived.dp_play_detail. Never called: sim.purge_expired_sessions(), and EngineArtifacts.attach_shared_views outside the tests. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>Each item has a reader, or it is deleted with its builder and its DDL.</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>Delete them, with a migration for the DDL. Keep any the owner wants for planned work, and name the ticket that will read it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="160" customHeight="1" s="15">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>SIM-632</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Give the backup path one name, and correct the staging and production templates</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>The app reads BACKUPS_ROOT (api/routes/metrics.py, docker-compose.yml) while the backup jobs read BACKUP_ROOT (pipeline/backup/data_stores.py, pipeline/backup/offsite.py, db/backup/pg_backup.sh). Both default to /backups, so the age gauges work today; a value set under one name alone splits them. Both env templates set LIVE_PIPELINE_ENABLED=true, which makes the app a second publisher beside the live service. .env.production.example sets ODDS_PROVIDER=theoddsapi, which no provider registers. The templates also carry seven keys no app code reads: WORKERS, SIM_MAX_WORKERS, ODDS_PROVIDER_API_KEY, ODDS_API_BASE, ASYNC_DB_DSN, MLB_API_BASE and PROMETHEUS_PUSHGATEWAY. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>One variable names the backup root, and the templates hold only keys the code reads, with values that start the stack.</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>Rename the app's variable to BACKUP_ROOT. Rewrite the two templates from .env.example.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="118" customHeight="1" s="15">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>SIM-633</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>Make the test targets run what their names say</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>make test-unit passes no -m "not slow", so it runs the slow tests at the 30 s timeout; CI's unit job excludes them. make test-integration runs in the app container, which has no Docker socket (only the scheduler mounts it), so testcontainers cannot start and every integration test skips. The games input of acceptance-nightly.yml says "max 12" and defaults to 12, but the balanced set has 45 games (beside SIM-581, the roster). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>make test-unit matches CI's unit job; make test-integration runs the integration lane or says it needs host Python; the workflow input describes the 45-game set.</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>Add -m "not slow" to test-unit and a test-slow target. Run the integration lane on host Python, as docs/technical/tests.md describes. Fix the input's text and default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="202" customHeight="1" s="15">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>SIM-634</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Small fixes found by the documentation rebuild</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>(1) frontend/index.html links a favicon, /baseball.svg, that frontend/public/ does not hold: a 404 on every page. (2) /ready (api/main.py) writes a redis entry only on a failure, so a healthy Redis is missing from its checks. (3) Six nginx blocks (/health, /ready, /metrics, /docs, /redoc, /openapi.json) set their own Host header, which drops the inherited X-Real-IP and X-Forwarded-For. (4) Nothing deletes the simviz:* explorer cache keys after a nightly rebuild, so a key serves old data for up to 24 h. (5) 12 of the 32 DuckDB migrations do not record themselves in migration_history. (6) Three stale texts: api/state.py calls the situation engine a FAISS engine (it is a KD-tree); the Makefile's gen-secrets comment says a blank key is left alone (gen_secrets.py fills it); scripts/probes/manager_profile_recompute.py says the app must be stopped (the recompute runs beside the app since SIM-524). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>Each of the six is fixed or retired.</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>One small commit per area. For (5), record the missing numbers in one new migration rather than editing old files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69"/>
+    <row r="70">
+      <c r="A70" s="7" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B60" s="8" t="inlineStr">
+      <c r="B70" s="8" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C60" s="9" t="inlineStr">
+      <c r="C70" s="9" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D60" s="12" t="inlineStr">
+      <c r="D70" s="12" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E60" s="10" t="inlineStr">
+      <c r="E70" s="10" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F60" s="11" t="n"/>
+      <c r="F70" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Re-rank the backlog: order the 59 new tickets by priority, move five between bands
The tickets filed by the code clean-up (SIM-575 to SIM-623) and the
documentation rebuild (SIM-625 to SIM-634) sat in ticket-number order inside
each band. P2 now holds the defects that change what the model computes and
the decisions on its inputs, which must land before the weight fit (SIM-548);
P3 is ranked by the cost of leaving each ticket. SIM-606, SIM-611 and SIM-587
move up to P2; SIM-581 and SIM-582 move down to P3. No ticket's text changed.
CLAUDE.md section 2 no longer names the old P2 range.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -690,31 +690,31 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>SIM-576</t>
+          <t>SIM-580</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Write the catcher engine's feature names in the catcher's league-average row</t>
+          <t>Make the pitcher arsenal fit reproducible: order the pitch rows before the mixture fit</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>The profile computor writes the catcher row of derived.league_averages with the keys framing_runs, blocking_runs and cs_rate. The catcher engine reads its eleven feature names with pj.get(f, 0.0) or 0.0, and only cs_rate matches. So the shrinkage pulls ten features toward 0.0: a constructed 300-pitch catcher reads pop time 1.95 -&gt; 1.857 s and arm strength 81 -&gt; 77.1 mph. The error reaches the catcher and catcher_throwing score matrices, which weight the steal and pickoff draws. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The pitch-vector query in _compute_pitcher_profiles (pipeline/batch/profiles/pitcher.py) has no ORDER BY. DuckDB's parallel Postgres scan returns the rows in a different order on every read, and the seeded mixture fit (random_state=42) depends on the row order. So every profile rebuild gives a different arsenal for nearly every pitcher (a different number of components for about one pitcher in five), and with it a different pitcher similarity matrix. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>The catcher's league row carries every engine feature. A missing key reads as NaN, as the steal engines do. The nightly matrices are rebuilt.</t>
+          <t>Two profile builds of the same code from the same data write the same arsenals, by content.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>In pipeline/batch/profiles (the catcher league row), write the engine's eleven feature keys. In similarity/engines/catcher_similarity.py _load_league_averages, read a missing key as NaN.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="127.5" customHeight="1" s="15">
+          <t>Add ORDER BY game_pk, at_bat_number, pitch_number to the query. It changes every arsenal once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1" s="15">
       <c r="A8" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -722,27 +722,27 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>SIM-577</t>
+          <t>SIM-606</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Write all thirteen features in the extra-base runner's league-average row</t>
+          <t>Pick the small-mixture-component merge target in standardized units</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>The baserunner row of derived.league_averages holds extra_base_attempt_rate, extra_base_success_rate, sb_success_rate, sprint_speed and the Savant rate. The engine reads thirteen features, so the four per-situation attempt rates, stop_rate and the four per-situation success rates shrink toward 0.0. The matrix build loads the thin profiles, so the effect is large there: a 5-chance runner's first-to-third attempt rate reads 0.35 -&gt; 0.088. The error reaches the runner_adv matrix, which weights the advancement draws. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>enforce_min_cluster_size runs before the standardization in the arsenal build, so spin rate (hundreds of rpm) decides the merge over velocity and movement. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>The runner's league row carries every engine feature, and a missing key reads as NaN. The nightly matrices are rebuilt.</t>
+          <t>The merge measures the gap in standardized units.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Write the engine's thirteen feature keys in the computor's baserunner league row; read a missing key as NaN in similarity/engines/baserunner_similarity.py.</t>
+          <t>Measure the gap over the mixture's feature_stds.</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="114" customHeight="1" s="15">
+    <row r="10" ht="127.5" customHeight="1" s="15">
       <c r="A10" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -786,27 +786,27 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SIM-579</t>
+          <t>SIM-577</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Select the pitcher's zone-take rate before the chase rate, so the two stay in feature order</t>
+          <t>Write all thirteen features in the extra-base runner's league-average row</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>In similarity/engines/pitcher_similarity.py _load_profiles, the SELECT returns chase_rate, zone_take_rate and the unpack names them zone_take_rate, chase_rate. So command_vec holds them in the opposite order to COMMAND_FEATURES and the league-average vector, and the shrinkage pulls each pitcher's chase rate toward the league's zone-take rate (weight 1 - alpha, at most 2.4% at 200 pitches). The kernel itself ignores the order. The error reaches the pitcher similarity matrix. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The baserunner row of derived.league_averages holds extra_base_attempt_rate, extra_base_success_rate, sb_success_rate, sprint_speed and the Savant rate. The engine reads thirteen features, so the four per-situation attempt rates, stop_rate and the four per-situation success rates shrink toward 0.0. The matrix build loads the thin profiles, so the effect is large there: a 5-chance runner's first-to-third attempt rate reads 0.35 -&gt; 0.088. The error reaches the runner_adv matrix, which weights the advancement draws. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>The SELECT order matches COMMAND_FEATURES, and a unit test pins it. The nightly matrices are rebuilt.</t>
+          <t>The runner's league row carries every engine feature, and a missing key reads as NaN. The nightly matrices are rebuilt.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Select zone_take_rate before chase_rate.</t>
+          <t>Write the engine's thirteen feature keys in the computor's baserunner league row; read a missing key as NaN in similarity/engines/baserunner_similarity.py.</t>
         </is>
       </c>
     </row>
@@ -818,31 +818,31 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SIM-580</t>
+          <t>SIM-576</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Make the pitcher arsenal fit reproducible: order the pitch rows before the mixture fit</t>
+          <t>Write the catcher engine's feature names in the catcher's league-average row</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>The pitch-vector query in _compute_pitcher_profiles (pipeline/batch/profiles/pitcher.py) has no ORDER BY. DuckDB's parallel Postgres scan returns the rows in a different order on every read, and the seeded mixture fit (random_state=42) depends on the row order. So every profile rebuild gives a different arsenal for nearly every pitcher (a different number of components for about one pitcher in five), and with it a different pitcher similarity matrix. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The profile computor writes the catcher row of derived.league_averages with the keys framing_runs, blocking_runs and cs_rate. The catcher engine reads its eleven feature names with pj.get(f, 0.0) or 0.0, and only cs_rate matches. So the shrinkage pulls ten features toward 0.0: a constructed 300-pitch catcher reads pop time 1.95 -&gt; 1.857 s and arm strength 81 -&gt; 77.1 mph. The error reaches the catcher and catcher_throwing score matrices, which weight the steal and pickoff draws. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Two profile builds of the same code from the same data write the same arsenals, by content.</t>
+          <t>The catcher's league row carries every engine feature. A missing key reads as NaN, as the steal engines do. The nightly matrices are rebuilt.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Add ORDER BY game_pk, at_bat_number, pitch_number to the query. It changes every arsenal once.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="87" customHeight="1" s="15">
+          <t>In pipeline/batch/profiles (the catcher league row), write the engine's eleven feature keys. In similarity/engines/catcher_similarity.py _load_league_averages, read a missing key as NaN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="114" customHeight="1" s="15">
       <c r="A12" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -850,31 +850,31 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>SIM-581</t>
+          <t>SIM-579</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Name only real tests in the nightly acceptance lane's required roster</t>
+          <t>Select the pitcher's zone-take rate before the chase rate, so the two stay in feature order</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>The REQUIRED roster of .github/workflows/acceptance-nightly.yml lists test_full_pool_out_advancement_runs_sim450, test_full_pool_steal_decision_runs_sim450 and test_reach_on_error_band_sim450. No test of those names exists, and the roster step fails when a required name did not run. So the nightly lane reds on every run, whatever the bands read. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>In similarity/engines/pitcher_similarity.py _load_profiles, the SELECT returns chase_rate, zone_take_rate and the unpack names them zone_take_rate, chase_rate. So command_vec holds them in the opposite order to COMMAND_FEATURES and the league-average vector, and the shrinkage pulls each pitcher's chase rate toward the league's zone-take rate (weight 1 - alpha, at most 2.4% at 200 pitches). The kernel itself ignores the order. The error reaches the pitcher similarity matrix. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>The roster names only real tests, and one nightly run passes its roster step.</t>
+          <t>The SELECT order matches COMMAND_FEATURES, and a unit test pins it. The nightly matrices are rebuilt.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Delete the three names, or name the tests that took their place.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="114" customHeight="1" s="15">
+          <t>Select zone_take_rate before chase_rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="127.5" customHeight="1" s="15">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -882,31 +882,31 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>SIM-582</t>
+          <t>SIM-611</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Add last_seen_at to the two odds archive tables, so the retirement copy fits again</t>
+          <t>Owner decisions: four similarity design points</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Migration 0029 added last_seen_at to raw.game_odds and raw.prop_odds and not to their archives (raw.game_odds_archive, raw.prop_odds_archive, migration 0028). The retirement script copies rows with INSERT ... SELECT *, which needs the same columns in the same order, so the next retirement fails. The integration test test_schema_migrations.py::test_sim555_stamp_indexes_and_archives reds on master fe81d79 and on the clean-up branch for this reason. Found by the code clean-up (SIM-493, the integration pass, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>Not defects, design points for the owner. (1) The catcher's shrinkage prior is 15 called pitches, so alpha is at least 0.95 for every kept catcher (framing stabilizes near 1,500). (2) stop_rate is exactly one minus the overall attempt rate, so that rate counts twice in the runner's aggression distance. (3) The batter's xba / xslg and the manager's hit-and-run and double-switch rates read 0.0 for everyone and still hold their share of the kernel weight. (4) CLAUDE.md section 1 calls CLV 'the gold-standard metric'; the owner ruled on 2026-09-28 that the model is not judged by it. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Both archives carry last_seen_at in the live table's position, the integration test passes, and a retirement run copies a row.</t>
+          <t>The owner rules on each point, and the code or CLAUDE.md follows.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>A new Alembic migration adds last_seen_at to both archives (nullable, so the copied rows keep their value), placed after book_line_at to match the live tables; check the column order with the test.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="73.5" customHeight="1" s="15">
+          <t>Raise the catcher prior; drop stop_rate; drop the all-zero features; rewrite CLAUDE.md section 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="87" customHeight="1" s="15">
       <c r="A14" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -914,91 +914,91 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
+          <t>SIM-587</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Decide which calibration values the draws use, and make the code follow</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>similarity/calibration/pitcher.py fits sigma_command and eb_n_prior_pitcher, and no code reads either, so the pitcher engine keeps RBF_SIGMA_COMMAND 1.0453 and EB_N_PRIOR 5. More broadly, the nightly actor matrices apply no calibration report (build_actor_sim_matrices): make calibrate changes only the API's engines. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>The owner decides which values the draws use, and the code and the docs follow.</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Read both fields in apply_calibration and apply /data/calibration.json in the matrix build; or document the module defaults as the draws' values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="73.5" customHeight="1" s="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
           <t>SIM-583</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Keep the calibrated win probability strictly between 0 and 1</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>build_validation_report fits the reliability curve with min_bin_count=1, so a bin of two games can map 0.75 to 1.0. Example: the curve [[0,0],[0.45,0.44],[0.55,0.56],[0.73,1.0],[1,1]] and home_win_pct 0.75 at n = 100 give home 1.0, away 0.0 and an interval of zero width. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>No calibrated probability is 0.0 or 1.0, and a unit test feeds the curve above.</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Fit the curve with a min_bin_count near 30, or clamp the mapped probability to [eps, 1 - eps].</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="127.5" customHeight="1" s="15">
-      <c r="A15" s="17" t="inlineStr">
+    <row r="16" ht="127.5" customHeight="1" s="15">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>SIM-584</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Stamp the accuracy report with the bundle the run read, not the live link</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>scripts/accuracy/selection.py bundle_provenance reads the manifest times under BASEBALL_PLAY_POOL_DIR/engine_artifacts (the live link). The factory reads BASEBALL_ENGINE_ARTIFACT_DIR when it is set (simulation/production_factory.py). Seen on 2026-10-20: two runs on the same pinned bundle, before and after the nightly rebuild, carry different manifest_mtimes and identical records, so pair_accuracy.py refuses to pair them; two runs on different pinned bundles on one day would pair. The weight fit (SIM-548) pairs these reports. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>The stamp names the bundle the run read, and a test pins the pinned-directory case.</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>Read the pinned directory first, as the factory does.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="81" customHeight="1" s="15">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>SIM-547</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/probes/manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
         </is>
       </c>
     </row>
@@ -1010,27 +1010,27 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>SIM-526</t>
+          <t>SIM-547</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Turn on the catcher pitch-receiving factor</t>
+          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
+          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
+          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
+          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/probes/manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
         </is>
       </c>
     </row>
@@ -1042,27 +1042,27 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>SIM-556</t>
+          <t>SIM-526</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
+          <t>Turn on the catcher pitch-receiving factor</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/probes/steal_weight_volume_probe.py with its records (docs/audit/records/steal_weight_volume_probe_2025.* and _2026.*; the arrays in results/steal_weight_volume/). Filed P3 by the owner on 2026-10-01.</t>
+          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
+          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/probes/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
+          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
         </is>
       </c>
     </row>
@@ -1074,571 +1074,571 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
+          <t>SIM-556</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/probes/steal_weight_volume_probe.py with its records (docs/audit/records/steal_weight_volume_probe_2025.* and _2026.*; the arrays in results/steal_weight_volume/). Filed P3 by the owner on 2026-10-01.</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/probes/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="81" customHeight="1" s="15">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
           <t>SIM-574</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Make each SIM_* flag's code default equal its production value, or record why it differs</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>The simulator reads its switches and weights from SIM_* environment flags. Each flag has a default in the code (the value an unset flag reads) and a production value set in the app service of docker-compose.yml. They differ for 24 of the flags compose sets (measured 2026-10-20): for example the pitch-draw cell index is off in code and on in production, and the fence stage, the fielding class filter and the manager draw are the same. So a script, a probe or a test that forgets one flag runs a different simulator from production, silently. The registry of the flags (simulation/flags.py, the code clean-up SIM-493) now lists every default in one table, which makes the gap visible but does not close it.</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>For every registered flag the code default equals the compose value, or the registry row says in one line why it differs (for example: the unit lane's byte-identical state). The unit lane's own pins in tests/conftest.py still hold its state. The fingerprint (scripts/behaviour_fingerprint.py) of production is unchanged, because compose already sets the production values.</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>Owner decision first: should an unset flag mean production or off? If production: change each default in simulation/flags.py to the compose value, keep tests/conftest.py's pins for the unit lane, and add a registry test that the defaults equal compose. If off: add the reason column to the registry and a test that compose sets every flag whose default differs.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="87" customHeight="1" s="15">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
+    <row r="21" ht="73.5" customHeight="1" s="15">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>SIM-608</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Store a price that returns to an earlier value</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>The odds writer dedups on a hash with no time (ON CONFLICT (game_pk, source, odds_hash)), so -110 at t0, -120 at t1, -110 at t2 closes the series at -120. Read from the code, not checked against stored data. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>A return to an earlier price is stored, and the series closes on the last price.</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Dedup only against the latest row of the same game, source, book, market and line type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="73.5" customHeight="1" s="15">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>SIM-607</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Read the line-movement direction book by book</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>betting/line_movement.py _net_direction pools every book, so the first and last quotes can come from two books: (t1, bp:1, -110/-110) and (t2, bp:2, -130/+110) give direction 'toward' and a CLV, though neither book moved. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>The direction is each book's own, then aggregated.</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Compute the direction per book, then aggregate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="132" customHeight="1" s="15">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>SIM-625</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Capture the opening lines every day</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>No scheduled job captures the opening lines. Nothing calls schedule_opening_line_job (pipeline/etl/opening_line_job.py), and the nightly closing-lines job (scripts/nightly_closing_lines.sh, 10:30 UTC) passes --line-types closing only. The venue backfill (schedule_venue_backfill_job) has no caller either. BettingPros serves the opener after the fact, so scripts/load_historical_odds.py (its default line types are opening and closing) recovers the missing rows: nothing is lost for good. The line-movement page reads the opening-to-closing series. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Each night's odds run stores the opening rows of the games it loads, and the venue backfill either runs on a schedule or is retired.</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Pass --line-types opening closing in scripts/nightly_closing_lines.sh. Then retire opening_line_job.py, or give it a scheduler entry; decide the venue backfill the same way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="60" customHeight="1" s="15">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>SIM-586</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Ask the schedule only for game types raw.games accepts</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>GAME_TYPES (pipeline/live/ingestion/constants.py) is R F D L W C P; the CHECK on raw.games allows R P S A D F L W. A game of type C on the slate fails its upsert. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>The live pipeline's game types and the table's CHECK agree, and a unit test compares them.</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Drop C from GAME_TYPES, or widen the CHECK with a migration if type C games should load.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="114" customHeight="1" s="15">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>SIM-582</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Add last_seen_at to the two odds archive tables, so the retirement copy fits again</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Migration 0029 added last_seen_at to raw.game_odds and raw.prop_odds and not to their archives (raw.game_odds_archive, raw.prop_odds_archive, migration 0028). The retirement script copies rows with INSERT ... SELECT *, which needs the same columns in the same order, so the next retirement fails. The integration test test_schema_migrations.py::test_sim555_stamp_indexes_and_archives reds on master fe81d79 and on the clean-up branch for this reason. Found by the code clean-up (SIM-493, the integration pass, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Both archives carry last_seen_at in the live table's position, the integration test passes, and a retirement run copies a row.</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>A new Alembic migration adds last_seen_at to both archives (nullable, so the copied rows keep their value), placed after book_line_at to match the live tables; check the column order with the test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="87" customHeight="1" s="15">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>SIM-581</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Name only real tests in the nightly acceptance lane's required roster</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>The REQUIRED roster of .github/workflows/acceptance-nightly.yml lists test_full_pool_out_advancement_runs_sim450, test_full_pool_steal_decision_runs_sim450 and test_reach_on_error_band_sim450. No test of those names exists, and the roster step fails when a required name did not run. So the nightly lane reds on every run, whatever the bands read. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>The roster names only real tests, and one nightly run passes its roster step.</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Delete the three names, or name the tests that took their place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="118" customHeight="1" s="15">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>SIM-633</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Make the test targets run what their names say</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>make test-unit passes no -m "not slow", so it runs the slow tests at the 30 s timeout; CI's unit job excludes them. make test-integration runs in the app container, which has no Docker socket (only the scheduler mounts it), so testcontainers cannot start and every integration test skips. The games input of acceptance-nightly.yml says "max 12" and defaults to 12, but the balanced set has 45 games (beside SIM-581, the roster). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>make test-unit matches CI's unit job; make test-integration runs the integration lane or says it needs host Python; the workflow input describes the 45-game set.</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Add -m "not slow" to test-unit and a test-slow target. Run the integration lane on host Python, as docs/technical/tests.md describes. Fix the input's text and default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="90" customHeight="1" s="15">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>SIM-626</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Point the GitHub workflows at master</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>docker-release.yml and frontend-release.yml run on a push to main (and on a published release), and the pull_request trigger of ci.yml lists main. The default branch is master, so a push never runs the two release workflows, and a pull request into master gets no pull-request run of CI (the push run still happens). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>A push to master runs both release workflows (or the owner retires them), and a pull request into master runs CI.</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Replace main with master in the three triggers, and in the trigger comment at the head of ci.yml.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="73.5" customHeight="1" s="15">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>SIM-619</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Run the batch-runner stress test in a CI job</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>tests/integration/test_batch_runner_stress.py carries only the slow marker. The CI slow lane runs tests/unit -m slow; the weekly integration lane and make test-integration select -m integration; the e2e job runs one file. No job runs it. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>One lane runs it.</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Mark it integration, or add its path to the slow lane.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="73.5" customHeight="1" s="15">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>SIM-602</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Make two API tests check what their names say</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>tests/unit/test_api_betting.py test_clv_snapshot_returns_only_series_with_clv makes a GET and asserts nothing. tests/unit/test_api_games_plays.py test_simulate_ok_without_duckdb_then_plays_404 never requests /plays. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Each test asserts what its name says.</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Add the assertions (the CLV series' filter; /plays answers 503 with no replay store), then rename the second test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="87" customHeight="1" s="15">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>SIM-601</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Make the Playwright smoke tests pass while the live app runs</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>frontend/e2e/smoke.spec.ts (three specs) fail on the owner's host: a request the test does not mock goes through the preview server's proxy to localhost:8000, the live app answers 401 and the page shows the login. With API_TARGET=http://127.0.0.1:9 all 21 tests pass; CI has no backend, so CI passes. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>The e2e suite passes with the live app running.</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Set API_TARGET to a closed port in playwright.config.ts's webServer.env, or end each spec with a catch-all **/api/** route that answers 404.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="104" customHeight="1" s="15">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>SIM-630</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Bring the Postgres schema file up to the migrations</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>db/schemas/01_postgres_schema.sql lags the Alembic migrations. It has no raw.savant_pitch_tracking (0020), no raw.game_bullpen (0025), none of the 0029 columns (raw.game_lineups.published_at, last_seen_at on the odds tables, the run-job columns) and none of the 0030 columns of sim.sim_runs (start_at_bat and the rest). At least eight unit tests read the file to check a schema fact. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>The file matches the schema that alembic upgrade head builds, and a test holds the two equal; or the file is retired and the tests read the migrations.</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Regenerate the file from a migrated database (pg_dump --schema-only), or retire it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="87" customHeight="1" s="15">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>SIM-585</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>Refuse CORS_ORIGINS=* while the API sends credentials</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>api/main.py sets allow_credentials=True for every origin list, and resolve_cors_origins (api/auth.py) returns ['*'] when an operator sets CORS_ORIGINS=*. Starlette then echoes the caller's Origin on a request with a cookie, so any site can read the API with the user's login. Production sets neither variable today, so the defect is latent. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
         <is>
           <t>CORS_ORIGINS=* either fails the boot or turns credentials off, and a unit test pins it.</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F33" s="5" t="inlineStr">
         <is>
           <t>Refuse '*' in resolve_cors_origins while credentials are on.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1" s="15">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>SIM-586</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Ask the schedule only for game types raw.games accepts</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>GAME_TYPES (pipeline/live/ingestion/constants.py) is R F D L W C P; the CHECK on raw.games allows R P S A D F L W. A game of type C on the slate fails its upsert. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>The live pipeline's game types and the table's CHECK agree, and a unit test compares them.</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>Drop C from GAME_TYPES, or widen the CHECK with a migration if type C games should load.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="87" customHeight="1" s="15">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>SIM-587</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Decide which calibration values the draws use, and make the code follow</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>similarity/calibration/pitcher.py fits sigma_command and eb_n_prior_pitcher, and no code reads either, so the pitcher engine keeps RBF_SIGMA_COMMAND 1.0453 and EB_N_PRIOR 5. More broadly, the nightly actor matrices apply no calibration report (build_actor_sim_matrices): make calibrate changes only the API's engines. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>The owner decides which values the draws use, and the code and the docs follow.</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>Read both fields in apply_calibration and apply /data/calibration.json in the matrix build; or document the module defaults as the draws' values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="46.5" customHeight="1" s="15">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>SIM-588</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Compute the z of the requested level in GameSimSummary.from_results</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>GameSimSummary.from_results(confidence_level=0.85) computes the 95% z and labels the intervals 0.85. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>Each level gets its own z, and a unit test checks 0.85.</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>Use NormalDist().inv_cdf((1 + level) / 2), or raise on a level outside the table.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="73.5" customHeight="1" s="15">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>SIM-589</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Treat both samples as samples in the replay chi-squared test</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>The two-sample path of replay_chi_squared.chi_squared_gof treats the reference sample as exact. Two independent samples of 1,000 Poisson(4.4) totals were rejected 52.5% of the time at alpha 0.05 over 400 trials. replay_and_test uses it. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>Two samples from one distribution are rejected near alpha.</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>Use scipy.stats.chi2_contingency on the pooled 2 x k table.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="60" customHeight="1" s="15">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>SIM-590</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Compare the historical replay against the right side's score</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>replay_historical_games always compares the simulated HOME score. A HistoricalGame row does not say which side its runs belong to, so an away team's runs meet the simulated home runs. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>A HistoricalGame row names its side, and the replay compares like with like.</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>Add a side field to HistoricalGame.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="73.5" customHeight="1" s="15">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>SIM-591</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>Charge the losing pitcher with the go-ahead run, as MLB does</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>pitcher_decisions charges the pitcher on the mound at the decisive play. In a tie, A walks a batter, B relieves him and allows a double that scores the runner, and the lead holds: MLB charges A; the simulator charges B. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>The decision follows the runner's responsible pitcher, and a unit test plays the example.</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>Carry each runner's responsible pitcher on the bases.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="73.5" customHeight="1" s="15">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>SIM-592</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>Put the batter on first after a forced reach with no batter id</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>_force_on_reach with no batter id leaves first base's runner on first after pushing him to second (b.first = state.batter_id if ... else b.first), so the base check raises; _resolve_walk assigns b.first = state.batter_id for the same case. Reachable only with a sampler and no lineup. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>The forced reach and the walk give the same bases.</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>Use the walk's assignment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="73.5" customHeight="1" s="15">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>SIM-593</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>Void the plate appearance after a third out on the bases in the single pre-pitch steal draw</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>With SIM_STEAL_PITCH_CLASS=0 (not production), a pickoff or a caught stealing that makes the third out before the pitch's result still ends the plate appearance, so the pitcher gets a batter faced and the batter an at-bat. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>The single draw voids the plate appearance as the running game on the pitch does.</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>Apply the no-pitch void of the class-aware draw.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="60" customHeight="1" s="15">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
+    <row r="34" ht="160" customHeight="1" s="15">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>SIM-632</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Give the backup path one name, and correct the staging and production templates</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>The app reads BACKUPS_ROOT (api/routes/metrics.py, docker-compose.yml) while the backup jobs read BACKUP_ROOT (pipeline/backup/data_stores.py, pipeline/backup/offsite.py, db/backup/pg_backup.sh). Both default to /backups, so the age gauges work today; a value set under one name alone splits them. Both env templates set LIVE_PIPELINE_ENABLED=true, which makes the app a second publisher beside the live service. .env.production.example sets ODDS_PROVIDER=theoddsapi, which no provider registers. The templates also carry seven keys no app code reads: WORKERS, SIM_MAX_WORKERS, ODDS_PROVIDER_API_KEY, ODDS_API_BASE, ASYNC_DB_DSN, MLB_API_BASE and PROMETHEUS_PUSHGATEWAY. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>One variable names the backup root, and the templates hold only keys the code reads, with values that start the stack.</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Rename the app's variable to BACKUP_ROOT. Rewrite the two templates from .env.example.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="104" customHeight="1" s="15">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>SIM-629</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>End a tied game at the inning limit without an extra pitch</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>simulate_game (simulation/sim_loop.py) checks state.inning &gt; max_innings only after a pitch that does not roll the half, and _game_over_after_half knows nothing of the limit. So a game tied after the API's 12 innings (max_innings 12 in simulation/sim_kwargs.py) starts the 13th, places the extra-innings runner on second and throws one pitch before it stops. That pitch can score a run or credit a box line. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>A game tied at the limit ends when the last allowed half completes, and a unit test pins it.</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Check the limit in the roll branch, right after _game_over_after_half.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="60" customHeight="1" s="15">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>SIM-594</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>Let the batter run on a called third strike that gets away</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>Rule 5.05(a)(2) lets the batter run on any uncaught third strike. _dropped_third_strike reads swinging strikes only. Two such rows exist in 2023-2026, both in 2026. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>A called third strike that gets away can be a dropped-third-strike reach.</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F36" s="5" t="inlineStr">
         <is>
           <t>Let _dropped_third_strike read a called third strike too.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="46.5" customHeight="1" s="15">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>SIM-595</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Fix the article in the what-if's ineligible-player message</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>whatif.apply_changes' message for an ineligible pinch hitter reads 'is not an bench hitter'. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>Each label reads with its own article.</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>Put the article inside each label.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="60" customHeight="1" s="15">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>SIM-596</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>Decide what the what-if does when the designated hitter takes the field</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>A designated hitter moved to the field leaves the fielder he replaced in the batting order with no position. The rule that ends the designated hitter is not modelled in simulation/whatif.py. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>The owner decides whether the what-if models the rule, and the code follows.</t>
-        </is>
-      </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>Model the rule: the pitcher bats in the replaced fielder's slot, or refuse the change.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="87" customHeight="1" s="15">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>SIM-597</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Write the pitching-change pool's role file in a fixed row order</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>roles.parquet (build_pitching_change_pool, pipeline/batch/artifacts/manager_pool.py) is written from a GROUP BY with no ORDER BY, so two builds of the same code from the same data write its rows in a different order. No reader uses the order, but the fingerprint's bundle mode reads a difference on every build. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>Two builds give the same file, by content.</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>Add ORDER BY pitcher_id, season. It changes no game.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="60" customHeight="1" s="15">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>SIM-598</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>Read the runners under the names the live service sends</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>frontend/src/hooks/useGameSocket.ts reads runner_on_first / _second / _third; the live service sends on_1b / on_2b / on_3b. The hook's on_1b to on_3b are always undefined. No page reads them today. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>A game_state_update with runners fills the hook's on_1b to on_3b.</t>
-        </is>
-      </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>Read gs.on_1b, gs.on_2b and gs.on_3b in mapWsState.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="73.5" customHeight="1" s="15">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>SIM-599</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>Describe the slate card's odds field as it is</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>The route description (api/routes/games_slate.py) and the model (api/routes/games_models.py) call the field 'reserved for the Phase-6 odds-provider integration (SIM-405)'. The field is always None: the card's lines come from /api/betting/games/{pk}/card-odds. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>Both texts say that, with a fresh API snapshot (CLAUDE.md section 15).</t>
-        </is>
-      </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>Rewrite both texts; run scripts/export_openapi.py in the image and npm run gen:api.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="46.5" customHeight="1" s="15">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>SIM-600</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>Name the current state in the API's version and health strings</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>api/main.py carries the app version 0.1.0-phase7, "phase": "6" on /health and "6 - Frontend Build (in progress)" on /. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>The strings name the current state, or go.</t>
-        </is>
-      </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>Drop the phase keys and set the version from one constant.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="87" customHeight="1" s="15">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>SIM-601</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>Make the Playwright smoke tests pass while the live app runs</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>frontend/e2e/smoke.spec.ts (three specs) fail on the owner's host: a request the test does not mock goes through the preview server's proxy to localhost:8000, the live app answers 401 and the page shows the login. With API_TARGET=http://127.0.0.1:9 all 21 tests pass; CI has no backend, so CI passes. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>The e2e suite passes with the live app running.</t>
-        </is>
-      </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>Set API_TARGET to a closed port in playwright.config.ts's webServer.env, or end each spec with a catch-all **/api/** route that answers 404.</t>
         </is>
       </c>
     </row>
@@ -1650,31 +1650,31 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>SIM-602</t>
+          <t>SIM-591</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Make two API tests check what their names say</t>
+          <t>Charge the losing pitcher with the go-ahead run, as MLB does</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>tests/unit/test_api_betting.py test_clv_snapshot_returns_only_series_with_clv makes a GET and asserts nothing. tests/unit/test_api_games_plays.py test_simulate_ok_without_duckdb_then_plays_404 never requests /plays. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>pitcher_decisions charges the pitcher on the mound at the decisive play. In a tie, A walks a batter, B relieves him and allows a double that scores the runner, and the lead holds: MLB charges A; the simulator charges B. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Each test asserts what its name says.</t>
+          <t>The decision follows the runner's responsible pitcher, and a unit test plays the example.</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Add the assertions (the CLV series' filter; /plays answers 503 with no replay store), then rename the second test.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="100.5" customHeight="1" s="15">
+          <t>Carry each runner's responsible pitcher on the bases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="73.5" customHeight="1" s="15">
       <c r="A38" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1682,31 +1682,31 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>SIM-603</t>
+          <t>SIM-592</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Return the fielder's infield sub-scores in the same order from query_pair as from query</t>
+          <t>Put the batter on first after a forced reach with no batter id</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>For an infielder, similarity/engines/fielder_similarity.py query_pair returns the specialty score in tertiary_score and the error score in quaternary_score; query returns them the other way round, as the Similarity Explorer's labels expect. Two shortstops with different error rates and equal specialty values: query gives 0.0710 / 1.0000, query_pair 1.0000 / 0.0710. The composite and the matrices are right. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>_force_on_reach with no batter id leaves first base's runner on first after pushing him to second (b.first = state.batter_id if ... else b.first), so the base check raises; _resolve_walk assigns b.first = state.batter_id for the same case. Reachable only with a sampler and no lineup. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>query and query_pair agree on every sub-score, and a unit test compares them.</t>
+          <t>The forced reach and the walk give the same bases.</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Map the infield tuple in SimilarityResult order.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="100.5" customHeight="1" s="15">
+          <t>Use the walk's assignment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="73.5" customHeight="1" s="15">
       <c r="A39" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1714,31 +1714,31 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>SIM-604</t>
+          <t>SIM-593</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Apply the per-hand 30-PA platoon rule in the batter engine's pair score</t>
+          <t>Void the plate appearance after a third out on the bases in the single pre-pitch steal draw</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>similarity/engines/batter_similarity.py _score_pair disagrees with score_all on a thin platoon split. A query with 30+ PA against either hand turns the platoon weights on for any vs_hand (10 PA vs L and 200 vs R with vs_hand='L': 0.8642 against 0.8900), and a candidate under 30 PA never gets the neutral 0.5. It serves query_pair (the Explorer's pair view and the diagnostics); the matrix is unaffected. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>With SIM_STEAL_PITCH_CLASS=0 (not production), a pickoff or a caught stealing that makes the third out before the pitch's result still ends the plate appearance, so the pitcher gets a batter faced and the batter an at-bat. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>_score_pair and score_all agree, and a unit test compares them.</t>
+          <t>The single draw voids the plate appearance as the running game on the pitch does.</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Use score_all's per-hand rule in _score_pair.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="73.5" customHeight="1" s="15">
+          <t>Apply the no-pitch void of the class-aware draw.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="46.5" customHeight="1" s="15">
       <c r="A40" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1746,63 +1746,63 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
+          <t>SIM-588</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Compute the z of the requested level in GameSimSummary.from_results</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>GameSimSummary.from_results(confidence_level=0.85) computes the 95% z and labels the intervals 0.85. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Each level gets its own z, and a unit test checks 0.85.</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>Use NormalDist().inv_cdf((1 + level) / 2), or raise on a level outside the table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="73.5" customHeight="1" s="15">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
           <t>SIM-605</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>Keep one pitcher engine's calibration from rewriting every pitcher engine</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr">
+      <c r="D41" s="5" t="inlineStr">
         <is>
           <t>PitcherSimilarityEngine.apply_calibration sets the module global ARSENAL_SCALE, and a report with no gamma resets it to 4.10. The API builds two instances. Latent: no production path calls it today. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E40" s="5" t="inlineStr">
+      <c r="E41" s="5" t="inlineStr">
         <is>
           <t>Each instance carries its own scale.</t>
         </is>
       </c>
-      <c r="F40" s="5" t="inlineStr">
+      <c r="F41" s="5" t="inlineStr">
         <is>
           <t>Pass the instance's scale into the three readers.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="60" customHeight="1" s="15">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>SIM-606</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>Pick the small-mixture-component merge target in standardized units</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>enforce_min_cluster_size runs before the standardization in the arsenal build, so spin rate (hundreds of rpm) decides the merge over velocity and movement. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>The merge measures the gap in standardized units.</t>
-        </is>
-      </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>Measure the gap over the mixture's feature_stds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="73.5" customHeight="1" s="15">
+    <row r="42" ht="90" customHeight="1" s="15">
       <c r="A42" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1810,27 +1810,27 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>SIM-607</t>
+          <t>SIM-628</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Read the line-movement direction book by book</t>
+          <t>Let the resumable sweep read the database address</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>betting/line_movement.py _net_direction pools every book, so the first and last quotes can come from two books: (t1, bp:1, -110/-110) and (t2, bp:2, -130/+110) give direction 'toward' and a CLV, though neither book moved. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The child process of scripts/resumable_sweep.py reads BASEBALL_DB_DSN from .env with env["BASEBALL_DB_DSN"]. Since the security hardening (SIM-443b), .env carries no such key: .env.example has it commented out, and the live .env has none. So a sweep stops with KeyError before its first game. This is separate from the retry after a crash (SIM-614). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>The direction is each book's own, then aggregated.</t>
+          <t>A sweep starts on the current .env.</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Compute the direction per book, then aggregate.</t>
+          <t>Read BASEBALL_DB_DSN from the process environment first (pipeline.db_dsn.require_dsn); read .env only when the key is set there.</t>
         </is>
       </c>
     </row>
@@ -1842,31 +1842,31 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>SIM-608</t>
+          <t>SIM-614</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Store a price that returns to an earlier value</t>
+          <t>Retry a sweep attempt that crashes before its first game</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>The odds writer dedups on a hash with no time (ON CONFLICT (game_pk, source, odds_hash)), so -110 at t0, -120 at t1, -110 at t2 closes the series at -120. Read from the code, not checked against stored data. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/resumable_sweep.py applies its zero-progress stop (gained == 0) after a crash too, so a segfault before the first game of an attempt ends the sweep (exit 1) instead of retrying. Found by reading the code; not exercised. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>A return to an earlier price is stored, and the series closes on the last price.</t>
+          <t>A crashed attempt with no gain retries up to --max-attempts.</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Dedup only against the latest row of the same game, source, book, market and line type.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="46.5" customHeight="1" s="15">
+          <t>Apply the stop only to an attempt that exited cleanly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="87" customHeight="1" s="15">
       <c r="A44" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1874,31 +1874,31 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>SIM-609</t>
+          <t>SIM-613</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Raise on a wrong market or side in the line-movement series</t>
+          <t>Print n/a in the hypothetical-return table when no bet qualifies</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>line_movement_from_quotes swallows _side_columns' ValueError, so a wrong market or side gives a silent empty series. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/accuracy/hypothetical_return.py _fmt_row formats the means and the range with :.4f and no guard for None. With no qualifying bet the table raises TypeError, and run() prints it before it writes the report and before the zero-games check, so the run ends in a traceback with no report and no exit code 5. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>A wrong market or side raises.</t>
+          <t>The table prints n/a, as the accuracy table does.</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Call _side_columns once before the loop.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="154.5" customHeight="1" s="15">
+          <t>Use the _fmt_or_na guard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="87" customHeight="1" s="15">
       <c r="A45" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1906,31 +1906,31 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>SIM-610</t>
+          <t>SIM-616</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Similarity and betting: seven small defects</t>
+          <t>Decide the minimum-sample read's two known limits</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>(1) SituationSimilarityEngine.query_batch([]) raises instead of returning []. (2) The engines' and the calibrator's __main__ blocks read a DuckDB path that does not exist (../../db/schemas/baseball_simulator.duckdb); the pitcher engine's block builds and prints nothing. (3) CalibrationReport.summary() prints no row for the batter's physical weights. (4) The Similarity Explorer's batter panel (api/routes/similarity_explorer.py) shows the four-way weights 0.40/0.35/0.15/0.10. (5) A log line in batted_ball_similarity.py says 'until SIM-051 ships'. (6) tests/regression/conftest.py scales the situation fixture's index twice. (7) No writer sets is_sharp_book, so sharp_consensus is always None. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/accuracy/confidence.py: the 0.02 floor assumes a coin-flip market, so its power is weaker than stated for a market far from 0.5 (a home-run prop); and a small sample whose observed spread is exactly zero reads as fully resolved. An adversarial review of the minimum-sample work (SIM-539) found both. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>Each of the seven is fixed or retired.</t>
+          <t>The owner decides whether to fix or accept them.</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>One edit each; retire sharp_consensus if no book will be marked sharp.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="127.5" customHeight="1" s="15">
+          <t>A per-market 4p(1-p) correction and an upper bound on the spread.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="73.5" customHeight="1" s="15">
       <c r="A46" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1938,27 +1938,27 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>SIM-611</t>
+          <t>SIM-589</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Owner decisions: four similarity design points</t>
+          <t>Treat both samples as samples in the replay chi-squared test</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Not defects, design points for the owner. (1) The catcher's shrinkage prior is 15 called pitches, so alpha is at least 0.95 for every kept catcher (framing stabilizes near 1,500). (2) stop_rate is exactly one minus the overall attempt rate, so that rate counts twice in the runner's aggression distance. (3) The batter's xba / xslg and the manager's hit-and-run and double-switch rates read 0.0 for everyone and still hold their share of the kernel weight. (4) CLAUDE.md section 1 calls CLV 'the gold-standard metric'; the owner ruled on 2026-09-28 that the model is not judged by it. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The two-sample path of replay_chi_squared.chi_squared_gof treats the reference sample as exact. Two independent samples of 1,000 Poisson(4.4) totals were rejected 52.5% of the time at alpha 0.05 over 400 trials. replay_and_test uses it. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>The owner rules on each point, and the code or CLAUDE.md follows.</t>
+          <t>Two samples from one distribution are rejected near alpha.</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Raise the catcher prior; drop stop_rate; drop the all-zero features; rewrite CLAUDE.md section 1.</t>
+          <t>Use scipy.stats.chi2_contingency on the pooled 2 x k table.</t>
         </is>
       </c>
     </row>
@@ -1970,31 +1970,31 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>SIM-612</t>
+          <t>SIM-590</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Read the pitch rebuild's before-smoke from results/</t>
+          <t>Compare the historical replay against the right side's score</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>scripts/pitch_pool_rebuild/export.py _smoke_games opens scripts/sim553_smoke_before.json; the groundwork moved run outputs to results/sim553/. The function always prints its placeholder. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>replay_historical_games always compares the simulated HOME score. A HistoricalGame row does not say which side its runs belong to, so an away team's runs meet the simulated home runs. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>It reads the results/ path.</t>
+          <t>A HistoricalGame row names its side, and the replay compares like with like.</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Change the one path.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="87" customHeight="1" s="15">
+          <t>Add a side field to HistoricalGame.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="60" customHeight="1" s="15">
       <c r="A48" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2002,27 +2002,27 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>SIM-613</t>
+          <t>SIM-618</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Print n/a in the hypothetical-return table when no bet qualifies</t>
+          <t>Keep one copy of the prop ground-truth readers</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>scripts/accuracy/hypothetical_return.py _fmt_row formats the means and the range with :.4f and no guard for None. With no qualifying bet the table raises TypeError, and run() prints it before it writes the report and before the zero-games check, so the run ends in a traceback with no report and no exit code 5. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/validate_props.py and scripts/accuracy/grading.py each define _fetch_official_boxscore and _fetch_pa_events. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>The table prints n/a, as the accuracy table does.</t>
+          <t>One reader, imported by both.</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>Use the _fmt_or_na guard.</t>
+          <t>Move it to simulation/prop_validation.py.</t>
         </is>
       </c>
     </row>
@@ -2034,31 +2034,31 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>SIM-614</t>
+          <t>SIM-621</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Retry a sweep attempt that crashes before its first game</t>
+          <t>Bench the per-pitch call the loop makes</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>scripts/resumable_sweep.py applies its zero-progress stop (gained == 0) after a crash too, so a segfault before the first game of an attempt ends the sweep (exit 1) instead of retrying. Found by reading the code; not exercised. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>tests/performance/bench_simulation.py times PitcherSimilarityEngine.query() as the per-pitch cost; the loop reads the dense pitcher matrix. bench_api_simulate.py says an authoritative gate runs on target hardware with the DB-backed factory; no job does. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>A crashed attempt with no gain retries up to --max-attempts.</t>
+          <t>The benches time what the loop runs, and the SLA text names the job that gates it.</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Apply the stop only to an attempt that exited cleanly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="73.5" customHeight="1" s="15">
+          <t>Bench the matrix read; correct the SLA text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="60" customHeight="1" s="15">
       <c r="A50" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2066,31 +2066,31 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>SIM-615</t>
+          <t>SIM-612</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Retire the odds-hash backfill probe</t>
+          <t>Read the pitch rebuild's before-smoke from results/</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>scripts/probes/backfill_odds_hash.py _dedup_rows orders by received_at, a column raw.game_odds does not have, so its DELETE fails; its ODDS_COLUMNS leaves out draw_ml. Both are dormant: the unique index and the NOT NULL hash of migration 0012 ended the probe's job. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/pitch_pool_rebuild/export.py _smoke_games opens scripts/sim553_smoke_before.json; the groundwork moved run outputs to results/sim553/. The function always prints its placeholder. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>The probe is retired.</t>
+          <t>It reads the results/ path.</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Delete the probe and its test.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="87" customHeight="1" s="15">
+          <t>Change the one path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="73.5" customHeight="1" s="15">
       <c r="A51" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2098,31 +2098,31 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>SIM-616</t>
+          <t>SIM-623</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Decide the minimum-sample read's two known limits</t>
+          <t>Replace the inning-grid test's pinned scores with an outcome check</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>scripts/accuracy/confidence.py: the 0.02 floor assumes a coin-flip market, so its power is weaker than stated for a market far from 0.5 (a home-run prop); and a small sample whose observed spread is exactly zero reads as fully resolved. An adversarial review of the minimum-sample work (SIM-539) found both. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>tests/unit/test_inning_grid.py pins the exact scores and pitch counts of ten seeds (OUTCOMES_AT_80E3F46). That works like the golden snapshots the owner ruled out on 2026-09-10: any intended change to the draw fails it. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>The owner decides whether to fix or accept them.</t>
+          <t>The test checks a property of the grid (its sum equals the final score, the halves match the outs), not ten remembered numbers.</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>A per-market 4p(1-p) correction and an upper bound on the spread.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="181.5" customHeight="1" s="15">
+          <t>Rewrite the assertions as invariants and delete the pinned table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="87" customHeight="1" s="15">
       <c r="A52" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2130,27 +2130,27 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>SIM-617</t>
+          <t>SIM-620</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Correct the runtime texts that state something false</t>
+          <t>Delete the regression gate's dead constants and its golden-file texts</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Left unedited by the clean-up's rule. (1) The park-guard messages name the deleted SIM_PARK_FACTOR: scripts/validate_props.py, scripts/accuracy_comparison.py, tests/acceptance/conftest.py and the --help of scripts/sim_stats.py. (2) The two pool rebuilds' exit-3 texts and the steal rebuild's lock message blame the app's worker server for the DuckDB lock (the app holds no handle since SIM-524), and two steal-rebuild texts say to merge code that is merged. (3) scripts/running_game_replay.py --help says a steal can land on any pitch in production. (4) Three texts point at a module docstring section that moved in the split. (5) scripts/measure_filter_cells.py writes into docs/audit/. (6) scripts/resumable_sweep.py --help cites a deleted record. (7) The rationale strings in tests/acceptance/bands.py cite BACKLOG.md, which is gone. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>tests/regression/regression_config.py: only SYMMETRY_TOLERANCE has a reader; eight constants have none (the conftest hard-codes the seed 2026), and one constant's docstring still speaks of golden files. The assert message at test_engine_regression.py:322 names golden files the gate does not have. The pyproject.toml marker text, the ci.yml header and make help were corrected by the documentation rebuild (SIM-624, 2026-10-21). Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>Each text says what is true.</t>
+          <t>The dead constants go, and the assert message says what the gate checks.</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>One edit per text; list the runtime-string changes in CHANGES.md.</t>
+          <t>Delete the dead constants and edit the assert message.</t>
         </is>
       </c>
     </row>
@@ -2162,31 +2162,31 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>SIM-618</t>
+          <t>SIM-622</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Keep one copy of the prop ground-truth readers</t>
+          <t>Use the pinned park factor in the sim-kwargs tests</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>scripts/validate_props.py and scripts/accuracy/grading.py each define _fetch_official_boxscore and _fetch_pa_events. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>tests/unit/test_sim_kwargs.py uses 0.8723846078 for venue 680 in six places; the pinned 2024 table in the same file holds 0.8725842237. The tests pass (the literal is only an input). Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>One reader, imported by both.</t>
+          <t>One value.</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Move it to simulation/prop_validation.py.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="73.5" customHeight="1" s="15">
+          <t>Read it from the table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="87" customHeight="1" s="15">
       <c r="A54" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2194,31 +2194,31 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>SIM-619</t>
+          <t>SIM-597</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Run the batch-runner stress test in a CI job</t>
+          <t>Write the pitching-change pool's role file in a fixed row order</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>tests/integration/test_batch_runner_stress.py carries only the slow marker. The CI slow lane runs tests/unit -m slow; the weekly integration lane and make test-integration select -m integration; the e2e job runs one file. No job runs it. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>roles.parquet (build_pitching_change_pool, pipeline/batch/artifacts/manager_pool.py) is written from a GROUP BY with no ORDER BY, so two builds of the same code from the same data write its rows in a different order. No reader uses the order, but the fingerprint's bundle mode reads a difference on every build. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>One lane runs it.</t>
+          <t>Two builds give the same file, by content.</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>Mark it integration, or add its path to the slow lane.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="87" customHeight="1" s="15">
+          <t>Add ORDER BY pitcher_id, season. It changes no game.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="118" customHeight="1" s="15">
       <c r="A55" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2226,27 +2226,27 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>SIM-620</t>
+          <t>SIM-631</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Delete the regression gate's dead constants and its golden-file texts</t>
+          <t>Delete or wire up the data nobody reads</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>tests/regression/regression_config.py: only SYMMETRY_TOLERANCE has a reader; eight constants have none (the conftest hard-codes the seed 2026), and one constant's docstring still speaks of golden files. The assert message at test_engine_regression.py:322 names golden files the gate does not have. The pyproject.toml marker text, the ci.yml header and make help were corrected by the documentation rebuild (SIM-624, 2026-10-21). Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>Built and never read: sim.stolen_base_pool (the profile computor builds it every night), the composite catcher actor matrix (built and concentration-checked; the draws read catcher_throwing), the sim.live_games view and raw.savant_first_base_receiving. Declared and never written: derived.outfield_play_detail, derived.infield_play_detail and derived.dp_play_detail. Never called: sim.purge_expired_sessions(), and EngineArtifacts.attach_shared_views outside the tests. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>The dead constants go, and the assert message says what the gate checks.</t>
+          <t>Each item has a reader, or it is deleted with its builder and its DDL.</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>Delete the dead constants and edit the assert message.</t>
+          <t>Delete them, with a migration for the DDL. Keep any the owner wants for planned work, and name the ticket that will read it.</t>
         </is>
       </c>
     </row>
@@ -2258,31 +2258,31 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>SIM-621</t>
+          <t>SIM-615</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Bench the per-pitch call the loop makes</t>
+          <t>Retire the odds-hash backfill probe</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>tests/performance/bench_simulation.py times PitcherSimilarityEngine.query() as the per-pitch cost; the loop reads the dense pitcher matrix. bench_api_simulate.py says an authoritative gate runs on target hardware with the DB-backed factory; no job does. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/probes/backfill_odds_hash.py _dedup_rows orders by received_at, a column raw.game_odds does not have, so its DELETE fails; its ODDS_COLUMNS leaves out draw_ml. Both are dormant: the unique index and the NOT NULL hash of migration 0012 ended the probe's job. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>The benches time what the loop runs, and the SLA text names the job that gates it.</t>
+          <t>The probe is retired.</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>Bench the matrix read; correct the SLA text.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="60" customHeight="1" s="15">
+          <t>Delete the probe and its test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="90" customHeight="1" s="15">
       <c r="A57" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2290,31 +2290,31 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>SIM-622</t>
+          <t>SIM-627</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Use the pinned park factor in the sim-kwargs tests</t>
+          <t>Retire the two odds routes that serve mock lines</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>tests/unit/test_sim_kwargs.py uses 0.8723846078 for venue 680 in six places; the pinned 2024 table in the same file holds 0.8725842237. The tests pass (the literal is only an input). Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>GET /api/odds/{game_pk} and GET /api/odds/today/all (pipeline/live/ingestion/odds_routes.py, mounted by api/main.py) always return MockOddsAPI lines, whatever ODDS_PROVIDER says. The rows carry is_mock: true, and no frontend code calls the routes. A client that ignores the flag reads fake prices as real ones. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>One value.</t>
+          <t>The routes are gone (or serve the stored book rows), and the API snapshot is regenerated.</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>Read it from the table.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="73.5" customHeight="1" s="15">
+          <t>Delete both routes, then run scripts/export_openapi.py in the app image and npm run gen:api (CLAUDE.md section 15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="181.5" customHeight="1" s="15">
       <c r="A58" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2322,31 +2322,31 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>SIM-623</t>
+          <t>SIM-617</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Replace the inning-grid test's pinned scores with an outcome check</t>
+          <t>Correct the runtime texts that state something false</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>tests/unit/test_inning_grid.py pins the exact scores and pitch counts of ten seeds (OUTCOMES_AT_80E3F46). That works like the golden snapshots the owner ruled out on 2026-09-10: any intended change to the draw fails it. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>Left unedited by the clean-up's rule. (1) The park-guard messages name the deleted SIM_PARK_FACTOR: scripts/validate_props.py, scripts/accuracy_comparison.py, tests/acceptance/conftest.py and the --help of scripts/sim_stats.py. (2) The two pool rebuilds' exit-3 texts and the steal rebuild's lock message blame the app's worker server for the DuckDB lock (the app holds no handle since SIM-524), and two steal-rebuild texts say to merge code that is merged. (3) scripts/running_game_replay.py --help says a steal can land on any pitch in production. (4) Three texts point at a module docstring section that moved in the split. (5) scripts/measure_filter_cells.py writes into docs/audit/. (6) scripts/resumable_sweep.py --help cites a deleted record. (7) The rationale strings in tests/acceptance/bands.py cite BACKLOG.md, which is gone. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>The test checks a property of the grid (its sum equals the final score, the halves match the outs), not ten remembered numbers.</t>
+          <t>Each text says what is true.</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>Rewrite the assertions as invariants and delete the pinned table.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="132" customHeight="1" s="15">
+          <t>One edit per text; list the runtime-string changes in CHANGES.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="154.5" customHeight="1" s="15">
       <c r="A59" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2354,31 +2354,31 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>SIM-625</t>
+          <t>SIM-610</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Capture the opening lines every day</t>
+          <t>Similarity and betting: seven small defects</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>No scheduled job captures the opening lines. Nothing calls schedule_opening_line_job (pipeline/etl/opening_line_job.py), and the nightly closing-lines job (scripts/nightly_closing_lines.sh, 10:30 UTC) passes --line-types closing only. The venue backfill (schedule_venue_backfill_job) has no caller either. BettingPros serves the opener after the fact, so scripts/load_historical_odds.py (its default line types are opening and closing) recovers the missing rows: nothing is lost for good. The line-movement page reads the opening-to-closing series. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>(1) SituationSimilarityEngine.query_batch([]) raises instead of returning []. (2) The engines' and the calibrator's __main__ blocks read a DuckDB path that does not exist (../../db/schemas/baseball_simulator.duckdb); the pitcher engine's block builds and prints nothing. (3) CalibrationReport.summary() prints no row for the batter's physical weights. (4) The Similarity Explorer's batter panel (api/routes/similarity_explorer.py) shows the four-way weights 0.40/0.35/0.15/0.10. (5) A log line in batted_ball_similarity.py says 'until SIM-051 ships'. (6) tests/regression/conftest.py scales the situation fixture's index twice. (7) No writer sets is_sharp_book, so sharp_consensus is always None. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>Each night's odds run stores the opening rows of the games it loads, and the venue backfill either runs on a schedule or is retired.</t>
+          <t>Each of the seven is fixed or retired.</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Pass --line-types opening closing in scripts/nightly_closing_lines.sh. Then retire opening_line_job.py, or give it a scheduler entry; decide the venue backfill the same way.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="90" customHeight="1" s="15">
+          <t>One edit each; retire sharp_consensus if no book will be marked sharp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="100.5" customHeight="1" s="15">
       <c r="A60" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2386,31 +2386,31 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>SIM-626</t>
+          <t>SIM-603</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Point the GitHub workflows at master</t>
+          <t>Return the fielder's infield sub-scores in the same order from query_pair as from query</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>docker-release.yml and frontend-release.yml run on a push to main (and on a published release), and the pull_request trigger of ci.yml lists main. The default branch is master, so a push never runs the two release workflows, and a pull request into master gets no pull-request run of CI (the push run still happens). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>For an infielder, similarity/engines/fielder_similarity.py query_pair returns the specialty score in tertiary_score and the error score in quaternary_score; query returns them the other way round, as the Similarity Explorer's labels expect. Two shortstops with different error rates and equal specialty values: query gives 0.0710 / 1.0000, query_pair 1.0000 / 0.0710. The composite and the matrices are right. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>A push to master runs both release workflows (or the owner retires them), and a pull request into master runs CI.</t>
+          <t>query and query_pair agree on every sub-score, and a unit test compares them.</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>Replace main with master in the three triggers, and in the trigger comment at the head of ci.yml.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="90" customHeight="1" s="15">
+          <t>Map the infield tuple in SimilarityResult order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="100.5" customHeight="1" s="15">
       <c r="A61" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2418,31 +2418,31 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>SIM-627</t>
+          <t>SIM-604</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Retire the two odds routes that serve mock lines</t>
+          <t>Apply the per-hand 30-PA platoon rule in the batter engine's pair score</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>GET /api/odds/{game_pk} and GET /api/odds/today/all (pipeline/live/ingestion/odds_routes.py, mounted by api/main.py) always return MockOddsAPI lines, whatever ODDS_PROVIDER says. The rows carry is_mock: true, and no frontend code calls the routes. A client that ignores the flag reads fake prices as real ones. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>similarity/engines/batter_similarity.py _score_pair disagrees with score_all on a thin platoon split. A query with 30+ PA against either hand turns the platoon weights on for any vs_hand (10 PA vs L and 200 vs R with vs_hand='L': 0.8642 against 0.8900), and a candidate under 30 PA never gets the neutral 0.5. It serves query_pair (the Explorer's pair view and the diagnostics); the matrix is unaffected. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>The routes are gone (or serve the stored book rows), and the API snapshot is regenerated.</t>
+          <t>_score_pair and score_all agree, and a unit test compares them.</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Delete both routes, then run scripts/export_openapi.py in the app image and npm run gen:api (CLAUDE.md section 15).</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="90" customHeight="1" s="15">
+          <t>Use score_all's per-hand rule in _score_pair.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="60" customHeight="1" s="15">
       <c r="A62" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2450,31 +2450,31 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>SIM-628</t>
+          <t>SIM-596</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Let the resumable sweep read the database address</t>
+          <t>Decide what the what-if does when the designated hitter takes the field</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>The child process of scripts/resumable_sweep.py reads BASEBALL_DB_DSN from .env with env["BASEBALL_DB_DSN"]. Since the security hardening (SIM-443b), .env carries no such key: .env.example has it commented out, and the live .env has none. So a sweep stops with KeyError before its first game. This is separate from the retry after a crash (SIM-614). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>A designated hitter moved to the field leaves the fielder he replaced in the batting order with no position. The rule that ends the designated hitter is not modelled in simulation/whatif.py. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>A sweep starts on the current .env.</t>
+          <t>The owner decides whether the what-if models the rule, and the code follows.</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>Read BASEBALL_DB_DSN from the process environment first (pipeline.db_dsn.require_dsn); read .env only when the key is set there.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="104" customHeight="1" s="15">
+          <t>Model the rule: the pitcher bats in the replaced fielder's slot, or refuse the change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="60" customHeight="1" s="15">
       <c r="A63" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2482,31 +2482,31 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>SIM-629</t>
+          <t>SIM-598</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>End a tied game at the inning limit without an extra pitch</t>
+          <t>Read the runners under the names the live service sends</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>simulate_game (simulation/sim_loop.py) checks state.inning &gt; max_innings only after a pitch that does not roll the half, and _game_over_after_half knows nothing of the limit. So a game tied after the API's 12 innings (max_innings 12 in simulation/sim_kwargs.py) starts the 13th, places the extra-innings runner on second and throws one pitch before it stops. That pitch can score a run or credit a box line. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>frontend/src/hooks/useGameSocket.ts reads runner_on_first / _second / _third; the live service sends on_1b / on_2b / on_3b. The hook's on_1b to on_3b are always undefined. No page reads them today. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>A game tied at the limit ends when the last allowed half completes, and a unit test pins it.</t>
+          <t>A game_state_update with runners fills the hook's on_1b to on_3b.</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>Check the limit in the roll branch, right after _game_over_after_half.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="104" customHeight="1" s="15">
+          <t>Read gs.on_1b, gs.on_2b and gs.on_3b in mapWsState.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="46.5" customHeight="1" s="15">
       <c r="A64" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2514,31 +2514,31 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>SIM-630</t>
+          <t>SIM-609</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Bring the Postgres schema file up to the migrations</t>
+          <t>Raise on a wrong market or side in the line-movement series</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>db/schemas/01_postgres_schema.sql lags the Alembic migrations. It has no raw.savant_pitch_tracking (0020), no raw.game_bullpen (0025), none of the 0029 columns (raw.game_lineups.published_at, last_seen_at on the odds tables, the run-job columns) and none of the 0030 columns of sim.sim_runs (start_at_bat and the rest). At least eight unit tests read the file to check a schema fact. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>line_movement_from_quotes swallows _side_columns' ValueError, so a wrong market or side gives a silent empty series. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>The file matches the schema that alembic upgrade head builds, and a test holds the two equal; or the file is retired and the tests read the migrations.</t>
+          <t>A wrong market or side raises.</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>Regenerate the file from a migrated database (pg_dump --schema-only), or retire it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="118" customHeight="1" s="15">
+          <t>Call _side_columns once before the loop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="73.5" customHeight="1" s="15">
       <c r="A65" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2546,31 +2546,31 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>SIM-631</t>
+          <t>SIM-599</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Delete or wire up the data nobody reads</t>
+          <t>Describe the slate card's odds field as it is</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>Built and never read: sim.stolen_base_pool (the profile computor builds it every night), the composite catcher actor matrix (built and concentration-checked; the draws read catcher_throwing), the sim.live_games view and raw.savant_first_base_receiving. Declared and never written: derived.outfield_play_detail, derived.infield_play_detail and derived.dp_play_detail. Never called: sim.purge_expired_sessions(), and EngineArtifacts.attach_shared_views outside the tests. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>The route description (api/routes/games_slate.py) and the model (api/routes/games_models.py) call the field 'reserved for the Phase-6 odds-provider integration (SIM-405)'. The field is always None: the card's lines come from /api/betting/games/{pk}/card-odds. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>Each item has a reader, or it is deleted with its builder and its DDL.</t>
+          <t>Both texts say that, with a fresh API snapshot (CLAUDE.md section 15).</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>Delete them, with a migration for the DDL. Keep any the owner wants for planned work, and name the ticket that will read it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="160" customHeight="1" s="15">
+          <t>Rewrite both texts; run scripts/export_openapi.py in the image and npm run gen:api.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="46.5" customHeight="1" s="15">
       <c r="A66" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2578,31 +2578,31 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>SIM-632</t>
+          <t>SIM-600</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Give the backup path one name, and correct the staging and production templates</t>
+          <t>Name the current state in the API's version and health strings</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>The app reads BACKUPS_ROOT (api/routes/metrics.py, docker-compose.yml) while the backup jobs read BACKUP_ROOT (pipeline/backup/data_stores.py, pipeline/backup/offsite.py, db/backup/pg_backup.sh). Both default to /backups, so the age gauges work today; a value set under one name alone splits them. Both env templates set LIVE_PIPELINE_ENABLED=true, which makes the app a second publisher beside the live service. .env.production.example sets ODDS_PROVIDER=theoddsapi, which no provider registers. The templates also carry seven keys no app code reads: WORKERS, SIM_MAX_WORKERS, ODDS_PROVIDER_API_KEY, ODDS_API_BASE, ASYNC_DB_DSN, MLB_API_BASE and PROMETHEUS_PUSHGATEWAY. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>api/main.py carries the app version 0.1.0-phase7, "phase": "6" on /health and "6 - Frontend Build (in progress)" on /. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>One variable names the backup root, and the templates hold only keys the code reads, with values that start the stack.</t>
+          <t>The strings name the current state, or go.</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>Rename the app's variable to BACKUP_ROOT. Rewrite the two templates from .env.example.</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="118" customHeight="1" s="15">
+          <t>Drop the phase keys and set the version from one constant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="202" customHeight="1" s="15">
       <c r="A67" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2610,31 +2610,31 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>SIM-633</t>
+          <t>SIM-634</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Make the test targets run what their names say</t>
+          <t>Small fixes found by the documentation rebuild</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>make test-unit passes no -m "not slow", so it runs the slow tests at the 30 s timeout; CI's unit job excludes them. make test-integration runs in the app container, which has no Docker socket (only the scheduler mounts it), so testcontainers cannot start and every integration test skips. The games input of acceptance-nightly.yml says "max 12" and defaults to 12, but the balanced set has 45 games (beside SIM-581, the roster). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>(1) frontend/index.html links a favicon, /baseball.svg, that frontend/public/ does not hold: a 404 on every page. (2) /ready (api/main.py) writes a redis entry only on a failure, so a healthy Redis is missing from its checks. (3) Six nginx blocks (/health, /ready, /metrics, /docs, /redoc, /openapi.json) set their own Host header, which drops the inherited X-Real-IP and X-Forwarded-For. (4) Nothing deletes the simviz:* explorer cache keys after a nightly rebuild, so a key serves old data for up to 24 h. (5) 12 of the 32 DuckDB migrations do not record themselves in migration_history. (6) Three stale texts: api/state.py calls the situation engine a FAISS engine (it is a KD-tree); the Makefile's gen-secrets comment says a blank key is left alone (gen_secrets.py fills it); scripts/probes/manager_profile_recompute.py says the app must be stopped (the recompute runs beside the app since SIM-524). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>make test-unit matches CI's unit job; make test-integration runs the integration lane or says it needs host Python; the workflow input describes the 45-game set.</t>
+          <t>Each of the six is fixed or retired.</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>Add -m "not slow" to test-unit and a test-slow target. Run the integration lane on host Python, as docs/technical/tests.md describes. Fix the input's text and default.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="202" customHeight="1" s="15">
+          <t>One small commit per area. For (5), record the missing numbers in one new migration rather than editing old files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="46.5" customHeight="1" s="15">
       <c r="A68" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2642,27 +2642,27 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>SIM-634</t>
+          <t>SIM-595</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Small fixes found by the documentation rebuild</t>
+          <t>Fix the article in the what-if's ineligible-player message</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>(1) frontend/index.html links a favicon, /baseball.svg, that frontend/public/ does not hold: a 404 on every page. (2) /ready (api/main.py) writes a redis entry only on a failure, so a healthy Redis is missing from its checks. (3) Six nginx blocks (/health, /ready, /metrics, /docs, /redoc, /openapi.json) set their own Host header, which drops the inherited X-Real-IP and X-Forwarded-For. (4) Nothing deletes the simviz:* explorer cache keys after a nightly rebuild, so a key serves old data for up to 24 h. (5) 12 of the 32 DuckDB migrations do not record themselves in migration_history. (6) Three stale texts: api/state.py calls the situation engine a FAISS engine (it is a KD-tree); the Makefile's gen-secrets comment says a blank key is left alone (gen_secrets.py fills it); scripts/probes/manager_profile_recompute.py says the app must be stopped (the recompute runs beside the app since SIM-524). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>whatif.apply_changes' message for an ineligible pinch hitter reads 'is not an bench hitter'. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t>Each of the six is fixed or retired.</t>
+          <t>Each label reads with its own article.</t>
         </is>
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>One small commit per area. For (5), record the missing numbers in one new migration rather than editing old files.</t>
+          <t>Put the article inside each label.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Delete the closed backlog row of the manager profiles in the API runs (SIM-575); record the deploy
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -560,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -650,7 +650,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="141" customHeight="1" s="15">
+    <row r="6" ht="114" customHeight="1" s="15">
       <c r="A6" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -658,31 +658,31 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>SIM-575</t>
+          <t>SIM-580</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Read each manager's profile in the API's runs, so the steal draw's manager weight is not flat</t>
+          <t>Make the pitcher arsenal fit reproducible: order the pitch rows before the mixture fit</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>The steal draw weighs each row by the batting manager's measured steal rate over the league mean. The API's runs (/simulate, the projections and the what-if) never read the manager profiles. build_sim_kwargs passes con=_get_sim_duckdb(request), and nothing sets app.state.sim_duckdb since the replay store moved to app.state.replay_duckdb. So resolve_manager_profiles_onto_state(state, None) returns at once, the kwargs carry manager_profiles == {0: {}, 1: {}}, and the manager weight reads 1.0 for every team. scripts/sim_stats.py and the accuracy comparison do read the profiles, so the lanes and the users run different simulators. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The pitch-vector query in _compute_pitcher_profiles (pipeline/batch/profiles/pitcher.py) has no ORDER BY. DuckDB's parallel Postgres scan returns the rows in a different order on every read, and the seeded mixture fit (random_state=42) depends on the row order. So every profile rebuild gives a different arsenal for nearly every pitcher (a different number of components for about one pitcher in five), and with it a different pitcher similarity matrix. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>An API run's kwargs carry each side's manager profile and the season's manager league means. A unit test builds the API's kwargs with no DuckDB connection on app.state and finds both.</t>
+          <t>Two profile builds of the same code from the same data write the same arsenals, by content.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Read the profiles through open_sim_duckdb(), as the park-factor snapshot does, or load them into the boot snapshot and read them from there.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="114" customHeight="1" s="15">
+          <t>Add ORDER BY game_pk, at_bat_number, pitch_number to the query. It changes every arsenal once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1" s="15">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -690,31 +690,31 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>SIM-580</t>
+          <t>SIM-606</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Make the pitcher arsenal fit reproducible: order the pitch rows before the mixture fit</t>
+          <t>Pick the small-mixture-component merge target in standardized units</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>The pitch-vector query in _compute_pitcher_profiles (pipeline/batch/profiles/pitcher.py) has no ORDER BY. DuckDB's parallel Postgres scan returns the rows in a different order on every read, and the seeded mixture fit (random_state=42) depends on the row order. So every profile rebuild gives a different arsenal for nearly every pitcher (a different number of components for about one pitcher in five), and with it a different pitcher similarity matrix. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>enforce_min_cluster_size runs before the standardization in the arsenal build, so spin rate (hundreds of rpm) decides the merge over velocity and movement. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Two profile builds of the same code from the same data write the same arsenals, by content.</t>
+          <t>The merge measures the gap in standardized units.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Add ORDER BY game_pk, at_bat_number, pitch_number to the query. It changes every arsenal once.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="60" customHeight="1" s="15">
+          <t>Measure the gap over the mixture's feature_stds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="114" customHeight="1" s="15">
       <c r="A8" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -722,31 +722,31 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>SIM-606</t>
+          <t>SIM-578</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Pick the small-mixture-component merge target in standardized units</t>
+          <t>Load a database NULL as NaN, not 0.0, in the baserunner, catcher, batter and manager engines</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>enforce_min_cluster_size runs before the standardization in the arsenal build, so spin rate (hundreds of rpm) decides the merge over velocity and movement. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The _v helpers of four engines read v or 0.0. A runner with no Savant row gets sprint speed 0 ft/s (still 20 ft/s after a 5-chance shrink, many deviations below the league's 27), so his speed score is about 0 against every measured runner. A runner who never tried reads 0% success; a NULL arm strength reads 0 mph; a manager-season with no bullpen-availability rows reads available_reliever_usage_rate near 0. The two steal engines already load NaN (the running-game work, SIM-531). Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>The merge measures the gap in standardized units.</t>
+          <t>Each of the four engines loads NULL as NaN, and its kernel or shrink handles a NaN feature. The nightly matrices are rebuilt.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Measure the gap over the mixture's feature_stds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="114" customHeight="1" s="15">
+          <t>Map None to NaN in each _v helper and add the features to each engine's NaN set, as the steal engines do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="127.5" customHeight="1" s="15">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -754,31 +754,31 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>SIM-578</t>
+          <t>SIM-577</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Load a database NULL as NaN, not 0.0, in the baserunner, catcher, batter and manager engines</t>
+          <t>Write all thirteen features in the extra-base runner's league-average row</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>The _v helpers of four engines read v or 0.0. A runner with no Savant row gets sprint speed 0 ft/s (still 20 ft/s after a 5-chance shrink, many deviations below the league's 27), so his speed score is about 0 against every measured runner. A runner who never tried reads 0% success; a NULL arm strength reads 0 mph; a manager-season with no bullpen-availability rows reads available_reliever_usage_rate near 0. The two steal engines already load NaN (the running-game work, SIM-531). Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The baserunner row of derived.league_averages holds extra_base_attempt_rate, extra_base_success_rate, sb_success_rate, sprint_speed and the Savant rate. The engine reads thirteen features, so the four per-situation attempt rates, stop_rate and the four per-situation success rates shrink toward 0.0. The matrix build loads the thin profiles, so the effect is large there: a 5-chance runner's first-to-third attempt rate reads 0.35 -&gt; 0.088. The error reaches the runner_adv matrix, which weights the advancement draws. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Each of the four engines loads NULL as NaN, and its kernel or shrink handles a NaN feature. The nightly matrices are rebuilt.</t>
+          <t>The runner's league row carries every engine feature, and a missing key reads as NaN. The nightly matrices are rebuilt.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Map None to NaN in each _v helper and add the features to each engine's NaN set, as the steal engines do.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="127.5" customHeight="1" s="15">
+          <t>Write the engine's thirteen feature keys in the computor's baserunner league row; read a missing key as NaN in similarity/engines/baserunner_similarity.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="114" customHeight="1" s="15">
       <c r="A10" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -786,27 +786,27 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SIM-577</t>
+          <t>SIM-576</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Write all thirteen features in the extra-base runner's league-average row</t>
+          <t>Write the catcher engine's feature names in the catcher's league-average row</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>The baserunner row of derived.league_averages holds extra_base_attempt_rate, extra_base_success_rate, sb_success_rate, sprint_speed and the Savant rate. The engine reads thirteen features, so the four per-situation attempt rates, stop_rate and the four per-situation success rates shrink toward 0.0. The matrix build loads the thin profiles, so the effect is large there: a 5-chance runner's first-to-third attempt rate reads 0.35 -&gt; 0.088. The error reaches the runner_adv matrix, which weights the advancement draws. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The profile computor writes the catcher row of derived.league_averages with the keys framing_runs, blocking_runs and cs_rate. The catcher engine reads its eleven feature names with pj.get(f, 0.0) or 0.0, and only cs_rate matches. So the shrinkage pulls ten features toward 0.0: a constructed 300-pitch catcher reads pop time 1.95 -&gt; 1.857 s and arm strength 81 -&gt; 77.1 mph. The error reaches the catcher and catcher_throwing score matrices, which weight the steal and pickoff draws. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>The runner's league row carries every engine feature, and a missing key reads as NaN. The nightly matrices are rebuilt.</t>
+          <t>The catcher's league row carries every engine feature. A missing key reads as NaN, as the steal engines do. The nightly matrices are rebuilt.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Write the engine's thirteen feature keys in the computor's baserunner league row; read a missing key as NaN in similarity/engines/baserunner_similarity.py.</t>
+          <t>In pipeline/batch/profiles (the catcher league row), write the engine's eleven feature keys. In similarity/engines/catcher_similarity.py _load_league_averages, read a missing key as NaN.</t>
         </is>
       </c>
     </row>
@@ -818,31 +818,31 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SIM-576</t>
+          <t>SIM-579</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Write the catcher engine's feature names in the catcher's league-average row</t>
+          <t>Select the pitcher's zone-take rate before the chase rate, so the two stay in feature order</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>The profile computor writes the catcher row of derived.league_averages with the keys framing_runs, blocking_runs and cs_rate. The catcher engine reads its eleven feature names with pj.get(f, 0.0) or 0.0, and only cs_rate matches. So the shrinkage pulls ten features toward 0.0: a constructed 300-pitch catcher reads pop time 1.95 -&gt; 1.857 s and arm strength 81 -&gt; 77.1 mph. The error reaches the catcher and catcher_throwing score matrices, which weight the steal and pickoff draws. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>In similarity/engines/pitcher_similarity.py _load_profiles, the SELECT returns chase_rate, zone_take_rate and the unpack names them zone_take_rate, chase_rate. So command_vec holds them in the opposite order to COMMAND_FEATURES and the league-average vector, and the shrinkage pulls each pitcher's chase rate toward the league's zone-take rate (weight 1 - alpha, at most 2.4% at 200 pitches). The kernel itself ignores the order. The error reaches the pitcher similarity matrix. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>The catcher's league row carries every engine feature. A missing key reads as NaN, as the steal engines do. The nightly matrices are rebuilt.</t>
+          <t>The SELECT order matches COMMAND_FEATURES, and a unit test pins it. The nightly matrices are rebuilt.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>In pipeline/batch/profiles (the catcher league row), write the engine's eleven feature keys. In similarity/engines/catcher_similarity.py _load_league_averages, read a missing key as NaN.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="114" customHeight="1" s="15">
+          <t>Select zone_take_rate before chase_rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="127.5" customHeight="1" s="15">
       <c r="A12" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -850,31 +850,31 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>SIM-579</t>
+          <t>SIM-611</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Select the pitcher's zone-take rate before the chase rate, so the two stay in feature order</t>
+          <t>Owner decisions: four similarity design points</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>In similarity/engines/pitcher_similarity.py _load_profiles, the SELECT returns chase_rate, zone_take_rate and the unpack names them zone_take_rate, chase_rate. So command_vec holds them in the opposite order to COMMAND_FEATURES and the league-average vector, and the shrinkage pulls each pitcher's chase rate toward the league's zone-take rate (weight 1 - alpha, at most 2.4% at 200 pitches). The kernel itself ignores the order. The error reaches the pitcher similarity matrix. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>Not defects, design points for the owner. (1) The catcher's shrinkage prior is 15 called pitches, so alpha is at least 0.95 for every kept catcher (framing stabilizes near 1,500). (2) stop_rate is exactly one minus the overall attempt rate, so that rate counts twice in the runner's aggression distance. (3) The batter's xba / xslg and the manager's hit-and-run and double-switch rates read 0.0 for everyone and still hold their share of the kernel weight. (4) CLAUDE.md section 1 calls CLV 'the gold-standard metric'; the owner ruled on 2026-09-28 that the model is not judged by it. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>The SELECT order matches COMMAND_FEATURES, and a unit test pins it. The nightly matrices are rebuilt.</t>
+          <t>The owner rules on each point, and the code or CLAUDE.md follows.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Select zone_take_rate before chase_rate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="127.5" customHeight="1" s="15">
+          <t>Raise the catcher prior; drop stop_rate; drop the all-zero features; rewrite CLAUDE.md section 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="87" customHeight="1" s="15">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -882,31 +882,31 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>SIM-611</t>
+          <t>SIM-587</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Owner decisions: four similarity design points</t>
+          <t>Decide which calibration values the draws use, and make the code follow</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Not defects, design points for the owner. (1) The catcher's shrinkage prior is 15 called pitches, so alpha is at least 0.95 for every kept catcher (framing stabilizes near 1,500). (2) stop_rate is exactly one minus the overall attempt rate, so that rate counts twice in the runner's aggression distance. (3) The batter's xba / xslg and the manager's hit-and-run and double-switch rates read 0.0 for everyone and still hold their share of the kernel weight. (4) CLAUDE.md section 1 calls CLV 'the gold-standard metric'; the owner ruled on 2026-09-28 that the model is not judged by it. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>similarity/calibration/pitcher.py fits sigma_command and eb_n_prior_pitcher, and no code reads either, so the pitcher engine keeps RBF_SIGMA_COMMAND 1.0453 and EB_N_PRIOR 5. More broadly, the nightly actor matrices apply no calibration report (build_actor_sim_matrices): make calibrate changes only the API's engines. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>The owner rules on each point, and the code or CLAUDE.md follows.</t>
+          <t>The owner decides which values the draws use, and the code and the docs follow.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Raise the catcher prior; drop stop_rate; drop the all-zero features; rewrite CLAUDE.md section 1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="87" customHeight="1" s="15">
+          <t>Read both fields in apply_calibration and apply /data/calibration.json in the matrix build; or document the module defaults as the draws' values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="73.5" customHeight="1" s="15">
       <c r="A14" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -914,31 +914,31 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>SIM-587</t>
+          <t>SIM-583</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Decide which calibration values the draws use, and make the code follow</t>
+          <t>Keep the calibrated win probability strictly between 0 and 1</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>similarity/calibration/pitcher.py fits sigma_command and eb_n_prior_pitcher, and no code reads either, so the pitcher engine keeps RBF_SIGMA_COMMAND 1.0453 and EB_N_PRIOR 5. More broadly, the nightly actor matrices apply no calibration report (build_actor_sim_matrices): make calibrate changes only the API's engines. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>build_validation_report fits the reliability curve with min_bin_count=1, so a bin of two games can map 0.75 to 1.0. Example: the curve [[0,0],[0.45,0.44],[0.55,0.56],[0.73,1.0],[1,1]] and home_win_pct 0.75 at n = 100 give home 1.0, away 0.0 and an interval of zero width. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>The owner decides which values the draws use, and the code and the docs follow.</t>
+          <t>No calibrated probability is 0.0 or 1.0, and a unit test feeds the curve above.</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Read both fields in apply_calibration and apply /data/calibration.json in the matrix build; or document the module defaults as the draws' values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="73.5" customHeight="1" s="15">
+          <t>Fit the curve with a min_bin_count near 30, or clamp the mapped probability to [eps, 1 - eps].</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="127.5" customHeight="1" s="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -946,59 +946,59 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>SIM-583</t>
+          <t>SIM-584</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Keep the calibrated win probability strictly between 0 and 1</t>
+          <t>Stamp the accuracy report with the bundle the run read, not the live link</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>build_validation_report fits the reliability curve with min_bin_count=1, so a bin of two games can map 0.75 to 1.0. Example: the curve [[0,0],[0.45,0.44],[0.55,0.56],[0.73,1.0],[1,1]] and home_win_pct 0.75 at n = 100 give home 1.0, away 0.0 and an interval of zero width. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/accuracy/selection.py bundle_provenance reads the manifest times under BASEBALL_PLAY_POOL_DIR/engine_artifacts (the live link). The factory reads BASEBALL_ENGINE_ARTIFACT_DIR when it is set (simulation/production_factory.py). Seen on 2026-10-20: two runs on the same pinned bundle, before and after the nightly rebuild, carry different manifest_mtimes and identical records, so pair_accuracy.py refuses to pair them; two runs on different pinned bundles on one day would pair. The weight fit (SIM-548) pairs these reports. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>No calibrated probability is 0.0 or 1.0, and a unit test feeds the curve above.</t>
+          <t>The stamp names the bundle the run read, and a test pins the pinned-directory case.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Fit the curve with a min_bin_count near 30, or clamp the mapped probability to [eps, 1 - eps].</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="127.5" customHeight="1" s="15">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Read the pinned directory first, as the factory does.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="81" customHeight="1" s="15">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>SIM-584</t>
+          <t>SIM-547</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Stamp the accuracy report with the bundle the run read, not the live link</t>
+          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>scripts/accuracy/selection.py bundle_provenance reads the manifest times under BASEBALL_PLAY_POOL_DIR/engine_artifacts (the live link). The factory reads BASEBALL_ENGINE_ARTIFACT_DIR when it is set (simulation/production_factory.py). Seen on 2026-10-20: two runs on the same pinned bundle, before and after the nightly rebuild, carry different manifest_mtimes and identical records, so pair_accuracy.py refuses to pair them; two runs on different pinned bundles on one day would pair. The weight fit (SIM-548) pairs these reports. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>The stamp names the bundle the run read, and a test pins the pinned-directory case.</t>
+          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Read the pinned directory first, as the factory does.</t>
+          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/probes/manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
         </is>
       </c>
     </row>
@@ -1010,27 +1010,27 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>SIM-547</t>
+          <t>SIM-526</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
+          <t>Turn on the catcher pitch-receiving factor</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
+          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
+          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/probes/manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
+          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
         </is>
       </c>
     </row>
@@ -1042,27 +1042,27 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>SIM-526</t>
+          <t>SIM-556</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Turn on the catcher pitch-receiving factor</t>
+          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
+          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/probes/steal_weight_volume_probe.py with its records (docs/audit/records/steal_weight_volume_probe_2025.* and _2026.*; the arrays in results/steal_weight_volume/). Filed P3 by the owner on 2026-10-01.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
+          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
+          <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/probes/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
         </is>
       </c>
     </row>
@@ -1074,31 +1074,31 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>SIM-556</t>
+          <t>SIM-574</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
+          <t>Make each SIM_* flag's code default equal its production value, or record why it differs</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/probes/steal_weight_volume_probe.py with its records (docs/audit/records/steal_weight_volume_probe_2025.* and _2026.*; the arrays in results/steal_weight_volume/). Filed P3 by the owner on 2026-10-01.</t>
+          <t>The simulator reads its switches and weights from SIM_* environment flags. Each flag has a default in the code (the value an unset flag reads) and a production value set in the app service of docker-compose.yml. They differ for 24 of the flags compose sets (measured 2026-10-20): for example the pitch-draw cell index is off in code and on in production, and the fence stage, the fielding class filter and the manager draw are the same. So a script, a probe or a test that forgets one flag runs a different simulator from production, silently. The registry of the flags (simulation/flags.py, the code clean-up SIM-493) now lists every default in one table, which makes the gap visible but does not close it.</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
+          <t>For every registered flag the code default equals the compose value, or the registry row says in one line why it differs (for example: the unit lane's byte-identical state). The unit lane's own pins in tests/conftest.py still hold its state. The fingerprint (scripts/behaviour_fingerprint.py) of production is unchanged, because compose already sets the production values.</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/probes/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="81" customHeight="1" s="15">
+          <t>Owner decision first: should an unset flag mean production or off? If production: change each default in simulation/flags.py to the compose value, keep tests/conftest.py's pins for the unit lane, and add a registry test that the defaults equal compose. If off: add the reason column to the registry and a test that compose sets every flag whose default differs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="73.5" customHeight="1" s="15">
       <c r="A20" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1106,27 +1106,27 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>SIM-574</t>
+          <t>SIM-608</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Make each SIM_* flag's code default equal its production value, or record why it differs</t>
+          <t>Store a price that returns to an earlier value</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>The simulator reads its switches and weights from SIM_* environment flags. Each flag has a default in the code (the value an unset flag reads) and a production value set in the app service of docker-compose.yml. They differ for 24 of the flags compose sets (measured 2026-10-20): for example the pitch-draw cell index is off in code and on in production, and the fence stage, the fielding class filter and the manager draw are the same. So a script, a probe or a test that forgets one flag runs a different simulator from production, silently. The registry of the flags (simulation/flags.py, the code clean-up SIM-493) now lists every default in one table, which makes the gap visible but does not close it.</t>
+          <t>The odds writer dedups on a hash with no time (ON CONFLICT (game_pk, source, odds_hash)), so -110 at t0, -120 at t1, -110 at t2 closes the series at -120. Read from the code, not checked against stored data. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>For every registered flag the code default equals the compose value, or the registry row says in one line why it differs (for example: the unit lane's byte-identical state). The unit lane's own pins in tests/conftest.py still hold its state. The fingerprint (scripts/behaviour_fingerprint.py) of production is unchanged, because compose already sets the production values.</t>
+          <t>A return to an earlier price is stored, and the series closes on the last price.</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Owner decision first: should an unset flag mean production or off? If production: change each default in simulation/flags.py to the compose value, keep tests/conftest.py's pins for the unit lane, and add a registry test that the defaults equal compose. If off: add the reason column to the registry and a test that compose sets every flag whose default differs.</t>
+          <t>Dedup only against the latest row of the same game, source, book, market and line type.</t>
         </is>
       </c>
     </row>
@@ -1138,31 +1138,31 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>SIM-608</t>
+          <t>SIM-607</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Store a price that returns to an earlier value</t>
+          <t>Read the line-movement direction book by book</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>The odds writer dedups on a hash with no time (ON CONFLICT (game_pk, source, odds_hash)), so -110 at t0, -120 at t1, -110 at t2 closes the series at -120. Read from the code, not checked against stored data. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>betting/line_movement.py _net_direction pools every book, so the first and last quotes can come from two books: (t1, bp:1, -110/-110) and (t2, bp:2, -130/+110) give direction 'toward' and a CLV, though neither book moved. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>A return to an earlier price is stored, and the series closes on the last price.</t>
+          <t>The direction is each book's own, then aggregated.</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Dedup only against the latest row of the same game, source, book, market and line type.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="73.5" customHeight="1" s="15">
+          <t>Compute the direction per book, then aggregate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="132" customHeight="1" s="15">
       <c r="A22" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1170,31 +1170,31 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>SIM-607</t>
+          <t>SIM-625</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Read the line-movement direction book by book</t>
+          <t>Capture the opening lines every day</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>betting/line_movement.py _net_direction pools every book, so the first and last quotes can come from two books: (t1, bp:1, -110/-110) and (t2, bp:2, -130/+110) give direction 'toward' and a CLV, though neither book moved. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>No scheduled job captures the opening lines. Nothing calls schedule_opening_line_job (pipeline/etl/opening_line_job.py), and the nightly closing-lines job (scripts/nightly_closing_lines.sh, 10:30 UTC) passes --line-types closing only. The venue backfill (schedule_venue_backfill_job) has no caller either. BettingPros serves the opener after the fact, so scripts/load_historical_odds.py (its default line types are opening and closing) recovers the missing rows: nothing is lost for good. The line-movement page reads the opening-to-closing series. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>The direction is each book's own, then aggregated.</t>
+          <t>Each night's odds run stores the opening rows of the games it loads, and the venue backfill either runs on a schedule or is retired.</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Compute the direction per book, then aggregate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="132" customHeight="1" s="15">
+          <t>Pass --line-types opening closing in scripts/nightly_closing_lines.sh. Then retire opening_line_job.py, or give it a scheduler entry; decide the venue backfill the same way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="60" customHeight="1" s="15">
       <c r="A23" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1202,31 +1202,31 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>SIM-625</t>
+          <t>SIM-586</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Capture the opening lines every day</t>
+          <t>Ask the schedule only for game types raw.games accepts</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>No scheduled job captures the opening lines. Nothing calls schedule_opening_line_job (pipeline/etl/opening_line_job.py), and the nightly closing-lines job (scripts/nightly_closing_lines.sh, 10:30 UTC) passes --line-types closing only. The venue backfill (schedule_venue_backfill_job) has no caller either. BettingPros serves the opener after the fact, so scripts/load_historical_odds.py (its default line types are opening and closing) recovers the missing rows: nothing is lost for good. The line-movement page reads the opening-to-closing series. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>GAME_TYPES (pipeline/live/ingestion/constants.py) is R F D L W C P; the CHECK on raw.games allows R P S A D F L W. A game of type C on the slate fails its upsert. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Each night's odds run stores the opening rows of the games it loads, and the venue backfill either runs on a schedule or is retired.</t>
+          <t>The live pipeline's game types and the table's CHECK agree, and a unit test compares them.</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Pass --line-types opening closing in scripts/nightly_closing_lines.sh. Then retire opening_line_job.py, or give it a scheduler entry; decide the venue backfill the same way.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="60" customHeight="1" s="15">
+          <t>Drop C from GAME_TYPES, or widen the CHECK with a migration if type C games should load.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="114" customHeight="1" s="15">
       <c r="A24" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1234,31 +1234,31 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>SIM-586</t>
+          <t>SIM-582</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Ask the schedule only for game types raw.games accepts</t>
+          <t>Add last_seen_at to the two odds archive tables, so the retirement copy fits again</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>GAME_TYPES (pipeline/live/ingestion/constants.py) is R F D L W C P; the CHECK on raw.games allows R P S A D F L W. A game of type C on the slate fails its upsert. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>Migration 0029 added last_seen_at to raw.game_odds and raw.prop_odds and not to their archives (raw.game_odds_archive, raw.prop_odds_archive, migration 0028). The retirement script copies rows with INSERT ... SELECT *, which needs the same columns in the same order, so the next retirement fails. The integration test test_schema_migrations.py::test_sim555_stamp_indexes_and_archives reds on master fe81d79 and on the clean-up branch for this reason. Found by the code clean-up (SIM-493, the integration pass, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>The live pipeline's game types and the table's CHECK agree, and a unit test compares them.</t>
+          <t>Both archives carry last_seen_at in the live table's position, the integration test passes, and a retirement run copies a row.</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Drop C from GAME_TYPES, or widen the CHECK with a migration if type C games should load.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="114" customHeight="1" s="15">
+          <t>A new Alembic migration adds last_seen_at to both archives (nullable, so the copied rows keep their value), placed after book_line_at to match the live tables; check the column order with the test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="87" customHeight="1" s="15">
       <c r="A25" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1266,31 +1266,31 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>SIM-582</t>
+          <t>SIM-581</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Add last_seen_at to the two odds archive tables, so the retirement copy fits again</t>
+          <t>Name only real tests in the nightly acceptance lane's required roster</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Migration 0029 added last_seen_at to raw.game_odds and raw.prop_odds and not to their archives (raw.game_odds_archive, raw.prop_odds_archive, migration 0028). The retirement script copies rows with INSERT ... SELECT *, which needs the same columns in the same order, so the next retirement fails. The integration test test_schema_migrations.py::test_sim555_stamp_indexes_and_archives reds on master fe81d79 and on the clean-up branch for this reason. Found by the code clean-up (SIM-493, the integration pass, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The REQUIRED roster of .github/workflows/acceptance-nightly.yml lists test_full_pool_out_advancement_runs_sim450, test_full_pool_steal_decision_runs_sim450 and test_reach_on_error_band_sim450. No test of those names exists, and the roster step fails when a required name did not run. So the nightly lane reds on every run, whatever the bands read. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Both archives carry last_seen_at in the live table's position, the integration test passes, and a retirement run copies a row.</t>
+          <t>The roster names only real tests, and one nightly run passes its roster step.</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>A new Alembic migration adds last_seen_at to both archives (nullable, so the copied rows keep their value), placed after book_line_at to match the live tables; check the column order with the test.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="87" customHeight="1" s="15">
+          <t>Delete the three names, or name the tests that took their place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="118" customHeight="1" s="15">
       <c r="A26" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1298,31 +1298,31 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>SIM-581</t>
+          <t>SIM-633</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Name only real tests in the nightly acceptance lane's required roster</t>
+          <t>Make the test targets run what their names say</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>The REQUIRED roster of .github/workflows/acceptance-nightly.yml lists test_full_pool_out_advancement_runs_sim450, test_full_pool_steal_decision_runs_sim450 and test_reach_on_error_band_sim450. No test of those names exists, and the roster step fails when a required name did not run. So the nightly lane reds on every run, whatever the bands read. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>make test-unit passes no -m "not slow", so it runs the slow tests at the 30 s timeout; CI's unit job excludes them. make test-integration runs in the app container, which has no Docker socket (only the scheduler mounts it), so testcontainers cannot start and every integration test skips. The games input of acceptance-nightly.yml says "max 12" and defaults to 12, but the balanced set has 45 games (beside SIM-581, the roster). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>The roster names only real tests, and one nightly run passes its roster step.</t>
+          <t>make test-unit matches CI's unit job; make test-integration runs the integration lane or says it needs host Python; the workflow input describes the 45-game set.</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Delete the three names, or name the tests that took their place.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="118" customHeight="1" s="15">
+          <t>Add -m "not slow" to test-unit and a test-slow target. Run the integration lane on host Python, as docs/technical/tests.md describes. Fix the input's text and default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="90" customHeight="1" s="15">
       <c r="A27" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1330,31 +1330,31 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>SIM-633</t>
+          <t>SIM-626</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Make the test targets run what their names say</t>
+          <t>Point the GitHub workflows at master</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>make test-unit passes no -m "not slow", so it runs the slow tests at the 30 s timeout; CI's unit job excludes them. make test-integration runs in the app container, which has no Docker socket (only the scheduler mounts it), so testcontainers cannot start and every integration test skips. The games input of acceptance-nightly.yml says "max 12" and defaults to 12, but the balanced set has 45 games (beside SIM-581, the roster). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>docker-release.yml and frontend-release.yml run on a push to main (and on a published release), and the pull_request trigger of ci.yml lists main. The default branch is master, so a push never runs the two release workflows, and a pull request into master gets no pull-request run of CI (the push run still happens). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>make test-unit matches CI's unit job; make test-integration runs the integration lane or says it needs host Python; the workflow input describes the 45-game set.</t>
+          <t>A push to master runs both release workflows (or the owner retires them), and a pull request into master runs CI.</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Add -m "not slow" to test-unit and a test-slow target. Run the integration lane on host Python, as docs/technical/tests.md describes. Fix the input's text and default.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="90" customHeight="1" s="15">
+          <t>Replace main with master in the three triggers, and in the trigger comment at the head of ci.yml.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="73.5" customHeight="1" s="15">
       <c r="A28" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1362,27 +1362,27 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>SIM-626</t>
+          <t>SIM-619</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Point the GitHub workflows at master</t>
+          <t>Run the batch-runner stress test in a CI job</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>docker-release.yml and frontend-release.yml run on a push to main (and on a published release), and the pull_request trigger of ci.yml lists main. The default branch is master, so a push never runs the two release workflows, and a pull request into master gets no pull-request run of CI (the push run still happens). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>tests/integration/test_batch_runner_stress.py carries only the slow marker. The CI slow lane runs tests/unit -m slow; the weekly integration lane and make test-integration select -m integration; the e2e job runs one file. No job runs it. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>A push to master runs both release workflows (or the owner retires them), and a pull request into master runs CI.</t>
+          <t>One lane runs it.</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Replace main with master in the three triggers, and in the trigger comment at the head of ci.yml.</t>
+          <t>Mark it integration, or add its path to the slow lane.</t>
         </is>
       </c>
     </row>
@@ -1394,31 +1394,31 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>SIM-619</t>
+          <t>SIM-602</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Run the batch-runner stress test in a CI job</t>
+          <t>Make two API tests check what their names say</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>tests/integration/test_batch_runner_stress.py carries only the slow marker. The CI slow lane runs tests/unit -m slow; the weekly integration lane and make test-integration select -m integration; the e2e job runs one file. No job runs it. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>tests/unit/test_api_betting.py test_clv_snapshot_returns_only_series_with_clv makes a GET and asserts nothing. tests/unit/test_api_games_plays.py test_simulate_ok_without_duckdb_then_plays_404 never requests /plays. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>One lane runs it.</t>
+          <t>Each test asserts what its name says.</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Mark it integration, or add its path to the slow lane.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="73.5" customHeight="1" s="15">
+          <t>Add the assertions (the CLV series' filter; /plays answers 503 with no replay store), then rename the second test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="87" customHeight="1" s="15">
       <c r="A30" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1426,31 +1426,31 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>SIM-602</t>
+          <t>SIM-601</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Make two API tests check what their names say</t>
+          <t>Make the Playwright smoke tests pass while the live app runs</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>tests/unit/test_api_betting.py test_clv_snapshot_returns_only_series_with_clv makes a GET and asserts nothing. tests/unit/test_api_games_plays.py test_simulate_ok_without_duckdb_then_plays_404 never requests /plays. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>frontend/e2e/smoke.spec.ts (three specs) fail on the owner's host: a request the test does not mock goes through the preview server's proxy to localhost:8000, the live app answers 401 and the page shows the login. With API_TARGET=http://127.0.0.1:9 all 21 tests pass; CI has no backend, so CI passes. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Each test asserts what its name says.</t>
+          <t>The e2e suite passes with the live app running.</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Add the assertions (the CLV series' filter; /plays answers 503 with no replay store), then rename the second test.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="87" customHeight="1" s="15">
+          <t>Set API_TARGET to a closed port in playwright.config.ts's webServer.env, or end each spec with a catch-all **/api/** route that answers 404.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="104" customHeight="1" s="15">
       <c r="A31" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1458,31 +1458,31 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>SIM-601</t>
+          <t>SIM-630</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Make the Playwright smoke tests pass while the live app runs</t>
+          <t>Bring the Postgres schema file up to the migrations</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>frontend/e2e/smoke.spec.ts (three specs) fail on the owner's host: a request the test does not mock goes through the preview server's proxy to localhost:8000, the live app answers 401 and the page shows the login. With API_TARGET=http://127.0.0.1:9 all 21 tests pass; CI has no backend, so CI passes. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>db/schemas/01_postgres_schema.sql lags the Alembic migrations. It has no raw.savant_pitch_tracking (0020), no raw.game_bullpen (0025), none of the 0029 columns (raw.game_lineups.published_at, last_seen_at on the odds tables, the run-job columns) and none of the 0030 columns of sim.sim_runs (start_at_bat and the rest). At least eight unit tests read the file to check a schema fact. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>The e2e suite passes with the live app running.</t>
+          <t>The file matches the schema that alembic upgrade head builds, and a test holds the two equal; or the file is retired and the tests read the migrations.</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Set API_TARGET to a closed port in playwright.config.ts's webServer.env, or end each spec with a catch-all **/api/** route that answers 404.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="104" customHeight="1" s="15">
+          <t>Regenerate the file from a migrated database (pg_dump --schema-only), or retire it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="87" customHeight="1" s="15">
       <c r="A32" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1490,31 +1490,31 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>SIM-630</t>
+          <t>SIM-585</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Bring the Postgres schema file up to the migrations</t>
+          <t>Refuse CORS_ORIGINS=* while the API sends credentials</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>db/schemas/01_postgres_schema.sql lags the Alembic migrations. It has no raw.savant_pitch_tracking (0020), no raw.game_bullpen (0025), none of the 0029 columns (raw.game_lineups.published_at, last_seen_at on the odds tables, the run-job columns) and none of the 0030 columns of sim.sim_runs (start_at_bat and the rest). At least eight unit tests read the file to check a schema fact. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>api/main.py sets allow_credentials=True for every origin list, and resolve_cors_origins (api/auth.py) returns ['*'] when an operator sets CORS_ORIGINS=*. Starlette then echoes the caller's Origin on a request with a cookie, so any site can read the API with the user's login. Production sets neither variable today, so the defect is latent. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>The file matches the schema that alembic upgrade head builds, and a test holds the two equal; or the file is retired and the tests read the migrations.</t>
+          <t>CORS_ORIGINS=* either fails the boot or turns credentials off, and a unit test pins it.</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Regenerate the file from a migrated database (pg_dump --schema-only), or retire it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="87" customHeight="1" s="15">
+          <t>Refuse '*' in resolve_cors_origins while credentials are on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="160" customHeight="1" s="15">
       <c r="A33" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1522,31 +1522,31 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>SIM-585</t>
+          <t>SIM-632</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Refuse CORS_ORIGINS=* while the API sends credentials</t>
+          <t>Give the backup path one name, and correct the staging and production templates</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>api/main.py sets allow_credentials=True for every origin list, and resolve_cors_origins (api/auth.py) returns ['*'] when an operator sets CORS_ORIGINS=*. Starlette then echoes the caller's Origin on a request with a cookie, so any site can read the API with the user's login. Production sets neither variable today, so the defect is latent. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The app reads BACKUPS_ROOT (api/routes/metrics.py, docker-compose.yml) while the backup jobs read BACKUP_ROOT (pipeline/backup/data_stores.py, pipeline/backup/offsite.py, db/backup/pg_backup.sh). Both default to /backups, so the age gauges work today; a value set under one name alone splits them. Both env templates set LIVE_PIPELINE_ENABLED=true, which makes the app a second publisher beside the live service. .env.production.example sets ODDS_PROVIDER=theoddsapi, which no provider registers. The templates also carry seven keys no app code reads: WORKERS, SIM_MAX_WORKERS, ODDS_PROVIDER_API_KEY, ODDS_API_BASE, ASYNC_DB_DSN, MLB_API_BASE and PROMETHEUS_PUSHGATEWAY. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>CORS_ORIGINS=* either fails the boot or turns credentials off, and a unit test pins it.</t>
+          <t>One variable names the backup root, and the templates hold only keys the code reads, with values that start the stack.</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Refuse '*' in resolve_cors_origins while credentials are on.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="160" customHeight="1" s="15">
+          <t>Rename the app's variable to BACKUP_ROOT. Rewrite the two templates from .env.example.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="104" customHeight="1" s="15">
       <c r="A34" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1554,31 +1554,31 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>SIM-632</t>
+          <t>SIM-629</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Give the backup path one name, and correct the staging and production templates</t>
+          <t>End a tied game at the inning limit without an extra pitch</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>The app reads BACKUPS_ROOT (api/routes/metrics.py, docker-compose.yml) while the backup jobs read BACKUP_ROOT (pipeline/backup/data_stores.py, pipeline/backup/offsite.py, db/backup/pg_backup.sh). Both default to /backups, so the age gauges work today; a value set under one name alone splits them. Both env templates set LIVE_PIPELINE_ENABLED=true, which makes the app a second publisher beside the live service. .env.production.example sets ODDS_PROVIDER=theoddsapi, which no provider registers. The templates also carry seven keys no app code reads: WORKERS, SIM_MAX_WORKERS, ODDS_PROVIDER_API_KEY, ODDS_API_BASE, ASYNC_DB_DSN, MLB_API_BASE and PROMETHEUS_PUSHGATEWAY. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>simulate_game (simulation/sim_loop.py) checks state.inning &gt; max_innings only after a pitch that does not roll the half, and _game_over_after_half knows nothing of the limit. So a game tied after the API's 12 innings (max_innings 12 in simulation/sim_kwargs.py) starts the 13th, places the extra-innings runner on second and throws one pitch before it stops. That pitch can score a run or credit a box line. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>One variable names the backup root, and the templates hold only keys the code reads, with values that start the stack.</t>
+          <t>A game tied at the limit ends when the last allowed half completes, and a unit test pins it.</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Rename the app's variable to BACKUP_ROOT. Rewrite the two templates from .env.example.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="104" customHeight="1" s="15">
+          <t>Check the limit in the roll branch, right after _game_over_after_half.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="60" customHeight="1" s="15">
       <c r="A35" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1586,31 +1586,31 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>SIM-629</t>
+          <t>SIM-594</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>End a tied game at the inning limit without an extra pitch</t>
+          <t>Let the batter run on a called third strike that gets away</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>simulate_game (simulation/sim_loop.py) checks state.inning &gt; max_innings only after a pitch that does not roll the half, and _game_over_after_half knows nothing of the limit. So a game tied after the API's 12 innings (max_innings 12 in simulation/sim_kwargs.py) starts the 13th, places the extra-innings runner on second and throws one pitch before it stops. That pitch can score a run or credit a box line. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>Rule 5.05(a)(2) lets the batter run on any uncaught third strike. _dropped_third_strike reads swinging strikes only. Two such rows exist in 2023-2026, both in 2026. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>A game tied at the limit ends when the last allowed half completes, and a unit test pins it.</t>
+          <t>A called third strike that gets away can be a dropped-third-strike reach.</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Check the limit in the roll branch, right after _game_over_after_half.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="60" customHeight="1" s="15">
+          <t>Let _dropped_third_strike read a called third strike too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="73.5" customHeight="1" s="15">
       <c r="A36" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1618,27 +1618,27 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>SIM-594</t>
+          <t>SIM-591</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Let the batter run on a called third strike that gets away</t>
+          <t>Charge the losing pitcher with the go-ahead run, as MLB does</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Rule 5.05(a)(2) lets the batter run on any uncaught third strike. _dropped_third_strike reads swinging strikes only. Two such rows exist in 2023-2026, both in 2026. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>pitcher_decisions charges the pitcher on the mound at the decisive play. In a tie, A walks a batter, B relieves him and allows a double that scores the runner, and the lead holds: MLB charges A; the simulator charges B. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>A called third strike that gets away can be a dropped-third-strike reach.</t>
+          <t>The decision follows the runner's responsible pitcher, and a unit test plays the example.</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Let _dropped_third_strike read a called third strike too.</t>
+          <t>Carry each runner's responsible pitcher on the bases.</t>
         </is>
       </c>
     </row>
@@ -1650,27 +1650,27 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>SIM-591</t>
+          <t>SIM-592</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Charge the losing pitcher with the go-ahead run, as MLB does</t>
+          <t>Put the batter on first after a forced reach with no batter id</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>pitcher_decisions charges the pitcher on the mound at the decisive play. In a tie, A walks a batter, B relieves him and allows a double that scores the runner, and the lead holds: MLB charges A; the simulator charges B. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>_force_on_reach with no batter id leaves first base's runner on first after pushing him to second (b.first = state.batter_id if ... else b.first), so the base check raises; _resolve_walk assigns b.first = state.batter_id for the same case. Reachable only with a sampler and no lineup. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>The decision follows the runner's responsible pitcher, and a unit test plays the example.</t>
+          <t>The forced reach and the walk give the same bases.</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Carry each runner's responsible pitcher on the bases.</t>
+          <t>Use the walk's assignment.</t>
         </is>
       </c>
     </row>
@@ -1682,31 +1682,31 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>SIM-592</t>
+          <t>SIM-593</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Put the batter on first after a forced reach with no batter id</t>
+          <t>Void the plate appearance after a third out on the bases in the single pre-pitch steal draw</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>_force_on_reach with no batter id leaves first base's runner on first after pushing him to second (b.first = state.batter_id if ... else b.first), so the base check raises; _resolve_walk assigns b.first = state.batter_id for the same case. Reachable only with a sampler and no lineup. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>With SIM_STEAL_PITCH_CLASS=0 (not production), a pickoff or a caught stealing that makes the third out before the pitch's result still ends the plate appearance, so the pitcher gets a batter faced and the batter an at-bat. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>The forced reach and the walk give the same bases.</t>
+          <t>The single draw voids the plate appearance as the running game on the pitch does.</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Use the walk's assignment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="73.5" customHeight="1" s="15">
+          <t>Apply the no-pitch void of the class-aware draw.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="46.5" customHeight="1" s="15">
       <c r="A39" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1714,31 +1714,31 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>SIM-593</t>
+          <t>SIM-588</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Void the plate appearance after a third out on the bases in the single pre-pitch steal draw</t>
+          <t>Compute the z of the requested level in GameSimSummary.from_results</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>With SIM_STEAL_PITCH_CLASS=0 (not production), a pickoff or a caught stealing that makes the third out before the pitch's result still ends the plate appearance, so the pitcher gets a batter faced and the batter an at-bat. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>GameSimSummary.from_results(confidence_level=0.85) computes the 95% z and labels the intervals 0.85. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>The single draw voids the plate appearance as the running game on the pitch does.</t>
+          <t>Each level gets its own z, and a unit test checks 0.85.</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Apply the no-pitch void of the class-aware draw.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="46.5" customHeight="1" s="15">
+          <t>Use NormalDist().inv_cdf((1 + level) / 2), or raise on a level outside the table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="73.5" customHeight="1" s="15">
       <c r="A40" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1746,31 +1746,31 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>SIM-588</t>
+          <t>SIM-605</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Compute the z of the requested level in GameSimSummary.from_results</t>
+          <t>Keep one pitcher engine's calibration from rewriting every pitcher engine</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>GameSimSummary.from_results(confidence_level=0.85) computes the 95% z and labels the intervals 0.85. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>PitcherSimilarityEngine.apply_calibration sets the module global ARSENAL_SCALE, and a report with no gamma resets it to 4.10. The API builds two instances. Latent: no production path calls it today. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Each level gets its own z, and a unit test checks 0.85.</t>
+          <t>Each instance carries its own scale.</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Use NormalDist().inv_cdf((1 + level) / 2), or raise on a level outside the table.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="73.5" customHeight="1" s="15">
+          <t>Pass the instance's scale into the three readers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="90" customHeight="1" s="15">
       <c r="A41" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1778,31 +1778,31 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>SIM-605</t>
+          <t>SIM-628</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Keep one pitcher engine's calibration from rewriting every pitcher engine</t>
+          <t>Let the resumable sweep read the database address</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>PitcherSimilarityEngine.apply_calibration sets the module global ARSENAL_SCALE, and a report with no gamma resets it to 4.10. The API builds two instances. Latent: no production path calls it today. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The child process of scripts/resumable_sweep.py reads BASEBALL_DB_DSN from .env with env["BASEBALL_DB_DSN"]. Since the security hardening (SIM-443b), .env carries no such key: .env.example has it commented out, and the live .env has none. So a sweep stops with KeyError before its first game. This is separate from the retry after a crash (SIM-614). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Each instance carries its own scale.</t>
+          <t>A sweep starts on the current .env.</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Pass the instance's scale into the three readers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="90" customHeight="1" s="15">
+          <t>Read BASEBALL_DB_DSN from the process environment first (pipeline.db_dsn.require_dsn); read .env only when the key is set there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="73.5" customHeight="1" s="15">
       <c r="A42" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1810,31 +1810,31 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>SIM-628</t>
+          <t>SIM-614</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Let the resumable sweep read the database address</t>
+          <t>Retry a sweep attempt that crashes before its first game</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>The child process of scripts/resumable_sweep.py reads BASEBALL_DB_DSN from .env with env["BASEBALL_DB_DSN"]. Since the security hardening (SIM-443b), .env carries no such key: .env.example has it commented out, and the live .env has none. So a sweep stops with KeyError before its first game. This is separate from the retry after a crash (SIM-614). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/resumable_sweep.py applies its zero-progress stop (gained == 0) after a crash too, so a segfault before the first game of an attempt ends the sweep (exit 1) instead of retrying. Found by reading the code; not exercised. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>A sweep starts on the current .env.</t>
+          <t>A crashed attempt with no gain retries up to --max-attempts.</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Read BASEBALL_DB_DSN from the process environment first (pipeline.db_dsn.require_dsn); read .env only when the key is set there.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="73.5" customHeight="1" s="15">
+          <t>Apply the stop only to an attempt that exited cleanly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="87" customHeight="1" s="15">
       <c r="A43" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1842,27 +1842,27 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>SIM-614</t>
+          <t>SIM-613</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Retry a sweep attempt that crashes before its first game</t>
+          <t>Print n/a in the hypothetical-return table when no bet qualifies</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>scripts/resumable_sweep.py applies its zero-progress stop (gained == 0) after a crash too, so a segfault before the first game of an attempt ends the sweep (exit 1) instead of retrying. Found by reading the code; not exercised. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/accuracy/hypothetical_return.py _fmt_row formats the means and the range with :.4f and no guard for None. With no qualifying bet the table raises TypeError, and run() prints it before it writes the report and before the zero-games check, so the run ends in a traceback with no report and no exit code 5. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>A crashed attempt with no gain retries up to --max-attempts.</t>
+          <t>The table prints n/a, as the accuracy table does.</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Apply the stop only to an attempt that exited cleanly.</t>
+          <t>Use the _fmt_or_na guard.</t>
         </is>
       </c>
     </row>
@@ -1874,31 +1874,31 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>SIM-613</t>
+          <t>SIM-616</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Print n/a in the hypothetical-return table when no bet qualifies</t>
+          <t>Decide the minimum-sample read's two known limits</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>scripts/accuracy/hypothetical_return.py _fmt_row formats the means and the range with :.4f and no guard for None. With no qualifying bet the table raises TypeError, and run() prints it before it writes the report and before the zero-games check, so the run ends in a traceback with no report and no exit code 5. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/accuracy/confidence.py: the 0.02 floor assumes a coin-flip market, so its power is weaker than stated for a market far from 0.5 (a home-run prop); and a small sample whose observed spread is exactly zero reads as fully resolved. An adversarial review of the minimum-sample work (SIM-539) found both. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>The table prints n/a, as the accuracy table does.</t>
+          <t>The owner decides whether to fix or accept them.</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Use the _fmt_or_na guard.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="87" customHeight="1" s="15">
+          <t>A per-market 4p(1-p) correction and an upper bound on the spread.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="73.5" customHeight="1" s="15">
       <c r="A45" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1906,31 +1906,31 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>SIM-616</t>
+          <t>SIM-589</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Decide the minimum-sample read's two known limits</t>
+          <t>Treat both samples as samples in the replay chi-squared test</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>scripts/accuracy/confidence.py: the 0.02 floor assumes a coin-flip market, so its power is weaker than stated for a market far from 0.5 (a home-run prop); and a small sample whose observed spread is exactly zero reads as fully resolved. An adversarial review of the minimum-sample work (SIM-539) found both. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The two-sample path of replay_chi_squared.chi_squared_gof treats the reference sample as exact. Two independent samples of 1,000 Poisson(4.4) totals were rejected 52.5% of the time at alpha 0.05 over 400 trials. replay_and_test uses it. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>The owner decides whether to fix or accept them.</t>
+          <t>Two samples from one distribution are rejected near alpha.</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>A per-market 4p(1-p) correction and an upper bound on the spread.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="73.5" customHeight="1" s="15">
+          <t>Use scipy.stats.chi2_contingency on the pooled 2 x k table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="60" customHeight="1" s="15">
       <c r="A46" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1938,27 +1938,27 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>SIM-589</t>
+          <t>SIM-590</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Treat both samples as samples in the replay chi-squared test</t>
+          <t>Compare the historical replay against the right side's score</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>The two-sample path of replay_chi_squared.chi_squared_gof treats the reference sample as exact. Two independent samples of 1,000 Poisson(4.4) totals were rejected 52.5% of the time at alpha 0.05 over 400 trials. replay_and_test uses it. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>replay_historical_games always compares the simulated HOME score. A HistoricalGame row does not say which side its runs belong to, so an away team's runs meet the simulated home runs. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Two samples from one distribution are rejected near alpha.</t>
+          <t>A HistoricalGame row names its side, and the replay compares like with like.</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Use scipy.stats.chi2_contingency on the pooled 2 x k table.</t>
+          <t>Add a side field to HistoricalGame.</t>
         </is>
       </c>
     </row>
@@ -1970,31 +1970,31 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>SIM-590</t>
+          <t>SIM-618</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Compare the historical replay against the right side's score</t>
+          <t>Keep one copy of the prop ground-truth readers</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>replay_historical_games always compares the simulated HOME score. A HistoricalGame row does not say which side its runs belong to, so an away team's runs meet the simulated home runs. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/validate_props.py and scripts/accuracy/grading.py each define _fetch_official_boxscore and _fetch_pa_events. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>A HistoricalGame row names its side, and the replay compares like with like.</t>
+          <t>One reader, imported by both.</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Add a side field to HistoricalGame.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="60" customHeight="1" s="15">
+          <t>Move it to simulation/prop_validation.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="73.5" customHeight="1" s="15">
       <c r="A48" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2002,31 +2002,31 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>SIM-618</t>
+          <t>SIM-621</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Keep one copy of the prop ground-truth readers</t>
+          <t>Bench the per-pitch call the loop makes</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>scripts/validate_props.py and scripts/accuracy/grading.py each define _fetch_official_boxscore and _fetch_pa_events. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>tests/performance/bench_simulation.py times PitcherSimilarityEngine.query() as the per-pitch cost; the loop reads the dense pitcher matrix. bench_api_simulate.py says an authoritative gate runs on target hardware with the DB-backed factory; no job does. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>One reader, imported by both.</t>
+          <t>The benches time what the loop runs, and the SLA text names the job that gates it.</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>Move it to simulation/prop_validation.py.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="73.5" customHeight="1" s="15">
+          <t>Bench the matrix read; correct the SLA text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="60" customHeight="1" s="15">
       <c r="A49" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2034,31 +2034,31 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>SIM-621</t>
+          <t>SIM-612</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Bench the per-pitch call the loop makes</t>
+          <t>Read the pitch rebuild's before-smoke from results/</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>tests/performance/bench_simulation.py times PitcherSimilarityEngine.query() as the per-pitch cost; the loop reads the dense pitcher matrix. bench_api_simulate.py says an authoritative gate runs on target hardware with the DB-backed factory; no job does. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/pitch_pool_rebuild/export.py _smoke_games opens scripts/sim553_smoke_before.json; the groundwork moved run outputs to results/sim553/. The function always prints its placeholder. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>The benches time what the loop runs, and the SLA text names the job that gates it.</t>
+          <t>It reads the results/ path.</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Bench the matrix read; correct the SLA text.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="60" customHeight="1" s="15">
+          <t>Change the one path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="73.5" customHeight="1" s="15">
       <c r="A50" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2066,31 +2066,31 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>SIM-612</t>
+          <t>SIM-623</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Read the pitch rebuild's before-smoke from results/</t>
+          <t>Replace the inning-grid test's pinned scores with an outcome check</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>scripts/pitch_pool_rebuild/export.py _smoke_games opens scripts/sim553_smoke_before.json; the groundwork moved run outputs to results/sim553/. The function always prints its placeholder. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>tests/unit/test_inning_grid.py pins the exact scores and pitch counts of ten seeds (OUTCOMES_AT_80E3F46). That works like the golden snapshots the owner ruled out on 2026-09-10: any intended change to the draw fails it. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>It reads the results/ path.</t>
+          <t>The test checks a property of the grid (its sum equals the final score, the halves match the outs), not ten remembered numbers.</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Change the one path.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="73.5" customHeight="1" s="15">
+          <t>Rewrite the assertions as invariants and delete the pinned table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="87" customHeight="1" s="15">
       <c r="A51" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2098,31 +2098,31 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>SIM-623</t>
+          <t>SIM-620</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Replace the inning-grid test's pinned scores with an outcome check</t>
+          <t>Delete the regression gate's dead constants and its golden-file texts</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>tests/unit/test_inning_grid.py pins the exact scores and pitch counts of ten seeds (OUTCOMES_AT_80E3F46). That works like the golden snapshots the owner ruled out on 2026-09-10: any intended change to the draw fails it. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>tests/regression/regression_config.py: only SYMMETRY_TOLERANCE has a reader; eight constants have none (the conftest hard-codes the seed 2026), and one constant's docstring still speaks of golden files. The assert message at test_engine_regression.py:322 names golden files the gate does not have. The pyproject.toml marker text, the ci.yml header and make help were corrected by the documentation rebuild (SIM-624, 2026-10-21). Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>The test checks a property of the grid (its sum equals the final score, the halves match the outs), not ten remembered numbers.</t>
+          <t>The dead constants go, and the assert message says what the gate checks.</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>Rewrite the assertions as invariants and delete the pinned table.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="87" customHeight="1" s="15">
+          <t>Delete the dead constants and edit the assert message.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="60" customHeight="1" s="15">
       <c r="A52" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2130,31 +2130,31 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>SIM-620</t>
+          <t>SIM-622</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Delete the regression gate's dead constants and its golden-file texts</t>
+          <t>Use the pinned park factor in the sim-kwargs tests</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>tests/regression/regression_config.py: only SYMMETRY_TOLERANCE has a reader; eight constants have none (the conftest hard-codes the seed 2026), and one constant's docstring still speaks of golden files. The assert message at test_engine_regression.py:322 names golden files the gate does not have. The pyproject.toml marker text, the ci.yml header and make help were corrected by the documentation rebuild (SIM-624, 2026-10-21). Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>tests/unit/test_sim_kwargs.py uses 0.8723846078 for venue 680 in six places; the pinned 2024 table in the same file holds 0.8725842237. The tests pass (the literal is only an input). Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>The dead constants go, and the assert message says what the gate checks.</t>
+          <t>One value.</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>Delete the dead constants and edit the assert message.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="60" customHeight="1" s="15">
+          <t>Read it from the table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="87" customHeight="1" s="15">
       <c r="A53" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2162,31 +2162,31 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>SIM-622</t>
+          <t>SIM-597</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Use the pinned park factor in the sim-kwargs tests</t>
+          <t>Write the pitching-change pool's role file in a fixed row order</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>tests/unit/test_sim_kwargs.py uses 0.8723846078 for venue 680 in six places; the pinned 2024 table in the same file holds 0.8725842237. The tests pass (the literal is only an input). Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>roles.parquet (build_pitching_change_pool, pipeline/batch/artifacts/manager_pool.py) is written from a GROUP BY with no ORDER BY, so two builds of the same code from the same data write its rows in a different order. No reader uses the order, but the fingerprint's bundle mode reads a difference on every build. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>One value.</t>
+          <t>Two builds give the same file, by content.</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Read it from the table.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="87" customHeight="1" s="15">
+          <t>Add ORDER BY pitcher_id, season. It changes no game.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="118" customHeight="1" s="15">
       <c r="A54" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2194,31 +2194,31 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>SIM-597</t>
+          <t>SIM-631</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Write the pitching-change pool's role file in a fixed row order</t>
+          <t>Delete or wire up the data nobody reads</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>roles.parquet (build_pitching_change_pool, pipeline/batch/artifacts/manager_pool.py) is written from a GROUP BY with no ORDER BY, so two builds of the same code from the same data write its rows in a different order. No reader uses the order, but the fingerprint's bundle mode reads a difference on every build. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>Built and never read: sim.stolen_base_pool (the profile computor builds it every night), the composite catcher actor matrix (built and concentration-checked; the draws read catcher_throwing), the sim.live_games view and raw.savant_first_base_receiving. Declared and never written: derived.outfield_play_detail, derived.infield_play_detail and derived.dp_play_detail. Never called: sim.purge_expired_sessions(), and EngineArtifacts.attach_shared_views outside the tests. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>Two builds give the same file, by content.</t>
+          <t>Each item has a reader, or it is deleted with its builder and its DDL.</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>Add ORDER BY pitcher_id, season. It changes no game.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="118" customHeight="1" s="15">
+          <t>Delete them, with a migration for the DDL. Keep any the owner wants for planned work, and name the ticket that will read it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="73.5" customHeight="1" s="15">
       <c r="A55" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2226,31 +2226,31 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>SIM-631</t>
+          <t>SIM-615</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Delete or wire up the data nobody reads</t>
+          <t>Retire the odds-hash backfill probe</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>Built and never read: sim.stolen_base_pool (the profile computor builds it every night), the composite catcher actor matrix (built and concentration-checked; the draws read catcher_throwing), the sim.live_games view and raw.savant_first_base_receiving. Declared and never written: derived.outfield_play_detail, derived.infield_play_detail and derived.dp_play_detail. Never called: sim.purge_expired_sessions(), and EngineArtifacts.attach_shared_views outside the tests. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/probes/backfill_odds_hash.py _dedup_rows orders by received_at, a column raw.game_odds does not have, so its DELETE fails; its ODDS_COLUMNS leaves out draw_ml. Both are dormant: the unique index and the NOT NULL hash of migration 0012 ended the probe's job. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>Each item has a reader, or it is deleted with its builder and its DDL.</t>
+          <t>The probe is retired.</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>Delete them, with a migration for the DDL. Keep any the owner wants for planned work, and name the ticket that will read it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="73.5" customHeight="1" s="15">
+          <t>Delete the probe and its test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="90" customHeight="1" s="15">
       <c r="A56" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2258,31 +2258,31 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>SIM-615</t>
+          <t>SIM-627</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Retire the odds-hash backfill probe</t>
+          <t>Retire the two odds routes that serve mock lines</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>scripts/probes/backfill_odds_hash.py _dedup_rows orders by received_at, a column raw.game_odds does not have, so its DELETE fails; its ODDS_COLUMNS leaves out draw_ml. Both are dormant: the unique index and the NOT NULL hash of migration 0012 ended the probe's job. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>GET /api/odds/{game_pk} and GET /api/odds/today/all (pipeline/live/ingestion/odds_routes.py, mounted by api/main.py) always return MockOddsAPI lines, whatever ODDS_PROVIDER says. The rows carry is_mock: true, and no frontend code calls the routes. A client that ignores the flag reads fake prices as real ones. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>The probe is retired.</t>
+          <t>The routes are gone (or serve the stored book rows), and the API snapshot is regenerated.</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>Delete the probe and its test.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="90" customHeight="1" s="15">
+          <t>Delete both routes, then run scripts/export_openapi.py in the app image and npm run gen:api (CLAUDE.md section 15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="181.5" customHeight="1" s="15">
       <c r="A57" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2290,31 +2290,31 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>SIM-627</t>
+          <t>SIM-617</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Retire the two odds routes that serve mock lines</t>
+          <t>Correct the runtime texts that state something false</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>GET /api/odds/{game_pk} and GET /api/odds/today/all (pipeline/live/ingestion/odds_routes.py, mounted by api/main.py) always return MockOddsAPI lines, whatever ODDS_PROVIDER says. The rows carry is_mock: true, and no frontend code calls the routes. A client that ignores the flag reads fake prices as real ones. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>Left unedited by the clean-up's rule. (1) The park-guard messages name the deleted SIM_PARK_FACTOR: scripts/validate_props.py, scripts/accuracy_comparison.py, tests/acceptance/conftest.py and the --help of scripts/sim_stats.py. (2) The two pool rebuilds' exit-3 texts and the steal rebuild's lock message blame the app's worker server for the DuckDB lock (the app holds no handle since SIM-524), and two steal-rebuild texts say to merge code that is merged. (3) scripts/running_game_replay.py --help says a steal can land on any pitch in production. (4) Three texts point at a module docstring section that moved in the split. (5) scripts/measure_filter_cells.py writes into docs/audit/. (6) scripts/resumable_sweep.py --help cites a deleted record. (7) The rationale strings in tests/acceptance/bands.py cite BACKLOG.md, which is gone. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>The routes are gone (or serve the stored book rows), and the API snapshot is regenerated.</t>
+          <t>Each text says what is true.</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>Delete both routes, then run scripts/export_openapi.py in the app image and npm run gen:api (CLAUDE.md section 15).</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="181.5" customHeight="1" s="15">
+          <t>One edit per text; list the runtime-string changes in CHANGES.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="154.5" customHeight="1" s="15">
       <c r="A58" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2322,31 +2322,31 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>SIM-617</t>
+          <t>SIM-610</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Correct the runtime texts that state something false</t>
+          <t>Similarity and betting: seven small defects</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Left unedited by the clean-up's rule. (1) The park-guard messages name the deleted SIM_PARK_FACTOR: scripts/validate_props.py, scripts/accuracy_comparison.py, tests/acceptance/conftest.py and the --help of scripts/sim_stats.py. (2) The two pool rebuilds' exit-3 texts and the steal rebuild's lock message blame the app's worker server for the DuckDB lock (the app holds no handle since SIM-524), and two steal-rebuild texts say to merge code that is merged. (3) scripts/running_game_replay.py --help says a steal can land on any pitch in production. (4) Three texts point at a module docstring section that moved in the split. (5) scripts/measure_filter_cells.py writes into docs/audit/. (6) scripts/resumable_sweep.py --help cites a deleted record. (7) The rationale strings in tests/acceptance/bands.py cite BACKLOG.md, which is gone. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>(1) SituationSimilarityEngine.query_batch([]) raises instead of returning []. (2) The engines' and the calibrator's __main__ blocks read a DuckDB path that does not exist (../../db/schemas/baseball_simulator.duckdb); the pitcher engine's block builds and prints nothing. (3) CalibrationReport.summary() prints no row for the batter's physical weights. (4) The Similarity Explorer's batter panel (api/routes/similarity_explorer.py) shows the four-way weights 0.40/0.35/0.15/0.10. (5) A log line in batted_ball_similarity.py says 'until SIM-051 ships'. (6) tests/regression/conftest.py scales the situation fixture's index twice. (7) No writer sets is_sharp_book, so sharp_consensus is always None. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>Each text says what is true.</t>
+          <t>Each of the seven is fixed or retired.</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>One edit per text; list the runtime-string changes in CHANGES.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="154.5" customHeight="1" s="15">
+          <t>One edit each; retire sharp_consensus if no book will be marked sharp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="100.5" customHeight="1" s="15">
       <c r="A59" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2354,27 +2354,27 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>SIM-610</t>
+          <t>SIM-603</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Similarity and betting: seven small defects</t>
+          <t>Return the fielder's infield sub-scores in the same order from query_pair as from query</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>(1) SituationSimilarityEngine.query_batch([]) raises instead of returning []. (2) The engines' and the calibrator's __main__ blocks read a DuckDB path that does not exist (../../db/schemas/baseball_simulator.duckdb); the pitcher engine's block builds and prints nothing. (3) CalibrationReport.summary() prints no row for the batter's physical weights. (4) The Similarity Explorer's batter panel (api/routes/similarity_explorer.py) shows the four-way weights 0.40/0.35/0.15/0.10. (5) A log line in batted_ball_similarity.py says 'until SIM-051 ships'. (6) tests/regression/conftest.py scales the situation fixture's index twice. (7) No writer sets is_sharp_book, so sharp_consensus is always None. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>For an infielder, similarity/engines/fielder_similarity.py query_pair returns the specialty score in tertiary_score and the error score in quaternary_score; query returns them the other way round, as the Similarity Explorer's labels expect. Two shortstops with different error rates and equal specialty values: query gives 0.0710 / 1.0000, query_pair 1.0000 / 0.0710. The composite and the matrices are right. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>Each of the seven is fixed or retired.</t>
+          <t>query and query_pair agree on every sub-score, and a unit test compares them.</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>One edit each; retire sharp_consensus if no book will be marked sharp.</t>
+          <t>Map the infield tuple in SimilarityResult order.</t>
         </is>
       </c>
     </row>
@@ -2386,31 +2386,31 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>SIM-603</t>
+          <t>SIM-604</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Return the fielder's infield sub-scores in the same order from query_pair as from query</t>
+          <t>Apply the per-hand 30-PA platoon rule in the batter engine's pair score</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>For an infielder, similarity/engines/fielder_similarity.py query_pair returns the specialty score in tertiary_score and the error score in quaternary_score; query returns them the other way round, as the Similarity Explorer's labels expect. Two shortstops with different error rates and equal specialty values: query gives 0.0710 / 1.0000, query_pair 1.0000 / 0.0710. The composite and the matrices are right. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>similarity/engines/batter_similarity.py _score_pair disagrees with score_all on a thin platoon split. A query with 30+ PA against either hand turns the platoon weights on for any vs_hand (10 PA vs L and 200 vs R with vs_hand='L': 0.8642 against 0.8900), and a candidate under 30 PA never gets the neutral 0.5. It serves query_pair (the Explorer's pair view and the diagnostics); the matrix is unaffected. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>query and query_pair agree on every sub-score, and a unit test compares them.</t>
+          <t>_score_pair and score_all agree, and a unit test compares them.</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>Map the infield tuple in SimilarityResult order.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="100.5" customHeight="1" s="15">
+          <t>Use score_all's per-hand rule in _score_pair.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="60" customHeight="1" s="15">
       <c r="A61" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2418,27 +2418,27 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>SIM-604</t>
+          <t>SIM-596</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Apply the per-hand 30-PA platoon rule in the batter engine's pair score</t>
+          <t>Decide what the what-if does when the designated hitter takes the field</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>similarity/engines/batter_similarity.py _score_pair disagrees with score_all on a thin platoon split. A query with 30+ PA against either hand turns the platoon weights on for any vs_hand (10 PA vs L and 200 vs R with vs_hand='L': 0.8642 against 0.8900), and a candidate under 30 PA never gets the neutral 0.5. It serves query_pair (the Explorer's pair view and the diagnostics); the matrix is unaffected. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>A designated hitter moved to the field leaves the fielder he replaced in the batting order with no position. The rule that ends the designated hitter is not modelled in simulation/whatif.py. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>_score_pair and score_all agree, and a unit test compares them.</t>
+          <t>The owner decides whether the what-if models the rule, and the code follows.</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Use score_all's per-hand rule in _score_pair.</t>
+          <t>Model the rule: the pitcher bats in the replaced fielder's slot, or refuse the change.</t>
         </is>
       </c>
     </row>
@@ -2450,31 +2450,31 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>SIM-596</t>
+          <t>SIM-598</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Decide what the what-if does when the designated hitter takes the field</t>
+          <t>Read the runners under the names the live service sends</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>A designated hitter moved to the field leaves the fielder he replaced in the batting order with no position. The rule that ends the designated hitter is not modelled in simulation/whatif.py. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>frontend/src/hooks/useGameSocket.ts reads runner_on_first / _second / _third; the live service sends on_1b / on_2b / on_3b. The hook's on_1b to on_3b are always undefined. No page reads them today. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>The owner decides whether the what-if models the rule, and the code follows.</t>
+          <t>A game_state_update with runners fills the hook's on_1b to on_3b.</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>Model the rule: the pitcher bats in the replaced fielder's slot, or refuse the change.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="60" customHeight="1" s="15">
+          <t>Read gs.on_1b, gs.on_2b and gs.on_3b in mapWsState.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="46.5" customHeight="1" s="15">
       <c r="A63" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2482,31 +2482,31 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>SIM-598</t>
+          <t>SIM-609</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Read the runners under the names the live service sends</t>
+          <t>Raise on a wrong market or side in the line-movement series</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/hooks/useGameSocket.ts reads runner_on_first / _second / _third; the live service sends on_1b / on_2b / on_3b. The hook's on_1b to on_3b are always undefined. No page reads them today. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>line_movement_from_quotes swallows _side_columns' ValueError, so a wrong market or side gives a silent empty series. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>A game_state_update with runners fills the hook's on_1b to on_3b.</t>
+          <t>A wrong market or side raises.</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>Read gs.on_1b, gs.on_2b and gs.on_3b in mapWsState.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="46.5" customHeight="1" s="15">
+          <t>Call _side_columns once before the loop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="73.5" customHeight="1" s="15">
       <c r="A64" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2514,31 +2514,31 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>SIM-609</t>
+          <t>SIM-599</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Raise on a wrong market or side in the line-movement series</t>
+          <t>Describe the slate card's odds field as it is</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>line_movement_from_quotes swallows _side_columns' ValueError, so a wrong market or side gives a silent empty series. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The route description (api/routes/games_slate.py) and the model (api/routes/games_models.py) call the field 'reserved for the Phase-6 odds-provider integration (SIM-405)'. The field is always None: the card's lines come from /api/betting/games/{pk}/card-odds. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>A wrong market or side raises.</t>
+          <t>Both texts say that, with a fresh API snapshot (CLAUDE.md section 15).</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>Call _side_columns once before the loop.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="73.5" customHeight="1" s="15">
+          <t>Rewrite both texts; run scripts/export_openapi.py in the image and npm run gen:api.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="46.5" customHeight="1" s="15">
       <c r="A65" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2546,31 +2546,31 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>SIM-599</t>
+          <t>SIM-600</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Describe the slate card's odds field as it is</t>
+          <t>Name the current state in the API's version and health strings</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>The route description (api/routes/games_slate.py) and the model (api/routes/games_models.py) call the field 'reserved for the Phase-6 odds-provider integration (SIM-405)'. The field is always None: the card's lines come from /api/betting/games/{pk}/card-odds. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>api/main.py carries the app version 0.1.0-phase7, "phase": "6" on /health and "6 - Frontend Build (in progress)" on /. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>Both texts say that, with a fresh API snapshot (CLAUDE.md section 15).</t>
+          <t>The strings name the current state, or go.</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>Rewrite both texts; run scripts/export_openapi.py in the image and npm run gen:api.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="46.5" customHeight="1" s="15">
+          <t>Drop the phase keys and set the version from one constant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="202" customHeight="1" s="15">
       <c r="A66" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2578,31 +2578,31 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>SIM-600</t>
+          <t>SIM-634</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Name the current state in the API's version and health strings</t>
+          <t>Small fixes found by the documentation rebuild</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>api/main.py carries the app version 0.1.0-phase7, "phase": "6" on /health and "6 - Frontend Build (in progress)" on /. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>(1) frontend/index.html links a favicon, /baseball.svg, that frontend/public/ does not hold: a 404 on every page. (2) /ready (api/main.py) writes a redis entry only on a failure, so a healthy Redis is missing from its checks. (3) Six nginx blocks (/health, /ready, /metrics, /docs, /redoc, /openapi.json) set their own Host header, which drops the inherited X-Real-IP and X-Forwarded-For. (4) Nothing deletes the simviz:* explorer cache keys after a nightly rebuild, so a key serves old data for up to 24 h. (5) 12 of the 32 DuckDB migrations do not record themselves in migration_history. (6) Three stale texts: api/state.py calls the situation engine a FAISS engine (it is a KD-tree); the Makefile's gen-secrets comment says a blank key is left alone (gen_secrets.py fills it); scripts/probes/manager_profile_recompute.py says the app must be stopped (the recompute runs beside the app since SIM-524). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>The strings name the current state, or go.</t>
+          <t>Each of the six is fixed or retired.</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>Drop the phase keys and set the version from one constant.</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="202" customHeight="1" s="15">
+          <t>One small commit per area. For (5), record the missing numbers in one new migration rather than editing old files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="46.5" customHeight="1" s="15">
       <c r="A67" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2610,91 +2610,60 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>SIM-634</t>
+          <t>SIM-595</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Small fixes found by the documentation rebuild</t>
+          <t>Fix the article in the what-if's ineligible-player message</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>(1) frontend/index.html links a favicon, /baseball.svg, that frontend/public/ does not hold: a 404 on every page. (2) /ready (api/main.py) writes a redis entry only on a failure, so a healthy Redis is missing from its checks. (3) Six nginx blocks (/health, /ready, /metrics, /docs, /redoc, /openapi.json) set their own Host header, which drops the inherited X-Real-IP and X-Forwarded-For. (4) Nothing deletes the simviz:* explorer cache keys after a nightly rebuild, so a key serves old data for up to 24 h. (5) 12 of the 32 DuckDB migrations do not record themselves in migration_history. (6) Three stale texts: api/state.py calls the situation engine a FAISS engine (it is a KD-tree); the Makefile's gen-secrets comment says a blank key is left alone (gen_secrets.py fills it); scripts/probes/manager_profile_recompute.py says the app must be stopped (the recompute runs beside the app since SIM-524). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>whatif.apply_changes' message for an ineligible pinch hitter reads 'is not an bench hitter'. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>Each of the six is fixed or retired.</t>
+          <t>Each label reads with its own article.</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>One small commit per area. For (5), record the missing numbers in one new migration rather than editing old files.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="46.5" customHeight="1" s="15">
-      <c r="A68" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B68" s="3" t="inlineStr">
-        <is>
-          <t>SIM-595</t>
-        </is>
-      </c>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>Fix the article in the what-if's ineligible-player message</t>
-        </is>
-      </c>
-      <c r="D68" s="5" t="inlineStr">
-        <is>
-          <t>whatif.apply_changes' message for an ineligible pinch hitter reads 'is not an bench hitter'. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E68" s="5" t="inlineStr">
-        <is>
-          <t>Each label reads with its own article.</t>
-        </is>
-      </c>
-      <c r="F68" s="5" t="inlineStr">
-        <is>
           <t>Put the article inside each label.</t>
         </is>
       </c>
     </row>
-    <row r="69"/>
-    <row r="70">
-      <c r="A70" s="7" t="inlineStr">
+    <row r="68" s="15"/>
+    <row r="69" s="15">
+      <c r="A69" s="7" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B70" s="8" t="inlineStr">
+      <c r="B69" s="8" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C70" s="9" t="inlineStr">
+      <c r="C69" s="9" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D70" s="12" t="inlineStr">
+      <c r="D69" s="12" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E70" s="10" t="inlineStr">
+      <c r="E69" s="10" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F70" s="11" t="n"/>
-    </row>
+      <c r="F69" s="11" t="n"/>
+    </row>
+    <row r="70" s="15"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>

<commit_message>
Delete the closed backlog row of the arsenal row order (SIM-580); file SIM-635 to SIM-639; record the deploy
BACKLOG.xlsx: the SIM-580 row is deleted. Five rows are filed from the arsenal
work's sweep: the pitch pool's and the batted-ball pool's export order for the
two density corrections (SIM-635, SIM-636, P2, after the four engine-input
fixes), the calibration's reliability pairs and bandwidth sample (SIM-637,
SIM-638, P3, the latent-risk group), and the crashed arsenal-fit worker that
exits 0 (SIM-639, P3, the wrong-data group). The next free ID is SIM-640.
CHANGES.md records the merge and the app's reload.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -560,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -581,7 +581,7 @@
     <row r="2" s="15">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>NEXT FREE TICKET ID: SIM-635</t>
+          <t>NEXT FREE TICKET ID: SIM-640</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="114" customHeight="1" s="15">
+    <row r="6" ht="60" customHeight="1" s="15">
       <c r="A6" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -658,31 +658,31 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>SIM-580</t>
+          <t>SIM-606</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Make the pitcher arsenal fit reproducible: order the pitch rows before the mixture fit</t>
+          <t>Pick the small-mixture-component merge target in standardized units</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>The pitch-vector query in _compute_pitcher_profiles (pipeline/batch/profiles/pitcher.py) has no ORDER BY. DuckDB's parallel Postgres scan returns the rows in a different order on every read, and the seeded mixture fit (random_state=42) depends on the row order. So every profile rebuild gives a different arsenal for nearly every pitcher (a different number of components for about one pitcher in five), and with it a different pitcher similarity matrix. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>enforce_min_cluster_size runs before the standardization in the arsenal build, so spin rate (hundreds of rpm) decides the merge over velocity and movement. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Two profile builds of the same code from the same data write the same arsenals, by content.</t>
+          <t>The merge measures the gap in standardized units.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Add ORDER BY game_pk, at_bat_number, pitch_number to the query. It changes every arsenal once.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="60" customHeight="1" s="15">
+          <t>Measure the gap over the mixture's feature_stds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="114" customHeight="1" s="15">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -690,31 +690,31 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>SIM-606</t>
+          <t>SIM-578</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Pick the small-mixture-component merge target in standardized units</t>
+          <t>Load a database NULL as NaN, not 0.0, in the baserunner, catcher, batter and manager engines</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>enforce_min_cluster_size runs before the standardization in the arsenal build, so spin rate (hundreds of rpm) decides the merge over velocity and movement. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The _v helpers of four engines read v or 0.0. A runner with no Savant row gets sprint speed 0 ft/s (still 20 ft/s after a 5-chance shrink, many deviations below the league's 27), so his speed score is about 0 against every measured runner. A runner who never tried reads 0% success; a NULL arm strength reads 0 mph; a manager-season with no bullpen-availability rows reads available_reliever_usage_rate near 0. The two steal engines already load NaN (the running-game work, SIM-531). Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>The merge measures the gap in standardized units.</t>
+          <t>Each of the four engines loads NULL as NaN, and its kernel or shrink handles a NaN feature. The nightly matrices are rebuilt.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Measure the gap over the mixture's feature_stds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="114" customHeight="1" s="15">
+          <t>Map None to NaN in each _v helper and add the features to each engine's NaN set, as the steal engines do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="127.5" customHeight="1" s="15">
       <c r="A8" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -722,31 +722,31 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>SIM-578</t>
+          <t>SIM-577</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Load a database NULL as NaN, not 0.0, in the baserunner, catcher, batter and manager engines</t>
+          <t>Write all thirteen features in the extra-base runner's league-average row</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>The _v helpers of four engines read v or 0.0. A runner with no Savant row gets sprint speed 0 ft/s (still 20 ft/s after a 5-chance shrink, many deviations below the league's 27), so his speed score is about 0 against every measured runner. A runner who never tried reads 0% success; a NULL arm strength reads 0 mph; a manager-season with no bullpen-availability rows reads available_reliever_usage_rate near 0. The two steal engines already load NaN (the running-game work, SIM-531). Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The baserunner row of derived.league_averages holds extra_base_attempt_rate, extra_base_success_rate, sb_success_rate, sprint_speed and the Savant rate. The engine reads thirteen features, so the four per-situation attempt rates, stop_rate and the four per-situation success rates shrink toward 0.0. The matrix build loads the thin profiles, so the effect is large there: a 5-chance runner's first-to-third attempt rate reads 0.35 -&gt; 0.088. The error reaches the runner_adv matrix, which weights the advancement draws. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Each of the four engines loads NULL as NaN, and its kernel or shrink handles a NaN feature. The nightly matrices are rebuilt.</t>
+          <t>The runner's league row carries every engine feature, and a missing key reads as NaN. The nightly matrices are rebuilt.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Map None to NaN in each _v helper and add the features to each engine's NaN set, as the steal engines do.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="127.5" customHeight="1" s="15">
+          <t>Write the engine's thirteen feature keys in the computor's baserunner league row; read a missing key as NaN in similarity/engines/baserunner_similarity.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="114" customHeight="1" s="15">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -754,27 +754,27 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>SIM-577</t>
+          <t>SIM-576</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Write all thirteen features in the extra-base runner's league-average row</t>
+          <t>Write the catcher engine's feature names in the catcher's league-average row</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>The baserunner row of derived.league_averages holds extra_base_attempt_rate, extra_base_success_rate, sb_success_rate, sprint_speed and the Savant rate. The engine reads thirteen features, so the four per-situation attempt rates, stop_rate and the four per-situation success rates shrink toward 0.0. The matrix build loads the thin profiles, so the effect is large there: a 5-chance runner's first-to-third attempt rate reads 0.35 -&gt; 0.088. The error reaches the runner_adv matrix, which weights the advancement draws. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The profile computor writes the catcher row of derived.league_averages with the keys framing_runs, blocking_runs and cs_rate. The catcher engine reads its eleven feature names with pj.get(f, 0.0) or 0.0, and only cs_rate matches. So the shrinkage pulls ten features toward 0.0: a constructed 300-pitch catcher reads pop time 1.95 -&gt; 1.857 s and arm strength 81 -&gt; 77.1 mph. The error reaches the catcher and catcher_throwing score matrices, which weight the steal and pickoff draws. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>The runner's league row carries every engine feature, and a missing key reads as NaN. The nightly matrices are rebuilt.</t>
+          <t>The catcher's league row carries every engine feature. A missing key reads as NaN, as the steal engines do. The nightly matrices are rebuilt.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Write the engine's thirteen feature keys in the computor's baserunner league row; read a missing key as NaN in similarity/engines/baserunner_similarity.py.</t>
+          <t>In pipeline/batch/profiles (the catcher league row), write the engine's eleven feature keys. In similarity/engines/catcher_similarity.py _load_league_averages, read a missing key as NaN.</t>
         </is>
       </c>
     </row>
@@ -786,31 +786,31 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SIM-576</t>
+          <t>SIM-579</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Write the catcher engine's feature names in the catcher's league-average row</t>
+          <t>Select the pitcher's zone-take rate before the chase rate, so the two stay in feature order</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>The profile computor writes the catcher row of derived.league_averages with the keys framing_runs, blocking_runs and cs_rate. The catcher engine reads its eleven feature names with pj.get(f, 0.0) or 0.0, and only cs_rate matches. So the shrinkage pulls ten features toward 0.0: a constructed 300-pitch catcher reads pop time 1.95 -&gt; 1.857 s and arm strength 81 -&gt; 77.1 mph. The error reaches the catcher and catcher_throwing score matrices, which weight the steal and pickoff draws. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>In similarity/engines/pitcher_similarity.py _load_profiles, the SELECT returns chase_rate, zone_take_rate and the unpack names them zone_take_rate, chase_rate. So command_vec holds them in the opposite order to COMMAND_FEATURES and the league-average vector, and the shrinkage pulls each pitcher's chase rate toward the league's zone-take rate (weight 1 - alpha, at most 2.4% at 200 pitches). The kernel itself ignores the order. The error reaches the pitcher similarity matrix. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>The catcher's league row carries every engine feature. A missing key reads as NaN, as the steal engines do. The nightly matrices are rebuilt.</t>
+          <t>The SELECT order matches COMMAND_FEATURES, and a unit test pins it. The nightly matrices are rebuilt.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>In pipeline/batch/profiles (the catcher league row), write the engine's eleven feature keys. In similarity/engines/catcher_similarity.py _load_league_averages, read a missing key as NaN.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="114" customHeight="1" s="15">
+          <t>Select zone_take_rate before chase_rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="219.5" customHeight="1" s="15">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -818,31 +818,31 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SIM-579</t>
+          <t>SIM-635</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Select the pitcher's zone-take rate before the chase rate, so the two stay in feature order</t>
+          <t>Export the pitch pool in pitch order, so the pitch-result draw's density weights stay the same between pool builds</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>In similarity/engines/pitcher_similarity.py _load_profiles, the SELECT returns chase_rate, zone_take_rate and the unpack names them zone_take_rate, chase_rate. So command_vec holds them in the opposite order to COMMAND_FEATURES and the league-average vector, and the shrinkage pulls each pitcher's chase rate toward the league's zone-take rate (weight 1 - alpha, at most 2.4% at 200 pitches). The kernel itself ignores the order. The error reaches the pitcher similarity matrix. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The pitch-result draw lowers the weight of a candidate pitch where the candidate set is crowded with similar pitches. It measures the crowding against 256 reference rows of the set (simulation/sampler/pitch_result.py:133-137). The draw picks the 256 rows by their POSITION in the set. Each set keeps the pool's stored order (simulation/sampler/pitch.py:271, a stable sort by cell). That order is not fixed. The pool insert reads a parallel scan of raw.pitches with no ORDER BY (pipeline/batch/profiles/pools.py:64-175). Both export scans have no ORDER BY either (pipeline/batch/artifacts/pitch_pool.py:36-39 and 77-83). So each pool build gives the draw other reference rows and other density weights. The nightly build rebuilds the current season's pool; a full rebuild rebuilds every season. Production runs the correction (SIM_PITCH_RESULT_SPLIT=1; SIM_RESULT_DENSITY_POWER defaults to 1.0). Two bundle builds from one DuckDB file already export the pool in one order; the order changes only between pool builds. Found by the arsenal row-order work (SIM-580, 2026-10-26); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>The SELECT order matches COMMAND_FEATURES, and a unit test pins it. The nightly matrices are rebuilt.</t>
+          <t>Two pool builds from the same data export the same pitch-pool rows in the same order. The density weights are then the same. A unit test pins the export order.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Select zone_take_rate before chase_rate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="127.5" customHeight="1" s="15">
+          <t>Add ORDER BY pitch_id (the table's key) to both pitch-pool export scans. The arrays and the meta file must keep one shared order. The fix changes every density weight once; land it before the weight fit (SIM-548).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="219.5" customHeight="1" s="15">
       <c r="A12" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -850,155 +850,155 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
+          <t>SIM-636</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Export the batted-ball pool in pitch order, so the fielding draw's density weights stay the same between pool builds</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>The fielding draw lowers the weight of a candidate batted ball where the candidate set is crowded with similar balls. It measures the crowding against 256 reference rows of the set (simulation/sampler/fielding.py:612-636). A generator seeded on the set's first row, last row and size picks the rows by POSITION. The set keeps the batted-ball pool's stored order. That order is not fixed. The outcome-pool insert joins the pitch pool to a parallel scan of raw.pitches with no ORDER BY (pipeline/batch/profiles/pools.py:205-393). The export's array query and its meta COPY have no ORDER BY either (pipeline/batch/artifacts/battedball_pool.py:114-117 and 162-175). So each pool build gives other density weights. The simulated mix of singles, doubles and home runs then moves with no change in code or data. Production runs the correction (SIM_BB_BORN_SIGMA=1.0; SIM_BB_BORN_DENSITY_POWER defaults to 1.0). The weight fit names this correction as a lever it tunes (SIM-548), so the correction must be stable first. Found by the arsenal row-order work (SIM-580, 2026-10-26); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Two pool builds from the same data export the same batted-ball rows in the same order. The fielding draw's density weights are then the same. A unit test pins the export order.</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Add ORDER BY pitch_id to the array query and to the meta COPY of battedball_pool.py. The two must keep one shared order. The fix changes every born-ball density weight once. It can land in the same commit as the pitch pool's export order (SIM-635).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="127.5" customHeight="1" s="15">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
           <t>SIM-611</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Owner decisions: four similarity design points</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Not defects, design points for the owner. (1) The catcher's shrinkage prior is 15 called pitches, so alpha is at least 0.95 for every kept catcher (framing stabilizes near 1,500). (2) stop_rate is exactly one minus the overall attempt rate, so that rate counts twice in the runner's aggression distance. (3) The batter's xba / xslg and the manager's hit-and-run and double-switch rates read 0.0 for everyone and still hold their share of the kernel weight. (4) CLAUDE.md section 1 calls CLV 'the gold-standard metric'; the owner ruled on 2026-09-28 that the model is not judged by it. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>The owner rules on each point, and the code or CLAUDE.md follows.</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Raise the catcher prior; drop stop_rate; drop the all-zero features; rewrite CLAUDE.md section 1.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="87" customHeight="1" s="15">
-      <c r="A13" s="17" t="inlineStr">
+    <row r="14" ht="87" customHeight="1" s="15">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>SIM-587</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Decide which calibration values the draws use, and make the code follow</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>similarity/calibration/pitcher.py fits sigma_command and eb_n_prior_pitcher, and no code reads either, so the pitcher engine keeps RBF_SIGMA_COMMAND 1.0453 and EB_N_PRIOR 5. More broadly, the nightly actor matrices apply no calibration report (build_actor_sim_matrices): make calibrate changes only the API's engines. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>The owner decides which values the draws use, and the code and the docs follow.</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>Read both fields in apply_calibration and apply /data/calibration.json in the matrix build; or document the module defaults as the draws' values.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="73.5" customHeight="1" s="15">
-      <c r="A14" s="17" t="inlineStr">
+    <row r="15" ht="73.5" customHeight="1" s="15">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>SIM-583</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Keep the calibrated win probability strictly between 0 and 1</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>build_validation_report fits the reliability curve with min_bin_count=1, so a bin of two games can map 0.75 to 1.0. Example: the curve [[0,0],[0.45,0.44],[0.55,0.56],[0.73,1.0],[1,1]] and home_win_pct 0.75 at n = 100 give home 1.0, away 0.0 and an interval of zero width. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>No calibrated probability is 0.0 or 1.0, and a unit test feeds the curve above.</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Fit the curve with a min_bin_count near 30, or clamp the mapped probability to [eps, 1 - eps].</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="127.5" customHeight="1" s="15">
-      <c r="A15" s="17" t="inlineStr">
+    <row r="16" ht="127.5" customHeight="1" s="15">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>SIM-584</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Stamp the accuracy report with the bundle the run read, not the live link</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>scripts/accuracy/selection.py bundle_provenance reads the manifest times under BASEBALL_PLAY_POOL_DIR/engine_artifacts (the live link). The factory reads BASEBALL_ENGINE_ARTIFACT_DIR when it is set (simulation/production_factory.py). Seen on 2026-10-20: two runs on the same pinned bundle, before and after the nightly rebuild, carry different manifest_mtimes and identical records, so pair_accuracy.py refuses to pair them; two runs on different pinned bundles on one day would pair. The weight fit (SIM-548) pairs these reports. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>The stamp names the bundle the run read, and a test pins the pinned-directory case.</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>Read the pinned directory first, as the factory does.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="81" customHeight="1" s="15">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>SIM-547</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/probes/manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
         </is>
       </c>
     </row>
@@ -1010,27 +1010,27 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>SIM-526</t>
+          <t>SIM-547</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Turn on the catcher pitch-receiving factor</t>
+          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
+          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
+          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
+          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/probes/manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
         </is>
       </c>
     </row>
@@ -1042,27 +1042,27 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>SIM-556</t>
+          <t>SIM-526</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
+          <t>Turn on the catcher pitch-receiving factor</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/probes/steal_weight_volume_probe.py with its records (docs/audit/records/steal_weight_volume_probe_2025.* and _2026.*; the arrays in results/steal_weight_volume/). Filed P3 by the owner on 2026-10-01.</t>
+          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
+          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/probes/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
+          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
         </is>
       </c>
     </row>
@@ -1074,59 +1074,59 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
+          <t>SIM-556</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/probes/steal_weight_volume_probe.py with its records (docs/audit/records/steal_weight_volume_probe_2025.* and _2026.*; the arrays in results/steal_weight_volume/). Filed P3 by the owner on 2026-10-01.</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/probes/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="81" customHeight="1" s="15">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
           <t>SIM-574</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Make each SIM_* flag's code default equal its production value, or record why it differs</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>The simulator reads its switches and weights from SIM_* environment flags. Each flag has a default in the code (the value an unset flag reads) and a production value set in the app service of docker-compose.yml. They differ for 24 of the flags compose sets (measured 2026-10-20): for example the pitch-draw cell index is off in code and on in production, and the fence stage, the fielding class filter and the manager draw are the same. So a script, a probe or a test that forgets one flag runs a different simulator from production, silently. The registry of the flags (simulation/flags.py, the code clean-up SIM-493) now lists every default in one table, which makes the gap visible but does not close it.</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>For every registered flag the code default equals the compose value, or the registry row says in one line why it differs (for example: the unit lane's byte-identical state). The unit lane's own pins in tests/conftest.py still hold its state. The fingerprint (scripts/behaviour_fingerprint.py) of production is unchanged, because compose already sets the production values.</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>Owner decision first: should an unset flag mean production or off? If production: change each default in simulation/flags.py to the compose value, keep tests/conftest.py's pins for the unit lane, and add a registry test that the defaults equal compose. If off: add the reason column to the registry and a test that compose sets every flag whose default differs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="73.5" customHeight="1" s="15">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>SIM-608</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Store a price that returns to an earlier value</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>The odds writer dedups on a hash with no time (ON CONFLICT (game_pk, source, odds_hash)), so -110 at t0, -120 at t1, -110 at t2 closes the series at -120. Read from the code, not checked against stored data. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>A return to an earlier price is stored, and the series closes on the last price.</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>Dedup only against the latest row of the same game, source, book, market and line type.</t>
         </is>
       </c>
     </row>
@@ -1138,347 +1138,347 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
+          <t>SIM-608</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Store a price that returns to an earlier value</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>The odds writer dedups on a hash with no time (ON CONFLICT (game_pk, source, odds_hash)), so -110 at t0, -120 at t1, -110 at t2 closes the series at -120. Read from the code, not checked against stored data. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>A return to an earlier price is stored, and the series closes on the last price.</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Dedup only against the latest row of the same game, source, book, market and line type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="73.5" customHeight="1" s="15">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
           <t>SIM-607</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Read the line-movement direction book by book</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>betting/line_movement.py _net_direction pools every book, so the first and last quotes can come from two books: (t1, bp:1, -110/-110) and (t2, bp:2, -130/+110) give direction 'toward' and a CLV, though neither book moved. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>The direction is each book's own, then aggregated.</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>Compute the direction per book, then aggregate.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="132" customHeight="1" s="15">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
+    <row r="23" ht="132" customHeight="1" s="15">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>SIM-625</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Capture the opening lines every day</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>No scheduled job captures the opening lines. Nothing calls schedule_opening_line_job (pipeline/etl/opening_line_job.py), and the nightly closing-lines job (scripts/nightly_closing_lines.sh, 10:30 UTC) passes --line-types closing only. The venue backfill (schedule_venue_backfill_job) has no caller either. BettingPros serves the opener after the fact, so scripts/load_historical_odds.py (its default line types are opening and closing) recovers the missing rows: nothing is lost for good. The line-movement page reads the opening-to-closing series. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>Each night's odds run stores the opening rows of the games it loads, and the venue backfill either runs on a schedule or is retired.</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>Pass --line-types opening closing in scripts/nightly_closing_lines.sh. Then retire opening_line_job.py, or give it a scheduler entry; decide the venue backfill the same way.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="60" customHeight="1" s="15">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
+    <row r="24" ht="60" customHeight="1" s="15">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>SIM-586</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Ask the schedule only for game types raw.games accepts</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>GAME_TYPES (pipeline/live/ingestion/constants.py) is R F D L W C P; the CHECK on raw.games allows R P S A D F L W. A game of type C on the slate fails its upsert. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>The live pipeline's game types and the table's CHECK agree, and a unit test compares them.</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>Drop C from GAME_TYPES, or widen the CHECK with a migration if type C games should load.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="114" customHeight="1" s="15">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
+    <row r="25" ht="190.5" customHeight="1" s="15">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>SIM-639</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Fail the profile step when an arsenal-fit worker crashes</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>The profile computor fits the pitcher arsenals in a process pool (the ProcessPoolExecutor loop of _compute_pitcher_profiles, pipeline/batch/profiles/pitcher.py, at the 'GMM worker chunk crashed' log line). When one worker dies (the random segfault class, CLAUDE.md section 2a), the pool breaks and every unfinished chunk raises. The computor logs the error and marks every pitcher of those chunks below the minimum sample (_flush_gmm_results in pipeline/batch/profiles/gmm.py). Those pitchers keep the placeholder model. They drop out of the pitcher engine and its score matrix. The step then exits 0, so the nightly's retry wrapper (scripts/with_retry.sh, three attempts) does not run it again. With one chunk per worker, one death can drop most pitchers of the season. Two builds of the same data then differ on a crash day. Found by the arsenal row-order work (SIM-580, 2026-10-26); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>A crashed worker chunk makes the profile step exit non-zero, and the nightly's retry wrapper runs it again. A unit test whose worker dies of a real segfault proves the non-zero exit and the 'Fatal Python error' line in the step's output. No pitcher with enough clean pitches is marked below the minimum sample because of a crash.</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Re-raise after the computor logs a crashed chunk or a broken pool, so the step exits non-zero. Keep the per-pitcher fallback only for a fit that fails on its own data (a model of None). A worker that segfaults prints nothing today, because no process turns faulthandler on. The re-raise alone exits 1 with no 'Fatal Python error' line, and with_retry.sh then stops. So start the pool with initializer=faulthandler.enable: a worker's segfault then writes the line, and the wrapper retries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="114" customHeight="1" s="15">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>SIM-582</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Add last_seen_at to the two odds archive tables, so the retirement copy fits again</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>Migration 0029 added last_seen_at to raw.game_odds and raw.prop_odds and not to their archives (raw.game_odds_archive, raw.prop_odds_archive, migration 0028). The retirement script copies rows with INSERT ... SELECT *, which needs the same columns in the same order, so the next retirement fails. The integration test test_schema_migrations.py::test_sim555_stamp_indexes_and_archives reds on master fe81d79 and on the clean-up branch for this reason. Found by the code clean-up (SIM-493, the integration pass, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>Both archives carry last_seen_at in the live table's position, the integration test passes, and a retirement run copies a row.</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>A new Alembic migration adds last_seen_at to both archives (nullable, so the copied rows keep their value), placed after book_line_at to match the live tables; check the column order with the test.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="87" customHeight="1" s="15">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
+    <row r="27" ht="87" customHeight="1" s="15">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>SIM-581</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Name only real tests in the nightly acceptance lane's required roster</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>The REQUIRED roster of .github/workflows/acceptance-nightly.yml lists test_full_pool_out_advancement_runs_sim450, test_full_pool_steal_decision_runs_sim450 and test_reach_on_error_band_sim450. No test of those names exists, and the roster step fails when a required name did not run. So the nightly lane reds on every run, whatever the bands read. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>The roster names only real tests, and one nightly run passes its roster step.</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>Delete the three names, or name the tests that took their place.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="118" customHeight="1" s="15">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
+    <row r="28" ht="118" customHeight="1" s="15">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>SIM-633</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Make the test targets run what their names say</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>make test-unit passes no -m "not slow", so it runs the slow tests at the 30 s timeout; CI's unit job excludes them. make test-integration runs in the app container, which has no Docker socket (only the scheduler mounts it), so testcontainers cannot start and every integration test skips. The games input of acceptance-nightly.yml says "max 12" and defaults to 12, but the balanced set has 45 games (beside SIM-581, the roster). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>make test-unit matches CI's unit job; make test-integration runs the integration lane or says it needs host Python; the workflow input describes the 45-game set.</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>Add -m "not slow" to test-unit and a test-slow target. Run the integration lane on host Python, as docs/technical/tests.md describes. Fix the input's text and default.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="90" customHeight="1" s="15">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
+    <row r="29" ht="90" customHeight="1" s="15">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>SIM-626</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Point the GitHub workflows at master</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>docker-release.yml and frontend-release.yml run on a push to main (and on a published release), and the pull_request trigger of ci.yml lists main. The default branch is master, so a push never runs the two release workflows, and a pull request into master gets no pull-request run of CI (the push run still happens). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>A push to master runs both release workflows (or the owner retires them), and a pull request into master runs CI.</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>Replace main with master in the three triggers, and in the trigger comment at the head of ci.yml.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="73.5" customHeight="1" s="15">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
+    <row r="30" ht="73.5" customHeight="1" s="15">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>SIM-619</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>Run the batch-runner stress test in a CI job</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>tests/integration/test_batch_runner_stress.py carries only the slow marker. The CI slow lane runs tests/unit -m slow; the weekly integration lane and make test-integration select -m integration; the e2e job runs one file. No job runs it. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>One lane runs it.</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="F30" s="5" t="inlineStr">
         <is>
           <t>Mark it integration, or add its path to the slow lane.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="73.5" customHeight="1" s="15">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
+    <row r="31" ht="73.5" customHeight="1" s="15">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>SIM-602</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>Make two API tests check what their names say</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>tests/unit/test_api_betting.py test_clv_snapshot_returns_only_series_with_clv makes a GET and asserts nothing. tests/unit/test_api_games_plays.py test_simulate_ok_without_duckdb_then_plays_404 never requests /plays. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>Each test asserts what its name says.</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>Add the assertions (the CLV series' filter; /plays answers 503 with no replay store), then rename the second test.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="87" customHeight="1" s="15">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>SIM-601</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Make the Playwright smoke tests pass while the live app runs</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>frontend/e2e/smoke.spec.ts (three specs) fail on the owner's host: a request the test does not mock goes through the preview server's proxy to localhost:8000, the live app answers 401 and the page shows the login. With API_TARGET=http://127.0.0.1:9 all 21 tests pass; CI has no backend, so CI passes. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>The e2e suite passes with the live app running.</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>Set API_TARGET to a closed port in playwright.config.ts's webServer.env, or end each spec with a catch-all **/api/** route that answers 404.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="104" customHeight="1" s="15">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>SIM-630</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>Bring the Postgres schema file up to the migrations</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>db/schemas/01_postgres_schema.sql lags the Alembic migrations. It has no raw.savant_pitch_tracking (0020), no raw.game_bullpen (0025), none of the 0029 columns (raw.game_lineups.published_at, last_seen_at on the odds tables, the run-job columns) and none of the 0030 columns of sim.sim_runs (start_at_bat and the rest). At least eight unit tests read the file to check a schema fact. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>The file matches the schema that alembic upgrade head builds, and a test holds the two equal; or the file is retired and the tests read the migrations.</t>
-        </is>
-      </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>Regenerate the file from a migrated database (pg_dump --schema-only), or retire it.</t>
         </is>
       </c>
     </row>
@@ -1490,251 +1490,251 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
+          <t>SIM-601</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Make the Playwright smoke tests pass while the live app runs</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>frontend/e2e/smoke.spec.ts (three specs) fail on the owner's host: a request the test does not mock goes through the preview server's proxy to localhost:8000, the live app answers 401 and the page shows the login. With API_TARGET=http://127.0.0.1:9 all 21 tests pass; CI has no backend, so CI passes. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>The e2e suite passes with the live app running.</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Set API_TARGET to a closed port in playwright.config.ts's webServer.env, or end each spec with a catch-all **/api/** route that answers 404.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="104" customHeight="1" s="15">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>SIM-630</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Bring the Postgres schema file up to the migrations</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>db/schemas/01_postgres_schema.sql lags the Alembic migrations. It has no raw.savant_pitch_tracking (0020), no raw.game_bullpen (0025), none of the 0029 columns (raw.game_lineups.published_at, last_seen_at on the odds tables, the run-job columns) and none of the 0030 columns of sim.sim_runs (start_at_bat and the rest). At least eight unit tests read the file to check a schema fact. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>The file matches the schema that alembic upgrade head builds, and a test holds the two equal; or the file is retired and the tests read the migrations.</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Regenerate the file from a migrated database (pg_dump --schema-only), or retire it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="87" customHeight="1" s="15">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
           <t>SIM-585</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>Refuse CORS_ORIGINS=* while the API sends credentials</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>api/main.py sets allow_credentials=True for every origin list, and resolve_cors_origins (api/auth.py) returns ['*'] when an operator sets CORS_ORIGINS=*. Starlette then echoes the caller's Origin on a request with a cookie, so any site can read the API with the user's login. Production sets neither variable today, so the defect is latent. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>CORS_ORIGINS=* either fails the boot or turns credentials off, and a unit test pins it.</t>
         </is>
       </c>
-      <c r="F32" s="5" t="inlineStr">
+      <c r="F34" s="5" t="inlineStr">
         <is>
           <t>Refuse '*' in resolve_cors_origins while credentials are on.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="160" customHeight="1" s="15">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
+    <row r="35" ht="160" customHeight="1" s="15">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>SIM-632</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Give the backup path one name, and correct the staging and production templates</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="D35" s="5" t="inlineStr">
         <is>
           <t>The app reads BACKUPS_ROOT (api/routes/metrics.py, docker-compose.yml) while the backup jobs read BACKUP_ROOT (pipeline/backup/data_stores.py, pipeline/backup/offsite.py, db/backup/pg_backup.sh). Both default to /backups, so the age gauges work today; a value set under one name alone splits them. Both env templates set LIVE_PIPELINE_ENABLED=true, which makes the app a second publisher beside the live service. .env.production.example sets ODDS_PROVIDER=theoddsapi, which no provider registers. The templates also carry seven keys no app code reads: WORKERS, SIM_MAX_WORKERS, ODDS_PROVIDER_API_KEY, ODDS_API_BASE, ASYNC_DB_DSN, MLB_API_BASE and PROMETHEUS_PUSHGATEWAY. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="E35" s="5" t="inlineStr">
         <is>
           <t>One variable names the backup root, and the templates hold only keys the code reads, with values that start the stack.</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="F35" s="5" t="inlineStr">
         <is>
           <t>Rename the app's variable to BACKUP_ROOT. Rewrite the two templates from .env.example.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="104" customHeight="1" s="15">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
+    <row r="36" ht="219.5" customHeight="1" s="15">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>SIM-637</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Pair consecutive seasons in the batter's and the runner's reliability-weight fit</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>make calibrate fits a reliability weight per feature group: how well the group repeats from one season to the next. The fit pairs two season rows of one player. The batter and baserunner calibrators pass no seasons to that fit (similarity/calibration/fitting.py:237-240 and 272-275). So each player's pair is the player's first two rows in the table's stored order, whatever their seasons. Their reads have no ORDER BY (similarity/calibration/batter.py:57-77, baserunner.py:50-66). Each profile build stores the rows in a new order. So two calibrations of the same data write other reliability weights to /data/calibration.json. Only the API's similarity engines read these values today (the /api/similarity routes and the Similarity Explorer page). The nightly score matrices apply no calibration report. A decision is open on which calibration values the draws use (SIM-587). If that decision applies the report to the matrix build, this ticket moves to P2 and lands before that change. Found by the arsenal row-order work (SIM-580, 2026-10-26); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>The batter's and the runner's reliability weights pair consecutive seasons of one player. Two calibrations from the same profiles give the same weights. A unit test pins a player whose rows are stored 2023, 2025, 2024.</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Pass seasons= to calibrate_reliability_weights in both calibrators, as the fielder's calibrator does. Pass each seasons array through the same mask as its rows (phys_mask, plat_mask, agg_measured). Rewrite the docstring at fitting.py:237-240.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="190.5" customHeight="1" s="15">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>SIM-638</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Order the calibrators' profile reads, so the fitted bandwidths stay the same between profile builds</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>make calibrate fits each kernel bandwidth (sigma: how fast a similarity score falls as two profiles grow apart). The fit (calibrate_sigma) takes the median distance over up to 50,000 pairs of rows (similarity/calibration/fitting.py:78-91). A seeded generator draws the pairs by row INDEX. Seven calibrators read their profile table with no ORDER BY: the batter, baserunner, runner-steal, catcher, manager, pitcher and pitcher-steal calibrators. Only the fielder's reads are ordered (similarity/calibration/fielder.py:103 and 131). Each profile build stores the rows in a new order. So the same indices pick other players, and the fitted bandwidths move by sampling noise. Only the API's similarity engines read the bandwidths today. This ticket moves to P2 if the decision on calibration values (SIM-587) applies the report to the matrix build. Found by the arsenal row-order work (SIM-580, 2026-10-26); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Two calibrations from the same profiles give the same bandwidths, whatever the stored row order. A unit test reverses a profile table's stored order and gets the same bandwidth.</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Add ORDER BY each table's key to the seven reads (for example pitcher_id, season for the pitcher).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="104" customHeight="1" s="15">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>SIM-629</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>End a tied game at the inning limit without an extra pitch</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
+      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>simulate_game (simulation/sim_loop.py) checks state.inning &gt; max_innings only after a pitch that does not roll the half, and _game_over_after_half knows nothing of the limit. So a game tied after the API's 12 innings (max_innings 12 in simulation/sim_kwargs.py) starts the 13th, places the extra-innings runner on second and throws one pitch before it stops. That pitch can score a run or credit a box line. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E34" s="5" t="inlineStr">
+      <c r="E38" s="5" t="inlineStr">
         <is>
           <t>A game tied at the limit ends when the last allowed half completes, and a unit test pins it.</t>
         </is>
       </c>
-      <c r="F34" s="5" t="inlineStr">
+      <c r="F38" s="5" t="inlineStr">
         <is>
           <t>Check the limit in the roll branch, right after _game_over_after_half.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="60" customHeight="1" s="15">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
+    <row r="39" ht="60" customHeight="1" s="15">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>SIM-594</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>Let the batter run on a called third strike that gets away</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="D39" s="5" t="inlineStr">
         <is>
           <t>Rule 5.05(a)(2) lets the batter run on any uncaught third strike. _dropped_third_strike reads swinging strikes only. Two such rows exist in 2023-2026, both in 2026. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E35" s="5" t="inlineStr">
+      <c r="E39" s="5" t="inlineStr">
         <is>
           <t>A called third strike that gets away can be a dropped-third-strike reach.</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
+      <c r="F39" s="5" t="inlineStr">
         <is>
           <t>Let _dropped_third_strike read a called third strike too.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="73.5" customHeight="1" s="15">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>SIM-591</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>Charge the losing pitcher with the go-ahead run, as MLB does</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>pitcher_decisions charges the pitcher on the mound at the decisive play. In a tie, A walks a batter, B relieves him and allows a double that scores the runner, and the lead holds: MLB charges A; the simulator charges B. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>The decision follows the runner's responsible pitcher, and a unit test plays the example.</t>
-        </is>
-      </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>Carry each runner's responsible pitcher on the bases.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="73.5" customHeight="1" s="15">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>SIM-592</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>Put the batter on first after a forced reach with no batter id</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>_force_on_reach with no batter id leaves first base's runner on first after pushing him to second (b.first = state.batter_id if ... else b.first), so the base check raises; _resolve_walk assigns b.first = state.batter_id for the same case. Reachable only with a sampler and no lineup. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>The forced reach and the walk give the same bases.</t>
-        </is>
-      </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>Use the walk's assignment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="73.5" customHeight="1" s="15">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>SIM-593</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>Void the plate appearance after a third out on the bases in the single pre-pitch steal draw</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>With SIM_STEAL_PITCH_CLASS=0 (not production), a pickoff or a caught stealing that makes the third out before the pitch's result still ends the plate appearance, so the pitcher gets a batter faced and the batter an at-bat. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>The single draw voids the plate appearance as the running game on the pitch does.</t>
-        </is>
-      </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>Apply the no-pitch void of the class-aware draw.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="46.5" customHeight="1" s="15">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>SIM-588</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>Compute the z of the requested level in GameSimSummary.from_results</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>GameSimSummary.from_results(confidence_level=0.85) computes the 95% z and labels the intervals 0.85. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Each level gets its own z, and a unit test checks 0.85.</t>
-        </is>
-      </c>
-      <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>Use NormalDist().inv_cdf((1 + level) / 2), or raise on a level outside the table.</t>
         </is>
       </c>
     </row>
@@ -1746,31 +1746,31 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>SIM-605</t>
+          <t>SIM-591</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Keep one pitcher engine's calibration from rewriting every pitcher engine</t>
+          <t>Charge the losing pitcher with the go-ahead run, as MLB does</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>PitcherSimilarityEngine.apply_calibration sets the module global ARSENAL_SCALE, and a report with no gamma resets it to 4.10. The API builds two instances. Latent: no production path calls it today. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>pitcher_decisions charges the pitcher on the mound at the decisive play. In a tie, A walks a batter, B relieves him and allows a double that scores the runner, and the lead holds: MLB charges A; the simulator charges B. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Each instance carries its own scale.</t>
+          <t>The decision follows the runner's responsible pitcher, and a unit test plays the example.</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Pass the instance's scale into the three readers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="90" customHeight="1" s="15">
+          <t>Carry each runner's responsible pitcher on the bases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="73.5" customHeight="1" s="15">
       <c r="A41" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1778,27 +1778,27 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>SIM-628</t>
+          <t>SIM-592</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Let the resumable sweep read the database address</t>
+          <t>Put the batter on first after a forced reach with no batter id</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>The child process of scripts/resumable_sweep.py reads BASEBALL_DB_DSN from .env with env["BASEBALL_DB_DSN"]. Since the security hardening (SIM-443b), .env carries no such key: .env.example has it commented out, and the live .env has none. So a sweep stops with KeyError before its first game. This is separate from the retry after a crash (SIM-614). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>_force_on_reach with no batter id leaves first base's runner on first after pushing him to second (b.first = state.batter_id if ... else b.first), so the base check raises; _resolve_walk assigns b.first = state.batter_id for the same case. Reachable only with a sampler and no lineup. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>A sweep starts on the current .env.</t>
+          <t>The forced reach and the walk give the same bases.</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Read BASEBALL_DB_DSN from the process environment first (pipeline.db_dsn.require_dsn); read .env only when the key is set there.</t>
+          <t>Use the walk's assignment.</t>
         </is>
       </c>
     </row>
@@ -1810,795 +1810,795 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
+          <t>SIM-593</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Void the plate appearance after a third out on the bases in the single pre-pitch steal draw</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>With SIM_STEAL_PITCH_CLASS=0 (not production), a pickoff or a caught stealing that makes the third out before the pitch's result still ends the plate appearance, so the pitcher gets a batter faced and the batter an at-bat. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>The single draw voids the plate appearance as the running game on the pitch does.</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>Apply the no-pitch void of the class-aware draw.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="46.5" customHeight="1" s="15">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>SIM-588</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Compute the z of the requested level in GameSimSummary.from_results</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>GameSimSummary.from_results(confidence_level=0.85) computes the 95% z and labels the intervals 0.85. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Each level gets its own z, and a unit test checks 0.85.</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>Use NormalDist().inv_cdf((1 + level) / 2), or raise on a level outside the table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="73.5" customHeight="1" s="15">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>SIM-605</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Keep one pitcher engine's calibration from rewriting every pitcher engine</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>PitcherSimilarityEngine.apply_calibration sets the module global ARSENAL_SCALE, and a report with no gamma resets it to 4.10. The API builds two instances. Latent: no production path calls it today. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Each instance carries its own scale.</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>Pass the instance's scale into the three readers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="90" customHeight="1" s="15">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>SIM-628</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Let the resumable sweep read the database address</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>The child process of scripts/resumable_sweep.py reads BASEBALL_DB_DSN from .env with env["BASEBALL_DB_DSN"]. Since the security hardening (SIM-443b), .env carries no such key: .env.example has it commented out, and the live .env has none. So a sweep stops with KeyError before its first game. This is separate from the retry after a crash (SIM-614). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>A sweep starts on the current .env.</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>Read BASEBALL_DB_DSN from the process environment first (pipeline.db_dsn.require_dsn); read .env only when the key is set there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="73.5" customHeight="1" s="15">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
           <t>SIM-614</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>Retry a sweep attempt that crashes before its first game</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="D46" s="5" t="inlineStr">
         <is>
           <t>scripts/resumable_sweep.py applies its zero-progress stop (gained == 0) after a crash too, so a segfault before the first game of an attempt ends the sweep (exit 1) instead of retrying. Found by reading the code; not exercised. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E42" s="5" t="inlineStr">
+      <c r="E46" s="5" t="inlineStr">
         <is>
           <t>A crashed attempt with no gain retries up to --max-attempts.</t>
         </is>
       </c>
-      <c r="F42" s="5" t="inlineStr">
+      <c r="F46" s="5" t="inlineStr">
         <is>
           <t>Apply the stop only to an attempt that exited cleanly.</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="87" customHeight="1" s="15">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
+    <row r="47" ht="87" customHeight="1" s="15">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>SIM-613</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>Print n/a in the hypothetical-return table when no bet qualifies</t>
         </is>
       </c>
-      <c r="D43" s="5" t="inlineStr">
+      <c r="D47" s="5" t="inlineStr">
         <is>
           <t>scripts/accuracy/hypothetical_return.py _fmt_row formats the means and the range with :.4f and no guard for None. With no qualifying bet the table raises TypeError, and run() prints it before it writes the report and before the zero-games check, so the run ends in a traceback with no report and no exit code 5. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E43" s="5" t="inlineStr">
+      <c r="E47" s="5" t="inlineStr">
         <is>
           <t>The table prints n/a, as the accuracy table does.</t>
         </is>
       </c>
-      <c r="F43" s="5" t="inlineStr">
+      <c r="F47" s="5" t="inlineStr">
         <is>
           <t>Use the _fmt_or_na guard.</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="87" customHeight="1" s="15">
-      <c r="A44" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
+    <row r="48" ht="87" customHeight="1" s="15">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>SIM-616</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>Decide the minimum-sample read's two known limits</t>
         </is>
       </c>
-      <c r="D44" s="5" t="inlineStr">
+      <c r="D48" s="5" t="inlineStr">
         <is>
           <t>scripts/accuracy/confidence.py: the 0.02 floor assumes a coin-flip market, so its power is weaker than stated for a market far from 0.5 (a home-run prop); and a small sample whose observed spread is exactly zero reads as fully resolved. An adversarial review of the minimum-sample work (SIM-539) found both. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E44" s="5" t="inlineStr">
+      <c r="E48" s="5" t="inlineStr">
         <is>
           <t>The owner decides whether to fix or accept them.</t>
         </is>
       </c>
-      <c r="F44" s="5" t="inlineStr">
+      <c r="F48" s="5" t="inlineStr">
         <is>
           <t>A per-market 4p(1-p) correction and an upper bound on the spread.</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="73.5" customHeight="1" s="15">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
+    <row r="49" ht="73.5" customHeight="1" s="15">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>SIM-589</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>Treat both samples as samples in the replay chi-squared test</t>
         </is>
       </c>
-      <c r="D45" s="5" t="inlineStr">
+      <c r="D49" s="5" t="inlineStr">
         <is>
           <t>The two-sample path of replay_chi_squared.chi_squared_gof treats the reference sample as exact. Two independent samples of 1,000 Poisson(4.4) totals were rejected 52.5% of the time at alpha 0.05 over 400 trials. replay_and_test uses it. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E45" s="5" t="inlineStr">
+      <c r="E49" s="5" t="inlineStr">
         <is>
           <t>Two samples from one distribution are rejected near alpha.</t>
         </is>
       </c>
-      <c r="F45" s="5" t="inlineStr">
+      <c r="F49" s="5" t="inlineStr">
         <is>
           <t>Use scipy.stats.chi2_contingency on the pooled 2 x k table.</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="60" customHeight="1" s="15">
-      <c r="A46" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="inlineStr">
+    <row r="50" ht="60" customHeight="1" s="15">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>SIM-590</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>Compare the historical replay against the right side's score</t>
         </is>
       </c>
-      <c r="D46" s="5" t="inlineStr">
+      <c r="D50" s="5" t="inlineStr">
         <is>
           <t>replay_historical_games always compares the simulated HOME score. A HistoricalGame row does not say which side its runs belong to, so an away team's runs meet the simulated home runs. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E46" s="5" t="inlineStr">
+      <c r="E50" s="5" t="inlineStr">
         <is>
           <t>A HistoricalGame row names its side, and the replay compares like with like.</t>
         </is>
       </c>
-      <c r="F46" s="5" t="inlineStr">
+      <c r="F50" s="5" t="inlineStr">
         <is>
           <t>Add a side field to HistoricalGame.</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="60" customHeight="1" s="15">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
+    <row r="51" ht="60" customHeight="1" s="15">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>SIM-618</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>Keep one copy of the prop ground-truth readers</t>
         </is>
       </c>
-      <c r="D47" s="5" t="inlineStr">
+      <c r="D51" s="5" t="inlineStr">
         <is>
           <t>scripts/validate_props.py and scripts/accuracy/grading.py each define _fetch_official_boxscore and _fetch_pa_events. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E47" s="5" t="inlineStr">
+      <c r="E51" s="5" t="inlineStr">
         <is>
           <t>One reader, imported by both.</t>
         </is>
       </c>
-      <c r="F47" s="5" t="inlineStr">
+      <c r="F51" s="5" t="inlineStr">
         <is>
           <t>Move it to simulation/prop_validation.py.</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="73.5" customHeight="1" s="15">
-      <c r="A48" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B48" s="3" t="inlineStr">
+    <row r="52" ht="73.5" customHeight="1" s="15">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>SIM-621</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>Bench the per-pitch call the loop makes</t>
         </is>
       </c>
-      <c r="D48" s="5" t="inlineStr">
+      <c r="D52" s="5" t="inlineStr">
         <is>
           <t>tests/performance/bench_simulation.py times PitcherSimilarityEngine.query() as the per-pitch cost; the loop reads the dense pitcher matrix. bench_api_simulate.py says an authoritative gate runs on target hardware with the DB-backed factory; no job does. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E48" s="5" t="inlineStr">
+      <c r="E52" s="5" t="inlineStr">
         <is>
           <t>The benches time what the loop runs, and the SLA text names the job that gates it.</t>
         </is>
       </c>
-      <c r="F48" s="5" t="inlineStr">
+      <c r="F52" s="5" t="inlineStr">
         <is>
           <t>Bench the matrix read; correct the SLA text.</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="60" customHeight="1" s="15">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="inlineStr">
+    <row r="53" ht="60" customHeight="1" s="15">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>SIM-612</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C53" s="4" t="inlineStr">
         <is>
           <t>Read the pitch rebuild's before-smoke from results/</t>
         </is>
       </c>
-      <c r="D49" s="5" t="inlineStr">
+      <c r="D53" s="5" t="inlineStr">
         <is>
           <t>scripts/pitch_pool_rebuild/export.py _smoke_games opens scripts/sim553_smoke_before.json; the groundwork moved run outputs to results/sim553/. The function always prints its placeholder. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E49" s="5" t="inlineStr">
+      <c r="E53" s="5" t="inlineStr">
         <is>
           <t>It reads the results/ path.</t>
         </is>
       </c>
-      <c r="F49" s="5" t="inlineStr">
+      <c r="F53" s="5" t="inlineStr">
         <is>
           <t>Change the one path.</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="73.5" customHeight="1" s="15">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="inlineStr">
+    <row r="54" ht="73.5" customHeight="1" s="15">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>SIM-623</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>Replace the inning-grid test's pinned scores with an outcome check</t>
         </is>
       </c>
-      <c r="D50" s="5" t="inlineStr">
+      <c r="D54" s="5" t="inlineStr">
         <is>
           <t>tests/unit/test_inning_grid.py pins the exact scores and pitch counts of ten seeds (OUTCOMES_AT_80E3F46). That works like the golden snapshots the owner ruled out on 2026-09-10: any intended change to the draw fails it. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E50" s="5" t="inlineStr">
+      <c r="E54" s="5" t="inlineStr">
         <is>
           <t>The test checks a property of the grid (its sum equals the final score, the halves match the outs), not ten remembered numbers.</t>
         </is>
       </c>
-      <c r="F50" s="5" t="inlineStr">
+      <c r="F54" s="5" t="inlineStr">
         <is>
           <t>Rewrite the assertions as invariants and delete the pinned table.</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="87" customHeight="1" s="15">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="inlineStr">
+    <row r="55" ht="87" customHeight="1" s="15">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>SIM-620</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>Delete the regression gate's dead constants and its golden-file texts</t>
         </is>
       </c>
-      <c r="D51" s="5" t="inlineStr">
+      <c r="D55" s="5" t="inlineStr">
         <is>
           <t>tests/regression/regression_config.py: only SYMMETRY_TOLERANCE has a reader; eight constants have none (the conftest hard-codes the seed 2026), and one constant's docstring still speaks of golden files. The assert message at test_engine_regression.py:322 names golden files the gate does not have. The pyproject.toml marker text, the ci.yml header and make help were corrected by the documentation rebuild (SIM-624, 2026-10-21). Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E51" s="5" t="inlineStr">
+      <c r="E55" s="5" t="inlineStr">
         <is>
           <t>The dead constants go, and the assert message says what the gate checks.</t>
         </is>
       </c>
-      <c r="F51" s="5" t="inlineStr">
+      <c r="F55" s="5" t="inlineStr">
         <is>
           <t>Delete the dead constants and edit the assert message.</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="60" customHeight="1" s="15">
-      <c r="A52" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B52" s="3" t="inlineStr">
+    <row r="56" ht="60" customHeight="1" s="15">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>SIM-622</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>Use the pinned park factor in the sim-kwargs tests</t>
         </is>
       </c>
-      <c r="D52" s="5" t="inlineStr">
+      <c r="D56" s="5" t="inlineStr">
         <is>
           <t>tests/unit/test_sim_kwargs.py uses 0.8723846078 for venue 680 in six places; the pinned 2024 table in the same file holds 0.8725842237. The tests pass (the literal is only an input). Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E52" s="5" t="inlineStr">
+      <c r="E56" s="5" t="inlineStr">
         <is>
           <t>One value.</t>
         </is>
       </c>
-      <c r="F52" s="5" t="inlineStr">
+      <c r="F56" s="5" t="inlineStr">
         <is>
           <t>Read it from the table.</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="87" customHeight="1" s="15">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B53" s="3" t="inlineStr">
+    <row r="57" ht="87" customHeight="1" s="15">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>SIM-597</t>
         </is>
       </c>
-      <c r="C53" s="4" t="inlineStr">
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>Write the pitching-change pool's role file in a fixed row order</t>
         </is>
       </c>
-      <c r="D53" s="5" t="inlineStr">
+      <c r="D57" s="5" t="inlineStr">
         <is>
           <t>roles.parquet (build_pitching_change_pool, pipeline/batch/artifacts/manager_pool.py) is written from a GROUP BY with no ORDER BY, so two builds of the same code from the same data write its rows in a different order. No reader uses the order, but the fingerprint's bundle mode reads a difference on every build. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E53" s="5" t="inlineStr">
+      <c r="E57" s="5" t="inlineStr">
         <is>
           <t>Two builds give the same file, by content.</t>
         </is>
       </c>
-      <c r="F53" s="5" t="inlineStr">
+      <c r="F57" s="5" t="inlineStr">
         <is>
           <t>Add ORDER BY pitcher_id, season. It changes no game.</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="118" customHeight="1" s="15">
-      <c r="A54" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B54" s="3" t="inlineStr">
+    <row r="58" ht="118" customHeight="1" s="15">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>SIM-631</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C58" s="4" t="inlineStr">
         <is>
           <t>Delete or wire up the data nobody reads</t>
         </is>
       </c>
-      <c r="D54" s="5" t="inlineStr">
+      <c r="D58" s="5" t="inlineStr">
         <is>
           <t>Built and never read: sim.stolen_base_pool (the profile computor builds it every night), the composite catcher actor matrix (built and concentration-checked; the draws read catcher_throwing), the sim.live_games view and raw.savant_first_base_receiving. Declared and never written: derived.outfield_play_detail, derived.infield_play_detail and derived.dp_play_detail. Never called: sim.purge_expired_sessions(), and EngineArtifacts.attach_shared_views outside the tests. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E54" s="5" t="inlineStr">
+      <c r="E58" s="5" t="inlineStr">
         <is>
           <t>Each item has a reader, or it is deleted with its builder and its DDL.</t>
         </is>
       </c>
-      <c r="F54" s="5" t="inlineStr">
+      <c r="F58" s="5" t="inlineStr">
         <is>
           <t>Delete them, with a migration for the DDL. Keep any the owner wants for planned work, and name the ticket that will read it.</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="73.5" customHeight="1" s="15">
-      <c r="A55" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="inlineStr">
+    <row r="59" ht="73.5" customHeight="1" s="15">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>SIM-615</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
+      <c r="C59" s="4" t="inlineStr">
         <is>
           <t>Retire the odds-hash backfill probe</t>
         </is>
       </c>
-      <c r="D55" s="5" t="inlineStr">
+      <c r="D59" s="5" t="inlineStr">
         <is>
           <t>scripts/probes/backfill_odds_hash.py _dedup_rows orders by received_at, a column raw.game_odds does not have, so its DELETE fails; its ODDS_COLUMNS leaves out draw_ml. Both are dormant: the unique index and the NOT NULL hash of migration 0012 ended the probe's job. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E55" s="5" t="inlineStr">
+      <c r="E59" s="5" t="inlineStr">
         <is>
           <t>The probe is retired.</t>
         </is>
       </c>
-      <c r="F55" s="5" t="inlineStr">
+      <c r="F59" s="5" t="inlineStr">
         <is>
           <t>Delete the probe and its test.</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="90" customHeight="1" s="15">
-      <c r="A56" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
+    <row r="60" ht="90" customHeight="1" s="15">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
         <is>
           <t>SIM-627</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>Retire the two odds routes that serve mock lines</t>
         </is>
       </c>
-      <c r="D56" s="5" t="inlineStr">
+      <c r="D60" s="5" t="inlineStr">
         <is>
           <t>GET /api/odds/{game_pk} and GET /api/odds/today/all (pipeline/live/ingestion/odds_routes.py, mounted by api/main.py) always return MockOddsAPI lines, whatever ODDS_PROVIDER says. The rows carry is_mock: true, and no frontend code calls the routes. A client that ignores the flag reads fake prices as real ones. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E56" s="5" t="inlineStr">
+      <c r="E60" s="5" t="inlineStr">
         <is>
           <t>The routes are gone (or serve the stored book rows), and the API snapshot is regenerated.</t>
         </is>
       </c>
-      <c r="F56" s="5" t="inlineStr">
+      <c r="F60" s="5" t="inlineStr">
         <is>
           <t>Delete both routes, then run scripts/export_openapi.py in the app image and npm run gen:api (CLAUDE.md section 15).</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="181.5" customHeight="1" s="15">
-      <c r="A57" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="inlineStr">
+    <row r="61" ht="181.5" customHeight="1" s="15">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
         <is>
           <t>SIM-617</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C61" s="4" t="inlineStr">
         <is>
           <t>Correct the runtime texts that state something false</t>
         </is>
       </c>
-      <c r="D57" s="5" t="inlineStr">
+      <c r="D61" s="5" t="inlineStr">
         <is>
           <t>Left unedited by the clean-up's rule. (1) The park-guard messages name the deleted SIM_PARK_FACTOR: scripts/validate_props.py, scripts/accuracy_comparison.py, tests/acceptance/conftest.py and the --help of scripts/sim_stats.py. (2) The two pool rebuilds' exit-3 texts and the steal rebuild's lock message blame the app's worker server for the DuckDB lock (the app holds no handle since SIM-524), and two steal-rebuild texts say to merge code that is merged. (3) scripts/running_game_replay.py --help says a steal can land on any pitch in production. (4) Three texts point at a module docstring section that moved in the split. (5) scripts/measure_filter_cells.py writes into docs/audit/. (6) scripts/resumable_sweep.py --help cites a deleted record. (7) The rationale strings in tests/acceptance/bands.py cite BACKLOG.md, which is gone. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E57" s="5" t="inlineStr">
+      <c r="E61" s="5" t="inlineStr">
         <is>
           <t>Each text says what is true.</t>
         </is>
       </c>
-      <c r="F57" s="5" t="inlineStr">
+      <c r="F61" s="5" t="inlineStr">
         <is>
           <t>One edit per text; list the runtime-string changes in CHANGES.md.</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="154.5" customHeight="1" s="15">
-      <c r="A58" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
+    <row r="62" ht="154.5" customHeight="1" s="15">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
         <is>
           <t>SIM-610</t>
         </is>
       </c>
-      <c r="C58" s="4" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>Similarity and betting: seven small defects</t>
         </is>
       </c>
-      <c r="D58" s="5" t="inlineStr">
+      <c r="D62" s="5" t="inlineStr">
         <is>
           <t>(1) SituationSimilarityEngine.query_batch([]) raises instead of returning []. (2) The engines' and the calibrator's __main__ blocks read a DuckDB path that does not exist (../../db/schemas/baseball_simulator.duckdb); the pitcher engine's block builds and prints nothing. (3) CalibrationReport.summary() prints no row for the batter's physical weights. (4) The Similarity Explorer's batter panel (api/routes/similarity_explorer.py) shows the four-way weights 0.40/0.35/0.15/0.10. (5) A log line in batted_ball_similarity.py says 'until SIM-051 ships'. (6) tests/regression/conftest.py scales the situation fixture's index twice. (7) No writer sets is_sharp_book, so sharp_consensus is always None. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E58" s="5" t="inlineStr">
+      <c r="E62" s="5" t="inlineStr">
         <is>
           <t>Each of the seven is fixed or retired.</t>
         </is>
       </c>
-      <c r="F58" s="5" t="inlineStr">
+      <c r="F62" s="5" t="inlineStr">
         <is>
           <t>One edit each; retire sharp_consensus if no book will be marked sharp.</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="100.5" customHeight="1" s="15">
-      <c r="A59" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
+    <row r="63" ht="100.5" customHeight="1" s="15">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
         <is>
           <t>SIM-603</t>
         </is>
       </c>
-      <c r="C59" s="4" t="inlineStr">
+      <c r="C63" s="4" t="inlineStr">
         <is>
           <t>Return the fielder's infield sub-scores in the same order from query_pair as from query</t>
         </is>
       </c>
-      <c r="D59" s="5" t="inlineStr">
+      <c r="D63" s="5" t="inlineStr">
         <is>
           <t>For an infielder, similarity/engines/fielder_similarity.py query_pair returns the specialty score in tertiary_score and the error score in quaternary_score; query returns them the other way round, as the Similarity Explorer's labels expect. Two shortstops with different error rates and equal specialty values: query gives 0.0710 / 1.0000, query_pair 1.0000 / 0.0710. The composite and the matrices are right. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E59" s="5" t="inlineStr">
+      <c r="E63" s="5" t="inlineStr">
         <is>
           <t>query and query_pair agree on every sub-score, and a unit test compares them.</t>
         </is>
       </c>
-      <c r="F59" s="5" t="inlineStr">
+      <c r="F63" s="5" t="inlineStr">
         <is>
           <t>Map the infield tuple in SimilarityResult order.</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="100.5" customHeight="1" s="15">
-      <c r="A60" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="inlineStr">
+    <row r="64" ht="100.5" customHeight="1" s="15">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
         <is>
           <t>SIM-604</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C64" s="4" t="inlineStr">
         <is>
           <t>Apply the per-hand 30-PA platoon rule in the batter engine's pair score</t>
         </is>
       </c>
-      <c r="D60" s="5" t="inlineStr">
+      <c r="D64" s="5" t="inlineStr">
         <is>
           <t>similarity/engines/batter_similarity.py _score_pair disagrees with score_all on a thin platoon split. A query with 30+ PA against either hand turns the platoon weights on for any vs_hand (10 PA vs L and 200 vs R with vs_hand='L': 0.8642 against 0.8900), and a candidate under 30 PA never gets the neutral 0.5. It serves query_pair (the Explorer's pair view and the diagnostics); the matrix is unaffected. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E60" s="5" t="inlineStr">
+      <c r="E64" s="5" t="inlineStr">
         <is>
           <t>_score_pair and score_all agree, and a unit test compares them.</t>
         </is>
       </c>
-      <c r="F60" s="5" t="inlineStr">
+      <c r="F64" s="5" t="inlineStr">
         <is>
           <t>Use score_all's per-hand rule in _score_pair.</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="60" customHeight="1" s="15">
-      <c r="A61" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="inlineStr">
+    <row r="65" ht="60" customHeight="1" s="15">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
         <is>
           <t>SIM-596</t>
         </is>
       </c>
-      <c r="C61" s="4" t="inlineStr">
+      <c r="C65" s="4" t="inlineStr">
         <is>
           <t>Decide what the what-if does when the designated hitter takes the field</t>
         </is>
       </c>
-      <c r="D61" s="5" t="inlineStr">
+      <c r="D65" s="5" t="inlineStr">
         <is>
           <t>A designated hitter moved to the field leaves the fielder he replaced in the batting order with no position. The rule that ends the designated hitter is not modelled in simulation/whatif.py. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E61" s="5" t="inlineStr">
+      <c r="E65" s="5" t="inlineStr">
         <is>
           <t>The owner decides whether the what-if models the rule, and the code follows.</t>
         </is>
       </c>
-      <c r="F61" s="5" t="inlineStr">
+      <c r="F65" s="5" t="inlineStr">
         <is>
           <t>Model the rule: the pitcher bats in the replaced fielder's slot, or refuse the change.</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="60" customHeight="1" s="15">
-      <c r="A62" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="inlineStr">
+    <row r="66" ht="60" customHeight="1" s="15">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>SIM-598</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
+      <c r="C66" s="4" t="inlineStr">
         <is>
           <t>Read the runners under the names the live service sends</t>
         </is>
       </c>
-      <c r="D62" s="5" t="inlineStr">
+      <c r="D66" s="5" t="inlineStr">
         <is>
           <t>frontend/src/hooks/useGameSocket.ts reads runner_on_first / _second / _third; the live service sends on_1b / on_2b / on_3b. The hook's on_1b to on_3b are always undefined. No page reads them today. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E62" s="5" t="inlineStr">
+      <c r="E66" s="5" t="inlineStr">
         <is>
           <t>A game_state_update with runners fills the hook's on_1b to on_3b.</t>
         </is>
       </c>
-      <c r="F62" s="5" t="inlineStr">
+      <c r="F66" s="5" t="inlineStr">
         <is>
           <t>Read gs.on_1b, gs.on_2b and gs.on_3b in mapWsState.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="46.5" customHeight="1" s="15">
-      <c r="A63" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B63" s="3" t="inlineStr">
-        <is>
-          <t>SIM-609</t>
-        </is>
-      </c>
-      <c r="C63" s="4" t="inlineStr">
-        <is>
-          <t>Raise on a wrong market or side in the line-movement series</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>line_movement_from_quotes swallows _side_columns' ValueError, so a wrong market or side gives a silent empty series. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E63" s="5" t="inlineStr">
-        <is>
-          <t>A wrong market or side raises.</t>
-        </is>
-      </c>
-      <c r="F63" s="5" t="inlineStr">
-        <is>
-          <t>Call _side_columns once before the loop.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="73.5" customHeight="1" s="15">
-      <c r="A64" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>SIM-599</t>
-        </is>
-      </c>
-      <c r="C64" s="4" t="inlineStr">
-        <is>
-          <t>Describe the slate card's odds field as it is</t>
-        </is>
-      </c>
-      <c r="D64" s="5" t="inlineStr">
-        <is>
-          <t>The route description (api/routes/games_slate.py) and the model (api/routes/games_models.py) call the field 'reserved for the Phase-6 odds-provider integration (SIM-405)'. The field is always None: the card's lines come from /api/betting/games/{pk}/card-odds. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="inlineStr">
-        <is>
-          <t>Both texts say that, with a fresh API snapshot (CLAUDE.md section 15).</t>
-        </is>
-      </c>
-      <c r="F64" s="5" t="inlineStr">
-        <is>
-          <t>Rewrite both texts; run scripts/export_openapi.py in the image and npm run gen:api.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="46.5" customHeight="1" s="15">
-      <c r="A65" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B65" s="3" t="inlineStr">
-        <is>
-          <t>SIM-600</t>
-        </is>
-      </c>
-      <c r="C65" s="4" t="inlineStr">
-        <is>
-          <t>Name the current state in the API's version and health strings</t>
-        </is>
-      </c>
-      <c r="D65" s="5" t="inlineStr">
-        <is>
-          <t>api/main.py carries the app version 0.1.0-phase7, "phase": "6" on /health and "6 - Frontend Build (in progress)" on /. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E65" s="5" t="inlineStr">
-        <is>
-          <t>The strings name the current state, or go.</t>
-        </is>
-      </c>
-      <c r="F65" s="5" t="inlineStr">
-        <is>
-          <t>Drop the phase keys and set the version from one constant.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="202" customHeight="1" s="15">
-      <c r="A66" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="inlineStr">
-        <is>
-          <t>SIM-634</t>
-        </is>
-      </c>
-      <c r="C66" s="4" t="inlineStr">
-        <is>
-          <t>Small fixes found by the documentation rebuild</t>
-        </is>
-      </c>
-      <c r="D66" s="5" t="inlineStr">
-        <is>
-          <t>(1) frontend/index.html links a favicon, /baseball.svg, that frontend/public/ does not hold: a 404 on every page. (2) /ready (api/main.py) writes a redis entry only on a failure, so a healthy Redis is missing from its checks. (3) Six nginx blocks (/health, /ready, /metrics, /docs, /redoc, /openapi.json) set their own Host header, which drops the inherited X-Real-IP and X-Forwarded-For. (4) Nothing deletes the simviz:* explorer cache keys after a nightly rebuild, so a key serves old data for up to 24 h. (5) 12 of the 32 DuckDB migrations do not record themselves in migration_history. (6) Three stale texts: api/state.py calls the situation engine a FAISS engine (it is a KD-tree); the Makefile's gen-secrets comment says a blank key is left alone (gen_secrets.py fills it); scripts/probes/manager_profile_recompute.py says the app must be stopped (the recompute runs beside the app since SIM-524). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E66" s="5" t="inlineStr">
-        <is>
-          <t>Each of the six is fixed or retired.</t>
-        </is>
-      </c>
-      <c r="F66" s="5" t="inlineStr">
-        <is>
-          <t>One small commit per area. For (5), record the missing numbers in one new migration rather than editing old files.</t>
         </is>
       </c>
     </row>
@@ -2610,60 +2610,187 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
+          <t>SIM-609</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>Raise on a wrong market or side in the line-movement series</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>line_movement_from_quotes swallows _side_columns' ValueError, so a wrong market or side gives a silent empty series. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>A wrong market or side raises.</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>Call _side_columns once before the loop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="73.5" customHeight="1" s="15">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>SIM-599</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Describe the slate card's odds field as it is</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>The route description (api/routes/games_slate.py) and the model (api/routes/games_models.py) call the field 'reserved for the Phase-6 odds-provider integration (SIM-405)'. The field is always None: the card's lines come from /api/betting/games/{pk}/card-odds. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>Both texts say that, with a fresh API snapshot (CLAUDE.md section 15).</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>Rewrite both texts; run scripts/export_openapi.py in the image and npm run gen:api.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="46.5" customHeight="1" s="15">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>SIM-600</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>Name the current state in the API's version and health strings</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>api/main.py carries the app version 0.1.0-phase7, "phase": "6" on /health and "6 - Frontend Build (in progress)" on /. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>The strings name the current state, or go.</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>Drop the phase keys and set the version from one constant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="202" customHeight="1" s="15">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>SIM-634</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>Small fixes found by the documentation rebuild</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>(1) frontend/index.html links a favicon, /baseball.svg, that frontend/public/ does not hold: a 404 on every page. (2) /ready (api/main.py) writes a redis entry only on a failure, so a healthy Redis is missing from its checks. (3) Six nginx blocks (/health, /ready, /metrics, /docs, /redoc, /openapi.json) set their own Host header, which drops the inherited X-Real-IP and X-Forwarded-For. (4) Nothing deletes the simviz:* explorer cache keys after a nightly rebuild, so a key serves old data for up to 24 h. (5) 12 of the 32 DuckDB migrations do not record themselves in migration_history. (6) Three stale texts: api/state.py calls the situation engine a FAISS engine (it is a KD-tree); the Makefile's gen-secrets comment says a blank key is left alone (gen_secrets.py fills it); scripts/probes/manager_profile_recompute.py says the app must be stopped (the recompute runs beside the app since SIM-524). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>Each of the six is fixed or retired.</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>One small commit per area. For (5), record the missing numbers in one new migration rather than editing old files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="46.5" customHeight="1" s="15">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
           <t>SIM-595</t>
         </is>
       </c>
-      <c r="C67" s="4" t="inlineStr">
+      <c r="C71" s="4" t="inlineStr">
         <is>
           <t>Fix the article in the what-if's ineligible-player message</t>
         </is>
       </c>
-      <c r="D67" s="5" t="inlineStr">
+      <c r="D71" s="5" t="inlineStr">
         <is>
           <t>whatif.apply_changes' message for an ineligible pinch hitter reads 'is not an bench hitter'. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
-      <c r="E67" s="5" t="inlineStr">
+      <c r="E71" s="5" t="inlineStr">
         <is>
           <t>Each label reads with its own article.</t>
         </is>
       </c>
-      <c r="F67" s="5" t="inlineStr">
+      <c r="F71" s="5" t="inlineStr">
         <is>
           <t>Put the article inside each label.</t>
         </is>
       </c>
     </row>
-    <row r="68" s="15"/>
-    <row r="69" s="15">
-      <c r="A69" s="7" t="inlineStr">
+    <row r="72" s="15"/>
+    <row r="73" s="15">
+      <c r="A73" s="7" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B69" s="8" t="inlineStr">
+      <c r="B73" s="8" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C69" s="9" t="inlineStr">
+      <c r="C73" s="9" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D69" s="12" t="inlineStr">
+      <c r="D73" s="12" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E69" s="10" t="inlineStr">
+      <c r="E73" s="10" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F69" s="11" t="n"/>
-    </row>
-    <row r="70" s="15"/>
+      <c r="F73" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>

<commit_message>
Delete the closed backlog row of the merge target in standardized units (SIM-606); record the merge
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -257,7 +257,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenTickets" displayName="OpenTickets" ref="A4:F14" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenTickets" displayName="OpenTickets" ref="A4:F13" headerRowCount="1">
   <autoFilter ref="A4:F14"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Priority"/>
@@ -560,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -650,7 +650,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1" s="15">
+    <row r="6" ht="114" customHeight="1" s="15">
       <c r="A6" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -658,31 +658,31 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>SIM-606</t>
+          <t>SIM-578</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Pick the small-mixture-component merge target in standardized units</t>
+          <t>Load a database NULL as NaN, not 0.0, in the baserunner, catcher, batter and manager engines</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>enforce_min_cluster_size runs before the standardization in the arsenal build, so spin rate (hundreds of rpm) decides the merge over velocity and movement. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The _v helpers of four engines read v or 0.0. A runner with no Savant row gets sprint speed 0 ft/s (still 20 ft/s after a 5-chance shrink, many deviations below the league's 27), so his speed score is about 0 against every measured runner. A runner who never tried reads 0% success; a NULL arm strength reads 0 mph; a manager-season with no bullpen-availability rows reads available_reliever_usage_rate near 0. The two steal engines already load NaN (the running-game work, SIM-531). Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>The merge measures the gap in standardized units.</t>
+          <t>Each of the four engines loads NULL as NaN, and its kernel or shrink handles a NaN feature. The nightly matrices are rebuilt.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Measure the gap over the mixture's feature_stds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="114" customHeight="1" s="15">
+          <t>Map None to NaN in each _v helper and add the features to each engine's NaN set, as the steal engines do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="127.5" customHeight="1" s="15">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -690,31 +690,31 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>SIM-578</t>
+          <t>SIM-577</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Load a database NULL as NaN, not 0.0, in the baserunner, catcher, batter and manager engines</t>
+          <t>Write all thirteen features in the extra-base runner's league-average row</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>The _v helpers of four engines read v or 0.0. A runner with no Savant row gets sprint speed 0 ft/s (still 20 ft/s after a 5-chance shrink, many deviations below the league's 27), so his speed score is about 0 against every measured runner. A runner who never tried reads 0% success; a NULL arm strength reads 0 mph; a manager-season with no bullpen-availability rows reads available_reliever_usage_rate near 0. The two steal engines already load NaN (the running-game work, SIM-531). Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The baserunner row of derived.league_averages holds extra_base_attempt_rate, extra_base_success_rate, sb_success_rate, sprint_speed and the Savant rate. The engine reads thirteen features, so the four per-situation attempt rates, stop_rate and the four per-situation success rates shrink toward 0.0. The matrix build loads the thin profiles, so the effect is large there: a 5-chance runner's first-to-third attempt rate reads 0.35 -&gt; 0.088. The error reaches the runner_adv matrix, which weights the advancement draws. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Each of the four engines loads NULL as NaN, and its kernel or shrink handles a NaN feature. The nightly matrices are rebuilt.</t>
+          <t>The runner's league row carries every engine feature, and a missing key reads as NaN. The nightly matrices are rebuilt.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Map None to NaN in each _v helper and add the features to each engine's NaN set, as the steal engines do.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="127.5" customHeight="1" s="15">
+          <t>Write the engine's thirteen feature keys in the computor's baserunner league row; read a missing key as NaN in similarity/engines/baserunner_similarity.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="114" customHeight="1" s="15">
       <c r="A8" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -722,27 +722,27 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>SIM-577</t>
+          <t>SIM-576</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Write all thirteen features in the extra-base runner's league-average row</t>
+          <t>Write the catcher engine's feature names in the catcher's league-average row</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>The baserunner row of derived.league_averages holds extra_base_attempt_rate, extra_base_success_rate, sb_success_rate, sprint_speed and the Savant rate. The engine reads thirteen features, so the four per-situation attempt rates, stop_rate and the four per-situation success rates shrink toward 0.0. The matrix build loads the thin profiles, so the effect is large there: a 5-chance runner's first-to-third attempt rate reads 0.35 -&gt; 0.088. The error reaches the runner_adv matrix, which weights the advancement draws. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The profile computor writes the catcher row of derived.league_averages with the keys framing_runs, blocking_runs and cs_rate. The catcher engine reads its eleven feature names with pj.get(f, 0.0) or 0.0, and only cs_rate matches. So the shrinkage pulls ten features toward 0.0: a constructed 300-pitch catcher reads pop time 1.95 -&gt; 1.857 s and arm strength 81 -&gt; 77.1 mph. The error reaches the catcher and catcher_throwing score matrices, which weight the steal and pickoff draws. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>The runner's league row carries every engine feature, and a missing key reads as NaN. The nightly matrices are rebuilt.</t>
+          <t>The catcher's league row carries every engine feature. A missing key reads as NaN, as the steal engines do. The nightly matrices are rebuilt.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Write the engine's thirteen feature keys in the computor's baserunner league row; read a missing key as NaN in similarity/engines/baserunner_similarity.py.</t>
+          <t>In pipeline/batch/profiles (the catcher league row), write the engine's eleven feature keys. In similarity/engines/catcher_similarity.py _load_league_averages, read a missing key as NaN.</t>
         </is>
       </c>
     </row>
@@ -754,31 +754,31 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>SIM-576</t>
+          <t>SIM-579</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Write the catcher engine's feature names in the catcher's league-average row</t>
+          <t>Select the pitcher's zone-take rate before the chase rate, so the two stay in feature order</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>The profile computor writes the catcher row of derived.league_averages with the keys framing_runs, blocking_runs and cs_rate. The catcher engine reads its eleven feature names with pj.get(f, 0.0) or 0.0, and only cs_rate matches. So the shrinkage pulls ten features toward 0.0: a constructed 300-pitch catcher reads pop time 1.95 -&gt; 1.857 s and arm strength 81 -&gt; 77.1 mph. The error reaches the catcher and catcher_throwing score matrices, which weight the steal and pickoff draws. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>In similarity/engines/pitcher_similarity.py _load_profiles, the SELECT returns chase_rate, zone_take_rate and the unpack names them zone_take_rate, chase_rate. So command_vec holds them in the opposite order to COMMAND_FEATURES and the league-average vector, and the shrinkage pulls each pitcher's chase rate toward the league's zone-take rate (weight 1 - alpha, at most 2.4% at 200 pitches). The kernel itself ignores the order. The error reaches the pitcher similarity matrix. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>The catcher's league row carries every engine feature. A missing key reads as NaN, as the steal engines do. The nightly matrices are rebuilt.</t>
+          <t>The SELECT order matches COMMAND_FEATURES, and a unit test pins it. The nightly matrices are rebuilt.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>In pipeline/batch/profiles (the catcher league row), write the engine's eleven feature keys. In similarity/engines/catcher_similarity.py _load_league_averages, read a missing key as NaN.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="114" customHeight="1" s="15">
+          <t>Select zone_take_rate before chase_rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="219.5" customHeight="1" s="15">
       <c r="A10" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -786,27 +786,27 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SIM-579</t>
+          <t>SIM-635</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Select the pitcher's zone-take rate before the chase rate, so the two stay in feature order</t>
+          <t>Export the pitch pool in pitch order, so the pitch-result draw's density weights stay the same between pool builds</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>In similarity/engines/pitcher_similarity.py _load_profiles, the SELECT returns chase_rate, zone_take_rate and the unpack names them zone_take_rate, chase_rate. So command_vec holds them in the opposite order to COMMAND_FEATURES and the league-average vector, and the shrinkage pulls each pitcher's chase rate toward the league's zone-take rate (weight 1 - alpha, at most 2.4% at 200 pitches). The kernel itself ignores the order. The error reaches the pitcher similarity matrix. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The pitch-result draw lowers the weight of a candidate pitch where the candidate set is crowded with similar pitches. It measures the crowding against 256 reference rows of the set (simulation/sampler/pitch_result.py:133-137). The draw picks the 256 rows by their POSITION in the set. Each set keeps the pool's stored order (simulation/sampler/pitch.py:271, a stable sort by cell). That order is not fixed. The pool insert reads a parallel scan of raw.pitches with no ORDER BY (pipeline/batch/profiles/pools.py:64-175). Both export scans have no ORDER BY either (pipeline/batch/artifacts/pitch_pool.py:36-39 and 77-83). So each pool build gives the draw other reference rows and other density weights. The nightly build rebuilds the current season's pool; a full rebuild rebuilds every season. Production runs the correction (SIM_PITCH_RESULT_SPLIT=1; SIM_RESULT_DENSITY_POWER defaults to 1.0). Two bundle builds from one DuckDB file already export the pool in one order; the order changes only between pool builds. Found by the arsenal row-order work (SIM-580, 2026-10-26); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>The SELECT order matches COMMAND_FEATURES, and a unit test pins it. The nightly matrices are rebuilt.</t>
+          <t>Two pool builds from the same data export the same pitch-pool rows in the same order. The density weights are then the same. A unit test pins the export order.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Select zone_take_rate before chase_rate.</t>
+          <t>Add ORDER BY pitch_id (the table's key) to both pitch-pool export scans. The arrays and the meta file must keep one shared order. The fix changes every density weight once; land it before the weight fit (SIM-548).</t>
         </is>
       </c>
     </row>
@@ -818,31 +818,31 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SIM-635</t>
+          <t>SIM-636</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Export the pitch pool in pitch order, so the pitch-result draw's density weights stay the same between pool builds</t>
+          <t>Export the batted-ball pool in pitch order, so the fielding draw's density weights stay the same between pool builds</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>The pitch-result draw lowers the weight of a candidate pitch where the candidate set is crowded with similar pitches. It measures the crowding against 256 reference rows of the set (simulation/sampler/pitch_result.py:133-137). The draw picks the 256 rows by their POSITION in the set. Each set keeps the pool's stored order (simulation/sampler/pitch.py:271, a stable sort by cell). That order is not fixed. The pool insert reads a parallel scan of raw.pitches with no ORDER BY (pipeline/batch/profiles/pools.py:64-175). Both export scans have no ORDER BY either (pipeline/batch/artifacts/pitch_pool.py:36-39 and 77-83). So each pool build gives the draw other reference rows and other density weights. The nightly build rebuilds the current season's pool; a full rebuild rebuilds every season. Production runs the correction (SIM_PITCH_RESULT_SPLIT=1; SIM_RESULT_DENSITY_POWER defaults to 1.0). Two bundle builds from one DuckDB file already export the pool in one order; the order changes only between pool builds. Found by the arsenal row-order work (SIM-580, 2026-10-26); the evidence is in its CHANGES.md entry.</t>
+          <t>The fielding draw lowers the weight of a candidate batted ball where the candidate set is crowded with similar balls. It measures the crowding against 256 reference rows of the set (simulation/sampler/fielding.py:612-636). A generator seeded on the set's first row, last row and size picks the rows by POSITION. The set keeps the batted-ball pool's stored order. That order is not fixed. The outcome-pool insert joins the pitch pool to a parallel scan of raw.pitches with no ORDER BY (pipeline/batch/profiles/pools.py:205-393). The export's array query and its meta COPY have no ORDER BY either (pipeline/batch/artifacts/battedball_pool.py:114-117 and 162-175). So each pool build gives other density weights. The simulated mix of singles, doubles and home runs then moves with no change in code or data. Production runs the correction (SIM_BB_BORN_SIGMA=1.0; SIM_BB_BORN_DENSITY_POWER defaults to 1.0). The weight fit names this correction as a lever it tunes (SIM-548), so the correction must be stable first. Found by the arsenal row-order work (SIM-580, 2026-10-26); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Two pool builds from the same data export the same pitch-pool rows in the same order. The density weights are then the same. A unit test pins the export order.</t>
+          <t>Two pool builds from the same data export the same batted-ball rows in the same order. The fielding draw's density weights are then the same. A unit test pins the export order.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Add ORDER BY pitch_id (the table's key) to both pitch-pool export scans. The arrays and the meta file must keep one shared order. The fix changes every density weight once; land it before the weight fit (SIM-548).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="219.5" customHeight="1" s="15">
+          <t>Add ORDER BY pitch_id to the array query and to the meta COPY of battedball_pool.py. The two must keep one shared order. The fix changes every born-ball density weight once. It can land in the same commit as the pitch pool's export order (SIM-635).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="127.5" customHeight="1" s="15">
       <c r="A12" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -850,31 +850,31 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>SIM-636</t>
+          <t>SIM-611</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Export the batted-ball pool in pitch order, so the fielding draw's density weights stay the same between pool builds</t>
+          <t>Owner decisions: four similarity design points</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>The fielding draw lowers the weight of a candidate batted ball where the candidate set is crowded with similar balls. It measures the crowding against 256 reference rows of the set (simulation/sampler/fielding.py:612-636). A generator seeded on the set's first row, last row and size picks the rows by POSITION. The set keeps the batted-ball pool's stored order. That order is not fixed. The outcome-pool insert joins the pitch pool to a parallel scan of raw.pitches with no ORDER BY (pipeline/batch/profiles/pools.py:205-393). The export's array query and its meta COPY have no ORDER BY either (pipeline/batch/artifacts/battedball_pool.py:114-117 and 162-175). So each pool build gives other density weights. The simulated mix of singles, doubles and home runs then moves with no change in code or data. Production runs the correction (SIM_BB_BORN_SIGMA=1.0; SIM_BB_BORN_DENSITY_POWER defaults to 1.0). The weight fit names this correction as a lever it tunes (SIM-548), so the correction must be stable first. Found by the arsenal row-order work (SIM-580, 2026-10-26); the evidence is in its CHANGES.md entry.</t>
+          <t>Not defects, design points for the owner. (1) The catcher's shrinkage prior is 15 called pitches, so alpha is at least 0.95 for every kept catcher (framing stabilizes near 1,500). (2) stop_rate is exactly one minus the overall attempt rate, so that rate counts twice in the runner's aggression distance. (3) The batter's xba / xslg and the manager's hit-and-run and double-switch rates read 0.0 for everyone and still hold their share of the kernel weight. (4) CLAUDE.md section 1 calls CLV 'the gold-standard metric'; the owner ruled on 2026-09-28 that the model is not judged by it. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Two pool builds from the same data export the same batted-ball rows in the same order. The fielding draw's density weights are then the same. A unit test pins the export order.</t>
+          <t>The owner rules on each point, and the code or CLAUDE.md follows.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Add ORDER BY pitch_id to the array query and to the meta COPY of battedball_pool.py. The two must keep one shared order. The fix changes every born-ball density weight once. It can land in the same commit as the pitch pool's export order (SIM-635).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="127.5" customHeight="1" s="15">
+          <t>Raise the catcher prior; drop stop_rate; drop the all-zero features; rewrite CLAUDE.md section 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="87" customHeight="1" s="15">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -882,31 +882,31 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>SIM-611</t>
+          <t>SIM-587</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Owner decisions: four similarity design points</t>
+          <t>Decide which calibration values the draws use, and make the code follow</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Not defects, design points for the owner. (1) The catcher's shrinkage prior is 15 called pitches, so alpha is at least 0.95 for every kept catcher (framing stabilizes near 1,500). (2) stop_rate is exactly one minus the overall attempt rate, so that rate counts twice in the runner's aggression distance. (3) The batter's xba / xslg and the manager's hit-and-run and double-switch rates read 0.0 for everyone and still hold their share of the kernel weight. (4) CLAUDE.md section 1 calls CLV 'the gold-standard metric'; the owner ruled on 2026-09-28 that the model is not judged by it. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>similarity/calibration/pitcher.py fits sigma_command and eb_n_prior_pitcher, and no code reads either, so the pitcher engine keeps RBF_SIGMA_COMMAND 1.0453 and EB_N_PRIOR 5. More broadly, the nightly actor matrices apply no calibration report (build_actor_sim_matrices): make calibrate changes only the API's engines. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>The owner rules on each point, and the code or CLAUDE.md follows.</t>
+          <t>The owner decides which values the draws use, and the code and the docs follow.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Raise the catcher prior; drop stop_rate; drop the all-zero features; rewrite CLAUDE.md section 1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="87" customHeight="1" s="15">
+          <t>Read both fields in apply_calibration and apply /data/calibration.json in the matrix build; or document the module defaults as the draws' values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="73.5" customHeight="1" s="15">
       <c r="A14" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -914,31 +914,31 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>SIM-587</t>
+          <t>SIM-583</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Decide which calibration values the draws use, and make the code follow</t>
+          <t>Keep the calibrated win probability strictly between 0 and 1</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>similarity/calibration/pitcher.py fits sigma_command and eb_n_prior_pitcher, and no code reads either, so the pitcher engine keeps RBF_SIGMA_COMMAND 1.0453 and EB_N_PRIOR 5. More broadly, the nightly actor matrices apply no calibration report (build_actor_sim_matrices): make calibrate changes only the API's engines. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>build_validation_report fits the reliability curve with min_bin_count=1, so a bin of two games can map 0.75 to 1.0. Example: the curve [[0,0],[0.45,0.44],[0.55,0.56],[0.73,1.0],[1,1]] and home_win_pct 0.75 at n = 100 give home 1.0, away 0.0 and an interval of zero width. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>The owner decides which values the draws use, and the code and the docs follow.</t>
+          <t>No calibrated probability is 0.0 or 1.0, and a unit test feeds the curve above.</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Read both fields in apply_calibration and apply /data/calibration.json in the matrix build; or document the module defaults as the draws' values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="73.5" customHeight="1" s="15">
+          <t>Fit the curve with a min_bin_count near 30, or clamp the mapped probability to [eps, 1 - eps].</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="127.5" customHeight="1" s="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
           <t>P2</t>
@@ -946,59 +946,59 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>SIM-583</t>
+          <t>SIM-584</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Keep the calibrated win probability strictly between 0 and 1</t>
+          <t>Stamp the accuracy report with the bundle the run read, not the live link</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>build_validation_report fits the reliability curve with min_bin_count=1, so a bin of two games can map 0.75 to 1.0. Example: the curve [[0,0],[0.45,0.44],[0.55,0.56],[0.73,1.0],[1,1]] and home_win_pct 0.75 at n = 100 give home 1.0, away 0.0 and an interval of zero width. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/accuracy/selection.py bundle_provenance reads the manifest times under BASEBALL_PLAY_POOL_DIR/engine_artifacts (the live link). The factory reads BASEBALL_ENGINE_ARTIFACT_DIR when it is set (simulation/production_factory.py). Seen on 2026-10-20: two runs on the same pinned bundle, before and after the nightly rebuild, carry different manifest_mtimes and identical records, so pair_accuracy.py refuses to pair them; two runs on different pinned bundles on one day would pair. The weight fit (SIM-548) pairs these reports. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>No calibrated probability is 0.0 or 1.0, and a unit test feeds the curve above.</t>
+          <t>The stamp names the bundle the run read, and a test pins the pinned-directory case.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Fit the curve with a min_bin_count near 30, or clamp the mapped probability to [eps, 1 - eps].</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="127.5" customHeight="1" s="15">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Read the pinned directory first, as the factory does.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="81" customHeight="1" s="15">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>SIM-584</t>
+          <t>SIM-547</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Stamp the accuracy report with the bundle the run read, not the live link</t>
+          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>scripts/accuracy/selection.py bundle_provenance reads the manifest times under BASEBALL_PLAY_POOL_DIR/engine_artifacts (the live link). The factory reads BASEBALL_ENGINE_ARTIFACT_DIR when it is set (simulation/production_factory.py). Seen on 2026-10-20: two runs on the same pinned bundle, before and after the nightly rebuild, carry different manifest_mtimes and identical records, so pair_accuracy.py refuses to pair them; two runs on different pinned bundles on one day would pair. The weight fit (SIM-548) pairs these reports. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>The stamp names the bundle the run read, and a test pins the pinned-directory case.</t>
+          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Read the pinned directory first, as the factory does.</t>
+          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/probes/manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
         </is>
       </c>
     </row>
@@ -1010,27 +1010,27 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>SIM-547</t>
+          <t>SIM-526</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Manager-draw follow-ons: the pen on the API, the preview-game fallbacks, the pen order and a finer rest fit</t>
+          <t>Turn on the catcher pitch-receiving factor</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>The pitching change now follows each team's real manager and real bullpen (flipped on 2026-09-13). Five small gaps remain. The game-state API response does not show the pen or where it came from. A game that has not started yet has no manager id and no bullpen listing, so the simulator treats it as an average manager with an invented pen. The pen lists the relievers who sat out today at the back, which the fallback pick reads as 'the closer is first'. The entering arm pitched yesterday 27% of the time against 16.5% in the real data, and its early-inning role reads 0.37 against 0.31.</t>
+          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>The API's live game state carries each side's pen and its source (box or synthetic). A preview game takes the team's most recent Final game's manager and its most recent listing with a staleness flag. The pen order no longer encodes who sat out today. A rest bandwidth of 0.25 days is measured with the manager probe and adopted if it brings the entering arm's 'pitched yesterday' share within 5 points of the pool's without breaking the other reliever reads.</t>
+          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Expose ResolvedLineup.bullpen / bullpen_source on LiveGameStateResponse (api/routes/games.py, api/schemas.py). In simulation/lineup_resolver.py, fall back to the team's latest Final game for the manager id (raw.games) and the listing (raw.game_bullpen) when the game's own are missing, and flag the staleness in bullpen_source. In pipeline/bullpen_usage.pen_from_listing, order the pen by the listing's own order (or by rest) instead of pitched-first. Run scripts/probes/manager_probe.py with rest=0.25 (and 0.35) against the r_base / r_rest05 arms and read the reliever line.</t>
+          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
         </is>
       </c>
     </row>
@@ -1042,27 +1042,27 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>SIM-526</t>
+          <t>SIM-556</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Turn on the catcher pitch-receiving factor</t>
+          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
+          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/probes/steal_weight_volume_probe.py with its records (docs/audit/records/steal_weight_volume_probe_2025.* and _2026.*; the arrays in results/steal_weight_volume/). Filed P3 by the owner on 2026-10-01.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
+          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
+          <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/probes/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
         </is>
       </c>
     </row>
@@ -1074,31 +1074,31 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>SIM-556</t>
+          <t>SIM-574</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Keep the number of steal attempts right when the steal draw weighs rows by how much their players resemble the live ones (the balance weight)</t>
+          <t>Make each SIM_* flag's code default equal its production value, or record why it differs</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>The simulator decides a steal by drawing one real past pitch from a pool. It weighs each candidate row by how much its runner, pitcher and catcher resemble the players in the game (the look-alike weights). Those weights lower the number of steal attempts. Base stealers are rare and resemble few other runners, so their rows are drawn less often than their share of the pool, and those rows hold most of the attempts. On a replay of 74,296 real pitches of 2026 the draw reads 1.225 steals per 100 chances against 1.462 in the pool (16% low); 2025 reads 14% low. The runner weight carries three quarters of the loss, the pitcher weight a fifth, the catcher weight the rest. This matches the two red steal-attempt bands of the acceptance lanes of 2026-09-21 and 2026-09-22 (-9.1% at second base, -17.9% at third). The draw's bell curve on the score margin has the same flaw the other way and adds 4%. A stronger weight alone does not repair it: at strengths 4 / 4 / 2 the total is 22% low, and at 12 / 12 / 2 it is 8.5% low with much worse odds per pitch. It is not the rows with no score and not the engines' sample-confidence multiplier (each moves the total by under half a point). Finding and evidence: docs/audit/2026-09-30-steal-weight-volume-finding.md and scripts/probes/steal_weight_volume_probe.py with its records (docs/audit/records/steal_weight_volume_probe_2025.* and _2026.*; the arrays in results/steal_weight_volume/). Filed P3 by the owner on 2026-10-01.</t>
+          <t>The simulator reads its switches and weights from SIM_* environment flags. Each flag has a default in the code (the value an unset flag reads) and a production value set in the app service of docker-compose.yml. They differ for 24 of the flags compose sets (measured 2026-10-20): for example the pitch-draw cell index is off in code and on in production, and the fence stage, the fielding class filter and the manager draw are the same. So a script, a probe or a test that forgets one flag runs a different simulator from production, silently. The registry of the flags (simulation/flags.py, the code clean-up SIM-493) now lists every default in one table, which makes the gap visible but does not close it.</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>The steal draw carries a balance weight on its three look-alike weights and on the score-margin curve, switched on in production. The pool replayed through each weight alone keeps between 0.98 and 1.02 of the pool's steal attempts, and the nightly matrix build prints that check. On the replay of real pitches the draw reads within 1% of the pool's rate at every strength tried (1 / 1 / 1, 4 / 4 / 2, 12 / 12 / 2), and the per-runner match between expected and real steals does not fall (0.710 today on 2026, 0.743 with the fix on the replay). One 45 x 130 acceptance lane reads the two steal-attempt bands inside their floors and the safe-share band still green. The owner has a recommendation on the strength of the runner weight in the steal draw: with the balance, 4 / 4 / 2 is the best row tested (base stealers 2.36 per 100 against a real 3.02; 1.78 at strength 1).</t>
+          <t>For every registered flag the code default equals the compose value, or the registry row says in one line why it differs (for example: the unit lane's byte-identical state). The unit lane's own pins in tests/conftest.py still hold its state. The fingerprint (scripts/behaviour_fingerprint.py) of production is unchanged, because compose already sets the production values.</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>In simulation/full_pool_sampler.py, add one number per player-season to the steal draw's weight (the balance weight). Fit it when the sampler loads, from the score matrix and the pool's row counts only (it never reads the attempted flag), by the alternating rescale (Sinkhorn): each player's rows must receive, over a season of draws, the share of the draw they hold. Fit it with only the simulated season's player-seasons as the live players and over the rows that season can draw (fitted on the whole pool it reads 5% low on 2026). Multiply it in _steal_actor_factor; cap it at 20; give a row with no score the mean scored weight at every power. Fit the same balance on the score-margin curve inside each count cell (eleven weights). One switch, SIM_STEAL_BALANCE, landing on with the cheap gates (the unit and regression lanes, a ten-game smoke of the steal channels), then the lane. Early in a season, add the season before to the live set (threshold not tested). Second step: run the same pool-replay check on the look-alike weights of the other draws (pitch, fielding, advancement, pitching change); the lane's red walks (+4.0%) and hit-by-pitch (+6.7%) bands are untested candidates. Reference fit: balance_weight_live in scripts/probes/steal_weight_volume_probe.py; the design is section 3 of the finding.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="81" customHeight="1" s="15">
+          <t>Owner decision first: should an unset flag mean production or off? If production: change each default in simulation/flags.py to the compose value, keep tests/conftest.py's pins for the unit lane, and add a registry test that the defaults equal compose. If off: add the reason column to the registry and a test that compose sets every flag whose default differs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="73.5" customHeight="1" s="15">
       <c r="A20" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1106,27 +1106,27 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>SIM-574</t>
+          <t>SIM-608</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Make each SIM_* flag's code default equal its production value, or record why it differs</t>
+          <t>Store a price that returns to an earlier value</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>The simulator reads its switches and weights from SIM_* environment flags. Each flag has a default in the code (the value an unset flag reads) and a production value set in the app service of docker-compose.yml. They differ for 24 of the flags compose sets (measured 2026-10-20): for example the pitch-draw cell index is off in code and on in production, and the fence stage, the fielding class filter and the manager draw are the same. So a script, a probe or a test that forgets one flag runs a different simulator from production, silently. The registry of the flags (simulation/flags.py, the code clean-up SIM-493) now lists every default in one table, which makes the gap visible but does not close it.</t>
+          <t>The odds writer dedups on a hash with no time (ON CONFLICT (game_pk, source, odds_hash)), so -110 at t0, -120 at t1, -110 at t2 closes the series at -120. Read from the code, not checked against stored data. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>For every registered flag the code default equals the compose value, or the registry row says in one line why it differs (for example: the unit lane's byte-identical state). The unit lane's own pins in tests/conftest.py still hold its state. The fingerprint (scripts/behaviour_fingerprint.py) of production is unchanged, because compose already sets the production values.</t>
+          <t>A return to an earlier price is stored, and the series closes on the last price.</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Owner decision first: should an unset flag mean production or off? If production: change each default in simulation/flags.py to the compose value, keep tests/conftest.py's pins for the unit lane, and add a registry test that the defaults equal compose. If off: add the reason column to the registry and a test that compose sets every flag whose default differs.</t>
+          <t>Dedup only against the latest row of the same game, source, book, market and line type.</t>
         </is>
       </c>
     </row>
@@ -1138,31 +1138,31 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>SIM-608</t>
+          <t>SIM-607</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Store a price that returns to an earlier value</t>
+          <t>Read the line-movement direction book by book</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>The odds writer dedups on a hash with no time (ON CONFLICT (game_pk, source, odds_hash)), so -110 at t0, -120 at t1, -110 at t2 closes the series at -120. Read from the code, not checked against stored data. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>betting/line_movement.py _net_direction pools every book, so the first and last quotes can come from two books: (t1, bp:1, -110/-110) and (t2, bp:2, -130/+110) give direction 'toward' and a CLV, though neither book moved. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>A return to an earlier price is stored, and the series closes on the last price.</t>
+          <t>The direction is each book's own, then aggregated.</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Dedup only against the latest row of the same game, source, book, market and line type.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="73.5" customHeight="1" s="15">
+          <t>Compute the direction per book, then aggregate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="132" customHeight="1" s="15">
       <c r="A22" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1170,31 +1170,31 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>SIM-607</t>
+          <t>SIM-625</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Read the line-movement direction book by book</t>
+          <t>Capture the opening lines every day</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>betting/line_movement.py _net_direction pools every book, so the first and last quotes can come from two books: (t1, bp:1, -110/-110) and (t2, bp:2, -130/+110) give direction 'toward' and a CLV, though neither book moved. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>No scheduled job captures the opening lines. Nothing calls schedule_opening_line_job (pipeline/etl/opening_line_job.py), and the nightly closing-lines job (scripts/nightly_closing_lines.sh, 10:30 UTC) passes --line-types closing only. The venue backfill (schedule_venue_backfill_job) has no caller either. BettingPros serves the opener after the fact, so scripts/load_historical_odds.py (its default line types are opening and closing) recovers the missing rows: nothing is lost for good. The line-movement page reads the opening-to-closing series. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>The direction is each book's own, then aggregated.</t>
+          <t>Each night's odds run stores the opening rows of the games it loads, and the venue backfill either runs on a schedule or is retired.</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Compute the direction per book, then aggregate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="132" customHeight="1" s="15">
+          <t>Pass --line-types opening closing in scripts/nightly_closing_lines.sh. Then retire opening_line_job.py, or give it a scheduler entry; decide the venue backfill the same way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="60" customHeight="1" s="15">
       <c r="A23" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1202,31 +1202,31 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>SIM-625</t>
+          <t>SIM-586</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Capture the opening lines every day</t>
+          <t>Ask the schedule only for game types raw.games accepts</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>No scheduled job captures the opening lines. Nothing calls schedule_opening_line_job (pipeline/etl/opening_line_job.py), and the nightly closing-lines job (scripts/nightly_closing_lines.sh, 10:30 UTC) passes --line-types closing only. The venue backfill (schedule_venue_backfill_job) has no caller either. BettingPros serves the opener after the fact, so scripts/load_historical_odds.py (its default line types are opening and closing) recovers the missing rows: nothing is lost for good. The line-movement page reads the opening-to-closing series. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>GAME_TYPES (pipeline/live/ingestion/constants.py) is R F D L W C P; the CHECK on raw.games allows R P S A D F L W. A game of type C on the slate fails its upsert. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Each night's odds run stores the opening rows of the games it loads, and the venue backfill either runs on a schedule or is retired.</t>
+          <t>The live pipeline's game types and the table's CHECK agree, and a unit test compares them.</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Pass --line-types opening closing in scripts/nightly_closing_lines.sh. Then retire opening_line_job.py, or give it a scheduler entry; decide the venue backfill the same way.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="60" customHeight="1" s="15">
+          <t>Drop C from GAME_TYPES, or widen the CHECK with a migration if type C games should load.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="190.5" customHeight="1" s="15">
       <c r="A24" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1234,31 +1234,31 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>SIM-586</t>
+          <t>SIM-639</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Ask the schedule only for game types raw.games accepts</t>
+          <t>Fail the profile step when an arsenal-fit worker crashes</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>GAME_TYPES (pipeline/live/ingestion/constants.py) is R F D L W C P; the CHECK on raw.games allows R P S A D F L W. A game of type C on the slate fails its upsert. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The profile computor fits the pitcher arsenals in a process pool (the ProcessPoolExecutor loop of _compute_pitcher_profiles, pipeline/batch/profiles/pitcher.py, at the 'GMM worker chunk crashed' log line). When one worker dies (the random segfault class, CLAUDE.md section 2a), the pool breaks and every unfinished chunk raises. The computor logs the error and marks every pitcher of those chunks below the minimum sample (_flush_gmm_results in pipeline/batch/profiles/gmm.py). Those pitchers keep the placeholder model. They drop out of the pitcher engine and its score matrix. The step then exits 0, so the nightly's retry wrapper (scripts/with_retry.sh, three attempts) does not run it again. With one chunk per worker, one death can drop most pitchers of the season. Two builds of the same data then differ on a crash day. Found by the arsenal row-order work (SIM-580, 2026-10-26); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>The live pipeline's game types and the table's CHECK agree, and a unit test compares them.</t>
+          <t>A crashed worker chunk makes the profile step exit non-zero, and the nightly's retry wrapper runs it again. A unit test whose worker dies of a real segfault proves the non-zero exit and the 'Fatal Python error' line in the step's output. No pitcher with enough clean pitches is marked below the minimum sample because of a crash.</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Drop C from GAME_TYPES, or widen the CHECK with a migration if type C games should load.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="190.5" customHeight="1" s="15">
+          <t>Re-raise after the computor logs a crashed chunk or a broken pool, so the step exits non-zero. Keep the per-pitcher fallback only for a fit that fails on its own data (a model of None). A worker that segfaults prints nothing today, because no process turns faulthandler on. The re-raise alone exits 1 with no 'Fatal Python error' line, and with_retry.sh then stops. So start the pool with initializer=faulthandler.enable: a worker's segfault then writes the line, and the wrapper retries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="114" customHeight="1" s="15">
       <c r="A25" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1266,31 +1266,31 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>SIM-639</t>
+          <t>SIM-582</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Fail the profile step when an arsenal-fit worker crashes</t>
+          <t>Add last_seen_at to the two odds archive tables, so the retirement copy fits again</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>The profile computor fits the pitcher arsenals in a process pool (the ProcessPoolExecutor loop of _compute_pitcher_profiles, pipeline/batch/profiles/pitcher.py, at the 'GMM worker chunk crashed' log line). When one worker dies (the random segfault class, CLAUDE.md section 2a), the pool breaks and every unfinished chunk raises. The computor logs the error and marks every pitcher of those chunks below the minimum sample (_flush_gmm_results in pipeline/batch/profiles/gmm.py). Those pitchers keep the placeholder model. They drop out of the pitcher engine and its score matrix. The step then exits 0, so the nightly's retry wrapper (scripts/with_retry.sh, three attempts) does not run it again. With one chunk per worker, one death can drop most pitchers of the season. Two builds of the same data then differ on a crash day. Found by the arsenal row-order work (SIM-580, 2026-10-26); the evidence is in its CHANGES.md entry.</t>
+          <t>Migration 0029 added last_seen_at to raw.game_odds and raw.prop_odds and not to their archives (raw.game_odds_archive, raw.prop_odds_archive, migration 0028). The retirement script copies rows with INSERT ... SELECT *, which needs the same columns in the same order, so the next retirement fails. The integration test test_schema_migrations.py::test_sim555_stamp_indexes_and_archives reds on master fe81d79 and on the clean-up branch for this reason. Found by the code clean-up (SIM-493, the integration pass, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>A crashed worker chunk makes the profile step exit non-zero, and the nightly's retry wrapper runs it again. A unit test whose worker dies of a real segfault proves the non-zero exit and the 'Fatal Python error' line in the step's output. No pitcher with enough clean pitches is marked below the minimum sample because of a crash.</t>
+          <t>Both archives carry last_seen_at in the live table's position, the integration test passes, and a retirement run copies a row.</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Re-raise after the computor logs a crashed chunk or a broken pool, so the step exits non-zero. Keep the per-pitcher fallback only for a fit that fails on its own data (a model of None). A worker that segfaults prints nothing today, because no process turns faulthandler on. The re-raise alone exits 1 with no 'Fatal Python error' line, and with_retry.sh then stops. So start the pool with initializer=faulthandler.enable: a worker's segfault then writes the line, and the wrapper retries.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="114" customHeight="1" s="15">
+          <t>A new Alembic migration adds last_seen_at to both archives (nullable, so the copied rows keep their value), placed after book_line_at to match the live tables; check the column order with the test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="87" customHeight="1" s="15">
       <c r="A26" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1298,31 +1298,31 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>SIM-582</t>
+          <t>SIM-581</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Add last_seen_at to the two odds archive tables, so the retirement copy fits again</t>
+          <t>Name only real tests in the nightly acceptance lane's required roster</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Migration 0029 added last_seen_at to raw.game_odds and raw.prop_odds and not to their archives (raw.game_odds_archive, raw.prop_odds_archive, migration 0028). The retirement script copies rows with INSERT ... SELECT *, which needs the same columns in the same order, so the next retirement fails. The integration test test_schema_migrations.py::test_sim555_stamp_indexes_and_archives reds on master fe81d79 and on the clean-up branch for this reason. Found by the code clean-up (SIM-493, the integration pass, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The REQUIRED roster of .github/workflows/acceptance-nightly.yml lists test_full_pool_out_advancement_runs_sim450, test_full_pool_steal_decision_runs_sim450 and test_reach_on_error_band_sim450. No test of those names exists, and the roster step fails when a required name did not run. So the nightly lane reds on every run, whatever the bands read. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Both archives carry last_seen_at in the live table's position, the integration test passes, and a retirement run copies a row.</t>
+          <t>The roster names only real tests, and one nightly run passes its roster step.</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>A new Alembic migration adds last_seen_at to both archives (nullable, so the copied rows keep their value), placed after book_line_at to match the live tables; check the column order with the test.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="87" customHeight="1" s="15">
+          <t>Delete the three names, or name the tests that took their place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="118" customHeight="1" s="15">
       <c r="A27" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1330,31 +1330,31 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>SIM-581</t>
+          <t>SIM-633</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Name only real tests in the nightly acceptance lane's required roster</t>
+          <t>Make the test targets run what their names say</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>The REQUIRED roster of .github/workflows/acceptance-nightly.yml lists test_full_pool_out_advancement_runs_sim450, test_full_pool_steal_decision_runs_sim450 and test_reach_on_error_band_sim450. No test of those names exists, and the roster step fails when a required name did not run. So the nightly lane reds on every run, whatever the bands read. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>make test-unit passes no -m "not slow", so it runs the slow tests at the 30 s timeout; CI's unit job excludes them. make test-integration runs in the app container, which has no Docker socket (only the scheduler mounts it), so testcontainers cannot start and every integration test skips. The games input of acceptance-nightly.yml says "max 12" and defaults to 12, but the balanced set has 45 games (beside SIM-581, the roster). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>The roster names only real tests, and one nightly run passes its roster step.</t>
+          <t>make test-unit matches CI's unit job; make test-integration runs the integration lane or says it needs host Python; the workflow input describes the 45-game set.</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Delete the three names, or name the tests that took their place.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="118" customHeight="1" s="15">
+          <t>Add -m "not slow" to test-unit and a test-slow target. Run the integration lane on host Python, as docs/technical/tests.md describes. Fix the input's text and default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="90" customHeight="1" s="15">
       <c r="A28" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1362,31 +1362,31 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>SIM-633</t>
+          <t>SIM-626</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Make the test targets run what their names say</t>
+          <t>Point the GitHub workflows at master</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>make test-unit passes no -m "not slow", so it runs the slow tests at the 30 s timeout; CI's unit job excludes them. make test-integration runs in the app container, which has no Docker socket (only the scheduler mounts it), so testcontainers cannot start and every integration test skips. The games input of acceptance-nightly.yml says "max 12" and defaults to 12, but the balanced set has 45 games (beside SIM-581, the roster). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>docker-release.yml and frontend-release.yml run on a push to main (and on a published release), and the pull_request trigger of ci.yml lists main. The default branch is master, so a push never runs the two release workflows, and a pull request into master gets no pull-request run of CI (the push run still happens). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>make test-unit matches CI's unit job; make test-integration runs the integration lane or says it needs host Python; the workflow input describes the 45-game set.</t>
+          <t>A push to master runs both release workflows (or the owner retires them), and a pull request into master runs CI.</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Add -m "not slow" to test-unit and a test-slow target. Run the integration lane on host Python, as docs/technical/tests.md describes. Fix the input's text and default.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="90" customHeight="1" s="15">
+          <t>Replace main with master in the three triggers, and in the trigger comment at the head of ci.yml.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="73.5" customHeight="1" s="15">
       <c r="A29" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1394,27 +1394,27 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>SIM-626</t>
+          <t>SIM-619</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Point the GitHub workflows at master</t>
+          <t>Run the batch-runner stress test in a CI job</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>docker-release.yml and frontend-release.yml run on a push to main (and on a published release), and the pull_request trigger of ci.yml lists main. The default branch is master, so a push never runs the two release workflows, and a pull request into master gets no pull-request run of CI (the push run still happens). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>tests/integration/test_batch_runner_stress.py carries only the slow marker. The CI slow lane runs tests/unit -m slow; the weekly integration lane and make test-integration select -m integration; the e2e job runs one file. No job runs it. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>A push to master runs both release workflows (or the owner retires them), and a pull request into master runs CI.</t>
+          <t>One lane runs it.</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Replace main with master in the three triggers, and in the trigger comment at the head of ci.yml.</t>
+          <t>Mark it integration, or add its path to the slow lane.</t>
         </is>
       </c>
     </row>
@@ -1426,31 +1426,31 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>SIM-619</t>
+          <t>SIM-602</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Run the batch-runner stress test in a CI job</t>
+          <t>Make two API tests check what their names say</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>tests/integration/test_batch_runner_stress.py carries only the slow marker. The CI slow lane runs tests/unit -m slow; the weekly integration lane and make test-integration select -m integration; the e2e job runs one file. No job runs it. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>tests/unit/test_api_betting.py test_clv_snapshot_returns_only_series_with_clv makes a GET and asserts nothing. tests/unit/test_api_games_plays.py test_simulate_ok_without_duckdb_then_plays_404 never requests /plays. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>One lane runs it.</t>
+          <t>Each test asserts what its name says.</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Mark it integration, or add its path to the slow lane.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="73.5" customHeight="1" s="15">
+          <t>Add the assertions (the CLV series' filter; /plays answers 503 with no replay store), then rename the second test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="87" customHeight="1" s="15">
       <c r="A31" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1458,31 +1458,31 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>SIM-602</t>
+          <t>SIM-601</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Make two API tests check what their names say</t>
+          <t>Make the Playwright smoke tests pass while the live app runs</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>tests/unit/test_api_betting.py test_clv_snapshot_returns_only_series_with_clv makes a GET and asserts nothing. tests/unit/test_api_games_plays.py test_simulate_ok_without_duckdb_then_plays_404 never requests /plays. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>frontend/e2e/smoke.spec.ts (three specs) fail on the owner's host: a request the test does not mock goes through the preview server's proxy to localhost:8000, the live app answers 401 and the page shows the login. With API_TARGET=http://127.0.0.1:9 all 21 tests pass; CI has no backend, so CI passes. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Each test asserts what its name says.</t>
+          <t>The e2e suite passes with the live app running.</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Add the assertions (the CLV series' filter; /plays answers 503 with no replay store), then rename the second test.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="87" customHeight="1" s="15">
+          <t>Set API_TARGET to a closed port in playwright.config.ts's webServer.env, or end each spec with a catch-all **/api/** route that answers 404.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="104" customHeight="1" s="15">
       <c r="A32" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1490,31 +1490,31 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>SIM-601</t>
+          <t>SIM-630</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Make the Playwright smoke tests pass while the live app runs</t>
+          <t>Bring the Postgres schema file up to the migrations</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>frontend/e2e/smoke.spec.ts (three specs) fail on the owner's host: a request the test does not mock goes through the preview server's proxy to localhost:8000, the live app answers 401 and the page shows the login. With API_TARGET=http://127.0.0.1:9 all 21 tests pass; CI has no backend, so CI passes. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>db/schemas/01_postgres_schema.sql lags the Alembic migrations. It has no raw.savant_pitch_tracking (0020), no raw.game_bullpen (0025), none of the 0029 columns (raw.game_lineups.published_at, last_seen_at on the odds tables, the run-job columns) and none of the 0030 columns of sim.sim_runs (start_at_bat and the rest). At least eight unit tests read the file to check a schema fact. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>The e2e suite passes with the live app running.</t>
+          <t>The file matches the schema that alembic upgrade head builds, and a test holds the two equal; or the file is retired and the tests read the migrations.</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Set API_TARGET to a closed port in playwright.config.ts's webServer.env, or end each spec with a catch-all **/api/** route that answers 404.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="104" customHeight="1" s="15">
+          <t>Regenerate the file from a migrated database (pg_dump --schema-only), or retire it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="87" customHeight="1" s="15">
       <c r="A33" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1522,31 +1522,31 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>SIM-630</t>
+          <t>SIM-585</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Bring the Postgres schema file up to the migrations</t>
+          <t>Refuse CORS_ORIGINS=* while the API sends credentials</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>db/schemas/01_postgres_schema.sql lags the Alembic migrations. It has no raw.savant_pitch_tracking (0020), no raw.game_bullpen (0025), none of the 0029 columns (raw.game_lineups.published_at, last_seen_at on the odds tables, the run-job columns) and none of the 0030 columns of sim.sim_runs (start_at_bat and the rest). At least eight unit tests read the file to check a schema fact. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>api/main.py sets allow_credentials=True for every origin list, and resolve_cors_origins (api/auth.py) returns ['*'] when an operator sets CORS_ORIGINS=*. Starlette then echoes the caller's Origin on a request with a cookie, so any site can read the API with the user's login. Production sets neither variable today, so the defect is latent. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>The file matches the schema that alembic upgrade head builds, and a test holds the two equal; or the file is retired and the tests read the migrations.</t>
+          <t>CORS_ORIGINS=* either fails the boot or turns credentials off, and a unit test pins it.</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Regenerate the file from a migrated database (pg_dump --schema-only), or retire it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="87" customHeight="1" s="15">
+          <t>Refuse '*' in resolve_cors_origins while credentials are on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="160" customHeight="1" s="15">
       <c r="A34" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1554,31 +1554,31 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>SIM-585</t>
+          <t>SIM-632</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Refuse CORS_ORIGINS=* while the API sends credentials</t>
+          <t>Give the backup path one name, and correct the staging and production templates</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>api/main.py sets allow_credentials=True for every origin list, and resolve_cors_origins (api/auth.py) returns ['*'] when an operator sets CORS_ORIGINS=*. Starlette then echoes the caller's Origin on a request with a cookie, so any site can read the API with the user's login. Production sets neither variable today, so the defect is latent. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The app reads BACKUPS_ROOT (api/routes/metrics.py, docker-compose.yml) while the backup jobs read BACKUP_ROOT (pipeline/backup/data_stores.py, pipeline/backup/offsite.py, db/backup/pg_backup.sh). Both default to /backups, so the age gauges work today; a value set under one name alone splits them. Both env templates set LIVE_PIPELINE_ENABLED=true, which makes the app a second publisher beside the live service. .env.production.example sets ODDS_PROVIDER=theoddsapi, which no provider registers. The templates also carry seven keys no app code reads: WORKERS, SIM_MAX_WORKERS, ODDS_PROVIDER_API_KEY, ODDS_API_BASE, ASYNC_DB_DSN, MLB_API_BASE and PROMETHEUS_PUSHGATEWAY. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>CORS_ORIGINS=* either fails the boot or turns credentials off, and a unit test pins it.</t>
+          <t>One variable names the backup root, and the templates hold only keys the code reads, with values that start the stack.</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Refuse '*' in resolve_cors_origins while credentials are on.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="160" customHeight="1" s="15">
+          <t>Rename the app's variable to BACKUP_ROOT. Rewrite the two templates from .env.example.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="219.5" customHeight="1" s="15">
       <c r="A35" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1586,31 +1586,31 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>SIM-632</t>
+          <t>SIM-637</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Give the backup path one name, and correct the staging and production templates</t>
+          <t>Pair consecutive seasons in the batter's and the runner's reliability-weight fit</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>The app reads BACKUPS_ROOT (api/routes/metrics.py, docker-compose.yml) while the backup jobs read BACKUP_ROOT (pipeline/backup/data_stores.py, pipeline/backup/offsite.py, db/backup/pg_backup.sh). Both default to /backups, so the age gauges work today; a value set under one name alone splits them. Both env templates set LIVE_PIPELINE_ENABLED=true, which makes the app a second publisher beside the live service. .env.production.example sets ODDS_PROVIDER=theoddsapi, which no provider registers. The templates also carry seven keys no app code reads: WORKERS, SIM_MAX_WORKERS, ODDS_PROVIDER_API_KEY, ODDS_API_BASE, ASYNC_DB_DSN, MLB_API_BASE and PROMETHEUS_PUSHGATEWAY. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>make calibrate fits a reliability weight per feature group: how well the group repeats from one season to the next. The fit pairs two season rows of one player. The batter and baserunner calibrators pass no seasons to that fit (similarity/calibration/fitting.py:237-240 and 272-275). So each player's pair is the player's first two rows in the table's stored order, whatever their seasons. Their reads have no ORDER BY (similarity/calibration/batter.py:57-77, baserunner.py:50-66). Each profile build stores the rows in a new order. So two calibrations of the same data write other reliability weights to /data/calibration.json. Only the API's similarity engines read these values today (the /api/similarity routes and the Similarity Explorer page). The nightly score matrices apply no calibration report. A decision is open on which calibration values the draws use (SIM-587). If that decision applies the report to the matrix build, this ticket moves to P2 and lands before that change. Found by the arsenal row-order work (SIM-580, 2026-10-26); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>One variable names the backup root, and the templates hold only keys the code reads, with values that start the stack.</t>
+          <t>The batter's and the runner's reliability weights pair consecutive seasons of one player. Two calibrations from the same profiles give the same weights. A unit test pins a player whose rows are stored 2023, 2025, 2024.</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Rename the app's variable to BACKUP_ROOT. Rewrite the two templates from .env.example.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="219.5" customHeight="1" s="15">
+          <t>Pass seasons= to calibrate_reliability_weights in both calibrators, as the fielder's calibrator does. Pass each seasons array through the same mask as its rows (phys_mask, plat_mask, agg_measured). Rewrite the docstring at fitting.py:237-240.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="190.5" customHeight="1" s="15">
       <c r="A36" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1618,31 +1618,31 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>SIM-637</t>
+          <t>SIM-638</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Pair consecutive seasons in the batter's and the runner's reliability-weight fit</t>
+          <t>Order the calibrators' profile reads, so the fitted bandwidths stay the same between profile builds</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>make calibrate fits a reliability weight per feature group: how well the group repeats from one season to the next. The fit pairs two season rows of one player. The batter and baserunner calibrators pass no seasons to that fit (similarity/calibration/fitting.py:237-240 and 272-275). So each player's pair is the player's first two rows in the table's stored order, whatever their seasons. Their reads have no ORDER BY (similarity/calibration/batter.py:57-77, baserunner.py:50-66). Each profile build stores the rows in a new order. So two calibrations of the same data write other reliability weights to /data/calibration.json. Only the API's similarity engines read these values today (the /api/similarity routes and the Similarity Explorer page). The nightly score matrices apply no calibration report. A decision is open on which calibration values the draws use (SIM-587). If that decision applies the report to the matrix build, this ticket moves to P2 and lands before that change. Found by the arsenal row-order work (SIM-580, 2026-10-26); the evidence is in its CHANGES.md entry.</t>
+          <t>make calibrate fits each kernel bandwidth (sigma: how fast a similarity score falls as two profiles grow apart). The fit (calibrate_sigma) takes the median distance over up to 50,000 pairs of rows (similarity/calibration/fitting.py:78-91). A seeded generator draws the pairs by row INDEX. Seven calibrators read their profile table with no ORDER BY: the batter, baserunner, runner-steal, catcher, manager, pitcher and pitcher-steal calibrators. Only the fielder's reads are ordered (similarity/calibration/fielder.py:103 and 131). Each profile build stores the rows in a new order. So the same indices pick other players, and the fitted bandwidths move by sampling noise. Only the API's similarity engines read the bandwidths today. This ticket moves to P2 if the decision on calibration values (SIM-587) applies the report to the matrix build. Found by the arsenal row-order work (SIM-580, 2026-10-26); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>The batter's and the runner's reliability weights pair consecutive seasons of one player. Two calibrations from the same profiles give the same weights. A unit test pins a player whose rows are stored 2023, 2025, 2024.</t>
+          <t>Two calibrations from the same profiles give the same bandwidths, whatever the stored row order. A unit test reverses a profile table's stored order and gets the same bandwidth.</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Pass seasons= to calibrate_reliability_weights in both calibrators, as the fielder's calibrator does. Pass each seasons array through the same mask as its rows (phys_mask, plat_mask, agg_measured). Rewrite the docstring at fitting.py:237-240.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="190.5" customHeight="1" s="15">
+          <t>Add ORDER BY each table's key to the seven reads (for example pitcher_id, season for the pitcher).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="104" customHeight="1" s="15">
       <c r="A37" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1650,31 +1650,31 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>SIM-638</t>
+          <t>SIM-629</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Order the calibrators' profile reads, so the fitted bandwidths stay the same between profile builds</t>
+          <t>End a tied game at the inning limit without an extra pitch</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>make calibrate fits each kernel bandwidth (sigma: how fast a similarity score falls as two profiles grow apart). The fit (calibrate_sigma) takes the median distance over up to 50,000 pairs of rows (similarity/calibration/fitting.py:78-91). A seeded generator draws the pairs by row INDEX. Seven calibrators read their profile table with no ORDER BY: the batter, baserunner, runner-steal, catcher, manager, pitcher and pitcher-steal calibrators. Only the fielder's reads are ordered (similarity/calibration/fielder.py:103 and 131). Each profile build stores the rows in a new order. So the same indices pick other players, and the fitted bandwidths move by sampling noise. Only the API's similarity engines read the bandwidths today. This ticket moves to P2 if the decision on calibration values (SIM-587) applies the report to the matrix build. Found by the arsenal row-order work (SIM-580, 2026-10-26); the evidence is in its CHANGES.md entry.</t>
+          <t>simulate_game (simulation/sim_loop.py) checks state.inning &gt; max_innings only after a pitch that does not roll the half, and _game_over_after_half knows nothing of the limit. So a game tied after the API's 12 innings (max_innings 12 in simulation/sim_kwargs.py) starts the 13th, places the extra-innings runner on second and throws one pitch before it stops. That pitch can score a run or credit a box line. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Two calibrations from the same profiles give the same bandwidths, whatever the stored row order. A unit test reverses a profile table's stored order and gets the same bandwidth.</t>
+          <t>A game tied at the limit ends when the last allowed half completes, and a unit test pins it.</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Add ORDER BY each table's key to the seven reads (for example pitcher_id, season for the pitcher).</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="104" customHeight="1" s="15">
+          <t>Check the limit in the roll branch, right after _game_over_after_half.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="60" customHeight="1" s="15">
       <c r="A38" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1682,31 +1682,31 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>SIM-629</t>
+          <t>SIM-594</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>End a tied game at the inning limit without an extra pitch</t>
+          <t>Let the batter run on a called third strike that gets away</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>simulate_game (simulation/sim_loop.py) checks state.inning &gt; max_innings only after a pitch that does not roll the half, and _game_over_after_half knows nothing of the limit. So a game tied after the API's 12 innings (max_innings 12 in simulation/sim_kwargs.py) starts the 13th, places the extra-innings runner on second and throws one pitch before it stops. That pitch can score a run or credit a box line. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>Rule 5.05(a)(2) lets the batter run on any uncaught third strike. _dropped_third_strike reads swinging strikes only. Two such rows exist in 2023-2026, both in 2026. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>A game tied at the limit ends when the last allowed half completes, and a unit test pins it.</t>
+          <t>A called third strike that gets away can be a dropped-third-strike reach.</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Check the limit in the roll branch, right after _game_over_after_half.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="60" customHeight="1" s="15">
+          <t>Let _dropped_third_strike read a called third strike too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="73.5" customHeight="1" s="15">
       <c r="A39" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1714,27 +1714,27 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>SIM-594</t>
+          <t>SIM-591</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Let the batter run on a called third strike that gets away</t>
+          <t>Charge the losing pitcher with the go-ahead run, as MLB does</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Rule 5.05(a)(2) lets the batter run on any uncaught third strike. _dropped_third_strike reads swinging strikes only. Two such rows exist in 2023-2026, both in 2026. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>pitcher_decisions charges the pitcher on the mound at the decisive play. In a tie, A walks a batter, B relieves him and allows a double that scores the runner, and the lead holds: MLB charges A; the simulator charges B. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>A called third strike that gets away can be a dropped-third-strike reach.</t>
+          <t>The decision follows the runner's responsible pitcher, and a unit test plays the example.</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Let _dropped_third_strike read a called third strike too.</t>
+          <t>Carry each runner's responsible pitcher on the bases.</t>
         </is>
       </c>
     </row>
@@ -1746,27 +1746,27 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>SIM-591</t>
+          <t>SIM-592</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Charge the losing pitcher with the go-ahead run, as MLB does</t>
+          <t>Put the batter on first after a forced reach with no batter id</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>pitcher_decisions charges the pitcher on the mound at the decisive play. In a tie, A walks a batter, B relieves him and allows a double that scores the runner, and the lead holds: MLB charges A; the simulator charges B. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>_force_on_reach with no batter id leaves first base's runner on first after pushing him to second (b.first = state.batter_id if ... else b.first), so the base check raises; _resolve_walk assigns b.first = state.batter_id for the same case. Reachable only with a sampler and no lineup. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>The decision follows the runner's responsible pitcher, and a unit test plays the example.</t>
+          <t>The forced reach and the walk give the same bases.</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Carry each runner's responsible pitcher on the bases.</t>
+          <t>Use the walk's assignment.</t>
         </is>
       </c>
     </row>
@@ -1778,31 +1778,31 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>SIM-592</t>
+          <t>SIM-593</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Put the batter on first after a forced reach with no batter id</t>
+          <t>Void the plate appearance after a third out on the bases in the single pre-pitch steal draw</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>_force_on_reach with no batter id leaves first base's runner on first after pushing him to second (b.first = state.batter_id if ... else b.first), so the base check raises; _resolve_walk assigns b.first = state.batter_id for the same case. Reachable only with a sampler and no lineup. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>With SIM_STEAL_PITCH_CLASS=0 (not production), a pickoff or a caught stealing that makes the third out before the pitch's result still ends the plate appearance, so the pitcher gets a batter faced and the batter an at-bat. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>The forced reach and the walk give the same bases.</t>
+          <t>The single draw voids the plate appearance as the running game on the pitch does.</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Use the walk's assignment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="73.5" customHeight="1" s="15">
+          <t>Apply the no-pitch void of the class-aware draw.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="46.5" customHeight="1" s="15">
       <c r="A42" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1810,31 +1810,31 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>SIM-593</t>
+          <t>SIM-588</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Void the plate appearance after a third out on the bases in the single pre-pitch steal draw</t>
+          <t>Compute the z of the requested level in GameSimSummary.from_results</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>With SIM_STEAL_PITCH_CLASS=0 (not production), a pickoff or a caught stealing that makes the third out before the pitch's result still ends the plate appearance, so the pitcher gets a batter faced and the batter an at-bat. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>GameSimSummary.from_results(confidence_level=0.85) computes the 95% z and labels the intervals 0.85. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>The single draw voids the plate appearance as the running game on the pitch does.</t>
+          <t>Each level gets its own z, and a unit test checks 0.85.</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Apply the no-pitch void of the class-aware draw.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="46.5" customHeight="1" s="15">
+          <t>Use NormalDist().inv_cdf((1 + level) / 2), or raise on a level outside the table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="73.5" customHeight="1" s="15">
       <c r="A43" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1842,31 +1842,31 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>SIM-588</t>
+          <t>SIM-605</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Compute the z of the requested level in GameSimSummary.from_results</t>
+          <t>Keep one pitcher engine's calibration from rewriting every pitcher engine</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>GameSimSummary.from_results(confidence_level=0.85) computes the 95% z and labels the intervals 0.85. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>PitcherSimilarityEngine.apply_calibration sets the module global ARSENAL_SCALE, and a report with no gamma resets it to 4.10. The API builds two instances. Latent: no production path calls it today. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>Each level gets its own z, and a unit test checks 0.85.</t>
+          <t>Each instance carries its own scale.</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Use NormalDist().inv_cdf((1 + level) / 2), or raise on a level outside the table.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="73.5" customHeight="1" s="15">
+          <t>Pass the instance's scale into the three readers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="90" customHeight="1" s="15">
       <c r="A44" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1874,31 +1874,31 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>SIM-605</t>
+          <t>SIM-628</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Keep one pitcher engine's calibration from rewriting every pitcher engine</t>
+          <t>Let the resumable sweep read the database address</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>PitcherSimilarityEngine.apply_calibration sets the module global ARSENAL_SCALE, and a report with no gamma resets it to 4.10. The API builds two instances. Latent: no production path calls it today. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The child process of scripts/resumable_sweep.py reads BASEBALL_DB_DSN from .env with env["BASEBALL_DB_DSN"]. Since the security hardening (SIM-443b), .env carries no such key: .env.example has it commented out, and the live .env has none. So a sweep stops with KeyError before its first game. This is separate from the retry after a crash (SIM-614). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>Each instance carries its own scale.</t>
+          <t>A sweep starts on the current .env.</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Pass the instance's scale into the three readers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="90" customHeight="1" s="15">
+          <t>Read BASEBALL_DB_DSN from the process environment first (pipeline.db_dsn.require_dsn); read .env only when the key is set there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="73.5" customHeight="1" s="15">
       <c r="A45" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1906,31 +1906,31 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>SIM-628</t>
+          <t>SIM-614</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Let the resumable sweep read the database address</t>
+          <t>Retry a sweep attempt that crashes before its first game</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>The child process of scripts/resumable_sweep.py reads BASEBALL_DB_DSN from .env with env["BASEBALL_DB_DSN"]. Since the security hardening (SIM-443b), .env carries no such key: .env.example has it commented out, and the live .env has none. So a sweep stops with KeyError before its first game. This is separate from the retry after a crash (SIM-614). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/resumable_sweep.py applies its zero-progress stop (gained == 0) after a crash too, so a segfault before the first game of an attempt ends the sweep (exit 1) instead of retrying. Found by reading the code; not exercised. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>A sweep starts on the current .env.</t>
+          <t>A crashed attempt with no gain retries up to --max-attempts.</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Read BASEBALL_DB_DSN from the process environment first (pipeline.db_dsn.require_dsn); read .env only when the key is set there.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="73.5" customHeight="1" s="15">
+          <t>Apply the stop only to an attempt that exited cleanly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="87" customHeight="1" s="15">
       <c r="A46" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -1938,27 +1938,27 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>SIM-614</t>
+          <t>SIM-613</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Retry a sweep attempt that crashes before its first game</t>
+          <t>Print n/a in the hypothetical-return table when no bet qualifies</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>scripts/resumable_sweep.py applies its zero-progress stop (gained == 0) after a crash too, so a segfault before the first game of an attempt ends the sweep (exit 1) instead of retrying. Found by reading the code; not exercised. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/accuracy/hypothetical_return.py _fmt_row formats the means and the range with :.4f and no guard for None. With no qualifying bet the table raises TypeError, and run() prints it before it writes the report and before the zero-games check, so the run ends in a traceback with no report and no exit code 5. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>A crashed attempt with no gain retries up to --max-attempts.</t>
+          <t>The table prints n/a, as the accuracy table does.</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Apply the stop only to an attempt that exited cleanly.</t>
+          <t>Use the _fmt_or_na guard.</t>
         </is>
       </c>
     </row>
@@ -1970,31 +1970,31 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>SIM-613</t>
+          <t>SIM-616</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Print n/a in the hypothetical-return table when no bet qualifies</t>
+          <t>Decide the minimum-sample read's two known limits</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>scripts/accuracy/hypothetical_return.py _fmt_row formats the means and the range with :.4f and no guard for None. With no qualifying bet the table raises TypeError, and run() prints it before it writes the report and before the zero-games check, so the run ends in a traceback with no report and no exit code 5. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/accuracy/confidence.py: the 0.02 floor assumes a coin-flip market, so its power is weaker than stated for a market far from 0.5 (a home-run prop); and a small sample whose observed spread is exactly zero reads as fully resolved. An adversarial review of the minimum-sample work (SIM-539) found both. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>The table prints n/a, as the accuracy table does.</t>
+          <t>The owner decides whether to fix or accept them.</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Use the _fmt_or_na guard.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="87" customHeight="1" s="15">
+          <t>A per-market 4p(1-p) correction and an upper bound on the spread.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="73.5" customHeight="1" s="15">
       <c r="A48" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2002,31 +2002,31 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>SIM-616</t>
+          <t>SIM-589</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Decide the minimum-sample read's two known limits</t>
+          <t>Treat both samples as samples in the replay chi-squared test</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>scripts/accuracy/confidence.py: the 0.02 floor assumes a coin-flip market, so its power is weaker than stated for a market far from 0.5 (a home-run prop); and a small sample whose observed spread is exactly zero reads as fully resolved. An adversarial review of the minimum-sample work (SIM-539) found both. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The two-sample path of replay_chi_squared.chi_squared_gof treats the reference sample as exact. Two independent samples of 1,000 Poisson(4.4) totals were rejected 52.5% of the time at alpha 0.05 over 400 trials. replay_and_test uses it. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>The owner decides whether to fix or accept them.</t>
+          <t>Two samples from one distribution are rejected near alpha.</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>A per-market 4p(1-p) correction and an upper bound on the spread.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="73.5" customHeight="1" s="15">
+          <t>Use scipy.stats.chi2_contingency on the pooled 2 x k table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="60" customHeight="1" s="15">
       <c r="A49" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2034,27 +2034,27 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>SIM-589</t>
+          <t>SIM-590</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Treat both samples as samples in the replay chi-squared test</t>
+          <t>Compare the historical replay against the right side's score</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>The two-sample path of replay_chi_squared.chi_squared_gof treats the reference sample as exact. Two independent samples of 1,000 Poisson(4.4) totals were rejected 52.5% of the time at alpha 0.05 over 400 trials. replay_and_test uses it. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>replay_historical_games always compares the simulated HOME score. A HistoricalGame row does not say which side its runs belong to, so an away team's runs meet the simulated home runs. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Two samples from one distribution are rejected near alpha.</t>
+          <t>A HistoricalGame row names its side, and the replay compares like with like.</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Use scipy.stats.chi2_contingency on the pooled 2 x k table.</t>
+          <t>Add a side field to HistoricalGame.</t>
         </is>
       </c>
     </row>
@@ -2066,31 +2066,31 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>SIM-590</t>
+          <t>SIM-618</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Compare the historical replay against the right side's score</t>
+          <t>Keep one copy of the prop ground-truth readers</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>replay_historical_games always compares the simulated HOME score. A HistoricalGame row does not say which side its runs belong to, so an away team's runs meet the simulated home runs. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/validate_props.py and scripts/accuracy/grading.py each define _fetch_official_boxscore and _fetch_pa_events. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>A HistoricalGame row names its side, and the replay compares like with like.</t>
+          <t>One reader, imported by both.</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Add a side field to HistoricalGame.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="60" customHeight="1" s="15">
+          <t>Move it to simulation/prop_validation.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="73.5" customHeight="1" s="15">
       <c r="A51" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2098,31 +2098,31 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>SIM-618</t>
+          <t>SIM-621</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Keep one copy of the prop ground-truth readers</t>
+          <t>Bench the per-pitch call the loop makes</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>scripts/validate_props.py and scripts/accuracy/grading.py each define _fetch_official_boxscore and _fetch_pa_events. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>tests/performance/bench_simulation.py times PitcherSimilarityEngine.query() as the per-pitch cost; the loop reads the dense pitcher matrix. bench_api_simulate.py says an authoritative gate runs on target hardware with the DB-backed factory; no job does. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>One reader, imported by both.</t>
+          <t>The benches time what the loop runs, and the SLA text names the job that gates it.</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>Move it to simulation/prop_validation.py.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="73.5" customHeight="1" s="15">
+          <t>Bench the matrix read; correct the SLA text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="60" customHeight="1" s="15">
       <c r="A52" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2130,31 +2130,31 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>SIM-621</t>
+          <t>SIM-612</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Bench the per-pitch call the loop makes</t>
+          <t>Read the pitch rebuild's before-smoke from results/</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>tests/performance/bench_simulation.py times PitcherSimilarityEngine.query() as the per-pitch cost; the loop reads the dense pitcher matrix. bench_api_simulate.py says an authoritative gate runs on target hardware with the DB-backed factory; no job does. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/pitch_pool_rebuild/export.py _smoke_games opens scripts/sim553_smoke_before.json; the groundwork moved run outputs to results/sim553/. The function always prints its placeholder. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>The benches time what the loop runs, and the SLA text names the job that gates it.</t>
+          <t>It reads the results/ path.</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>Bench the matrix read; correct the SLA text.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="60" customHeight="1" s="15">
+          <t>Change the one path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="73.5" customHeight="1" s="15">
       <c r="A53" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2162,31 +2162,31 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>SIM-612</t>
+          <t>SIM-623</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Read the pitch rebuild's before-smoke from results/</t>
+          <t>Replace the inning-grid test's pinned scores with an outcome check</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>scripts/pitch_pool_rebuild/export.py _smoke_games opens scripts/sim553_smoke_before.json; the groundwork moved run outputs to results/sim553/. The function always prints its placeholder. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>tests/unit/test_inning_grid.py pins the exact scores and pitch counts of ten seeds (OUTCOMES_AT_80E3F46). That works like the golden snapshots the owner ruled out on 2026-09-10: any intended change to the draw fails it. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>It reads the results/ path.</t>
+          <t>The test checks a property of the grid (its sum equals the final score, the halves match the outs), not ten remembered numbers.</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Change the one path.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="73.5" customHeight="1" s="15">
+          <t>Rewrite the assertions as invariants and delete the pinned table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="87" customHeight="1" s="15">
       <c r="A54" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2194,31 +2194,31 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>SIM-623</t>
+          <t>SIM-620</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Replace the inning-grid test's pinned scores with an outcome check</t>
+          <t>Delete the regression gate's dead constants and its golden-file texts</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>tests/unit/test_inning_grid.py pins the exact scores and pitch counts of ten seeds (OUTCOMES_AT_80E3F46). That works like the golden snapshots the owner ruled out on 2026-09-10: any intended change to the draw fails it. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>tests/regression/regression_config.py: only SYMMETRY_TOLERANCE has a reader; eight constants have none (the conftest hard-codes the seed 2026), and one constant's docstring still speaks of golden files. The assert message at test_engine_regression.py:322 names golden files the gate does not have. The pyproject.toml marker text, the ci.yml header and make help were corrected by the documentation rebuild (SIM-624, 2026-10-21). Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>The test checks a property of the grid (its sum equals the final score, the halves match the outs), not ten remembered numbers.</t>
+          <t>The dead constants go, and the assert message says what the gate checks.</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>Rewrite the assertions as invariants and delete the pinned table.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="87" customHeight="1" s="15">
+          <t>Delete the dead constants and edit the assert message.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="60" customHeight="1" s="15">
       <c r="A55" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2226,31 +2226,31 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>SIM-620</t>
+          <t>SIM-622</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Delete the regression gate's dead constants and its golden-file texts</t>
+          <t>Use the pinned park factor in the sim-kwargs tests</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>tests/regression/regression_config.py: only SYMMETRY_TOLERANCE has a reader; eight constants have none (the conftest hard-codes the seed 2026), and one constant's docstring still speaks of golden files. The assert message at test_engine_regression.py:322 names golden files the gate does not have. The pyproject.toml marker text, the ci.yml header and make help were corrected by the documentation rebuild (SIM-624, 2026-10-21). Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>tests/unit/test_sim_kwargs.py uses 0.8723846078 for venue 680 in six places; the pinned 2024 table in the same file holds 0.8725842237. The tests pass (the literal is only an input). Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>The dead constants go, and the assert message says what the gate checks.</t>
+          <t>One value.</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>Delete the dead constants and edit the assert message.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="60" customHeight="1" s="15">
+          <t>Read it from the table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="87" customHeight="1" s="15">
       <c r="A56" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2258,31 +2258,31 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>SIM-622</t>
+          <t>SIM-597</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Use the pinned park factor in the sim-kwargs tests</t>
+          <t>Write the pitching-change pool's role file in a fixed row order</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>tests/unit/test_sim_kwargs.py uses 0.8723846078 for venue 680 in six places; the pinned 2024 table in the same file holds 0.8725842237. The tests pass (the literal is only an input). Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>roles.parquet (build_pitching_change_pool, pipeline/batch/artifacts/manager_pool.py) is written from a GROUP BY with no ORDER BY, so two builds of the same code from the same data write its rows in a different order. No reader uses the order, but the fingerprint's bundle mode reads a difference on every build. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>One value.</t>
+          <t>Two builds give the same file, by content.</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>Read it from the table.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="87" customHeight="1" s="15">
+          <t>Add ORDER BY pitcher_id, season. It changes no game.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="118" customHeight="1" s="15">
       <c r="A57" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2290,31 +2290,31 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>SIM-597</t>
+          <t>SIM-631</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Write the pitching-change pool's role file in a fixed row order</t>
+          <t>Delete or wire up the data nobody reads</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>roles.parquet (build_pitching_change_pool, pipeline/batch/artifacts/manager_pool.py) is written from a GROUP BY with no ORDER BY, so two builds of the same code from the same data write its rows in a different order. No reader uses the order, but the fingerprint's bundle mode reads a difference on every build. Found by the code clean-up (SIM-493, B2 pipeline, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>Built and never read: sim.stolen_base_pool (the profile computor builds it every night), the composite catcher actor matrix (built and concentration-checked; the draws read catcher_throwing), the sim.live_games view and raw.savant_first_base_receiving. Declared and never written: derived.outfield_play_detail, derived.infield_play_detail and derived.dp_play_detail. Never called: sim.purge_expired_sessions(), and EngineArtifacts.attach_shared_views outside the tests. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>Two builds give the same file, by content.</t>
+          <t>Each item has a reader, or it is deleted with its builder and its DDL.</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>Add ORDER BY pitcher_id, season. It changes no game.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="118" customHeight="1" s="15">
+          <t>Delete them, with a migration for the DDL. Keep any the owner wants for planned work, and name the ticket that will read it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="73.5" customHeight="1" s="15">
       <c r="A58" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2322,31 +2322,31 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>SIM-631</t>
+          <t>SIM-615</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Delete or wire up the data nobody reads</t>
+          <t>Retire the odds-hash backfill probe</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Built and never read: sim.stolen_base_pool (the profile computor builds it every night), the composite catcher actor matrix (built and concentration-checked; the draws read catcher_throwing), the sim.live_games view and raw.savant_first_base_receiving. Declared and never written: derived.outfield_play_detail, derived.infield_play_detail and derived.dp_play_detail. Never called: sim.purge_expired_sessions(), and EngineArtifacts.attach_shared_views outside the tests. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>scripts/probes/backfill_odds_hash.py _dedup_rows orders by received_at, a column raw.game_odds does not have, so its DELETE fails; its ODDS_COLUMNS leaves out draw_ml. Both are dormant: the unique index and the NOT NULL hash of migration 0012 ended the probe's job. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>Each item has a reader, or it is deleted with its builder and its DDL.</t>
+          <t>The probe is retired.</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>Delete them, with a migration for the DDL. Keep any the owner wants for planned work, and name the ticket that will read it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="73.5" customHeight="1" s="15">
+          <t>Delete the probe and its test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="90" customHeight="1" s="15">
       <c r="A59" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2354,31 +2354,31 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>SIM-615</t>
+          <t>SIM-627</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Retire the odds-hash backfill probe</t>
+          <t>Retire the two odds routes that serve mock lines</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>scripts/probes/backfill_odds_hash.py _dedup_rows orders by received_at, a column raw.game_odds does not have, so its DELETE fails; its ODDS_COLUMNS leaves out draw_ml. Both are dormant: the unique index and the NOT NULL hash of migration 0012 ended the probe's job. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>GET /api/odds/{game_pk} and GET /api/odds/today/all (pipeline/live/ingestion/odds_routes.py, mounted by api/main.py) always return MockOddsAPI lines, whatever ODDS_PROVIDER says. The rows carry is_mock: true, and no frontend code calls the routes. A client that ignores the flag reads fake prices as real ones. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>The probe is retired.</t>
+          <t>The routes are gone (or serve the stored book rows), and the API snapshot is regenerated.</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Delete the probe and its test.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="90" customHeight="1" s="15">
+          <t>Delete both routes, then run scripts/export_openapi.py in the app image and npm run gen:api (CLAUDE.md section 15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="181.5" customHeight="1" s="15">
       <c r="A60" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2386,31 +2386,31 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>SIM-627</t>
+          <t>SIM-617</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Retire the two odds routes that serve mock lines</t>
+          <t>Correct the runtime texts that state something false</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>GET /api/odds/{game_pk} and GET /api/odds/today/all (pipeline/live/ingestion/odds_routes.py, mounted by api/main.py) always return MockOddsAPI lines, whatever ODDS_PROVIDER says. The rows carry is_mock: true, and no frontend code calls the routes. A client that ignores the flag reads fake prices as real ones. Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>Left unedited by the clean-up's rule. (1) The park-guard messages name the deleted SIM_PARK_FACTOR: scripts/validate_props.py, scripts/accuracy_comparison.py, tests/acceptance/conftest.py and the --help of scripts/sim_stats.py. (2) The two pool rebuilds' exit-3 texts and the steal rebuild's lock message blame the app's worker server for the DuckDB lock (the app holds no handle since SIM-524), and two steal-rebuild texts say to merge code that is merged. (3) scripts/running_game_replay.py --help says a steal can land on any pitch in production. (4) Three texts point at a module docstring section that moved in the split. (5) scripts/measure_filter_cells.py writes into docs/audit/. (6) scripts/resumable_sweep.py --help cites a deleted record. (7) The rationale strings in tests/acceptance/bands.py cite BACKLOG.md, which is gone. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>The routes are gone (or serve the stored book rows), and the API snapshot is regenerated.</t>
+          <t>Each text says what is true.</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>Delete both routes, then run scripts/export_openapi.py in the app image and npm run gen:api (CLAUDE.md section 15).</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="181.5" customHeight="1" s="15">
+          <t>One edit per text; list the runtime-string changes in CHANGES.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="154.5" customHeight="1" s="15">
       <c r="A61" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2418,31 +2418,31 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>SIM-617</t>
+          <t>SIM-610</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Correct the runtime texts that state something false</t>
+          <t>Similarity and betting: seven small defects</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Left unedited by the clean-up's rule. (1) The park-guard messages name the deleted SIM_PARK_FACTOR: scripts/validate_props.py, scripts/accuracy_comparison.py, tests/acceptance/conftest.py and the --help of scripts/sim_stats.py. (2) The two pool rebuilds' exit-3 texts and the steal rebuild's lock message blame the app's worker server for the DuckDB lock (the app holds no handle since SIM-524), and two steal-rebuild texts say to merge code that is merged. (3) scripts/running_game_replay.py --help says a steal can land on any pitch in production. (4) Three texts point at a module docstring section that moved in the split. (5) scripts/measure_filter_cells.py writes into docs/audit/. (6) scripts/resumable_sweep.py --help cites a deleted record. (7) The rationale strings in tests/acceptance/bands.py cite BACKLOG.md, which is gone. Found by the code clean-up (SIM-493, B5 scripts and test harness, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>(1) SituationSimilarityEngine.query_batch([]) raises instead of returning []. (2) The engines' and the calibrator's __main__ blocks read a DuckDB path that does not exist (../../db/schemas/baseball_simulator.duckdb); the pitcher engine's block builds and prints nothing. (3) CalibrationReport.summary() prints no row for the batter's physical weights. (4) The Similarity Explorer's batter panel (api/routes/similarity_explorer.py) shows the four-way weights 0.40/0.35/0.15/0.10. (5) A log line in batted_ball_similarity.py says 'until SIM-051 ships'. (6) tests/regression/conftest.py scales the situation fixture's index twice. (7) No writer sets is_sharp_book, so sharp_consensus is always None. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>Each text says what is true.</t>
+          <t>Each of the seven is fixed or retired.</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>One edit per text; list the runtime-string changes in CHANGES.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="154.5" customHeight="1" s="15">
+          <t>One edit each; retire sharp_consensus if no book will be marked sharp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="100.5" customHeight="1" s="15">
       <c r="A62" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2450,27 +2450,27 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>SIM-610</t>
+          <t>SIM-603</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Similarity and betting: seven small defects</t>
+          <t>Return the fielder's infield sub-scores in the same order from query_pair as from query</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>(1) SituationSimilarityEngine.query_batch([]) raises instead of returning []. (2) The engines' and the calibrator's __main__ blocks read a DuckDB path that does not exist (../../db/schemas/baseball_simulator.duckdb); the pitcher engine's block builds and prints nothing. (3) CalibrationReport.summary() prints no row for the batter's physical weights. (4) The Similarity Explorer's batter panel (api/routes/similarity_explorer.py) shows the four-way weights 0.40/0.35/0.15/0.10. (5) A log line in batted_ball_similarity.py says 'until SIM-051 ships'. (6) tests/regression/conftest.py scales the situation fixture's index twice. (7) No writer sets is_sharp_book, so sharp_consensus is always None. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>For an infielder, similarity/engines/fielder_similarity.py query_pair returns the specialty score in tertiary_score and the error score in quaternary_score; query returns them the other way round, as the Similarity Explorer's labels expect. Two shortstops with different error rates and equal specialty values: query gives 0.0710 / 1.0000, query_pair 1.0000 / 0.0710. The composite and the matrices are right. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>Each of the seven is fixed or retired.</t>
+          <t>query and query_pair agree on every sub-score, and a unit test compares them.</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>One edit each; retire sharp_consensus if no book will be marked sharp.</t>
+          <t>Map the infield tuple in SimilarityResult order.</t>
         </is>
       </c>
     </row>
@@ -2482,31 +2482,31 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>SIM-603</t>
+          <t>SIM-604</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Return the fielder's infield sub-scores in the same order from query_pair as from query</t>
+          <t>Apply the per-hand 30-PA platoon rule in the batter engine's pair score</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>For an infielder, similarity/engines/fielder_similarity.py query_pair returns the specialty score in tertiary_score and the error score in quaternary_score; query returns them the other way round, as the Similarity Explorer's labels expect. Two shortstops with different error rates and equal specialty values: query gives 0.0710 / 1.0000, query_pair 1.0000 / 0.0710. The composite and the matrices are right. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>similarity/engines/batter_similarity.py _score_pair disagrees with score_all on a thin platoon split. A query with 30+ PA against either hand turns the platoon weights on for any vs_hand (10 PA vs L and 200 vs R with vs_hand='L': 0.8642 against 0.8900), and a candidate under 30 PA never gets the neutral 0.5. It serves query_pair (the Explorer's pair view and the diagnostics); the matrix is unaffected. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>query and query_pair agree on every sub-score, and a unit test compares them.</t>
+          <t>_score_pair and score_all agree, and a unit test compares them.</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>Map the infield tuple in SimilarityResult order.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="100.5" customHeight="1" s="15">
+          <t>Use score_all's per-hand rule in _score_pair.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="60" customHeight="1" s="15">
       <c r="A64" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2514,27 +2514,27 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>SIM-604</t>
+          <t>SIM-596</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Apply the per-hand 30-PA platoon rule in the batter engine's pair score</t>
+          <t>Decide what the what-if does when the designated hitter takes the field</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>similarity/engines/batter_similarity.py _score_pair disagrees with score_all on a thin platoon split. A query with 30+ PA against either hand turns the platoon weights on for any vs_hand (10 PA vs L and 200 vs R with vs_hand='L': 0.8642 against 0.8900), and a candidate under 30 PA never gets the neutral 0.5. It serves query_pair (the Explorer's pair view and the diagnostics); the matrix is unaffected. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>A designated hitter moved to the field leaves the fielder he replaced in the batting order with no position. The rule that ends the designated hitter is not modelled in simulation/whatif.py. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>_score_pair and score_all agree, and a unit test compares them.</t>
+          <t>The owner decides whether the what-if models the rule, and the code follows.</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>Use score_all's per-hand rule in _score_pair.</t>
+          <t>Model the rule: the pitcher bats in the replaced fielder's slot, or refuse the change.</t>
         </is>
       </c>
     </row>
@@ -2546,31 +2546,31 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>SIM-596</t>
+          <t>SIM-598</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Decide what the what-if does when the designated hitter takes the field</t>
+          <t>Read the runners under the names the live service sends</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>A designated hitter moved to the field leaves the fielder he replaced in the batting order with no position. The rule that ends the designated hitter is not modelled in simulation/whatif.py. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>frontend/src/hooks/useGameSocket.ts reads runner_on_first / _second / _third; the live service sends on_1b / on_2b / on_3b. The hook's on_1b to on_3b are always undefined. No page reads them today. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>The owner decides whether the what-if models the rule, and the code follows.</t>
+          <t>A game_state_update with runners fills the hook's on_1b to on_3b.</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>Model the rule: the pitcher bats in the replaced fielder's slot, or refuse the change.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="60" customHeight="1" s="15">
+          <t>Read gs.on_1b, gs.on_2b and gs.on_3b in mapWsState.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="46.5" customHeight="1" s="15">
       <c r="A66" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2578,31 +2578,31 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>SIM-598</t>
+          <t>SIM-609</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Read the runners under the names the live service sends</t>
+          <t>Raise on a wrong market or side in the line-movement series</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/hooks/useGameSocket.ts reads runner_on_first / _second / _third; the live service sends on_1b / on_2b / on_3b. The hook's on_1b to on_3b are always undefined. No page reads them today. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>line_movement_from_quotes swallows _side_columns' ValueError, so a wrong market or side gives a silent empty series. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>A game_state_update with runners fills the hook's on_1b to on_3b.</t>
+          <t>A wrong market or side raises.</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>Read gs.on_1b, gs.on_2b and gs.on_3b in mapWsState.</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="46.5" customHeight="1" s="15">
+          <t>Call _side_columns once before the loop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="73.5" customHeight="1" s="15">
       <c r="A67" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2610,31 +2610,31 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>SIM-609</t>
+          <t>SIM-599</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Raise on a wrong market or side in the line-movement series</t>
+          <t>Describe the slate card's odds field as it is</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>line_movement_from_quotes swallows _side_columns' ValueError, so a wrong market or side gives a silent empty series. Found by the code clean-up (SIM-493, B4 similarity and betting, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>The route description (api/routes/games_slate.py) and the model (api/routes/games_models.py) call the field 'reserved for the Phase-6 odds-provider integration (SIM-405)'. The field is always None: the card's lines come from /api/betting/games/{pk}/card-odds. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>A wrong market or side raises.</t>
+          <t>Both texts say that, with a fresh API snapshot (CLAUDE.md section 15).</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>Call _side_columns once before the loop.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="73.5" customHeight="1" s="15">
+          <t>Rewrite both texts; run scripts/export_openapi.py in the image and npm run gen:api.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="46.5" customHeight="1" s="15">
       <c r="A68" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2642,31 +2642,31 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>SIM-599</t>
+          <t>SIM-600</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Describe the slate card's odds field as it is</t>
+          <t>Name the current state in the API's version and health strings</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>The route description (api/routes/games_slate.py) and the model (api/routes/games_models.py) call the field 'reserved for the Phase-6 odds-provider integration (SIM-405)'. The field is always None: the card's lines come from /api/betting/games/{pk}/card-odds. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>api/main.py carries the app version 0.1.0-phase7, "phase": "6" on /health and "6 - Frontend Build (in progress)" on /. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t>Both texts say that, with a fresh API snapshot (CLAUDE.md section 15).</t>
+          <t>The strings name the current state, or go.</t>
         </is>
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>Rewrite both texts; run scripts/export_openapi.py in the image and npm run gen:api.</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="46.5" customHeight="1" s="15">
+          <t>Drop the phase keys and set the version from one constant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="202" customHeight="1" s="15">
       <c r="A69" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2674,31 +2674,31 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>SIM-600</t>
+          <t>SIM-634</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>Name the current state in the API's version and health strings</t>
+          <t>Small fixes found by the documentation rebuild</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>api/main.py carries the app version 0.1.0-phase7, "phase": "6" on /health and "6 - Frontend Build (in progress)" on /. Found by the code clean-up (SIM-493, B3 API and frontend, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
+          <t>(1) frontend/index.html links a favicon, /baseball.svg, that frontend/public/ does not hold: a 404 on every page. (2) /ready (api/main.py) writes a redis entry only on a failure, so a healthy Redis is missing from its checks. (3) Six nginx blocks (/health, /ready, /metrics, /docs, /redoc, /openapi.json) set their own Host header, which drops the inherited X-Real-IP and X-Forwarded-For. (4) Nothing deletes the simviz:* explorer cache keys after a nightly rebuild, so a key serves old data for up to 24 h. (5) 12 of the 32 DuckDB migrations do not record themselves in migration_history. (6) Three stale texts: api/state.py calls the situation engine a FAISS engine (it is a KD-tree); the Makefile's gen-secrets comment says a blank key is left alone (gen_secrets.py fills it); scripts/probes/manager_profile_recompute.py says the app must be stopped (the recompute runs beside the app since SIM-524). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>The strings name the current state, or go.</t>
+          <t>Each of the six is fixed or retired.</t>
         </is>
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>Drop the phase keys and set the version from one constant.</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="202" customHeight="1" s="15">
+          <t>One small commit per area. For (5), record the missing numbers in one new migration rather than editing old files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="46.5" customHeight="1" s="15">
       <c r="A70" s="6" t="inlineStr">
         <is>
           <t>P3</t>
@@ -2706,91 +2706,60 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>SIM-634</t>
+          <t>SIM-595</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Small fixes found by the documentation rebuild</t>
+          <t>Fix the article in the what-if's ineligible-player message</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>(1) frontend/index.html links a favicon, /baseball.svg, that frontend/public/ does not hold: a 404 on every page. (2) /ready (api/main.py) writes a redis entry only on a failure, so a healthy Redis is missing from its checks. (3) Six nginx blocks (/health, /ready, /metrics, /docs, /redoc, /openapi.json) set their own Host header, which drops the inherited X-Real-IP and X-Forwarded-For. (4) Nothing deletes the simviz:* explorer cache keys after a nightly rebuild, so a key serves old data for up to 24 h. (5) 12 of the 32 DuckDB migrations do not record themselves in migration_history. (6) Three stale texts: api/state.py calls the situation engine a FAISS engine (it is a KD-tree); the Makefile's gen-secrets comment says a blank key is left alone (gen_secrets.py fills it); scripts/probes/manager_profile_recompute.py says the app must be stopped (the recompute runs beside the app since SIM-524). Found by the documentation rebuild (SIM-624, 2026-10-21); the evidence is in its CHANGES.md entry.</t>
+          <t>whatif.apply_changes' message for an ineligible pinch hitter reads 'is not an bench hitter'. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>Each of the six is fixed or retired.</t>
+          <t>Each label reads with its own article.</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>One small commit per area. For (5), record the missing numbers in one new migration rather than editing old files.</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="46.5" customHeight="1" s="15">
-      <c r="A71" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B71" s="3" t="inlineStr">
-        <is>
-          <t>SIM-595</t>
-        </is>
-      </c>
-      <c r="C71" s="4" t="inlineStr">
-        <is>
-          <t>Fix the article in the what-if's ineligible-player message</t>
-        </is>
-      </c>
-      <c r="D71" s="5" t="inlineStr">
-        <is>
-          <t>whatif.apply_changes' message for an ineligible pinch hitter reads 'is not an bench hitter'. Found by the code clean-up (SIM-493, B1 simulation, 2026-10-20); the evidence is in its CHANGES.md entry.</t>
-        </is>
-      </c>
-      <c r="E71" s="5" t="inlineStr">
-        <is>
-          <t>Each label reads with its own article.</t>
-        </is>
-      </c>
-      <c r="F71" s="5" t="inlineStr">
-        <is>
           <t>Put the article inside each label.</t>
         </is>
       </c>
     </row>
-    <row r="72" s="15"/>
-    <row r="73" s="15">
-      <c r="A73" s="7" t="inlineStr">
+    <row r="71" s="15"/>
+    <row r="72" s="15">
+      <c r="A72" s="7" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B73" s="8" t="inlineStr">
+      <c r="B72" s="8" t="inlineStr">
         <is>
           <t>P0 — immediate</t>
         </is>
       </c>
-      <c r="C73" s="9" t="inlineStr">
+      <c r="C72" s="9" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D73" s="12" t="inlineStr">
+      <c r="D72" s="12" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E73" s="10" t="inlineStr">
+      <c r="E72" s="10" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F73" s="11" t="n"/>
-    </row>
+      <c r="F72" s="11" t="n"/>
+    </row>
+    <row r="73" s="15"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>